<commit_message>
Record 2 August: 999 sends across both surfaces
App 586 sends, web and mobile web 413. Both files verified before loading:
every channel column of the pivot matches the SUM row it was given with, and
every row agrees with its own Total.

The absent Sl. no. values in the app log are the failed sends, which are not
exported - so the log is 586 successes out of ids 1..615, not a log with 29
rows missing. The earlier caveat about "22 rows never seen" on 1 August was
wrong for the same reason and is dropped.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9KsXegBwxB1sWdCzRVLrr
</commit_message>
<xml_diff>
--- a/reports/daily_tracking.xlsx
+++ b/reports/daily_tracking.xlsx
@@ -224,7 +224,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -247,7 +247,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
     </row>
@@ -339,28 +339,56 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B3" s="2">
+        <v>999</v>
+      </c>
+      <c r="C3" s="2">
+        <v>586</v>
+      </c>
+      <c r="D3" s="2">
+        <v>413</v>
+      </c>
+      <c r="E3" s="2">
+        <v>958</v>
+      </c>
+      <c r="F3" s="2">
+        <v>41</v>
+      </c>
+      <c r="G3" s="2">
+        <v>321</v>
+      </c>
+      <c r="H3" s="2">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B3" s="5">
-        <v>1059</v>
-      </c>
-      <c r="C3" s="5">
-        <v>591</v>
-      </c>
-      <c r="D3" s="5">
-        <v>468</v>
-      </c>
-      <c r="E3" s="5">
-        <v>1018</v>
-      </c>
-      <c r="F3" s="5">
-        <v>41</v>
-      </c>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
+      <c r="B4" s="5">
+        <v>2058</v>
+      </c>
+      <c r="C4" s="5">
+        <v>1177</v>
+      </c>
+      <c r="D4" s="5">
+        <v>881</v>
+      </c>
+      <c r="E4" s="5">
+        <v>1976</v>
+      </c>
+      <c r="F4" s="5">
+        <v>82</v>
+      </c>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -375,18 +403,18 @@
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
     <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="17" customWidth="1"/>
-    <col min="11" max="11" width="24" customWidth="1"/>
-    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="11" max="11" width="17" customWidth="1"/>
+    <col min="12" max="12" width="17" customWidth="1"/>
     <col min="13" max="13" width="11" customWidth="1"/>
-    <col min="14" max="14" width="21" customWidth="1"/>
-    <col min="15" max="15" width="11" customWidth="1"/>
-    <col min="16" max="16" width="17" customWidth="1"/>
-    <col min="17" max="17" width="17" customWidth="1"/>
-    <col min="18" max="18" width="11" customWidth="1"/>
+    <col min="14" max="14" width="18" customWidth="1"/>
+    <col min="15" max="15" width="21" customWidth="1"/>
+    <col min="16" max="16" width="11" customWidth="1"/>
+    <col min="17" max="17" width="11" customWidth="1"/>
+    <col min="18" max="18" width="17" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -422,14 +450,14 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Everyday greetings</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Friendship</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Love &amp; romance</t>
@@ -437,47 +465,47 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Congratulations</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Inspirational &amp; sympathy</t>
-        </is>
-      </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Keeping in touch</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Cute</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Family &amp; loved ones</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Pets</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Business &amp; work</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>World languages</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Flowers</t>
         </is>
       </c>
     </row>
@@ -512,89 +540,147 @@
         <v>19</v>
       </c>
       <c r="J2" s="2">
+        <v>10</v>
+      </c>
+      <c r="K2" s="2">
         <v>12</v>
       </c>
-      <c r="K2" s="2">
-        <v>10</v>
-      </c>
       <c r="L2" s="2">
+        <v>2</v>
+      </c>
+      <c r="M2" s="2">
+        <v>1</v>
+      </c>
+      <c r="N2" s="2">
         <v>6</v>
-      </c>
-      <c r="M2" s="2">
-        <v>4</v>
-      </c>
-      <c r="N2" s="2">
-        <v>3</v>
       </c>
       <c r="O2" s="2">
         <v>3</v>
       </c>
       <c r="P2" s="2">
+        <v>4</v>
+      </c>
+      <c r="Q2" s="2">
+        <v>3</v>
+      </c>
+      <c r="R2" s="2">
         <v>2</v>
       </c>
-      <c r="Q2" s="2">
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B3" s="2">
+        <v>958</v>
+      </c>
+      <c r="C3" s="2">
+        <v>544</v>
+      </c>
+      <c r="D3" s="2">
+        <v>167</v>
+      </c>
+      <c r="E3" s="2">
+        <v>35</v>
+      </c>
+      <c r="F3" s="2">
+        <v>52</v>
+      </c>
+      <c r="G3" s="2">
+        <v>41</v>
+      </c>
+      <c r="H3" s="2">
+        <v>40</v>
+      </c>
+      <c r="I3" s="2">
+        <v>24</v>
+      </c>
+      <c r="J3" s="2">
+        <v>19</v>
+      </c>
+      <c r="K3" s="2">
+        <v>11</v>
+      </c>
+      <c r="L3" s="2">
+        <v>10</v>
+      </c>
+      <c r="M3" s="2">
+        <v>8</v>
+      </c>
+      <c r="N3" s="2">
         <v>2</v>
       </c>
-      <c r="R2" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="O3" s="2">
+        <v>3</v>
+      </c>
+      <c r="P3" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>1</v>
+      </c>
+      <c r="R3" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B3" s="5">
-        <v>1018</v>
-      </c>
-      <c r="C3" s="5">
-        <v>572</v>
-      </c>
-      <c r="D3" s="5">
-        <v>241</v>
-      </c>
-      <c r="E3" s="5">
-        <v>57</v>
-      </c>
-      <c r="F3" s="5">
-        <v>30</v>
-      </c>
-      <c r="G3" s="5">
-        <v>28</v>
-      </c>
-      <c r="H3" s="5">
-        <v>28</v>
-      </c>
-      <c r="I3" s="5">
-        <v>19</v>
-      </c>
-      <c r="J3" s="5">
+      <c r="B4" s="5">
+        <v>1976</v>
+      </c>
+      <c r="C4" s="5">
+        <v>1116</v>
+      </c>
+      <c r="D4" s="5">
+        <v>408</v>
+      </c>
+      <c r="E4" s="5">
+        <v>92</v>
+      </c>
+      <c r="F4" s="5">
+        <v>82</v>
+      </c>
+      <c r="G4" s="5">
+        <v>69</v>
+      </c>
+      <c r="H4" s="5">
+        <v>68</v>
+      </c>
+      <c r="I4" s="5">
+        <v>43</v>
+      </c>
+      <c r="J4" s="5">
+        <v>29</v>
+      </c>
+      <c r="K4" s="5">
+        <v>23</v>
+      </c>
+      <c r="L4" s="5">
         <v>12</v>
       </c>
-      <c r="K3" s="5">
-        <v>10</v>
-      </c>
-      <c r="L3" s="5">
+      <c r="M4" s="5">
+        <v>9</v>
+      </c>
+      <c r="N4" s="5">
+        <v>8</v>
+      </c>
+      <c r="O4" s="5">
         <v>6</v>
       </c>
-      <c r="M3" s="5">
+      <c r="P4" s="5">
+        <v>5</v>
+      </c>
+      <c r="Q4" s="5">
         <v>4</v>
       </c>
-      <c r="N3" s="5">
-        <v>3</v>
-      </c>
-      <c r="O3" s="5">
-        <v>3</v>
-      </c>
-      <c r="P3" s="5">
+      <c r="R4" s="5">
         <v>2</v>
-      </c>
-      <c r="Q3" s="5">
-        <v>2</v>
-      </c>
-      <c r="R3" s="5">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1190,6 +1276,508 @@
       </c>
       <c r="H18" s="4"/>
     </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>birth</t>
+        </is>
+      </c>
+      <c r="D19" s="2">
+        <v>343</v>
+      </c>
+      <c r="E19" s="2">
+        <v>201</v>
+      </c>
+      <c r="F19" s="2">
+        <v>544</v>
+      </c>
+      <c r="G19" s="3">
+        <v>0.5678496868475992</v>
+      </c>
+      <c r="H19" s="2">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="D20" s="2">
+        <v>106</v>
+      </c>
+      <c r="E20" s="2">
+        <v>61</v>
+      </c>
+      <c r="F20" s="2">
+        <v>167</v>
+      </c>
+      <c r="G20" s="3">
+        <v>0.174321503131524</v>
+      </c>
+      <c r="H20" s="2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>thank</t>
+        </is>
+      </c>
+      <c r="D21" s="2">
+        <v>21</v>
+      </c>
+      <c r="E21" s="2">
+        <v>31</v>
+      </c>
+      <c r="F21" s="2">
+        <v>52</v>
+      </c>
+      <c r="G21" s="3">
+        <v>0.054279749478079335</v>
+      </c>
+      <c r="H21" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>friend</t>
+        </is>
+      </c>
+      <c r="D22" s="2">
+        <v>9</v>
+      </c>
+      <c r="E22" s="2">
+        <v>32</v>
+      </c>
+      <c r="F22" s="2">
+        <v>41</v>
+      </c>
+      <c r="G22" s="3">
+        <v>0.04279749478079332</v>
+      </c>
+      <c r="H22" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>gen</t>
+        </is>
+      </c>
+      <c r="D23" s="2">
+        <v>33</v>
+      </c>
+      <c r="E23" s="2">
+        <v>7</v>
+      </c>
+      <c r="F23" s="2">
+        <v>40</v>
+      </c>
+      <c r="G23" s="3">
+        <v>0.04175365344467641</v>
+      </c>
+      <c r="H23" s="2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>anniv</t>
+        </is>
+      </c>
+      <c r="D24" s="2">
+        <v>19</v>
+      </c>
+      <c r="E24" s="2">
+        <v>16</v>
+      </c>
+      <c r="F24" s="2">
+        <v>35</v>
+      </c>
+      <c r="G24" s="3">
+        <v>0.03653444676409186</v>
+      </c>
+      <c r="H24" s="2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D25" s="2">
+        <v>18</v>
+      </c>
+      <c r="E25" s="2">
+        <v>6</v>
+      </c>
+      <c r="F25" s="2">
+        <v>24</v>
+      </c>
+      <c r="G25" s="3">
+        <v>0.025052192066805846</v>
+      </c>
+      <c r="H25" s="2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>insp</t>
+        </is>
+      </c>
+      <c r="D26" s="2">
+        <v>12</v>
+      </c>
+      <c r="E26" s="2">
+        <v>7</v>
+      </c>
+      <c r="F26" s="2">
+        <v>19</v>
+      </c>
+      <c r="G26" s="3">
+        <v>0.019832985386221295</v>
+      </c>
+      <c r="H26" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>congrats</t>
+        </is>
+      </c>
+      <c r="D27" s="2">
+        <v>5</v>
+      </c>
+      <c r="E27" s="2">
+        <v>6</v>
+      </c>
+      <c r="F27" s="2">
+        <v>11</v>
+      </c>
+      <c r="G27" s="3">
+        <v>0.011482254697286013</v>
+      </c>
+      <c r="H27" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="D28" s="2">
+        <v>8</v>
+      </c>
+      <c r="E28" s="2">
+        <v>2</v>
+      </c>
+      <c r="F28" s="2">
+        <v>10</v>
+      </c>
+      <c r="G28" s="3">
+        <v>0.010438413361169102</v>
+      </c>
+      <c r="H28" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>flwr</t>
+        </is>
+      </c>
+      <c r="D29" s="2">
+        <v>7</v>
+      </c>
+      <c r="E29" s="2">
+        <v>1</v>
+      </c>
+      <c r="F29" s="2">
+        <v>8</v>
+      </c>
+      <c r="G29" s="3">
+        <v>0.008350730688935281</v>
+      </c>
+      <c r="H29" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>fkt</t>
+        </is>
+      </c>
+      <c r="D30" s="2">
+        <v>1</v>
+      </c>
+      <c r="E30" s="2">
+        <v>2</v>
+      </c>
+      <c r="F30" s="2">
+        <v>3</v>
+      </c>
+      <c r="G30" s="3">
+        <v>0.003131524008350731</v>
+      </c>
+      <c r="H30" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>intouch</t>
+        </is>
+      </c>
+      <c r="D31" s="2">
+        <v>2</v>
+      </c>
+      <c r="E31" s="2">
+        <v>0</v>
+      </c>
+      <c r="F31" s="2">
+        <v>2</v>
+      </c>
+      <c r="G31" s="3">
+        <v>0.0020876826722338203</v>
+      </c>
+      <c r="H31" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>cute</t>
+        </is>
+      </c>
+      <c r="D32" s="2">
+        <v>1</v>
+      </c>
+      <c r="E32" s="2">
+        <v>0</v>
+      </c>
+      <c r="F32" s="2">
+        <v>1</v>
+      </c>
+      <c r="G32" s="3">
+        <v>0.0010438413361169101</v>
+      </c>
+      <c r="H32" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="D33" s="2">
+        <v>1</v>
+      </c>
+      <c r="E33" s="2">
+        <v>0</v>
+      </c>
+      <c r="F33" s="2">
+        <v>1</v>
+      </c>
+      <c r="G33" s="3">
+        <v>0.0010438413361169101</v>
+      </c>
+      <c r="H33" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-02</t>
+        </is>
+      </c>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="5">
+        <v>586</v>
+      </c>
+      <c r="E34" s="5">
+        <v>372</v>
+      </c>
+      <c r="F34" s="5">
+        <v>958</v>
+      </c>
+      <c r="G34" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="H34" s="4"/>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -3799,6 +4387,2904 @@
       </c>
       <c r="F93" s="4"/>
     </row>
+    <row r="94">
+      <c r="A94" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B94" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C94" s="0" t="inlineStr">
+        <is>
+          <t>happybirthday</t>
+        </is>
+      </c>
+      <c r="D94" s="0" t="inlineStr">
+        <is>
+          <t>birth_happybirthday</t>
+        </is>
+      </c>
+      <c r="E94" s="2">
+        <v>432</v>
+      </c>
+      <c r="F94" s="2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B95" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C95" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_happy</t>
+        </is>
+      </c>
+      <c r="D95" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_happy</t>
+        </is>
+      </c>
+      <c r="E95" s="2">
+        <v>69</v>
+      </c>
+      <c r="F95" s="2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B96" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C96" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="D96" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="E96" s="2">
+        <v>23</v>
+      </c>
+      <c r="F96" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B97" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C97" s="0" t="inlineStr">
+        <is>
+          <t>bestfriends</t>
+        </is>
+      </c>
+      <c r="D97" s="0" t="inlineStr">
+        <is>
+          <t>friend_bestfriends</t>
+        </is>
+      </c>
+      <c r="E97" s="2">
+        <v>23</v>
+      </c>
+      <c r="F97" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B98" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C98" s="0" t="inlineStr">
+        <is>
+          <t>birthday</t>
+        </is>
+      </c>
+      <c r="D98" s="0" t="inlineStr">
+        <is>
+          <t>thank_birthday</t>
+        </is>
+      </c>
+      <c r="E98" s="2">
+        <v>19</v>
+      </c>
+      <c r="F98" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B99" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C99" s="0" t="inlineStr">
+        <is>
+          <t>belated</t>
+        </is>
+      </c>
+      <c r="D99" s="0" t="inlineStr">
+        <is>
+          <t>birth_belated</t>
+        </is>
+      </c>
+      <c r="E99" s="2">
+        <v>17</v>
+      </c>
+      <c r="F99" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B100" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C100" s="0" t="inlineStr">
+        <is>
+          <t>morning</t>
+        </is>
+      </c>
+      <c r="D100" s="0" t="inlineStr">
+        <is>
+          <t>gen_morning</t>
+        </is>
+      </c>
+      <c r="E100" s="2">
+        <v>17</v>
+      </c>
+      <c r="F100" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B101" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C101" s="0" t="inlineStr">
+        <is>
+          <t>anniversaryetc</t>
+        </is>
+      </c>
+      <c r="D101" s="0" t="inlineStr">
+        <is>
+          <t>anniv_anniversaryetc</t>
+        </is>
+      </c>
+      <c r="E101" s="2">
+        <v>15</v>
+      </c>
+      <c r="F101" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B102" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C102" s="0" t="inlineStr">
+        <is>
+          <t>fun</t>
+        </is>
+      </c>
+      <c r="D102" s="0" t="inlineStr">
+        <is>
+          <t>birth_fun</t>
+        </is>
+      </c>
+      <c r="E102" s="2">
+        <v>12</v>
+      </c>
+      <c r="F102" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B103" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C103" s="0" t="inlineStr">
+        <is>
+          <t>sonanddaughter</t>
+        </is>
+      </c>
+      <c r="D103" s="0" t="inlineStr">
+        <is>
+          <t>birth_sonanddaughter</t>
+        </is>
+      </c>
+      <c r="E103" s="2">
+        <v>12</v>
+      </c>
+      <c r="F103" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B104" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C104" s="0" t="inlineStr">
+        <is>
+          <t>songs</t>
+        </is>
+      </c>
+      <c r="D104" s="0" t="inlineStr">
+        <is>
+          <t>birth_songs</t>
+        </is>
+      </c>
+      <c r="E104" s="2">
+        <v>12</v>
+      </c>
+      <c r="F104" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B105" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C105" s="0" t="inlineStr">
+        <is>
+          <t>eaug_cardssister</t>
+        </is>
+      </c>
+      <c r="D105" s="0" t="inlineStr">
+        <is>
+          <t>eaug_cardssister</t>
+        </is>
+      </c>
+      <c r="E105" s="2">
+        <v>12</v>
+      </c>
+      <c r="F105" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B106" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C106" s="0" t="inlineStr">
+        <is>
+          <t>sympathy</t>
+        </is>
+      </c>
+      <c r="D106" s="0" t="inlineStr">
+        <is>
+          <t>insp_sympathy</t>
+        </is>
+      </c>
+      <c r="E106" s="2">
+        <v>12</v>
+      </c>
+      <c r="F106" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B107" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C107" s="0" t="inlineStr">
+        <is>
+          <t>inspirational</t>
+        </is>
+      </c>
+      <c r="D107" s="0" t="inlineStr">
+        <is>
+          <t>thank_inspirational</t>
+        </is>
+      </c>
+      <c r="E107" s="2">
+        <v>12</v>
+      </c>
+      <c r="F107" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B108" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C108" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="D108" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="E108" s="2">
+        <v>10</v>
+      </c>
+      <c r="F108" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B109" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C109" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_thanku</t>
+        </is>
+      </c>
+      <c r="D109" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_thanku</t>
+        </is>
+      </c>
+      <c r="E109" s="2">
+        <v>10</v>
+      </c>
+      <c r="F109" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B110" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C110" s="0" t="inlineStr">
+        <is>
+          <t>eaug_girlfriendsday</t>
+        </is>
+      </c>
+      <c r="D110" s="0" t="inlineStr">
+        <is>
+          <t>eaug_girlfriendsday</t>
+        </is>
+      </c>
+      <c r="E110" s="2">
+        <v>10</v>
+      </c>
+      <c r="F110" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B111" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C111" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D111" s="0" t="inlineStr">
+        <is>
+          <t>gen_getwell</t>
+        </is>
+      </c>
+      <c r="E111" s="2">
+        <v>10</v>
+      </c>
+      <c r="F111" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B112" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C112" s="0" t="inlineStr">
+        <is>
+          <t>everyday</t>
+        </is>
+      </c>
+      <c r="D112" s="0" t="inlineStr">
+        <is>
+          <t>thank_everyday</t>
+        </is>
+      </c>
+      <c r="E112" s="2">
+        <v>10</v>
+      </c>
+      <c r="F112" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B113" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C113" s="0" t="inlineStr">
+        <is>
+          <t>flowers</t>
+        </is>
+      </c>
+      <c r="D113" s="0" t="inlineStr">
+        <is>
+          <t>birth_flowers</t>
+        </is>
+      </c>
+      <c r="E113" s="2">
+        <v>8</v>
+      </c>
+      <c r="F113" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B114" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C114" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D114" s="0" t="inlineStr">
+        <is>
+          <t>birth_milestone</t>
+        </is>
+      </c>
+      <c r="E114" s="2">
+        <v>8</v>
+      </c>
+      <c r="F114" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B115" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C115" s="0" t="inlineStr">
+        <is>
+          <t>wishes</t>
+        </is>
+      </c>
+      <c r="D115" s="0" t="inlineStr">
+        <is>
+          <t>birth_wishes</t>
+        </is>
+      </c>
+      <c r="E115" s="2">
+        <v>8</v>
+      </c>
+      <c r="F115" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B116" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C116" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="D116" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="E116" s="2">
+        <v>8</v>
+      </c>
+      <c r="F116" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B117" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C117" s="0" t="inlineStr">
+        <is>
+          <t>extfamily</t>
+        </is>
+      </c>
+      <c r="D117" s="0" t="inlineStr">
+        <is>
+          <t>birth_extfamily</t>
+        </is>
+      </c>
+      <c r="E117" s="2">
+        <v>7</v>
+      </c>
+      <c r="F117" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B118" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C118" s="0" t="inlineStr">
+        <is>
+          <t>friendsforever</t>
+        </is>
+      </c>
+      <c r="D118" s="0" t="inlineStr">
+        <is>
+          <t>friend_friendsforever</t>
+        </is>
+      </c>
+      <c r="E118" s="2">
+        <v>7</v>
+      </c>
+      <c r="F118" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B119" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C119" s="0" t="inlineStr">
+        <is>
+          <t>thinkingofyou</t>
+        </is>
+      </c>
+      <c r="D119" s="0" t="inlineStr">
+        <is>
+          <t>gen_thinkingofyou</t>
+        </is>
+      </c>
+      <c r="E119" s="2">
+        <v>7</v>
+      </c>
+      <c r="F119" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B120" s="0" t="inlineStr">
+        <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="C120" s="0" t="inlineStr">
+        <is>
+          <t>hindi_indian</t>
+        </is>
+      </c>
+      <c r="D120" s="0" t="inlineStr">
+        <is>
+          <t>w_hindi_indian</t>
+        </is>
+      </c>
+      <c r="E120" s="2">
+        <v>7</v>
+      </c>
+      <c r="F120" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B121" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C121" s="0" t="inlineStr">
+        <is>
+          <t>friends</t>
+        </is>
+      </c>
+      <c r="D121" s="0" t="inlineStr">
+        <is>
+          <t>birth_friends</t>
+        </is>
+      </c>
+      <c r="E121" s="2">
+        <v>6</v>
+      </c>
+      <c r="F121" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B122" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C122" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_heart</t>
+        </is>
+      </c>
+      <c r="D122" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_heart</t>
+        </is>
+      </c>
+      <c r="E122" s="2">
+        <v>6</v>
+      </c>
+      <c r="F122" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B123" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C123" s="0" t="inlineStr">
+        <is>
+          <t>flrwishes</t>
+        </is>
+      </c>
+      <c r="D123" s="0" t="inlineStr">
+        <is>
+          <t>flwr_flrwishes</t>
+        </is>
+      </c>
+      <c r="E123" s="2">
+        <v>6</v>
+      </c>
+      <c r="F123" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B124" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C124" s="0" t="inlineStr">
+        <is>
+          <t>friendship</t>
+        </is>
+      </c>
+      <c r="D124" s="0" t="inlineStr">
+        <is>
+          <t>thank_friendship</t>
+        </is>
+      </c>
+      <c r="E124" s="2">
+        <v>6</v>
+      </c>
+      <c r="F124" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B125" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C125" s="0" t="inlineStr">
+        <is>
+          <t>bronsis</t>
+        </is>
+      </c>
+      <c r="D125" s="0" t="inlineStr">
+        <is>
+          <t>birth_bronsis</t>
+        </is>
+      </c>
+      <c r="E125" s="2">
+        <v>5</v>
+      </c>
+      <c r="F125" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B126" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C126" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipweek</t>
+        </is>
+      </c>
+      <c r="D126" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipweek</t>
+        </is>
+      </c>
+      <c r="E126" s="2">
+        <v>5</v>
+      </c>
+      <c r="F126" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B127" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C127" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_general</t>
+        </is>
+      </c>
+      <c r="D127" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_general</t>
+        </is>
+      </c>
+      <c r="E127" s="2">
+        <v>5</v>
+      </c>
+      <c r="F127" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B128" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C128" s="0" t="inlineStr">
+        <is>
+          <t>momndad</t>
+        </is>
+      </c>
+      <c r="D128" s="0" t="inlineStr">
+        <is>
+          <t>birth_momndad</t>
+        </is>
+      </c>
+      <c r="E128" s="2">
+        <v>4</v>
+      </c>
+      <c r="F128" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B129" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C129" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_more</t>
+        </is>
+      </c>
+      <c r="D129" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_more</t>
+        </is>
+      </c>
+      <c r="E129" s="2">
+        <v>4</v>
+      </c>
+      <c r="F129" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B130" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C130" s="0" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="D130" s="0" t="inlineStr">
+        <is>
+          <t>insp_health</t>
+        </is>
+      </c>
+      <c r="E130" s="2">
+        <v>4</v>
+      </c>
+      <c r="F130" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B131" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C131" s="0" t="inlineStr">
+        <is>
+          <t>belated</t>
+        </is>
+      </c>
+      <c r="D131" s="0" t="inlineStr">
+        <is>
+          <t>anniv_belated</t>
+        </is>
+      </c>
+      <c r="E131" s="2">
+        <v>3</v>
+      </c>
+      <c r="F131" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B132" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C132" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_family</t>
+        </is>
+      </c>
+      <c r="D132" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_family</t>
+        </is>
+      </c>
+      <c r="E132" s="2">
+        <v>3</v>
+      </c>
+      <c r="F132" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B133" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C133" s="0" t="inlineStr">
+        <is>
+          <t>blessings</t>
+        </is>
+      </c>
+      <c r="D133" s="0" t="inlineStr">
+        <is>
+          <t>birth_blessings</t>
+        </is>
+      </c>
+      <c r="E133" s="2">
+        <v>3</v>
+      </c>
+      <c r="F133" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B134" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C134" s="0" t="inlineStr">
+        <is>
+          <t>forher</t>
+        </is>
+      </c>
+      <c r="D134" s="0" t="inlineStr">
+        <is>
+          <t>birth_forher</t>
+        </is>
+      </c>
+      <c r="E134" s="2">
+        <v>3</v>
+      </c>
+      <c r="F134" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B135" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C135" s="0" t="inlineStr">
+        <is>
+          <t>foreveryone</t>
+        </is>
+      </c>
+      <c r="D135" s="0" t="inlineStr">
+        <is>
+          <t>congrats_foreveryone</t>
+        </is>
+      </c>
+      <c r="E135" s="2">
+        <v>3</v>
+      </c>
+      <c r="F135" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B136" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C136" s="0" t="inlineStr">
+        <is>
+          <t>onotheroccasions</t>
+        </is>
+      </c>
+      <c r="D136" s="0" t="inlineStr">
+        <is>
+          <t>congrats_onotheroccasions</t>
+        </is>
+      </c>
+      <c r="E136" s="2">
+        <v>3</v>
+      </c>
+      <c r="F136" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B137" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C137" s="0" t="inlineStr">
+        <is>
+          <t>retirement</t>
+        </is>
+      </c>
+      <c r="D137" s="0" t="inlineStr">
+        <is>
+          <t>congrats_retirement</t>
+        </is>
+      </c>
+      <c r="E137" s="2">
+        <v>3</v>
+      </c>
+      <c r="F137" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B138" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C138" s="0" t="inlineStr">
+        <is>
+          <t>eaug_flwrmonthaug</t>
+        </is>
+      </c>
+      <c r="D138" s="0" t="inlineStr">
+        <is>
+          <t>eaug_flwrmonthaug</t>
+        </is>
+      </c>
+      <c r="E138" s="2">
+        <v>3</v>
+      </c>
+      <c r="F138" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B139" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C139" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_flowers</t>
+        </is>
+      </c>
+      <c r="D139" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_flowers</t>
+        </is>
+      </c>
+      <c r="E139" s="2">
+        <v>3</v>
+      </c>
+      <c r="F139" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B140" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C140" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalwatermelon_day</t>
+        </is>
+      </c>
+      <c r="D140" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalwatermelon_day</t>
+        </is>
+      </c>
+      <c r="E140" s="2">
+        <v>3</v>
+      </c>
+      <c r="F140" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B141" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C141" s="0" t="inlineStr">
+        <is>
+          <t>specialfriend</t>
+        </is>
+      </c>
+      <c r="D141" s="0" t="inlineStr">
+        <is>
+          <t>friend_specialfriend</t>
+        </is>
+      </c>
+      <c r="E141" s="2">
+        <v>3</v>
+      </c>
+      <c r="F141" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B142" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C142" s="0" t="inlineStr">
+        <is>
+          <t>lovepoems</t>
+        </is>
+      </c>
+      <c r="D142" s="0" t="inlineStr">
+        <is>
+          <t>love_lovepoems</t>
+        </is>
+      </c>
+      <c r="E142" s="2">
+        <v>3</v>
+      </c>
+      <c r="F142" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B143" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C143" s="0" t="inlineStr">
+        <is>
+          <t>wed_wed_congrats</t>
+        </is>
+      </c>
+      <c r="D143" s="0" t="inlineStr">
+        <is>
+          <t>wed_wed_congrats</t>
+        </is>
+      </c>
+      <c r="E143" s="2">
+        <v>3</v>
+      </c>
+      <c r="F143" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B144" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C144" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="D144" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="E144" s="2">
+        <v>2</v>
+      </c>
+      <c r="F144" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B145" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C145" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="D145" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="E145" s="2">
+        <v>2</v>
+      </c>
+      <c r="F145" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B146" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C146" s="0" t="inlineStr">
+        <is>
+          <t>forhim</t>
+        </is>
+      </c>
+      <c r="D146" s="0" t="inlineStr">
+        <is>
+          <t>birth_forhim</t>
+        </is>
+      </c>
+      <c r="E146" s="2">
+        <v>2</v>
+      </c>
+      <c r="F146" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B147" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C147" s="0" t="inlineStr">
+        <is>
+          <t>hubbywife</t>
+        </is>
+      </c>
+      <c r="D147" s="0" t="inlineStr">
+        <is>
+          <t>birth_hubbywife</t>
+        </is>
+      </c>
+      <c r="E147" s="2">
+        <v>2</v>
+      </c>
+      <c r="F147" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B148" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C148" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_soulmates</t>
+        </is>
+      </c>
+      <c r="D148" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_soulmates</t>
+        </is>
+      </c>
+      <c r="E148" s="2">
+        <v>2</v>
+      </c>
+      <c r="F148" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B149" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C149" s="0" t="inlineStr">
+        <is>
+          <t>eaug_icecream_sandwich_day</t>
+        </is>
+      </c>
+      <c r="D149" s="0" t="inlineStr">
+        <is>
+          <t>eaug_icecream_sandwich_day</t>
+        </is>
+      </c>
+      <c r="E149" s="2">
+        <v>2</v>
+      </c>
+      <c r="F149" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B150" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C150" s="0" t="inlineStr">
+        <is>
+          <t>edec_christworldday_english</t>
+        </is>
+      </c>
+      <c r="D150" s="0" t="inlineStr">
+        <is>
+          <t>edec_christworldday_english</t>
+        </is>
+      </c>
+      <c r="E150" s="2">
+        <v>2</v>
+      </c>
+      <c r="F150" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B151" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C151" s="0" t="inlineStr">
+        <is>
+          <t>ejan_thankyoucards</t>
+        </is>
+      </c>
+      <c r="D151" s="0" t="inlineStr">
+        <is>
+          <t>ejan_thankyoucards</t>
+        </is>
+      </c>
+      <c r="E151" s="2">
+        <v>2</v>
+      </c>
+      <c r="F151" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B152" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C152" s="0" t="inlineStr">
+        <is>
+          <t>esep_nathoneymonth</t>
+        </is>
+      </c>
+      <c r="D152" s="0" t="inlineStr">
+        <is>
+          <t>esep_nathoneymonth</t>
+        </is>
+      </c>
+      <c r="E152" s="2">
+        <v>2</v>
+      </c>
+      <c r="F152" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B153" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C153" s="0" t="inlineStr">
+        <is>
+          <t>friendshipetc</t>
+        </is>
+      </c>
+      <c r="D153" s="0" t="inlineStr">
+        <is>
+          <t>friend_friendshipetc</t>
+        </is>
+      </c>
+      <c r="E153" s="2">
+        <v>2</v>
+      </c>
+      <c r="F153" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B154" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C154" s="0" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="D154" s="0" t="inlineStr">
+        <is>
+          <t>friend_hello</t>
+        </is>
+      </c>
+      <c r="E154" s="2">
+        <v>2</v>
+      </c>
+      <c r="F154" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B155" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C155" s="0" t="inlineStr">
+        <is>
+          <t>missingyou</t>
+        </is>
+      </c>
+      <c r="D155" s="0" t="inlineStr">
+        <is>
+          <t>friend_missingyou</t>
+        </is>
+      </c>
+      <c r="E155" s="2">
+        <v>2</v>
+      </c>
+      <c r="F155" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B156" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C156" s="0" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="D156" s="0" t="inlineStr">
+        <is>
+          <t>gen_luck</t>
+        </is>
+      </c>
+      <c r="E156" s="2">
+        <v>2</v>
+      </c>
+      <c r="F156" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B157" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C157" s="0" t="inlineStr">
+        <is>
+          <t>dating</t>
+        </is>
+      </c>
+      <c r="D157" s="0" t="inlineStr">
+        <is>
+          <t>love_dating</t>
+        </is>
+      </c>
+      <c r="E157" s="2">
+        <v>2</v>
+      </c>
+      <c r="F157" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B158" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C158" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="D158" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="E158" s="2">
+        <v>2</v>
+      </c>
+      <c r="F158" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B159" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C159" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_kisses</t>
+        </is>
+      </c>
+      <c r="D159" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_kisses</t>
+        </is>
+      </c>
+      <c r="E159" s="2">
+        <v>2</v>
+      </c>
+      <c r="F159" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B160" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C160" s="0" t="inlineStr">
+        <is>
+          <t>flower</t>
+        </is>
+      </c>
+      <c r="D160" s="0" t="inlineStr">
+        <is>
+          <t>thank_flower</t>
+        </is>
+      </c>
+      <c r="E160" s="2">
+        <v>2</v>
+      </c>
+      <c r="F160" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B161" s="0" t="inlineStr">
+        <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="C161" s="0" t="inlineStr">
+        <is>
+          <t>german_birthday</t>
+        </is>
+      </c>
+      <c r="D161" s="0" t="inlineStr">
+        <is>
+          <t>w_german_birthday</t>
+        </is>
+      </c>
+      <c r="E161" s="2">
+        <v>2</v>
+      </c>
+      <c r="F161" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B162" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C162" s="0" t="inlineStr">
+        <is>
+          <t>balloons</t>
+        </is>
+      </c>
+      <c r="D162" s="0" t="inlineStr">
+        <is>
+          <t>birth_balloons</t>
+        </is>
+      </c>
+      <c r="E162" s="2">
+        <v>1</v>
+      </c>
+      <c r="F162" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B163" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C163" s="0" t="inlineStr">
+        <is>
+          <t>kids</t>
+        </is>
+      </c>
+      <c r="D163" s="0" t="inlineStr">
+        <is>
+          <t>birth_kids</t>
+        </is>
+      </c>
+      <c r="E163" s="2">
+        <v>1</v>
+      </c>
+      <c r="F163" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B164" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C164" s="0" t="inlineStr">
+        <is>
+          <t>missyou</t>
+        </is>
+      </c>
+      <c r="D164" s="0" t="inlineStr">
+        <is>
+          <t>birth_missyou</t>
+        </is>
+      </c>
+      <c r="E164" s="2">
+        <v>1</v>
+      </c>
+      <c r="F164" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B165" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C165" s="0" t="inlineStr">
+        <is>
+          <t>newcarandlicense</t>
+        </is>
+      </c>
+      <c r="D165" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newcarandlicense</t>
+        </is>
+      </c>
+      <c r="E165" s="2">
+        <v>1</v>
+      </c>
+      <c r="F165" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B166" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C166" s="0" t="inlineStr">
+        <is>
+          <t>newjob</t>
+        </is>
+      </c>
+      <c r="D166" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newjob</t>
+        </is>
+      </c>
+      <c r="E166" s="2">
+        <v>1</v>
+      </c>
+      <c r="F166" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B167" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C167" s="0" t="inlineStr">
+        <is>
+          <t>kiss</t>
+        </is>
+      </c>
+      <c r="D167" s="0" t="inlineStr">
+        <is>
+          <t>cute_kiss</t>
+        </is>
+      </c>
+      <c r="E167" s="2">
+        <v>1</v>
+      </c>
+      <c r="F167" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B168" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C168" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_makesmile</t>
+        </is>
+      </c>
+      <c r="D168" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_makesmile</t>
+        </is>
+      </c>
+      <c r="E168" s="2">
+        <v>1</v>
+      </c>
+      <c r="F168" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B169" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C169" s="0" t="inlineStr">
+        <is>
+          <t>eaug_justbecauseday</t>
+        </is>
+      </c>
+      <c r="D169" s="0" t="inlineStr">
+        <is>
+          <t>eaug_justbecauseday</t>
+        </is>
+      </c>
+      <c r="E169" s="2">
+        <v>1</v>
+      </c>
+      <c r="F169" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B170" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C170" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalraspberry_cream_pie_day</t>
+        </is>
+      </c>
+      <c r="D170" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalraspberry_cream_pie_day</t>
+        </is>
+      </c>
+      <c r="E170" s="2">
+        <v>1</v>
+      </c>
+      <c r="F170" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B171" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C171" s="0" t="inlineStr">
+        <is>
+          <t>eaug_romanceday</t>
+        </is>
+      </c>
+      <c r="D171" s="0" t="inlineStr">
+        <is>
+          <t>eaug_romanceday</t>
+        </is>
+      </c>
+      <c r="E171" s="2">
+        <v>1</v>
+      </c>
+      <c r="F171" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B172" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C172" s="0" t="inlineStr">
+        <is>
+          <t>eaug_thankyouday</t>
+        </is>
+      </c>
+      <c r="D172" s="0" t="inlineStr">
+        <is>
+          <t>eaug_thankyouday</t>
+        </is>
+      </c>
+      <c r="E172" s="2">
+        <v>1</v>
+      </c>
+      <c r="F172" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B173" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C173" s="0" t="inlineStr">
+        <is>
+          <t>efeb_friendweek</t>
+        </is>
+      </c>
+      <c r="D173" s="0" t="inlineStr">
+        <is>
+          <t>efeb_friendweek</t>
+        </is>
+      </c>
+      <c r="E173" s="2">
+        <v>1</v>
+      </c>
+      <c r="F173" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B174" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C174" s="0" t="inlineStr">
+        <is>
+          <t>lovedones</t>
+        </is>
+      </c>
+      <c r="D174" s="0" t="inlineStr">
+        <is>
+          <t>fkt_lovedones</t>
+        </is>
+      </c>
+      <c r="E174" s="2">
+        <v>1</v>
+      </c>
+      <c r="F174" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B175" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C175" s="0" t="inlineStr">
+        <is>
+          <t>loveyoudad</t>
+        </is>
+      </c>
+      <c r="D175" s="0" t="inlineStr">
+        <is>
+          <t>fkt_loveyoudad</t>
+        </is>
+      </c>
+      <c r="E175" s="2">
+        <v>1</v>
+      </c>
+      <c r="F175" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B176" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C176" s="0" t="inlineStr">
+        <is>
+          <t>sisters</t>
+        </is>
+      </c>
+      <c r="D176" s="0" t="inlineStr">
+        <is>
+          <t>fkt_sisters</t>
+        </is>
+      </c>
+      <c r="E176" s="2">
+        <v>1</v>
+      </c>
+      <c r="F176" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B177" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C177" s="0" t="inlineStr">
+        <is>
+          <t>friend</t>
+        </is>
+      </c>
+      <c r="D177" s="0" t="inlineStr">
+        <is>
+          <t>flwr_friend</t>
+        </is>
+      </c>
+      <c r="E177" s="2">
+        <v>1</v>
+      </c>
+      <c r="F177" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B178" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C178" s="0" t="inlineStr">
+        <is>
+          <t>roses</t>
+        </is>
+      </c>
+      <c r="D178" s="0" t="inlineStr">
+        <is>
+          <t>flwr_roses</t>
+        </is>
+      </c>
+      <c r="E178" s="2">
+        <v>1</v>
+      </c>
+      <c r="F178" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B179" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C179" s="0" t="inlineStr">
+        <is>
+          <t>hugsncaring</t>
+        </is>
+      </c>
+      <c r="D179" s="0" t="inlineStr">
+        <is>
+          <t>friend_hugsncaring</t>
+        </is>
+      </c>
+      <c r="E179" s="2">
+        <v>1</v>
+      </c>
+      <c r="F179" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B180" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C180" s="0" t="inlineStr">
+        <is>
+          <t>smiles</t>
+        </is>
+      </c>
+      <c r="D180" s="0" t="inlineStr">
+        <is>
+          <t>friend_smiles</t>
+        </is>
+      </c>
+      <c r="E180" s="2">
+        <v>1</v>
+      </c>
+      <c r="F180" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B181" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C181" s="0" t="inlineStr">
+        <is>
+          <t>goodnight</t>
+        </is>
+      </c>
+      <c r="D181" s="0" t="inlineStr">
+        <is>
+          <t>gen_goodnight</t>
+        </is>
+      </c>
+      <c r="E181" s="2">
+        <v>1</v>
+      </c>
+      <c r="F181" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B182" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C182" s="0" t="inlineStr">
+        <is>
+          <t>sorry</t>
+        </is>
+      </c>
+      <c r="D182" s="0" t="inlineStr">
+        <is>
+          <t>gen_sorry</t>
+        </is>
+      </c>
+      <c r="E182" s="2">
+        <v>1</v>
+      </c>
+      <c r="F182" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B183" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C183" s="0" t="inlineStr">
+        <is>
+          <t>voyage</t>
+        </is>
+      </c>
+      <c r="D183" s="0" t="inlineStr">
+        <is>
+          <t>gen_voyage</t>
+        </is>
+      </c>
+      <c r="E183" s="2">
+        <v>1</v>
+      </c>
+      <c r="F183" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B184" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C184" s="0" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="D184" s="0" t="inlineStr">
+        <is>
+          <t>gen_weekend</t>
+        </is>
+      </c>
+      <c r="E184" s="2">
+        <v>1</v>
+      </c>
+      <c r="F184" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B185" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C185" s="0" t="inlineStr">
+        <is>
+          <t>encour</t>
+        </is>
+      </c>
+      <c r="D185" s="0" t="inlineStr">
+        <is>
+          <t>insp_encour</t>
+        </is>
+      </c>
+      <c r="E185" s="2">
+        <v>1</v>
+      </c>
+      <c r="F185" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B186" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C186" s="0" t="inlineStr">
+        <is>
+          <t>poetry</t>
+        </is>
+      </c>
+      <c r="D186" s="0" t="inlineStr">
+        <is>
+          <t>insp_poetry</t>
+        </is>
+      </c>
+      <c r="E186" s="2">
+        <v>1</v>
+      </c>
+      <c r="F186" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B187" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C187" s="0" t="inlineStr">
+        <is>
+          <t>recovery</t>
+        </is>
+      </c>
+      <c r="D187" s="0" t="inlineStr">
+        <is>
+          <t>insp_recovery</t>
+        </is>
+      </c>
+      <c r="E187" s="2">
+        <v>1</v>
+      </c>
+      <c r="F187" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B188" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C188" s="0" t="inlineStr">
+        <is>
+          <t>acrossthemiles</t>
+        </is>
+      </c>
+      <c r="D188" s="0" t="inlineStr">
+        <is>
+          <t>intouch_acrossthemiles</t>
+        </is>
+      </c>
+      <c r="E188" s="2">
+        <v>1</v>
+      </c>
+      <c r="F188" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B189" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C189" s="0" t="inlineStr">
+        <is>
+          <t>thinkingofyou</t>
+        </is>
+      </c>
+      <c r="D189" s="0" t="inlineStr">
+        <is>
+          <t>intouch_thinkingofyou</t>
+        </is>
+      </c>
+      <c r="E189" s="2">
+        <v>1</v>
+      </c>
+      <c r="F189" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B190" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C190" s="0" t="inlineStr">
+        <is>
+          <t>newlove</t>
+        </is>
+      </c>
+      <c r="D190" s="0" t="inlineStr">
+        <is>
+          <t>love_newlove</t>
+        </is>
+      </c>
+      <c r="E190" s="2">
+        <v>1</v>
+      </c>
+      <c r="F190" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B191" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C191" s="0" t="inlineStr">
+        <is>
+          <t>youarespecial</t>
+        </is>
+      </c>
+      <c r="D191" s="0" t="inlineStr">
+        <is>
+          <t>love_youarespecial</t>
+        </is>
+      </c>
+      <c r="E191" s="2">
+        <v>1</v>
+      </c>
+      <c r="F191" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B192" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C192" s="0" t="inlineStr">
+        <is>
+          <t>hihello</t>
+        </is>
+      </c>
+      <c r="D192" s="0" t="inlineStr">
+        <is>
+          <t>pet_hihello</t>
+        </is>
+      </c>
+      <c r="E192" s="2">
+        <v>1</v>
+      </c>
+      <c r="F192" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B193" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C193" s="0" t="inlineStr">
+        <is>
+          <t>congratulations</t>
+        </is>
+      </c>
+      <c r="D193" s="0" t="inlineStr">
+        <is>
+          <t>thank_congratulations</t>
+        </is>
+      </c>
+      <c r="E193" s="2">
+        <v>1</v>
+      </c>
+      <c r="F193" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B194" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C194" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D194" s="0" t="inlineStr">
+        <is>
+          <t>thank_love</t>
+        </is>
+      </c>
+      <c r="E194" s="2">
+        <v>1</v>
+      </c>
+      <c r="F194" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B195" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C195" s="0" t="inlineStr">
+        <is>
+          <t>wedding</t>
+        </is>
+      </c>
+      <c r="D195" s="0" t="inlineStr">
+        <is>
+          <t>thank_wedding</t>
+        </is>
+      </c>
+      <c r="E195" s="2">
+        <v>1</v>
+      </c>
+      <c r="F195" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B196" s="0" t="inlineStr">
+        <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="C196" s="0" t="inlineStr">
+        <is>
+          <t>spanish_secretariesday</t>
+        </is>
+      </c>
+      <c r="D196" s="0" t="inlineStr">
+        <is>
+          <t>w_spanish_secretariesday</t>
+        </is>
+      </c>
+      <c r="E196" s="2">
+        <v>1</v>
+      </c>
+      <c r="F196" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-02</t>
+        </is>
+      </c>
+      <c r="B197" s="4"/>
+      <c r="C197" s="4"/>
+      <c r="D197" s="4"/>
+      <c r="E197" s="5">
+        <v>958</v>
+      </c>
+      <c r="F197" s="4"/>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -3815,6 +7301,7 @@
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3863,6 +7350,11 @@
           <t>Skype</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Google_Plus_Post</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
@@ -3894,36 +7386,76 @@
       <c r="I2" s="2">
         <v>12</v>
       </c>
+      <c r="J2" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B3" s="2">
+        <v>999</v>
+      </c>
+      <c r="C3" s="2">
+        <v>355</v>
+      </c>
+      <c r="D3" s="2">
+        <v>266</v>
+      </c>
+      <c r="E3" s="2">
+        <v>174</v>
+      </c>
+      <c r="F3" s="2">
+        <v>118</v>
+      </c>
+      <c r="G3" s="2">
+        <v>38</v>
+      </c>
+      <c r="H3" s="2">
+        <v>34</v>
+      </c>
+      <c r="I3" s="2">
+        <v>13</v>
+      </c>
+      <c r="J3" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B3" s="5">
-        <v>1059</v>
-      </c>
-      <c r="C3" s="5">
-        <v>404</v>
-      </c>
-      <c r="D3" s="5">
-        <v>280</v>
-      </c>
-      <c r="E3" s="5">
-        <v>177</v>
-      </c>
-      <c r="F3" s="5">
-        <v>108</v>
-      </c>
-      <c r="G3" s="5">
-        <v>47</v>
-      </c>
-      <c r="H3" s="5">
-        <v>31</v>
-      </c>
-      <c r="I3" s="5">
-        <v>12</v>
+      <c r="B4" s="5">
+        <v>2058</v>
+      </c>
+      <c r="C4" s="5">
+        <v>759</v>
+      </c>
+      <c r="D4" s="5">
+        <v>546</v>
+      </c>
+      <c r="E4" s="5">
+        <v>351</v>
+      </c>
+      <c r="F4" s="5">
+        <v>226</v>
+      </c>
+      <c r="G4" s="5">
+        <v>85</v>
+      </c>
+      <c r="H4" s="5">
+        <v>65</v>
+      </c>
+      <c r="I4" s="5">
+        <v>25</v>
+      </c>
+      <c r="J4" s="5">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record 3 August: 765 sends, three days now tracked
App 494 sends, web and mobile web 271. The pivot's nine channel columns match
the SUM row it came with, and every row agrees with its own Total.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9KsXegBwxB1sWdCzRVLrr
</commit_message>
<xml_diff>
--- a/reports/daily_tracking.xlsx
+++ b/reports/daily_tracking.xlsx
@@ -224,7 +224,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -247,7 +247,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -367,28 +367,56 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2">
+        <v>765</v>
+      </c>
+      <c r="C4" s="2">
+        <v>494</v>
+      </c>
+      <c r="D4" s="2">
+        <v>271</v>
+      </c>
+      <c r="E4" s="2">
+        <v>726</v>
+      </c>
+      <c r="F4" s="2">
+        <v>39</v>
+      </c>
+      <c r="G4" s="2">
+        <v>256</v>
+      </c>
+      <c r="H4" s="2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B4" s="5">
-        <v>2058</v>
-      </c>
-      <c r="C4" s="5">
-        <v>1177</v>
-      </c>
-      <c r="D4" s="5">
-        <v>881</v>
-      </c>
-      <c r="E4" s="5">
-        <v>1976</v>
-      </c>
-      <c r="F4" s="5">
-        <v>82</v>
-      </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
+      <c r="B5" s="5">
+        <v>2823</v>
+      </c>
+      <c r="C5" s="5">
+        <v>1671</v>
+      </c>
+      <c r="D5" s="5">
+        <v>1152</v>
+      </c>
+      <c r="E5" s="5">
+        <v>2702</v>
+      </c>
+      <c r="F5" s="5">
+        <v>121</v>
+      </c>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -403,16 +431,16 @@
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="16" customWidth="1"/>
     <col min="10" max="10" width="24" customWidth="1"/>
     <col min="11" max="11" width="17" customWidth="1"/>
     <col min="12" max="12" width="17" customWidth="1"/>
     <col min="13" max="13" width="11" customWidth="1"/>
-    <col min="14" max="14" width="18" customWidth="1"/>
-    <col min="15" max="15" width="21" customWidth="1"/>
-    <col min="16" max="16" width="11" customWidth="1"/>
+    <col min="14" max="14" width="11" customWidth="1"/>
+    <col min="15" max="15" width="18" customWidth="1"/>
+    <col min="16" max="16" width="21" customWidth="1"/>
     <col min="17" max="17" width="11" customWidth="1"/>
     <col min="18" max="18" width="17" customWidth="1"/>
   </cols>
@@ -450,14 +478,14 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Friendship</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Everyday greetings</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Love &amp; romance</t>
@@ -480,22 +508,22 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Flowers</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Keeping in touch</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Family &amp; loved ones</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Cute</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
@@ -549,16 +577,16 @@
         <v>2</v>
       </c>
       <c r="M2" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N2" s="2">
+        <v>1</v>
+      </c>
+      <c r="O2" s="2">
         <v>6</v>
       </c>
-      <c r="O2" s="2">
+      <c r="P2" s="2">
         <v>3</v>
-      </c>
-      <c r="P2" s="2">
-        <v>4</v>
       </c>
       <c r="Q2" s="2">
         <v>3</v>
@@ -589,10 +617,10 @@
         <v>52</v>
       </c>
       <c r="G3" s="2">
+        <v>40</v>
+      </c>
+      <c r="H3" s="2">
         <v>41</v>
-      </c>
-      <c r="H3" s="2">
-        <v>40</v>
       </c>
       <c r="I3" s="2">
         <v>24</v>
@@ -607,16 +635,16 @@
         <v>10</v>
       </c>
       <c r="M3" s="2">
+        <v>1</v>
+      </c>
+      <c r="N3" s="2">
         <v>8</v>
       </c>
-      <c r="N3" s="2">
+      <c r="O3" s="2">
         <v>2</v>
       </c>
-      <c r="O3" s="2">
+      <c r="P3" s="2">
         <v>3</v>
-      </c>
-      <c r="P3" s="2">
-        <v>1</v>
       </c>
       <c r="Q3" s="2">
         <v>1</v>
@@ -626,60 +654,118 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2">
+        <v>726</v>
+      </c>
+      <c r="C4" s="2">
+        <v>491</v>
+      </c>
+      <c r="D4" s="2">
+        <v>45</v>
+      </c>
+      <c r="E4" s="2">
+        <v>57</v>
+      </c>
+      <c r="F4" s="2">
+        <v>30</v>
+      </c>
+      <c r="G4" s="2">
+        <v>36</v>
+      </c>
+      <c r="H4" s="2">
+        <v>11</v>
+      </c>
+      <c r="I4" s="2">
+        <v>18</v>
+      </c>
+      <c r="J4" s="2">
+        <v>16</v>
+      </c>
+      <c r="K4" s="2">
+        <v>17</v>
+      </c>
+      <c r="L4" s="2">
+        <v>0</v>
+      </c>
+      <c r="M4" s="2">
+        <v>5</v>
+      </c>
+      <c r="N4" s="2">
+        <v>0</v>
+      </c>
+      <c r="O4" s="2">
+        <v>0</v>
+      </c>
+      <c r="P4" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="2">
+        <v>0</v>
+      </c>
+      <c r="R4" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B4" s="5">
-        <v>1976</v>
-      </c>
-      <c r="C4" s="5">
-        <v>1116</v>
-      </c>
-      <c r="D4" s="5">
-        <v>408</v>
-      </c>
-      <c r="E4" s="5">
-        <v>92</v>
-      </c>
-      <c r="F4" s="5">
-        <v>82</v>
-      </c>
-      <c r="G4" s="5">
-        <v>69</v>
-      </c>
-      <c r="H4" s="5">
-        <v>68</v>
-      </c>
-      <c r="I4" s="5">
-        <v>43</v>
-      </c>
-      <c r="J4" s="5">
-        <v>29</v>
-      </c>
-      <c r="K4" s="5">
-        <v>23</v>
-      </c>
-      <c r="L4" s="5">
+      <c r="B5" s="5">
+        <v>2702</v>
+      </c>
+      <c r="C5" s="5">
+        <v>1607</v>
+      </c>
+      <c r="D5" s="5">
+        <v>453</v>
+      </c>
+      <c r="E5" s="5">
+        <v>149</v>
+      </c>
+      <c r="F5" s="5">
+        <v>112</v>
+      </c>
+      <c r="G5" s="5">
+        <v>104</v>
+      </c>
+      <c r="H5" s="5">
+        <v>80</v>
+      </c>
+      <c r="I5" s="5">
+        <v>61</v>
+      </c>
+      <c r="J5" s="5">
+        <v>45</v>
+      </c>
+      <c r="K5" s="5">
+        <v>40</v>
+      </c>
+      <c r="L5" s="5">
         <v>12</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M5" s="5">
+        <v>10</v>
+      </c>
+      <c r="N5" s="5">
         <v>9</v>
       </c>
-      <c r="N4" s="5">
+      <c r="O5" s="5">
         <v>8</v>
       </c>
-      <c r="O4" s="5">
+      <c r="P5" s="5">
         <v>6</v>
       </c>
-      <c r="P4" s="5">
-        <v>5</v>
-      </c>
-      <c r="Q4" s="5">
+      <c r="Q5" s="5">
         <v>4</v>
       </c>
-      <c r="R4" s="5">
+      <c r="R5" s="5">
         <v>2</v>
       </c>
     </row>
@@ -1778,6 +1864,348 @@
       </c>
       <c r="H34" s="4"/>
     </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>birth</t>
+        </is>
+      </c>
+      <c r="D35" s="2">
+        <v>335</v>
+      </c>
+      <c r="E35" s="2">
+        <v>156</v>
+      </c>
+      <c r="F35" s="2">
+        <v>491</v>
+      </c>
+      <c r="G35" s="3">
+        <v>0.6763085399449036</v>
+      </c>
+      <c r="H35" s="2">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>anniv</t>
+        </is>
+      </c>
+      <c r="D36" s="2">
+        <v>39</v>
+      </c>
+      <c r="E36" s="2">
+        <v>18</v>
+      </c>
+      <c r="F36" s="2">
+        <v>57</v>
+      </c>
+      <c r="G36" s="3">
+        <v>0.07851239669421488</v>
+      </c>
+      <c r="H36" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="D37" s="2">
+        <v>39</v>
+      </c>
+      <c r="E37" s="2">
+        <v>6</v>
+      </c>
+      <c r="F37" s="2">
+        <v>45</v>
+      </c>
+      <c r="G37" s="3">
+        <v>0.06198347107438017</v>
+      </c>
+      <c r="H37" s="2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>gen</t>
+        </is>
+      </c>
+      <c r="D38" s="2">
+        <v>27</v>
+      </c>
+      <c r="E38" s="2">
+        <v>9</v>
+      </c>
+      <c r="F38" s="2">
+        <v>36</v>
+      </c>
+      <c r="G38" s="3">
+        <v>0.049586776859504134</v>
+      </c>
+      <c r="H38" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>thank</t>
+        </is>
+      </c>
+      <c r="D39" s="2">
+        <v>5</v>
+      </c>
+      <c r="E39" s="2">
+        <v>25</v>
+      </c>
+      <c r="F39" s="2">
+        <v>30</v>
+      </c>
+      <c r="G39" s="3">
+        <v>0.04132231404958678</v>
+      </c>
+      <c r="H39" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D40" s="2">
+        <v>15</v>
+      </c>
+      <c r="E40" s="2">
+        <v>3</v>
+      </c>
+      <c r="F40" s="2">
+        <v>18</v>
+      </c>
+      <c r="G40" s="3">
+        <v>0.024793388429752067</v>
+      </c>
+      <c r="H40" s="2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>congrats</t>
+        </is>
+      </c>
+      <c r="D41" s="2">
+        <v>6</v>
+      </c>
+      <c r="E41" s="2">
+        <v>11</v>
+      </c>
+      <c r="F41" s="2">
+        <v>17</v>
+      </c>
+      <c r="G41" s="3">
+        <v>0.023415977961432508</v>
+      </c>
+      <c r="H41" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>insp</t>
+        </is>
+      </c>
+      <c r="D42" s="2">
+        <v>16</v>
+      </c>
+      <c r="E42" s="2">
+        <v>0</v>
+      </c>
+      <c r="F42" s="2">
+        <v>16</v>
+      </c>
+      <c r="G42" s="3">
+        <v>0.02203856749311295</v>
+      </c>
+      <c r="H42" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>friend</t>
+        </is>
+      </c>
+      <c r="D43" s="2">
+        <v>9</v>
+      </c>
+      <c r="E43" s="2">
+        <v>2</v>
+      </c>
+      <c r="F43" s="2">
+        <v>11</v>
+      </c>
+      <c r="G43" s="3">
+        <v>0.015151515151515152</v>
+      </c>
+      <c r="H43" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>cute</t>
+        </is>
+      </c>
+      <c r="D44" s="2">
+        <v>3</v>
+      </c>
+      <c r="E44" s="2">
+        <v>2</v>
+      </c>
+      <c r="F44" s="2">
+        <v>5</v>
+      </c>
+      <c r="G44" s="3">
+        <v>0.006887052341597796</v>
+      </c>
+      <c r="H44" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-03</t>
+        </is>
+      </c>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="5">
+        <v>494</v>
+      </c>
+      <c r="E45" s="5">
+        <v>232</v>
+      </c>
+      <c r="F45" s="5">
+        <v>726</v>
+      </c>
+      <c r="G45" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="H45" s="4"/>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -7284,6 +7712,2120 @@
         <v>958</v>
       </c>
       <c r="F197" s="4"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B198" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C198" s="0" t="inlineStr">
+        <is>
+          <t>happybirthday</t>
+        </is>
+      </c>
+      <c r="D198" s="0" t="inlineStr">
+        <is>
+          <t>birth_happybirthday</t>
+        </is>
+      </c>
+      <c r="E198" s="2">
+        <v>368</v>
+      </c>
+      <c r="F198" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B199" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C199" s="0" t="inlineStr">
+        <is>
+          <t>anniversaryetc</t>
+        </is>
+      </c>
+      <c r="D199" s="0" t="inlineStr">
+        <is>
+          <t>anniv_anniversaryetc</t>
+        </is>
+      </c>
+      <c r="E199" s="2">
+        <v>42</v>
+      </c>
+      <c r="F199" s="2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B200" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C200" s="0" t="inlineStr">
+        <is>
+          <t>wishes</t>
+        </is>
+      </c>
+      <c r="D200" s="0" t="inlineStr">
+        <is>
+          <t>birth_wishes</t>
+        </is>
+      </c>
+      <c r="E200" s="2">
+        <v>24</v>
+      </c>
+      <c r="F200" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B201" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C201" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalwatermelon_day</t>
+        </is>
+      </c>
+      <c r="D201" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalwatermelon_day</t>
+        </is>
+      </c>
+      <c r="E201" s="2">
+        <v>24</v>
+      </c>
+      <c r="F201" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B202" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C202" s="0" t="inlineStr">
+        <is>
+          <t>birthday</t>
+        </is>
+      </c>
+      <c r="D202" s="0" t="inlineStr">
+        <is>
+          <t>thank_birthday</t>
+        </is>
+      </c>
+      <c r="E202" s="2">
+        <v>17</v>
+      </c>
+      <c r="F202" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B203" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C203" s="0" t="inlineStr">
+        <is>
+          <t>fun</t>
+        </is>
+      </c>
+      <c r="D203" s="0" t="inlineStr">
+        <is>
+          <t>birth_fun</t>
+        </is>
+      </c>
+      <c r="E203" s="2">
+        <v>16</v>
+      </c>
+      <c r="F203" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B204" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C204" s="0" t="inlineStr">
+        <is>
+          <t>songs</t>
+        </is>
+      </c>
+      <c r="D204" s="0" t="inlineStr">
+        <is>
+          <t>birth_songs</t>
+        </is>
+      </c>
+      <c r="E204" s="2">
+        <v>13</v>
+      </c>
+      <c r="F204" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B205" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C205" s="0" t="inlineStr">
+        <is>
+          <t>morning</t>
+        </is>
+      </c>
+      <c r="D205" s="0" t="inlineStr">
+        <is>
+          <t>gen_morning</t>
+        </is>
+      </c>
+      <c r="E205" s="2">
+        <v>13</v>
+      </c>
+      <c r="F205" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B206" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C206" s="0" t="inlineStr">
+        <is>
+          <t>sympathy</t>
+        </is>
+      </c>
+      <c r="D206" s="0" t="inlineStr">
+        <is>
+          <t>insp_sympathy</t>
+        </is>
+      </c>
+      <c r="E206" s="2">
+        <v>12</v>
+      </c>
+      <c r="F206" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B207" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C207" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D207" s="0" t="inlineStr">
+        <is>
+          <t>birth_milestone</t>
+        </is>
+      </c>
+      <c r="E207" s="2">
+        <v>10</v>
+      </c>
+      <c r="F207" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B208" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C208" s="0" t="inlineStr">
+        <is>
+          <t>belated</t>
+        </is>
+      </c>
+      <c r="D208" s="0" t="inlineStr">
+        <is>
+          <t>birth_belated</t>
+        </is>
+      </c>
+      <c r="E208" s="2">
+        <v>9</v>
+      </c>
+      <c r="F208" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B209" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C209" s="0" t="inlineStr">
+        <is>
+          <t>blessings</t>
+        </is>
+      </c>
+      <c r="D209" s="0" t="inlineStr">
+        <is>
+          <t>birth_blessings</t>
+        </is>
+      </c>
+      <c r="E209" s="2">
+        <v>9</v>
+      </c>
+      <c r="F209" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B210" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C210" s="0" t="inlineStr">
+        <is>
+          <t>newbaby</t>
+        </is>
+      </c>
+      <c r="D210" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newbaby</t>
+        </is>
+      </c>
+      <c r="E210" s="2">
+        <v>9</v>
+      </c>
+      <c r="F210" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B211" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C211" s="0" t="inlineStr">
+        <is>
+          <t>bestfriends</t>
+        </is>
+      </c>
+      <c r="D211" s="0" t="inlineStr">
+        <is>
+          <t>friend_bestfriends</t>
+        </is>
+      </c>
+      <c r="E211" s="2">
+        <v>9</v>
+      </c>
+      <c r="F211" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B212" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C212" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="D212" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="E212" s="2">
+        <v>8</v>
+      </c>
+      <c r="F212" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B213" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C213" s="0" t="inlineStr">
+        <is>
+          <t>sonanddaughter</t>
+        </is>
+      </c>
+      <c r="D213" s="0" t="inlineStr">
+        <is>
+          <t>birth_sonanddaughter</t>
+        </is>
+      </c>
+      <c r="E213" s="2">
+        <v>8</v>
+      </c>
+      <c r="F213" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B214" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C214" s="0" t="inlineStr">
+        <is>
+          <t>friends</t>
+        </is>
+      </c>
+      <c r="D214" s="0" t="inlineStr">
+        <is>
+          <t>birth_friends</t>
+        </is>
+      </c>
+      <c r="E214" s="2">
+        <v>6</v>
+      </c>
+      <c r="F214" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B215" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C215" s="0" t="inlineStr">
+        <is>
+          <t>thinkingofyou</t>
+        </is>
+      </c>
+      <c r="D215" s="0" t="inlineStr">
+        <is>
+          <t>gen_thinkingofyou</t>
+        </is>
+      </c>
+      <c r="E215" s="2">
+        <v>6</v>
+      </c>
+      <c r="F215" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B216" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C216" s="0" t="inlineStr">
+        <is>
+          <t>bronsis</t>
+        </is>
+      </c>
+      <c r="D216" s="0" t="inlineStr">
+        <is>
+          <t>birth_bronsis</t>
+        </is>
+      </c>
+      <c r="E216" s="2">
+        <v>5</v>
+      </c>
+      <c r="F216" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B217" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C217" s="0" t="inlineStr">
+        <is>
+          <t>extfamily</t>
+        </is>
+      </c>
+      <c r="D217" s="0" t="inlineStr">
+        <is>
+          <t>birth_extfamily</t>
+        </is>
+      </c>
+      <c r="E217" s="2">
+        <v>5</v>
+      </c>
+      <c r="F217" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B218" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C218" s="0" t="inlineStr">
+        <is>
+          <t>foreveryone</t>
+        </is>
+      </c>
+      <c r="D218" s="0" t="inlineStr">
+        <is>
+          <t>congrats_foreveryone</t>
+        </is>
+      </c>
+      <c r="E218" s="2">
+        <v>5</v>
+      </c>
+      <c r="F218" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B219" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C219" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D219" s="0" t="inlineStr">
+        <is>
+          <t>gen_getwell</t>
+        </is>
+      </c>
+      <c r="E219" s="2">
+        <v>5</v>
+      </c>
+      <c r="F219" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B220" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C220" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="D220" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="E220" s="2">
+        <v>5</v>
+      </c>
+      <c r="F220" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B221" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C221" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D221" s="0" t="inlineStr">
+        <is>
+          <t>thank_love</t>
+        </is>
+      </c>
+      <c r="E221" s="2">
+        <v>5</v>
+      </c>
+      <c r="F221" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B222" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C222" s="0" t="inlineStr">
+        <is>
+          <t>balloons</t>
+        </is>
+      </c>
+      <c r="D222" s="0" t="inlineStr">
+        <is>
+          <t>birth_balloons</t>
+        </is>
+      </c>
+      <c r="E222" s="2">
+        <v>4</v>
+      </c>
+      <c r="F222" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B223" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C223" s="0" t="inlineStr">
+        <is>
+          <t>flowers</t>
+        </is>
+      </c>
+      <c r="D223" s="0" t="inlineStr">
+        <is>
+          <t>birth_flowers</t>
+        </is>
+      </c>
+      <c r="E223" s="2">
+        <v>4</v>
+      </c>
+      <c r="F223" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B224" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C224" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="D224" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="E224" s="2">
+        <v>4</v>
+      </c>
+      <c r="F224" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B225" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C225" s="0" t="inlineStr">
+        <is>
+          <t>everyday</t>
+        </is>
+      </c>
+      <c r="D225" s="0" t="inlineStr">
+        <is>
+          <t>thank_everyday</t>
+        </is>
+      </c>
+      <c r="E225" s="2">
+        <v>4</v>
+      </c>
+      <c r="F225" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B226" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C226" s="0" t="inlineStr">
+        <is>
+          <t>gifts</t>
+        </is>
+      </c>
+      <c r="D226" s="0" t="inlineStr">
+        <is>
+          <t>anniv_gifts</t>
+        </is>
+      </c>
+      <c r="E226" s="2">
+        <v>3</v>
+      </c>
+      <c r="F226" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B227" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C227" s="0" t="inlineStr">
+        <is>
+          <t>newjob</t>
+        </is>
+      </c>
+      <c r="D227" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newjob</t>
+        </is>
+      </c>
+      <c r="E227" s="2">
+        <v>3</v>
+      </c>
+      <c r="F227" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B228" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C228" s="0" t="inlineStr">
+        <is>
+          <t>teddy</t>
+        </is>
+      </c>
+      <c r="D228" s="0" t="inlineStr">
+        <is>
+          <t>cute_teddy</t>
+        </is>
+      </c>
+      <c r="E228" s="2">
+        <v>3</v>
+      </c>
+      <c r="F228" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B229" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C229" s="0" t="inlineStr">
+        <is>
+          <t>eaug_dollarday</t>
+        </is>
+      </c>
+      <c r="D229" s="0" t="inlineStr">
+        <is>
+          <t>eaug_dollarday</t>
+        </is>
+      </c>
+      <c r="E229" s="2">
+        <v>3</v>
+      </c>
+      <c r="F229" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B230" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C230" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalzucchini_day</t>
+        </is>
+      </c>
+      <c r="D230" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalzucchini_day</t>
+        </is>
+      </c>
+      <c r="E230" s="2">
+        <v>3</v>
+      </c>
+      <c r="F230" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B231" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C231" s="0" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="D231" s="0" t="inlineStr">
+        <is>
+          <t>gen_hi</t>
+        </is>
+      </c>
+      <c r="E231" s="2">
+        <v>3</v>
+      </c>
+      <c r="F231" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B232" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C232" s="0" t="inlineStr">
+        <is>
+          <t>monblues</t>
+        </is>
+      </c>
+      <c r="D232" s="0" t="inlineStr">
+        <is>
+          <t>gen_monblues</t>
+        </is>
+      </c>
+      <c r="E232" s="2">
+        <v>3</v>
+      </c>
+      <c r="F232" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B233" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C233" s="0" t="inlineStr">
+        <is>
+          <t>encour</t>
+        </is>
+      </c>
+      <c r="D233" s="0" t="inlineStr">
+        <is>
+          <t>insp_encour</t>
+        </is>
+      </c>
+      <c r="E233" s="2">
+        <v>3</v>
+      </c>
+      <c r="F233" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B234" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C234" s="0" t="inlineStr">
+        <is>
+          <t>youarespecial</t>
+        </is>
+      </c>
+      <c r="D234" s="0" t="inlineStr">
+        <is>
+          <t>love_youarespecial</t>
+        </is>
+      </c>
+      <c r="E234" s="2">
+        <v>3</v>
+      </c>
+      <c r="F234" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B235" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C235" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="D235" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="E235" s="2">
+        <v>2</v>
+      </c>
+      <c r="F235" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B236" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C236" s="0" t="inlineStr">
+        <is>
+          <t>forhim</t>
+        </is>
+      </c>
+      <c r="D236" s="0" t="inlineStr">
+        <is>
+          <t>birth_forhim</t>
+        </is>
+      </c>
+      <c r="E236" s="2">
+        <v>2</v>
+      </c>
+      <c r="F236" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B237" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C237" s="0" t="inlineStr">
+        <is>
+          <t>kids</t>
+        </is>
+      </c>
+      <c r="D237" s="0" t="inlineStr">
+        <is>
+          <t>birth_kids</t>
+        </is>
+      </c>
+      <c r="E237" s="2">
+        <v>2</v>
+      </c>
+      <c r="F237" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B238" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C238" s="0" t="inlineStr">
+        <is>
+          <t>zodiac</t>
+        </is>
+      </c>
+      <c r="D238" s="0" t="inlineStr">
+        <is>
+          <t>birth_zodiac</t>
+        </is>
+      </c>
+      <c r="E238" s="2">
+        <v>2</v>
+      </c>
+      <c r="F238" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B239" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C239" s="0" t="inlineStr">
+        <is>
+          <t>hugs</t>
+        </is>
+      </c>
+      <c r="D239" s="0" t="inlineStr">
+        <is>
+          <t>cute_hugs</t>
+        </is>
+      </c>
+      <c r="E239" s="2">
+        <v>2</v>
+      </c>
+      <c r="F239" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B240" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C240" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_happy</t>
+        </is>
+      </c>
+      <c r="D240" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_happy</t>
+        </is>
+      </c>
+      <c r="E240" s="2">
+        <v>2</v>
+      </c>
+      <c r="F240" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B241" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C241" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="D241" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="E241" s="2">
+        <v>2</v>
+      </c>
+      <c r="F241" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B242" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C242" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalwhite_wine_day</t>
+        </is>
+      </c>
+      <c r="D242" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalwhite_wine_day</t>
+        </is>
+      </c>
+      <c r="E242" s="2">
+        <v>2</v>
+      </c>
+      <c r="F242" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B243" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C243" s="0" t="inlineStr">
+        <is>
+          <t>ejan_thankyoucards</t>
+        </is>
+      </c>
+      <c r="D243" s="0" t="inlineStr">
+        <is>
+          <t>ejan_thankyoucards</t>
+        </is>
+      </c>
+      <c r="E243" s="2">
+        <v>2</v>
+      </c>
+      <c r="F243" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B244" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C244" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_general</t>
+        </is>
+      </c>
+      <c r="D244" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_general</t>
+        </is>
+      </c>
+      <c r="E244" s="2">
+        <v>2</v>
+      </c>
+      <c r="F244" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B245" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C245" s="0" t="inlineStr">
+        <is>
+          <t>inspirational</t>
+        </is>
+      </c>
+      <c r="D245" s="0" t="inlineStr">
+        <is>
+          <t>thank_inspirational</t>
+        </is>
+      </c>
+      <c r="E245" s="2">
+        <v>2</v>
+      </c>
+      <c r="F245" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B246" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C246" s="0" t="inlineStr">
+        <is>
+          <t>wedding</t>
+        </is>
+      </c>
+      <c r="D246" s="0" t="inlineStr">
+        <is>
+          <t>thank_wedding</t>
+        </is>
+      </c>
+      <c r="E246" s="2">
+        <v>2</v>
+      </c>
+      <c r="F246" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B247" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C247" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="D247" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="E247" s="2">
+        <v>1</v>
+      </c>
+      <c r="F247" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B248" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C248" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_family</t>
+        </is>
+      </c>
+      <c r="D248" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_family</t>
+        </is>
+      </c>
+      <c r="E248" s="2">
+        <v>1</v>
+      </c>
+      <c r="F248" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B249" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C249" s="0" t="inlineStr">
+        <is>
+          <t>hubbywife</t>
+        </is>
+      </c>
+      <c r="D249" s="0" t="inlineStr">
+        <is>
+          <t>birth_hubbywife</t>
+        </is>
+      </c>
+      <c r="E249" s="2">
+        <v>1</v>
+      </c>
+      <c r="F249" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B250" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C250" s="0" t="inlineStr">
+        <is>
+          <t>momndad</t>
+        </is>
+      </c>
+      <c r="D250" s="0" t="inlineStr">
+        <is>
+          <t>birth_momndad</t>
+        </is>
+      </c>
+      <c r="E250" s="2">
+        <v>1</v>
+      </c>
+      <c r="F250" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B251" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C251" s="0" t="inlineStr">
+        <is>
+          <t>pets</t>
+        </is>
+      </c>
+      <c r="D251" s="0" t="inlineStr">
+        <is>
+          <t>birth_pets</t>
+        </is>
+      </c>
+      <c r="E251" s="2">
+        <v>1</v>
+      </c>
+      <c r="F251" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B252" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C252" s="0" t="inlineStr">
+        <is>
+          <t>specials</t>
+        </is>
+      </c>
+      <c r="D252" s="0" t="inlineStr">
+        <is>
+          <t>birth_specials</t>
+        </is>
+      </c>
+      <c r="E252" s="2">
+        <v>1</v>
+      </c>
+      <c r="F252" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B253" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C253" s="0" t="inlineStr">
+        <is>
+          <t>eaug_cardssister</t>
+        </is>
+      </c>
+      <c r="D253" s="0" t="inlineStr">
+        <is>
+          <t>eaug_cardssister</t>
+        </is>
+      </c>
+      <c r="E253" s="2">
+        <v>1</v>
+      </c>
+      <c r="F253" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B254" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C254" s="0" t="inlineStr">
+        <is>
+          <t>eaug_girlfriendsday</t>
+        </is>
+      </c>
+      <c r="D254" s="0" t="inlineStr">
+        <is>
+          <t>eaug_girlfriendsday</t>
+        </is>
+      </c>
+      <c r="E254" s="2">
+        <v>1</v>
+      </c>
+      <c r="F254" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B255" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C255" s="0" t="inlineStr">
+        <is>
+          <t>eaug_romawaremonth</t>
+        </is>
+      </c>
+      <c r="D255" s="0" t="inlineStr">
+        <is>
+          <t>eaug_romawaremonth</t>
+        </is>
+      </c>
+      <c r="E255" s="2">
+        <v>1</v>
+      </c>
+      <c r="F255" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B256" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C256" s="0" t="inlineStr">
+        <is>
+          <t>edec_c_thankyou</t>
+        </is>
+      </c>
+      <c r="D256" s="0" t="inlineStr">
+        <is>
+          <t>edec_c_thankyou</t>
+        </is>
+      </c>
+      <c r="E256" s="2">
+        <v>1</v>
+      </c>
+      <c r="F256" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B257" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C257" s="0" t="inlineStr">
+        <is>
+          <t>ejan_sendahugday_love</t>
+        </is>
+      </c>
+      <c r="D257" s="0" t="inlineStr">
+        <is>
+          <t>ejan_sendahugday_love</t>
+        </is>
+      </c>
+      <c r="E257" s="2">
+        <v>1</v>
+      </c>
+      <c r="F257" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B258" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C258" s="0" t="inlineStr">
+        <is>
+          <t>ejul_livebetterday</t>
+        </is>
+      </c>
+      <c r="D258" s="0" t="inlineStr">
+        <is>
+          <t>ejul_livebetterday</t>
+        </is>
+      </c>
+      <c r="E258" s="2">
+        <v>1</v>
+      </c>
+      <c r="F258" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B259" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C259" s="0" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="D259" s="0" t="inlineStr">
+        <is>
+          <t>friend_hello</t>
+        </is>
+      </c>
+      <c r="E259" s="2">
+        <v>1</v>
+      </c>
+      <c r="F259" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B260" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C260" s="0" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
+      <c r="D260" s="0" t="inlineStr">
+        <is>
+          <t>friend_thoughts</t>
+        </is>
+      </c>
+      <c r="E260" s="2">
+        <v>1</v>
+      </c>
+      <c r="F260" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B261" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C261" s="0" t="inlineStr">
+        <is>
+          <t>blessings</t>
+        </is>
+      </c>
+      <c r="D261" s="0" t="inlineStr">
+        <is>
+          <t>gen_blessings</t>
+        </is>
+      </c>
+      <c r="E261" s="2">
+        <v>1</v>
+      </c>
+      <c r="F261" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B262" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C262" s="0" t="inlineStr">
+        <is>
+          <t>cheerup</t>
+        </is>
+      </c>
+      <c r="D262" s="0" t="inlineStr">
+        <is>
+          <t>gen_cheerup</t>
+        </is>
+      </c>
+      <c r="E262" s="2">
+        <v>1</v>
+      </c>
+      <c r="F262" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B263" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C263" s="0" t="inlineStr">
+        <is>
+          <t>goodnight</t>
+        </is>
+      </c>
+      <c r="D263" s="0" t="inlineStr">
+        <is>
+          <t>gen_goodnight</t>
+        </is>
+      </c>
+      <c r="E263" s="2">
+        <v>1</v>
+      </c>
+      <c r="F263" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B264" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C264" s="0" t="inlineStr">
+        <is>
+          <t>missyou</t>
+        </is>
+      </c>
+      <c r="D264" s="0" t="inlineStr">
+        <is>
+          <t>gen_missyou</t>
+        </is>
+      </c>
+      <c r="E264" s="2">
+        <v>1</v>
+      </c>
+      <c r="F264" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B265" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C265" s="0" t="inlineStr">
+        <is>
+          <t>sorry</t>
+        </is>
+      </c>
+      <c r="D265" s="0" t="inlineStr">
+        <is>
+          <t>gen_sorry</t>
+        </is>
+      </c>
+      <c r="E265" s="2">
+        <v>1</v>
+      </c>
+      <c r="F265" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B266" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C266" s="0" t="inlineStr">
+        <is>
+          <t>voyage</t>
+        </is>
+      </c>
+      <c r="D266" s="0" t="inlineStr">
+        <is>
+          <t>gen_voyage</t>
+        </is>
+      </c>
+      <c r="E266" s="2">
+        <v>1</v>
+      </c>
+      <c r="F266" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B267" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C267" s="0" t="inlineStr">
+        <is>
+          <t>recovery</t>
+        </is>
+      </c>
+      <c r="D267" s="0" t="inlineStr">
+        <is>
+          <t>insp_recovery</t>
+        </is>
+      </c>
+      <c r="E267" s="2">
+        <v>1</v>
+      </c>
+      <c r="F267" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B268" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C268" s="0" t="inlineStr">
+        <is>
+          <t>cute</t>
+        </is>
+      </c>
+      <c r="D268" s="0" t="inlineStr">
+        <is>
+          <t>love_cute</t>
+        </is>
+      </c>
+      <c r="E268" s="2">
+        <v>1</v>
+      </c>
+      <c r="F268" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B269" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C269" s="0" t="inlineStr">
+        <is>
+          <t>dating</t>
+        </is>
+      </c>
+      <c r="D269" s="0" t="inlineStr">
+        <is>
+          <t>love_dating</t>
+        </is>
+      </c>
+      <c r="E269" s="2">
+        <v>1</v>
+      </c>
+      <c r="F269" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B270" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C270" s="0" t="inlineStr">
+        <is>
+          <t>lovepoems</t>
+        </is>
+      </c>
+      <c r="D270" s="0" t="inlineStr">
+        <is>
+          <t>love_lovepoems</t>
+        </is>
+      </c>
+      <c r="E270" s="2">
+        <v>1</v>
+      </c>
+      <c r="F270" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B271" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C271" s="0" t="inlineStr">
+        <is>
+          <t>sweetheart</t>
+        </is>
+      </c>
+      <c r="D271" s="0" t="inlineStr">
+        <is>
+          <t>love_sweetheart</t>
+        </is>
+      </c>
+      <c r="E271" s="2">
+        <v>1</v>
+      </c>
+      <c r="F271" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B272" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C272" s="0" t="inlineStr">
+        <is>
+          <t>wed_weddingetc</t>
+        </is>
+      </c>
+      <c r="D272" s="0" t="inlineStr">
+        <is>
+          <t>wed_weddingetc</t>
+        </is>
+      </c>
+      <c r="E272" s="2">
+        <v>1</v>
+      </c>
+      <c r="F272" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-03</t>
+        </is>
+      </c>
+      <c r="B273" s="4"/>
+      <c r="C273" s="4"/>
+      <c r="D273" s="4"/>
+      <c r="E273" s="5">
+        <v>726</v>
+      </c>
+      <c r="F273" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -7425,36 +9967,70 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2">
+        <v>765</v>
+      </c>
+      <c r="C4" s="2">
+        <v>242</v>
+      </c>
+      <c r="D4" s="2">
+        <v>238</v>
+      </c>
+      <c r="E4" s="2">
+        <v>148</v>
+      </c>
+      <c r="F4" s="2">
+        <v>84</v>
+      </c>
+      <c r="G4" s="2">
+        <v>19</v>
+      </c>
+      <c r="H4" s="2">
+        <v>31</v>
+      </c>
+      <c r="I4" s="2">
+        <v>3</v>
+      </c>
+      <c r="J4" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B4" s="5">
-        <v>2058</v>
-      </c>
-      <c r="C4" s="5">
-        <v>759</v>
-      </c>
-      <c r="D4" s="5">
-        <v>546</v>
-      </c>
-      <c r="E4" s="5">
-        <v>351</v>
-      </c>
-      <c r="F4" s="5">
-        <v>226</v>
-      </c>
-      <c r="G4" s="5">
-        <v>85</v>
-      </c>
-      <c r="H4" s="5">
-        <v>65</v>
-      </c>
-      <c r="I4" s="5">
-        <v>25</v>
-      </c>
-      <c r="J4" s="5">
+      <c r="B5" s="5">
+        <v>2823</v>
+      </c>
+      <c r="C5" s="5">
+        <v>1001</v>
+      </c>
+      <c r="D5" s="5">
+        <v>784</v>
+      </c>
+      <c r="E5" s="5">
+        <v>499</v>
+      </c>
+      <c r="F5" s="5">
+        <v>310</v>
+      </c>
+      <c r="G5" s="5">
+        <v>104</v>
+      </c>
+      <c r="H5" s="5">
+        <v>96</v>
+      </c>
+      <c r="I5" s="5">
+        <v>28</v>
+      </c>
+      <c r="J5" s="5">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Record 4 August: 805 sends, four days now tracked
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9KsXegBwxB1sWdCzRVLrr
</commit_message>
<xml_diff>
--- a/reports/daily_tracking.xlsx
+++ b/reports/daily_tracking.xlsx
@@ -224,7 +224,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -247,7 +247,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
     </row>
@@ -395,28 +395,56 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B5" s="2">
+        <v>805</v>
+      </c>
+      <c r="C5" s="2">
+        <v>554</v>
+      </c>
+      <c r="D5" s="2">
+        <v>251</v>
+      </c>
+      <c r="E5" s="2">
+        <v>770</v>
+      </c>
+      <c r="F5" s="2">
+        <v>35</v>
+      </c>
+      <c r="G5" s="2">
+        <v>252</v>
+      </c>
+      <c r="H5" s="2">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B5" s="5">
-        <v>2823</v>
-      </c>
-      <c r="C5" s="5">
-        <v>1671</v>
-      </c>
-      <c r="D5" s="5">
-        <v>1152</v>
-      </c>
-      <c r="E5" s="5">
-        <v>2702</v>
-      </c>
-      <c r="F5" s="5">
-        <v>121</v>
-      </c>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
+      <c r="B6" s="5">
+        <v>3628</v>
+      </c>
+      <c r="C6" s="5">
+        <v>2225</v>
+      </c>
+      <c r="D6" s="5">
+        <v>1403</v>
+      </c>
+      <c r="E6" s="5">
+        <v>3472</v>
+      </c>
+      <c r="F6" s="5">
+        <v>156</v>
+      </c>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -438,9 +466,9 @@
     <col min="11" max="11" width="17" customWidth="1"/>
     <col min="12" max="12" width="17" customWidth="1"/>
     <col min="13" max="13" width="11" customWidth="1"/>
-    <col min="14" max="14" width="11" customWidth="1"/>
-    <col min="15" max="15" width="18" customWidth="1"/>
-    <col min="16" max="16" width="21" customWidth="1"/>
+    <col min="14" max="14" width="21" customWidth="1"/>
+    <col min="15" max="15" width="11" customWidth="1"/>
+    <col min="16" max="16" width="18" customWidth="1"/>
     <col min="17" max="17" width="11" customWidth="1"/>
     <col min="18" max="18" width="17" customWidth="1"/>
   </cols>
@@ -513,17 +541,17 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>Flowers</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Keeping in touch</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Family &amp; loved ones</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
@@ -580,13 +608,13 @@
         <v>4</v>
       </c>
       <c r="N2" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O2" s="2">
+        <v>1</v>
+      </c>
+      <c r="P2" s="2">
         <v>6</v>
-      </c>
-      <c r="P2" s="2">
-        <v>3</v>
       </c>
       <c r="Q2" s="2">
         <v>3</v>
@@ -638,13 +666,13 @@
         <v>1</v>
       </c>
       <c r="N3" s="2">
+        <v>3</v>
+      </c>
+      <c r="O3" s="2">
         <v>8</v>
       </c>
-      <c r="O3" s="2">
+      <c r="P3" s="2">
         <v>2</v>
-      </c>
-      <c r="P3" s="2">
-        <v>3</v>
       </c>
       <c r="Q3" s="2">
         <v>1</v>
@@ -712,60 +740,118 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B5" s="2">
+        <v>770</v>
+      </c>
+      <c r="C5" s="2">
+        <v>555</v>
+      </c>
+      <c r="D5" s="2">
+        <v>29</v>
+      </c>
+      <c r="E5" s="2">
+        <v>46</v>
+      </c>
+      <c r="F5" s="2">
+        <v>28</v>
+      </c>
+      <c r="G5" s="2">
+        <v>34</v>
+      </c>
+      <c r="H5" s="2">
+        <v>22</v>
+      </c>
+      <c r="I5" s="2">
+        <v>26</v>
+      </c>
+      <c r="J5" s="2">
+        <v>15</v>
+      </c>
+      <c r="K5" s="2">
+        <v>4</v>
+      </c>
+      <c r="L5" s="2">
+        <v>2</v>
+      </c>
+      <c r="M5" s="2">
+        <v>1</v>
+      </c>
+      <c r="N5" s="2">
+        <v>5</v>
+      </c>
+      <c r="O5" s="2">
+        <v>0</v>
+      </c>
+      <c r="P5" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="2">
+        <v>2</v>
+      </c>
+      <c r="R5" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B5" s="5">
-        <v>2702</v>
-      </c>
-      <c r="C5" s="5">
-        <v>1607</v>
-      </c>
-      <c r="D5" s="5">
-        <v>453</v>
-      </c>
-      <c r="E5" s="5">
-        <v>149</v>
-      </c>
-      <c r="F5" s="5">
-        <v>112</v>
-      </c>
-      <c r="G5" s="5">
-        <v>104</v>
-      </c>
-      <c r="H5" s="5">
-        <v>80</v>
-      </c>
-      <c r="I5" s="5">
-        <v>61</v>
-      </c>
-      <c r="J5" s="5">
-        <v>45</v>
-      </c>
-      <c r="K5" s="5">
-        <v>40</v>
-      </c>
-      <c r="L5" s="5">
-        <v>12</v>
-      </c>
-      <c r="M5" s="5">
-        <v>10</v>
-      </c>
-      <c r="N5" s="5">
+      <c r="B6" s="5">
+        <v>3472</v>
+      </c>
+      <c r="C6" s="5">
+        <v>2162</v>
+      </c>
+      <c r="D6" s="5">
+        <v>482</v>
+      </c>
+      <c r="E6" s="5">
+        <v>195</v>
+      </c>
+      <c r="F6" s="5">
+        <v>140</v>
+      </c>
+      <c r="G6" s="5">
+        <v>138</v>
+      </c>
+      <c r="H6" s="5">
+        <v>102</v>
+      </c>
+      <c r="I6" s="5">
+        <v>87</v>
+      </c>
+      <c r="J6" s="5">
+        <v>60</v>
+      </c>
+      <c r="K6" s="5">
+        <v>44</v>
+      </c>
+      <c r="L6" s="5">
+        <v>14</v>
+      </c>
+      <c r="M6" s="5">
+        <v>11</v>
+      </c>
+      <c r="N6" s="5">
+        <v>11</v>
+      </c>
+      <c r="O6" s="5">
         <v>9</v>
       </c>
-      <c r="O5" s="5">
-        <v>8</v>
-      </c>
-      <c r="P5" s="5">
+      <c r="P6" s="5">
+        <v>9</v>
+      </c>
+      <c r="Q6" s="5">
         <v>6</v>
       </c>
-      <c r="Q5" s="5">
-        <v>4</v>
-      </c>
-      <c r="R5" s="5">
+      <c r="R6" s="5">
         <v>2</v>
       </c>
     </row>
@@ -2206,6 +2292,476 @@
       </c>
       <c r="H45" s="4"/>
     </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>birth</t>
+        </is>
+      </c>
+      <c r="D46" s="2">
+        <v>398</v>
+      </c>
+      <c r="E46" s="2">
+        <v>157</v>
+      </c>
+      <c r="F46" s="2">
+        <v>555</v>
+      </c>
+      <c r="G46" s="3">
+        <v>0.7207792207792207</v>
+      </c>
+      <c r="H46" s="2">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>anniv</t>
+        </is>
+      </c>
+      <c r="D47" s="2">
+        <v>34</v>
+      </c>
+      <c r="E47" s="2">
+        <v>12</v>
+      </c>
+      <c r="F47" s="2">
+        <v>46</v>
+      </c>
+      <c r="G47" s="3">
+        <v>0.05974025974025974</v>
+      </c>
+      <c r="H47" s="2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>gen</t>
+        </is>
+      </c>
+      <c r="D48" s="2">
+        <v>21</v>
+      </c>
+      <c r="E48" s="2">
+        <v>13</v>
+      </c>
+      <c r="F48" s="2">
+        <v>34</v>
+      </c>
+      <c r="G48" s="3">
+        <v>0.04415584415584416</v>
+      </c>
+      <c r="H48" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="D49" s="2">
+        <v>23</v>
+      </c>
+      <c r="E49" s="2">
+        <v>6</v>
+      </c>
+      <c r="F49" s="2">
+        <v>29</v>
+      </c>
+      <c r="G49" s="3">
+        <v>0.03766233766233766</v>
+      </c>
+      <c r="H49" s="2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>thank</t>
+        </is>
+      </c>
+      <c r="D50" s="2">
+        <v>9</v>
+      </c>
+      <c r="E50" s="2">
+        <v>19</v>
+      </c>
+      <c r="F50" s="2">
+        <v>28</v>
+      </c>
+      <c r="G50" s="3">
+        <v>0.03636363636363636</v>
+      </c>
+      <c r="H50" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D51" s="2">
+        <v>20</v>
+      </c>
+      <c r="E51" s="2">
+        <v>6</v>
+      </c>
+      <c r="F51" s="2">
+        <v>26</v>
+      </c>
+      <c r="G51" s="3">
+        <v>0.033766233766233764</v>
+      </c>
+      <c r="H51" s="2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B52" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C52" s="0" t="inlineStr">
+        <is>
+          <t>friend</t>
+        </is>
+      </c>
+      <c r="D52" s="2">
+        <v>22</v>
+      </c>
+      <c r="E52" s="2">
+        <v>0</v>
+      </c>
+      <c r="F52" s="2">
+        <v>22</v>
+      </c>
+      <c r="G52" s="3">
+        <v>0.02857142857142857</v>
+      </c>
+      <c r="H52" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B53" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C53" s="0" t="inlineStr">
+        <is>
+          <t>insp</t>
+        </is>
+      </c>
+      <c r="D53" s="2">
+        <v>13</v>
+      </c>
+      <c r="E53" s="2">
+        <v>2</v>
+      </c>
+      <c r="F53" s="2">
+        <v>15</v>
+      </c>
+      <c r="G53" s="3">
+        <v>0.01948051948051948</v>
+      </c>
+      <c r="H53" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B54" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C54" s="0" t="inlineStr">
+        <is>
+          <t>fkt</t>
+        </is>
+      </c>
+      <c r="D54" s="2">
+        <v>5</v>
+      </c>
+      <c r="E54" s="2">
+        <v>0</v>
+      </c>
+      <c r="F54" s="2">
+        <v>5</v>
+      </c>
+      <c r="G54" s="3">
+        <v>0.006493506493506494</v>
+      </c>
+      <c r="H54" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B55" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C55" s="0" t="inlineStr">
+        <is>
+          <t>congrats</t>
+        </is>
+      </c>
+      <c r="D55" s="2">
+        <v>4</v>
+      </c>
+      <c r="E55" s="2">
+        <v>0</v>
+      </c>
+      <c r="F55" s="2">
+        <v>4</v>
+      </c>
+      <c r="G55" s="3">
+        <v>0.005194805194805195</v>
+      </c>
+      <c r="H55" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B56" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C56" s="0" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="D56" s="2">
+        <v>2</v>
+      </c>
+      <c r="E56" s="2">
+        <v>0</v>
+      </c>
+      <c r="F56" s="2">
+        <v>2</v>
+      </c>
+      <c r="G56" s="3">
+        <v>0.0025974025974025974</v>
+      </c>
+      <c r="H56" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B57" s="0" t="inlineStr">
+        <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="C57" s="0" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="D57" s="2">
+        <v>1</v>
+      </c>
+      <c r="E57" s="2">
+        <v>1</v>
+      </c>
+      <c r="F57" s="2">
+        <v>2</v>
+      </c>
+      <c r="G57" s="3">
+        <v>0.0025974025974025974</v>
+      </c>
+      <c r="H57" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B58" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C58" s="0" t="inlineStr">
+        <is>
+          <t>cute</t>
+        </is>
+      </c>
+      <c r="D58" s="2">
+        <v>1</v>
+      </c>
+      <c r="E58" s="2">
+        <v>0</v>
+      </c>
+      <c r="F58" s="2">
+        <v>1</v>
+      </c>
+      <c r="G58" s="3">
+        <v>0.0012987012987012987</v>
+      </c>
+      <c r="H58" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B59" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C59" s="0" t="inlineStr">
+        <is>
+          <t>intouch</t>
+        </is>
+      </c>
+      <c r="D59" s="2">
+        <v>1</v>
+      </c>
+      <c r="E59" s="2">
+        <v>0</v>
+      </c>
+      <c r="F59" s="2">
+        <v>1</v>
+      </c>
+      <c r="G59" s="3">
+        <v>0.0012987012987012987</v>
+      </c>
+      <c r="H59" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-04</t>
+        </is>
+      </c>
+      <c r="B60" s="4"/>
+      <c r="C60" s="4"/>
+      <c r="D60" s="5">
+        <v>554</v>
+      </c>
+      <c r="E60" s="5">
+        <v>216</v>
+      </c>
+      <c r="F60" s="5">
+        <v>770</v>
+      </c>
+      <c r="G60" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="H60" s="4"/>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -9826,6 +10382,2232 @@
         <v>726</v>
       </c>
       <c r="F273" s="4"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B274" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C274" s="0" t="inlineStr">
+        <is>
+          <t>happybirthday</t>
+        </is>
+      </c>
+      <c r="D274" s="0" t="inlineStr">
+        <is>
+          <t>birth_happybirthday</t>
+        </is>
+      </c>
+      <c r="E274" s="2">
+        <v>417</v>
+      </c>
+      <c r="F274" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B275" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C275" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="D275" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="E275" s="2">
+        <v>36</v>
+      </c>
+      <c r="F275" s="2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B276" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C276" s="0" t="inlineStr">
+        <is>
+          <t>bronsis</t>
+        </is>
+      </c>
+      <c r="D276" s="0" t="inlineStr">
+        <is>
+          <t>birth_bronsis</t>
+        </is>
+      </c>
+      <c r="E276" s="2">
+        <v>18</v>
+      </c>
+      <c r="F276" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B277" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C277" s="0" t="inlineStr">
+        <is>
+          <t>fun</t>
+        </is>
+      </c>
+      <c r="D277" s="0" t="inlineStr">
+        <is>
+          <t>birth_fun</t>
+        </is>
+      </c>
+      <c r="E277" s="2">
+        <v>18</v>
+      </c>
+      <c r="F277" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B278" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C278" s="0" t="inlineStr">
+        <is>
+          <t>songs</t>
+        </is>
+      </c>
+      <c r="D278" s="0" t="inlineStr">
+        <is>
+          <t>birth_songs</t>
+        </is>
+      </c>
+      <c r="E278" s="2">
+        <v>18</v>
+      </c>
+      <c r="F278" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B279" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C279" s="0" t="inlineStr">
+        <is>
+          <t>wishes</t>
+        </is>
+      </c>
+      <c r="D279" s="0" t="inlineStr">
+        <is>
+          <t>birth_wishes</t>
+        </is>
+      </c>
+      <c r="E279" s="2">
+        <v>18</v>
+      </c>
+      <c r="F279" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B280" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C280" s="0" t="inlineStr">
+        <is>
+          <t>birthday</t>
+        </is>
+      </c>
+      <c r="D280" s="0" t="inlineStr">
+        <is>
+          <t>thank_birthday</t>
+        </is>
+      </c>
+      <c r="E280" s="2">
+        <v>17</v>
+      </c>
+      <c r="F280" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B281" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C281" s="0" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="D281" s="0" t="inlineStr">
+        <is>
+          <t>friend_hello</t>
+        </is>
+      </c>
+      <c r="E281" s="2">
+        <v>13</v>
+      </c>
+      <c r="F281" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B282" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C282" s="0" t="inlineStr">
+        <is>
+          <t>thinkingofyou</t>
+        </is>
+      </c>
+      <c r="D282" s="0" t="inlineStr">
+        <is>
+          <t>gen_thinkingofyou</t>
+        </is>
+      </c>
+      <c r="E282" s="2">
+        <v>13</v>
+      </c>
+      <c r="F282" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B283" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C283" s="0" t="inlineStr">
+        <is>
+          <t>sympathy</t>
+        </is>
+      </c>
+      <c r="D283" s="0" t="inlineStr">
+        <is>
+          <t>insp_sympathy</t>
+        </is>
+      </c>
+      <c r="E283" s="2">
+        <v>13</v>
+      </c>
+      <c r="F283" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B284" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C284" s="0" t="inlineStr">
+        <is>
+          <t>friends</t>
+        </is>
+      </c>
+      <c r="D284" s="0" t="inlineStr">
+        <is>
+          <t>birth_friends</t>
+        </is>
+      </c>
+      <c r="E284" s="2">
+        <v>11</v>
+      </c>
+      <c r="F284" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B285" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C285" s="0" t="inlineStr">
+        <is>
+          <t>belated</t>
+        </is>
+      </c>
+      <c r="D285" s="0" t="inlineStr">
+        <is>
+          <t>birth_belated</t>
+        </is>
+      </c>
+      <c r="E285" s="2">
+        <v>10</v>
+      </c>
+      <c r="F285" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B286" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C286" s="0" t="inlineStr">
+        <is>
+          <t>sonanddaughter</t>
+        </is>
+      </c>
+      <c r="D286" s="0" t="inlineStr">
+        <is>
+          <t>birth_sonanddaughter</t>
+        </is>
+      </c>
+      <c r="E286" s="2">
+        <v>10</v>
+      </c>
+      <c r="F286" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B287" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C287" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D287" s="0" t="inlineStr">
+        <is>
+          <t>gen_getwell</t>
+        </is>
+      </c>
+      <c r="E287" s="2">
+        <v>9</v>
+      </c>
+      <c r="F287" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B288" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C288" s="0" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
+      <c r="D288" s="0" t="inlineStr">
+        <is>
+          <t>friend_thoughts</t>
+        </is>
+      </c>
+      <c r="E288" s="2">
+        <v>8</v>
+      </c>
+      <c r="F288" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B289" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C289" s="0" t="inlineStr">
+        <is>
+          <t>blessings</t>
+        </is>
+      </c>
+      <c r="D289" s="0" t="inlineStr">
+        <is>
+          <t>birth_blessings</t>
+        </is>
+      </c>
+      <c r="E289" s="2">
+        <v>7</v>
+      </c>
+      <c r="F289" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B290" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C290" s="0" t="inlineStr">
+        <is>
+          <t>extfamily</t>
+        </is>
+      </c>
+      <c r="D290" s="0" t="inlineStr">
+        <is>
+          <t>birth_extfamily</t>
+        </is>
+      </c>
+      <c r="E290" s="2">
+        <v>7</v>
+      </c>
+      <c r="F290" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B291" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C291" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D291" s="0" t="inlineStr">
+        <is>
+          <t>birth_milestone</t>
+        </is>
+      </c>
+      <c r="E291" s="2">
+        <v>7</v>
+      </c>
+      <c r="F291" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B292" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C292" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalwhite_wine_day</t>
+        </is>
+      </c>
+      <c r="D292" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalwhite_wine_day</t>
+        </is>
+      </c>
+      <c r="E292" s="2">
+        <v>7</v>
+      </c>
+      <c r="F292" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B293" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C293" s="0" t="inlineStr">
+        <is>
+          <t>dating</t>
+        </is>
+      </c>
+      <c r="D293" s="0" t="inlineStr">
+        <is>
+          <t>love_dating</t>
+        </is>
+      </c>
+      <c r="E293" s="2">
+        <v>6</v>
+      </c>
+      <c r="F293" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B294" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C294" s="0" t="inlineStr">
+        <is>
+          <t>hubbywife</t>
+        </is>
+      </c>
+      <c r="D294" s="0" t="inlineStr">
+        <is>
+          <t>birth_hubbywife</t>
+        </is>
+      </c>
+      <c r="E294" s="2">
+        <v>5</v>
+      </c>
+      <c r="F294" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B295" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C295" s="0" t="inlineStr">
+        <is>
+          <t>kids</t>
+        </is>
+      </c>
+      <c r="D295" s="0" t="inlineStr">
+        <is>
+          <t>birth_kids</t>
+        </is>
+      </c>
+      <c r="E295" s="2">
+        <v>5</v>
+      </c>
+      <c r="F295" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B296" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C296" s="0" t="inlineStr">
+        <is>
+          <t>eaug_cardssister</t>
+        </is>
+      </c>
+      <c r="D296" s="0" t="inlineStr">
+        <is>
+          <t>eaug_cardssister</t>
+        </is>
+      </c>
+      <c r="E296" s="2">
+        <v>5</v>
+      </c>
+      <c r="F296" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B297" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C297" s="0" t="inlineStr">
+        <is>
+          <t>eaug_coastguard_day</t>
+        </is>
+      </c>
+      <c r="D297" s="0" t="inlineStr">
+        <is>
+          <t>eaug_coastguard_day</t>
+        </is>
+      </c>
+      <c r="E297" s="2">
+        <v>4</v>
+      </c>
+      <c r="F297" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B298" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C298" s="0" t="inlineStr">
+        <is>
+          <t>sisters</t>
+        </is>
+      </c>
+      <c r="D298" s="0" t="inlineStr">
+        <is>
+          <t>fkt_sisters</t>
+        </is>
+      </c>
+      <c r="E298" s="2">
+        <v>4</v>
+      </c>
+      <c r="F298" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B299" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C299" s="0" t="inlineStr">
+        <is>
+          <t>missyou</t>
+        </is>
+      </c>
+      <c r="D299" s="0" t="inlineStr">
+        <is>
+          <t>gen_missyou</t>
+        </is>
+      </c>
+      <c r="E299" s="2">
+        <v>4</v>
+      </c>
+      <c r="F299" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B300" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C300" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="D300" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="E300" s="2">
+        <v>4</v>
+      </c>
+      <c r="F300" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B301" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C301" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_general</t>
+        </is>
+      </c>
+      <c r="D301" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_general</t>
+        </is>
+      </c>
+      <c r="E301" s="2">
+        <v>4</v>
+      </c>
+      <c r="F301" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B302" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C302" s="0" t="inlineStr">
+        <is>
+          <t>everyday</t>
+        </is>
+      </c>
+      <c r="D302" s="0" t="inlineStr">
+        <is>
+          <t>thank_everyday</t>
+        </is>
+      </c>
+      <c r="E302" s="2">
+        <v>4</v>
+      </c>
+      <c r="F302" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B303" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C303" s="0" t="inlineStr">
+        <is>
+          <t>anniversaryetc</t>
+        </is>
+      </c>
+      <c r="D303" s="0" t="inlineStr">
+        <is>
+          <t>anniv_anniversaryetc</t>
+        </is>
+      </c>
+      <c r="E303" s="2">
+        <v>3</v>
+      </c>
+      <c r="F303" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B304" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C304" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_family</t>
+        </is>
+      </c>
+      <c r="D304" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_family</t>
+        </is>
+      </c>
+      <c r="E304" s="2">
+        <v>3</v>
+      </c>
+      <c r="F304" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B305" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C305" s="0" t="inlineStr">
+        <is>
+          <t>foreveryone</t>
+        </is>
+      </c>
+      <c r="D305" s="0" t="inlineStr">
+        <is>
+          <t>congrats_foreveryone</t>
+        </is>
+      </c>
+      <c r="E305" s="2">
+        <v>3</v>
+      </c>
+      <c r="F305" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B306" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C306" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="D306" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="E306" s="2">
+        <v>3</v>
+      </c>
+      <c r="F306" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B307" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C307" s="0" t="inlineStr">
+        <is>
+          <t>youarespecial</t>
+        </is>
+      </c>
+      <c r="D307" s="0" t="inlineStr">
+        <is>
+          <t>love_youarespecial</t>
+        </is>
+      </c>
+      <c r="E307" s="2">
+        <v>3</v>
+      </c>
+      <c r="F307" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B308" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C308" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="D308" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="E308" s="2">
+        <v>2</v>
+      </c>
+      <c r="F308" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B309" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C309" s="0" t="inlineStr">
+        <is>
+          <t>flowers</t>
+        </is>
+      </c>
+      <c r="D309" s="0" t="inlineStr">
+        <is>
+          <t>birth_flowers</t>
+        </is>
+      </c>
+      <c r="E309" s="2">
+        <v>2</v>
+      </c>
+      <c r="F309" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B310" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C310" s="0" t="inlineStr">
+        <is>
+          <t>goodnight</t>
+        </is>
+      </c>
+      <c r="D310" s="0" t="inlineStr">
+        <is>
+          <t>gen_goodnight</t>
+        </is>
+      </c>
+      <c r="E310" s="2">
+        <v>2</v>
+      </c>
+      <c r="F310" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B311" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C311" s="0" t="inlineStr">
+        <is>
+          <t>hvgtday</t>
+        </is>
+      </c>
+      <c r="D311" s="0" t="inlineStr">
+        <is>
+          <t>gen_hvgtday</t>
+        </is>
+      </c>
+      <c r="E311" s="2">
+        <v>2</v>
+      </c>
+      <c r="F311" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B312" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C312" s="0" t="inlineStr">
+        <is>
+          <t>morning</t>
+        </is>
+      </c>
+      <c r="D312" s="0" t="inlineStr">
+        <is>
+          <t>gen_morning</t>
+        </is>
+      </c>
+      <c r="E312" s="2">
+        <v>2</v>
+      </c>
+      <c r="F312" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B313" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C313" s="0" t="inlineStr">
+        <is>
+          <t>cute</t>
+        </is>
+      </c>
+      <c r="D313" s="0" t="inlineStr">
+        <is>
+          <t>love_cute</t>
+        </is>
+      </c>
+      <c r="E313" s="2">
+        <v>2</v>
+      </c>
+      <c r="F313" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B314" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C314" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D314" s="0" t="inlineStr">
+        <is>
+          <t>thank_love</t>
+        </is>
+      </c>
+      <c r="E314" s="2">
+        <v>2</v>
+      </c>
+      <c r="F314" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B315" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C315" s="0" t="inlineStr">
+        <is>
+          <t>wedding</t>
+        </is>
+      </c>
+      <c r="D315" s="0" t="inlineStr">
+        <is>
+          <t>thank_wedding</t>
+        </is>
+      </c>
+      <c r="E315" s="2">
+        <v>2</v>
+      </c>
+      <c r="F315" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B316" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C316" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D316" s="0" t="inlineStr">
+        <is>
+          <t>anniv_milestone</t>
+        </is>
+      </c>
+      <c r="E316" s="2">
+        <v>1</v>
+      </c>
+      <c r="F316" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B317" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C317" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="D317" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="E317" s="2">
+        <v>1</v>
+      </c>
+      <c r="F317" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B318" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C318" s="0" t="inlineStr">
+        <is>
+          <t>collassociates</t>
+        </is>
+      </c>
+      <c r="D318" s="0" t="inlineStr">
+        <is>
+          <t>birth_collassociates</t>
+        </is>
+      </c>
+      <c r="E318" s="2">
+        <v>1</v>
+      </c>
+      <c r="F318" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B319" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C319" s="0" t="inlineStr">
+        <is>
+          <t>missyou</t>
+        </is>
+      </c>
+      <c r="D319" s="0" t="inlineStr">
+        <is>
+          <t>birth_missyou</t>
+        </is>
+      </c>
+      <c r="E319" s="2">
+        <v>1</v>
+      </c>
+      <c r="F319" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B320" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C320" s="0" t="inlineStr">
+        <is>
+          <t>businessandworkplace</t>
+        </is>
+      </c>
+      <c r="D320" s="0" t="inlineStr">
+        <is>
+          <t>congrats_businessandworkplace</t>
+        </is>
+      </c>
+      <c r="E320" s="2">
+        <v>1</v>
+      </c>
+      <c r="F320" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B321" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C321" s="0" t="inlineStr">
+        <is>
+          <t>teddy</t>
+        </is>
+      </c>
+      <c r="D321" s="0" t="inlineStr">
+        <is>
+          <t>cute_teddy</t>
+        </is>
+      </c>
+      <c r="E321" s="2">
+        <v>1</v>
+      </c>
+      <c r="F321" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B322" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C322" s="0" t="inlineStr">
+        <is>
+          <t>eaug_beachparty_day</t>
+        </is>
+      </c>
+      <c r="D322" s="0" t="inlineStr">
+        <is>
+          <t>eaug_beachparty_day</t>
+        </is>
+      </c>
+      <c r="E322" s="2">
+        <v>1</v>
+      </c>
+      <c r="F322" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B323" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C323" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_happy</t>
+        </is>
+      </c>
+      <c r="D323" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_happy</t>
+        </is>
+      </c>
+      <c r="E323" s="2">
+        <v>1</v>
+      </c>
+      <c r="F323" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B324" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C324" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="D324" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="E324" s="2">
+        <v>1</v>
+      </c>
+      <c r="F324" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B325" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C325" s="0" t="inlineStr">
+        <is>
+          <t>eaug_internationalyouth_day</t>
+        </is>
+      </c>
+      <c r="D325" s="0" t="inlineStr">
+        <is>
+          <t>eaug_internationalyouth_day</t>
+        </is>
+      </c>
+      <c r="E325" s="2">
+        <v>1</v>
+      </c>
+      <c r="F325" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B326" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C326" s="0" t="inlineStr">
+        <is>
+          <t>eaug_justbecauseday</t>
+        </is>
+      </c>
+      <c r="D326" s="0" t="inlineStr">
+        <is>
+          <t>eaug_justbecauseday</t>
+        </is>
+      </c>
+      <c r="E326" s="2">
+        <v>1</v>
+      </c>
+      <c r="F326" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B327" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C327" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalchocolate_chip_cookie_day</t>
+        </is>
+      </c>
+      <c r="D327" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalchocolate_chip_cookie_day</t>
+        </is>
+      </c>
+      <c r="E327" s="2">
+        <v>1</v>
+      </c>
+      <c r="F327" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B328" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C328" s="0" t="inlineStr">
+        <is>
+          <t>ejan_thankyoucards</t>
+        </is>
+      </c>
+      <c r="D328" s="0" t="inlineStr">
+        <is>
+          <t>ejan_thankyoucards</t>
+        </is>
+      </c>
+      <c r="E328" s="2">
+        <v>1</v>
+      </c>
+      <c r="F328" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B329" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C329" s="0" t="inlineStr">
+        <is>
+          <t>ejun_friendinneed</t>
+        </is>
+      </c>
+      <c r="D329" s="0" t="inlineStr">
+        <is>
+          <t>ejun_friendinneed</t>
+        </is>
+      </c>
+      <c r="E329" s="2">
+        <v>1</v>
+      </c>
+      <c r="F329" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B330" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C330" s="0" t="inlineStr">
+        <is>
+          <t>enov_allsaintsday</t>
+        </is>
+      </c>
+      <c r="D330" s="0" t="inlineStr">
+        <is>
+          <t>enov_allsaintsday</t>
+        </is>
+      </c>
+      <c r="E330" s="2">
+        <v>1</v>
+      </c>
+      <c r="F330" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B331" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C331" s="0" t="inlineStr">
+        <is>
+          <t>eoct_sweetday_missyou</t>
+        </is>
+      </c>
+      <c r="D331" s="0" t="inlineStr">
+        <is>
+          <t>eoct_sweetday_missyou</t>
+        </is>
+      </c>
+      <c r="E331" s="2">
+        <v>1</v>
+      </c>
+      <c r="F331" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B332" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C332" s="0" t="inlineStr">
+        <is>
+          <t>esep_allangelsday</t>
+        </is>
+      </c>
+      <c r="D332" s="0" t="inlineStr">
+        <is>
+          <t>esep_allangelsday</t>
+        </is>
+      </c>
+      <c r="E332" s="2">
+        <v>1</v>
+      </c>
+      <c r="F332" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B333" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C333" s="0" t="inlineStr">
+        <is>
+          <t>huswife</t>
+        </is>
+      </c>
+      <c r="D333" s="0" t="inlineStr">
+        <is>
+          <t>fkt_huswife</t>
+        </is>
+      </c>
+      <c r="E333" s="2">
+        <v>1</v>
+      </c>
+      <c r="F333" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B334" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C334" s="0" t="inlineStr">
+        <is>
+          <t>bestfriends</t>
+        </is>
+      </c>
+      <c r="D334" s="0" t="inlineStr">
+        <is>
+          <t>friend_bestfriends</t>
+        </is>
+      </c>
+      <c r="E334" s="2">
+        <v>1</v>
+      </c>
+      <c r="F334" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B335" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C335" s="0" t="inlineStr">
+        <is>
+          <t>joke</t>
+        </is>
+      </c>
+      <c r="D335" s="0" t="inlineStr">
+        <is>
+          <t>gen_joke</t>
+        </is>
+      </c>
+      <c r="E335" s="2">
+        <v>1</v>
+      </c>
+      <c r="F335" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B336" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C336" s="0" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="D336" s="0" t="inlineStr">
+        <is>
+          <t>gen_luck</t>
+        </is>
+      </c>
+      <c r="E336" s="2">
+        <v>1</v>
+      </c>
+      <c r="F336" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B337" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C337" s="0" t="inlineStr">
+        <is>
+          <t>angels</t>
+        </is>
+      </c>
+      <c r="D337" s="0" t="inlineStr">
+        <is>
+          <t>insp_angels</t>
+        </is>
+      </c>
+      <c r="E337" s="2">
+        <v>1</v>
+      </c>
+      <c r="F337" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B338" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C338" s="0" t="inlineStr">
+        <is>
+          <t>recovery</t>
+        </is>
+      </c>
+      <c r="D338" s="0" t="inlineStr">
+        <is>
+          <t>insp_recovery</t>
+        </is>
+      </c>
+      <c r="E338" s="2">
+        <v>1</v>
+      </c>
+      <c r="F338" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B339" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C339" s="0" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="D339" s="0" t="inlineStr">
+        <is>
+          <t>intouch_hi</t>
+        </is>
+      </c>
+      <c r="E339" s="2">
+        <v>1</v>
+      </c>
+      <c r="F339" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B340" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C340" s="0" t="inlineStr">
+        <is>
+          <t>foreverlove</t>
+        </is>
+      </c>
+      <c r="D340" s="0" t="inlineStr">
+        <is>
+          <t>love_foreverlove</t>
+        </is>
+      </c>
+      <c r="E340" s="2">
+        <v>1</v>
+      </c>
+      <c r="F340" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B341" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C341" s="0" t="inlineStr">
+        <is>
+          <t>hugs</t>
+        </is>
+      </c>
+      <c r="D341" s="0" t="inlineStr">
+        <is>
+          <t>love_hugs</t>
+        </is>
+      </c>
+      <c r="E341" s="2">
+        <v>1</v>
+      </c>
+      <c r="F341" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B342" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C342" s="0" t="inlineStr">
+        <is>
+          <t>iamsorry</t>
+        </is>
+      </c>
+      <c r="D342" s="0" t="inlineStr">
+        <is>
+          <t>love_iamsorry</t>
+        </is>
+      </c>
+      <c r="E342" s="2">
+        <v>1</v>
+      </c>
+      <c r="F342" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B343" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C343" s="0" t="inlineStr">
+        <is>
+          <t>newlove</t>
+        </is>
+      </c>
+      <c r="D343" s="0" t="inlineStr">
+        <is>
+          <t>love_newlove</t>
+        </is>
+      </c>
+      <c r="E343" s="2">
+        <v>1</v>
+      </c>
+      <c r="F343" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B344" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C344" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D344" s="0" t="inlineStr">
+        <is>
+          <t>pet_getwell</t>
+        </is>
+      </c>
+      <c r="E344" s="2">
+        <v>1</v>
+      </c>
+      <c r="F344" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B345" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C345" s="0" t="inlineStr">
+        <is>
+          <t>lossofpet</t>
+        </is>
+      </c>
+      <c r="D345" s="0" t="inlineStr">
+        <is>
+          <t>pet_lossofpet</t>
+        </is>
+      </c>
+      <c r="E345" s="2">
+        <v>1</v>
+      </c>
+      <c r="F345" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B346" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C346" s="0" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="D346" s="0" t="inlineStr">
+        <is>
+          <t>thank_family</t>
+        </is>
+      </c>
+      <c r="E346" s="2">
+        <v>1</v>
+      </c>
+      <c r="F346" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B347" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C347" s="0" t="inlineStr">
+        <is>
+          <t>friendship</t>
+        </is>
+      </c>
+      <c r="D347" s="0" t="inlineStr">
+        <is>
+          <t>thank_friendship</t>
+        </is>
+      </c>
+      <c r="E347" s="2">
+        <v>1</v>
+      </c>
+      <c r="F347" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B348" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C348" s="0" t="inlineStr">
+        <is>
+          <t>inspirational</t>
+        </is>
+      </c>
+      <c r="D348" s="0" t="inlineStr">
+        <is>
+          <t>thank_inspirational</t>
+        </is>
+      </c>
+      <c r="E348" s="2">
+        <v>1</v>
+      </c>
+      <c r="F348" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B349" s="0" t="inlineStr">
+        <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="C349" s="0" t="inlineStr">
+        <is>
+          <t>german_birthday</t>
+        </is>
+      </c>
+      <c r="D349" s="0" t="inlineStr">
+        <is>
+          <t>w_german_birthday</t>
+        </is>
+      </c>
+      <c r="E349" s="2">
+        <v>1</v>
+      </c>
+      <c r="F349" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B350" s="0" t="inlineStr">
+        <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="C350" s="0" t="inlineStr">
+        <is>
+          <t>spanish_love</t>
+        </is>
+      </c>
+      <c r="D350" s="0" t="inlineStr">
+        <is>
+          <t>w_spanish_love</t>
+        </is>
+      </c>
+      <c r="E350" s="2">
+        <v>1</v>
+      </c>
+      <c r="F350" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B351" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C351" s="0" t="inlineStr">
+        <is>
+          <t>wed_weddingetc</t>
+        </is>
+      </c>
+      <c r="D351" s="0" t="inlineStr">
+        <is>
+          <t>wed_weddingetc</t>
+        </is>
+      </c>
+      <c r="E351" s="2">
+        <v>1</v>
+      </c>
+      <c r="F351" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B352" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C352" s="0" t="inlineStr">
+        <is>
+          <t>wed_wishes</t>
+        </is>
+      </c>
+      <c r="D352" s="0" t="inlineStr">
+        <is>
+          <t>wed_wishes</t>
+        </is>
+      </c>
+      <c r="E352" s="2">
+        <v>1</v>
+      </c>
+      <c r="F352" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-04</t>
+        </is>
+      </c>
+      <c r="B353" s="4"/>
+      <c r="C353" s="4"/>
+      <c r="D353" s="4"/>
+      <c r="E353" s="5">
+        <v>770</v>
+      </c>
+      <c r="F353" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -9879,12 +12661,12 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Telegram</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Facebook</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -9920,10 +12702,10 @@
         <v>108</v>
       </c>
       <c r="G2" s="2">
+        <v>31</v>
+      </c>
+      <c r="H2" s="2">
         <v>47</v>
-      </c>
-      <c r="H2" s="2">
-        <v>31</v>
       </c>
       <c r="I2" s="2">
         <v>12</v>
@@ -9954,10 +12736,10 @@
         <v>118</v>
       </c>
       <c r="G3" s="2">
+        <v>34</v>
+      </c>
+      <c r="H3" s="2">
         <v>38</v>
-      </c>
-      <c r="H3" s="2">
-        <v>34</v>
       </c>
       <c r="I3" s="2">
         <v>13</v>
@@ -9988,10 +12770,10 @@
         <v>84</v>
       </c>
       <c r="G4" s="2">
+        <v>31</v>
+      </c>
+      <c r="H4" s="2">
         <v>19</v>
-      </c>
-      <c r="H4" s="2">
-        <v>31</v>
       </c>
       <c r="I4" s="2">
         <v>3</v>
@@ -10001,36 +12783,70 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B5" s="2">
+        <v>805</v>
+      </c>
+      <c r="C5" s="2">
+        <v>247</v>
+      </c>
+      <c r="D5" s="2">
+        <v>268</v>
+      </c>
+      <c r="E5" s="2">
+        <v>160</v>
+      </c>
+      <c r="F5" s="2">
+        <v>72</v>
+      </c>
+      <c r="G5" s="2">
+        <v>38</v>
+      </c>
+      <c r="H5" s="2">
+        <v>20</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B5" s="5">
-        <v>2823</v>
-      </c>
-      <c r="C5" s="5">
-        <v>1001</v>
-      </c>
-      <c r="D5" s="5">
-        <v>784</v>
-      </c>
-      <c r="E5" s="5">
-        <v>499</v>
-      </c>
-      <c r="F5" s="5">
-        <v>310</v>
-      </c>
-      <c r="G5" s="5">
-        <v>104</v>
-      </c>
-      <c r="H5" s="5">
-        <v>96</v>
-      </c>
-      <c r="I5" s="5">
+      <c r="B6" s="5">
+        <v>3628</v>
+      </c>
+      <c r="C6" s="5">
+        <v>1248</v>
+      </c>
+      <c r="D6" s="5">
+        <v>1052</v>
+      </c>
+      <c r="E6" s="5">
+        <v>659</v>
+      </c>
+      <c r="F6" s="5">
+        <v>382</v>
+      </c>
+      <c r="G6" s="5">
+        <v>134</v>
+      </c>
+      <c r="H6" s="5">
+        <v>124</v>
+      </c>
+      <c r="I6" s="5">
         <v>28</v>
       </c>
-      <c r="J5" s="5">
+      <c r="J6" s="5">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Record 8 August: 839 sends, eight days now tracked
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9KsXegBwxB1sWdCzRVLrr
</commit_message>
<xml_diff>
--- a/reports/daily_tracking.xlsx
+++ b/reports/daily_tracking.xlsx
@@ -224,7 +224,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
@@ -247,7 +247,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
@@ -507,28 +507,56 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B9" s="2">
+        <v>839</v>
+      </c>
+      <c r="C9" s="2">
+        <v>576</v>
+      </c>
+      <c r="D9" s="2">
+        <v>263</v>
+      </c>
+      <c r="E9" s="2">
+        <v>776</v>
+      </c>
+      <c r="F9" s="2">
+        <v>63</v>
+      </c>
+      <c r="G9" s="2">
+        <v>257</v>
+      </c>
+      <c r="H9" s="2">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="5">
-        <v>5868</v>
-      </c>
-      <c r="C9" s="5">
-        <v>3726</v>
-      </c>
-      <c r="D9" s="5">
-        <v>2142</v>
-      </c>
-      <c r="E9" s="5">
-        <v>5620</v>
-      </c>
-      <c r="F9" s="5">
-        <v>248</v>
-      </c>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
+      <c r="B10" s="5">
+        <v>6707</v>
+      </c>
+      <c r="C10" s="5">
+        <v>4302</v>
+      </c>
+      <c r="D10" s="5">
+        <v>2405</v>
+      </c>
+      <c r="E10" s="5">
+        <v>6396</v>
+      </c>
+      <c r="F10" s="5">
+        <v>311</v>
+      </c>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -544,17 +572,17 @@
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
     <col min="10" max="10" width="24" customWidth="1"/>
     <col min="11" max="11" width="17" customWidth="1"/>
     <col min="12" max="12" width="11" customWidth="1"/>
     <col min="13" max="13" width="21" customWidth="1"/>
-    <col min="14" max="14" width="17" customWidth="1"/>
-    <col min="15" max="15" width="11" customWidth="1"/>
+    <col min="14" max="14" width="11" customWidth="1"/>
+    <col min="15" max="15" width="17" customWidth="1"/>
     <col min="16" max="16" width="11" customWidth="1"/>
-    <col min="17" max="17" width="18" customWidth="1"/>
-    <col min="18" max="18" width="17" customWidth="1"/>
+    <col min="17" max="17" width="17" customWidth="1"/>
+    <col min="18" max="18" width="18" customWidth="1"/>
     <col min="19" max="19" width="23" customWidth="1"/>
   </cols>
   <sheetData>
@@ -596,14 +624,14 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Friendship</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Love &amp; romance</t>
-        </is>
-      </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Inspirational &amp; sympathy</t>
@@ -626,14 +654,14 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>World languages</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Pets</t>
-        </is>
-      </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Cute</t>
@@ -641,12 +669,12 @@
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>Keeping in touch</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Business &amp; work</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
@@ -680,10 +708,10 @@
         <v>30</v>
       </c>
       <c r="H2" s="2">
+        <v>19</v>
+      </c>
+      <c r="I2" s="2">
         <v>28</v>
-      </c>
-      <c r="I2" s="2">
-        <v>19</v>
       </c>
       <c r="J2" s="2">
         <v>10</v>
@@ -698,19 +726,19 @@
         <v>3</v>
       </c>
       <c r="N2" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O2" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P2" s="2">
         <v>4</v>
       </c>
       <c r="Q2" s="2">
+        <v>2</v>
+      </c>
+      <c r="R2" s="2">
         <v>6</v>
-      </c>
-      <c r="R2" s="2">
-        <v>2</v>
       </c>
       <c r="S2" s="2">
         <v>0</v>
@@ -741,10 +769,10 @@
         <v>52</v>
       </c>
       <c r="H3" s="2">
+        <v>24</v>
+      </c>
+      <c r="I3" s="2">
         <v>41</v>
-      </c>
-      <c r="I3" s="2">
-        <v>24</v>
       </c>
       <c r="J3" s="2">
         <v>19</v>
@@ -759,19 +787,19 @@
         <v>3</v>
       </c>
       <c r="N3" s="2">
+        <v>1</v>
+      </c>
+      <c r="O3" s="2">
         <v>10</v>
       </c>
-      <c r="O3" s="2">
-        <v>1</v>
-      </c>
       <c r="P3" s="2">
         <v>1</v>
       </c>
       <c r="Q3" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R3" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S3" s="2">
         <v>0</v>
@@ -802,10 +830,10 @@
         <v>30</v>
       </c>
       <c r="H4" s="2">
+        <v>18</v>
+      </c>
+      <c r="I4" s="2">
         <v>11</v>
-      </c>
-      <c r="I4" s="2">
-        <v>18</v>
       </c>
       <c r="J4" s="2">
         <v>16</v>
@@ -863,10 +891,10 @@
         <v>28</v>
       </c>
       <c r="H5" s="2">
+        <v>26</v>
+      </c>
+      <c r="I5" s="2">
         <v>22</v>
-      </c>
-      <c r="I5" s="2">
-        <v>26</v>
       </c>
       <c r="J5" s="2">
         <v>15</v>
@@ -890,10 +918,10 @@
         <v>1</v>
       </c>
       <c r="Q5" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R5" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S5" s="2">
         <v>0</v>
@@ -924,10 +952,10 @@
         <v>24</v>
       </c>
       <c r="H6" s="2">
+        <v>13</v>
+      </c>
+      <c r="I6" s="2">
         <v>11</v>
-      </c>
-      <c r="I6" s="2">
-        <v>13</v>
       </c>
       <c r="J6" s="2">
         <v>15</v>
@@ -942,19 +970,19 @@
         <v>1</v>
       </c>
       <c r="N6" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O6" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P6" s="2">
         <v>0</v>
       </c>
       <c r="Q6" s="2">
+        <v>2</v>
+      </c>
+      <c r="R6" s="2">
         <v>0</v>
-      </c>
-      <c r="R6" s="2">
-        <v>2</v>
       </c>
       <c r="S6" s="2">
         <v>1</v>
@@ -985,10 +1013,10 @@
         <v>20</v>
       </c>
       <c r="H7" s="2">
+        <v>11</v>
+      </c>
+      <c r="I7" s="2">
         <v>16</v>
-      </c>
-      <c r="I7" s="2">
-        <v>11</v>
       </c>
       <c r="J7" s="2">
         <v>12</v>
@@ -1003,19 +1031,19 @@
         <v>8</v>
       </c>
       <c r="N7" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O7" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P7" s="2">
         <v>0</v>
       </c>
       <c r="Q7" s="2">
+        <v>3</v>
+      </c>
+      <c r="R7" s="2">
         <v>0</v>
-      </c>
-      <c r="R7" s="2">
-        <v>3</v>
       </c>
       <c r="S7" s="2">
         <v>0</v>
@@ -1046,10 +1074,10 @@
         <v>30</v>
       </c>
       <c r="H8" s="2">
+        <v>17</v>
+      </c>
+      <c r="I8" s="2">
         <v>7</v>
-      </c>
-      <c r="I8" s="2">
-        <v>17</v>
       </c>
       <c r="J8" s="2">
         <v>14</v>
@@ -1064,82 +1092,143 @@
         <v>6</v>
       </c>
       <c r="N8" s="2">
+        <v>3</v>
+      </c>
+      <c r="O8" s="2">
         <v>0</v>
       </c>
-      <c r="O8" s="2">
+      <c r="P8" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="2">
+        <v>1</v>
+      </c>
+      <c r="R8" s="2">
+        <v>0</v>
+      </c>
+      <c r="S8" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B9" s="2">
+        <v>776</v>
+      </c>
+      <c r="C9" s="2">
+        <v>500</v>
+      </c>
+      <c r="D9" s="2">
+        <v>48</v>
+      </c>
+      <c r="E9" s="2">
+        <v>52</v>
+      </c>
+      <c r="F9" s="2">
+        <v>42</v>
+      </c>
+      <c r="G9" s="2">
+        <v>41</v>
+      </c>
+      <c r="H9" s="2">
+        <v>20</v>
+      </c>
+      <c r="I9" s="2">
+        <v>5</v>
+      </c>
+      <c r="J9" s="2">
+        <v>12</v>
+      </c>
+      <c r="K9" s="2">
+        <v>8</v>
+      </c>
+      <c r="L9" s="2">
+        <v>39</v>
+      </c>
+      <c r="M9" s="2">
+        <v>1</v>
+      </c>
+      <c r="N9" s="2">
+        <v>4</v>
+      </c>
+      <c r="O9" s="2">
+        <v>0</v>
+      </c>
+      <c r="P9" s="2">
         <v>3</v>
       </c>
-      <c r="P8" s="2">
-        <v>1</v>
-      </c>
-      <c r="Q8" s="2">
+      <c r="Q9" s="2">
+        <v>1</v>
+      </c>
+      <c r="R9" s="2">
         <v>0</v>
       </c>
-      <c r="R8" s="2">
-        <v>1</v>
-      </c>
-      <c r="S8" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="S9" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="5">
-        <v>5620</v>
-      </c>
-      <c r="C9" s="5">
-        <v>3697</v>
-      </c>
-      <c r="D9" s="5">
-        <v>588</v>
-      </c>
-      <c r="E9" s="5">
-        <v>328</v>
-      </c>
-      <c r="F9" s="5">
-        <v>238</v>
-      </c>
-      <c r="G9" s="5">
-        <v>214</v>
-      </c>
-      <c r="H9" s="5">
-        <v>136</v>
-      </c>
-      <c r="I9" s="5">
-        <v>128</v>
-      </c>
-      <c r="J9" s="5">
-        <v>101</v>
-      </c>
-      <c r="K9" s="5">
-        <v>70</v>
-      </c>
-      <c r="L9" s="5">
-        <v>32</v>
-      </c>
-      <c r="M9" s="5">
-        <v>26</v>
-      </c>
-      <c r="N9" s="5">
+      <c r="B10" s="5">
+        <v>6396</v>
+      </c>
+      <c r="C10" s="5">
+        <v>4197</v>
+      </c>
+      <c r="D10" s="5">
+        <v>636</v>
+      </c>
+      <c r="E10" s="5">
+        <v>380</v>
+      </c>
+      <c r="F10" s="5">
+        <v>280</v>
+      </c>
+      <c r="G10" s="5">
+        <v>255</v>
+      </c>
+      <c r="H10" s="5">
+        <v>148</v>
+      </c>
+      <c r="I10" s="5">
+        <v>141</v>
+      </c>
+      <c r="J10" s="5">
+        <v>113</v>
+      </c>
+      <c r="K10" s="5">
+        <v>78</v>
+      </c>
+      <c r="L10" s="5">
+        <v>71</v>
+      </c>
+      <c r="M10" s="5">
+        <v>27</v>
+      </c>
+      <c r="N10" s="5">
+        <v>19</v>
+      </c>
+      <c r="O10" s="5">
         <v>16</v>
       </c>
-      <c r="O9" s="5">
+      <c r="P10" s="5">
         <v>15</v>
       </c>
-      <c r="P9" s="5">
-        <v>12</v>
-      </c>
-      <c r="Q9" s="5">
+      <c r="Q10" s="5">
         <v>9</v>
       </c>
-      <c r="R9" s="5">
-        <v>8</v>
-      </c>
-      <c r="S9" s="5">
+      <c r="R10" s="5">
+        <v>9</v>
+      </c>
+      <c r="S10" s="5">
         <v>2</v>
       </c>
     </row>
@@ -4492,6 +4581,476 @@
       </c>
       <c r="H106" s="4"/>
     </row>
+    <row r="107">
+      <c r="A107" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B107" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C107" s="0" t="inlineStr">
+        <is>
+          <t>birth</t>
+        </is>
+      </c>
+      <c r="D107" s="2">
+        <v>372</v>
+      </c>
+      <c r="E107" s="2">
+        <v>128</v>
+      </c>
+      <c r="F107" s="2">
+        <v>500</v>
+      </c>
+      <c r="G107" s="3">
+        <v>0.6443298969072165</v>
+      </c>
+      <c r="H107" s="2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B108" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C108" s="0" t="inlineStr">
+        <is>
+          <t>anniv</t>
+        </is>
+      </c>
+      <c r="D108" s="2">
+        <v>36</v>
+      </c>
+      <c r="E108" s="2">
+        <v>16</v>
+      </c>
+      <c r="F108" s="2">
+        <v>52</v>
+      </c>
+      <c r="G108" s="3">
+        <v>0.06701030927835051</v>
+      </c>
+      <c r="H108" s="2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B109" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C109" s="0" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="D109" s="2">
+        <v>40</v>
+      </c>
+      <c r="E109" s="2">
+        <v>8</v>
+      </c>
+      <c r="F109" s="2">
+        <v>48</v>
+      </c>
+      <c r="G109" s="3">
+        <v>0.061855670103092786</v>
+      </c>
+      <c r="H109" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B110" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C110" s="0" t="inlineStr">
+        <is>
+          <t>gen</t>
+        </is>
+      </c>
+      <c r="D110" s="2">
+        <v>28</v>
+      </c>
+      <c r="E110" s="2">
+        <v>14</v>
+      </c>
+      <c r="F110" s="2">
+        <v>42</v>
+      </c>
+      <c r="G110" s="3">
+        <v>0.05412371134020619</v>
+      </c>
+      <c r="H110" s="2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B111" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C111" s="0" t="inlineStr">
+        <is>
+          <t>thank</t>
+        </is>
+      </c>
+      <c r="D111" s="2">
+        <v>18</v>
+      </c>
+      <c r="E111" s="2">
+        <v>23</v>
+      </c>
+      <c r="F111" s="2">
+        <v>41</v>
+      </c>
+      <c r="G111" s="3">
+        <v>0.05283505154639175</v>
+      </c>
+      <c r="H111" s="2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B112" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C112" s="0" t="inlineStr">
+        <is>
+          <t>flwr</t>
+        </is>
+      </c>
+      <c r="D112" s="2">
+        <v>38</v>
+      </c>
+      <c r="E112" s="2">
+        <v>1</v>
+      </c>
+      <c r="F112" s="2">
+        <v>39</v>
+      </c>
+      <c r="G112" s="3">
+        <v>0.05025773195876289</v>
+      </c>
+      <c r="H112" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B113" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C113" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D113" s="2">
+        <v>14</v>
+      </c>
+      <c r="E113" s="2">
+        <v>6</v>
+      </c>
+      <c r="F113" s="2">
+        <v>20</v>
+      </c>
+      <c r="G113" s="3">
+        <v>0.02577319587628866</v>
+      </c>
+      <c r="H113" s="2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B114" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C114" s="0" t="inlineStr">
+        <is>
+          <t>insp</t>
+        </is>
+      </c>
+      <c r="D114" s="2">
+        <v>10</v>
+      </c>
+      <c r="E114" s="2">
+        <v>2</v>
+      </c>
+      <c r="F114" s="2">
+        <v>12</v>
+      </c>
+      <c r="G114" s="3">
+        <v>0.015463917525773196</v>
+      </c>
+      <c r="H114" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B115" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C115" s="0" t="inlineStr">
+        <is>
+          <t>congrats</t>
+        </is>
+      </c>
+      <c r="D115" s="2">
+        <v>6</v>
+      </c>
+      <c r="E115" s="2">
+        <v>2</v>
+      </c>
+      <c r="F115" s="2">
+        <v>8</v>
+      </c>
+      <c r="G115" s="3">
+        <v>0.010309278350515464</v>
+      </c>
+      <c r="H115" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B116" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C116" s="0" t="inlineStr">
+        <is>
+          <t>friend</t>
+        </is>
+      </c>
+      <c r="D116" s="2">
+        <v>5</v>
+      </c>
+      <c r="E116" s="2">
+        <v>0</v>
+      </c>
+      <c r="F116" s="2">
+        <v>5</v>
+      </c>
+      <c r="G116" s="3">
+        <v>0.006443298969072165</v>
+      </c>
+      <c r="H116" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B117" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C117" s="0" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="D117" s="2">
+        <v>4</v>
+      </c>
+      <c r="E117" s="2">
+        <v>0</v>
+      </c>
+      <c r="F117" s="2">
+        <v>4</v>
+      </c>
+      <c r="G117" s="3">
+        <v>0.005154639175257732</v>
+      </c>
+      <c r="H117" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B118" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C118" s="0" t="inlineStr">
+        <is>
+          <t>cute</t>
+        </is>
+      </c>
+      <c r="D118" s="2">
+        <v>3</v>
+      </c>
+      <c r="E118" s="2">
+        <v>0</v>
+      </c>
+      <c r="F118" s="2">
+        <v>3</v>
+      </c>
+      <c r="G118" s="3">
+        <v>0.003865979381443299</v>
+      </c>
+      <c r="H118" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B119" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C119" s="0" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+      <c r="D119" s="2">
+        <v>1</v>
+      </c>
+      <c r="E119" s="2">
+        <v>0</v>
+      </c>
+      <c r="F119" s="2">
+        <v>1</v>
+      </c>
+      <c r="G119" s="3">
+        <v>0.001288659793814433</v>
+      </c>
+      <c r="H119" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B120" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C120" s="0" t="inlineStr">
+        <is>
+          <t>fkt</t>
+        </is>
+      </c>
+      <c r="D120" s="2">
+        <v>1</v>
+      </c>
+      <c r="E120" s="2">
+        <v>0</v>
+      </c>
+      <c r="F120" s="2">
+        <v>1</v>
+      </c>
+      <c r="G120" s="3">
+        <v>0.001288659793814433</v>
+      </c>
+      <c r="H120" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-08</t>
+        </is>
+      </c>
+      <c r="B121" s="4"/>
+      <c r="C121" s="4"/>
+      <c r="D121" s="5">
+        <v>576</v>
+      </c>
+      <c r="E121" s="5">
+        <v>200</v>
+      </c>
+      <c r="F121" s="5">
+        <v>776</v>
+      </c>
+      <c r="G121" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="H121" s="4"/>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -20820,6 +21379,2260 @@
         <v>731</v>
       </c>
       <c r="F586" s="4"/>
+    </row>
+    <row r="587">
+      <c r="A587" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B587" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C587" s="0" t="inlineStr">
+        <is>
+          <t>happybirthday</t>
+        </is>
+      </c>
+      <c r="D587" s="0" t="inlineStr">
+        <is>
+          <t>birth_happybirthday</t>
+        </is>
+      </c>
+      <c r="E587" s="2">
+        <v>403</v>
+      </c>
+      <c r="F587" s="2">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B588" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C588" s="0" t="inlineStr">
+        <is>
+          <t>flrwishes</t>
+        </is>
+      </c>
+      <c r="D588" s="0" t="inlineStr">
+        <is>
+          <t>flwr_flrwishes</t>
+        </is>
+      </c>
+      <c r="E588" s="2">
+        <v>38</v>
+      </c>
+      <c r="F588" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B589" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C589" s="0" t="inlineStr">
+        <is>
+          <t>anniversaryetc</t>
+        </is>
+      </c>
+      <c r="D589" s="0" t="inlineStr">
+        <is>
+          <t>anniv_anniversaryetc</t>
+        </is>
+      </c>
+      <c r="E589" s="2">
+        <v>36</v>
+      </c>
+      <c r="F589" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B590" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C590" s="0" t="inlineStr">
+        <is>
+          <t>birthday</t>
+        </is>
+      </c>
+      <c r="D590" s="0" t="inlineStr">
+        <is>
+          <t>thank_birthday</t>
+        </is>
+      </c>
+      <c r="E590" s="2">
+        <v>26</v>
+      </c>
+      <c r="F590" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B591" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C591" s="0" t="inlineStr">
+        <is>
+          <t>fun</t>
+        </is>
+      </c>
+      <c r="D591" s="0" t="inlineStr">
+        <is>
+          <t>birth_fun</t>
+        </is>
+      </c>
+      <c r="E591" s="2">
+        <v>20</v>
+      </c>
+      <c r="F591" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B592" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C592" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="D592" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="E592" s="2">
+        <v>14</v>
+      </c>
+      <c r="F592" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B593" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C593" s="0" t="inlineStr">
+        <is>
+          <t>thinkingofyou</t>
+        </is>
+      </c>
+      <c r="D593" s="0" t="inlineStr">
+        <is>
+          <t>gen_thinkingofyou</t>
+        </is>
+      </c>
+      <c r="E593" s="2">
+        <v>14</v>
+      </c>
+      <c r="F593" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B594" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C594" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalzucchini_day</t>
+        </is>
+      </c>
+      <c r="D594" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalzucchini_day</t>
+        </is>
+      </c>
+      <c r="E594" s="2">
+        <v>13</v>
+      </c>
+      <c r="F594" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B595" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C595" s="0" t="inlineStr">
+        <is>
+          <t>friends</t>
+        </is>
+      </c>
+      <c r="D595" s="0" t="inlineStr">
+        <is>
+          <t>birth_friends</t>
+        </is>
+      </c>
+      <c r="E595" s="2">
+        <v>12</v>
+      </c>
+      <c r="F595" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B596" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C596" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_general</t>
+        </is>
+      </c>
+      <c r="D596" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_general</t>
+        </is>
+      </c>
+      <c r="E596" s="2">
+        <v>12</v>
+      </c>
+      <c r="F596" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B597" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C597" s="0" t="inlineStr">
+        <is>
+          <t>blessings</t>
+        </is>
+      </c>
+      <c r="D597" s="0" t="inlineStr">
+        <is>
+          <t>birth_blessings</t>
+        </is>
+      </c>
+      <c r="E597" s="2">
+        <v>10</v>
+      </c>
+      <c r="F597" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B598" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C598" s="0" t="inlineStr">
+        <is>
+          <t>sympathy</t>
+        </is>
+      </c>
+      <c r="D598" s="0" t="inlineStr">
+        <is>
+          <t>insp_sympathy</t>
+        </is>
+      </c>
+      <c r="E598" s="2">
+        <v>9</v>
+      </c>
+      <c r="F598" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B599" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C599" s="0" t="inlineStr">
+        <is>
+          <t>belated</t>
+        </is>
+      </c>
+      <c r="D599" s="0" t="inlineStr">
+        <is>
+          <t>birth_belated</t>
+        </is>
+      </c>
+      <c r="E599" s="2">
+        <v>7</v>
+      </c>
+      <c r="F599" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B600" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C600" s="0" t="inlineStr">
+        <is>
+          <t>everyday</t>
+        </is>
+      </c>
+      <c r="D600" s="0" t="inlineStr">
+        <is>
+          <t>thank_everyday</t>
+        </is>
+      </c>
+      <c r="E600" s="2">
+        <v>7</v>
+      </c>
+      <c r="F600" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B601" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C601" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D601" s="0" t="inlineStr">
+        <is>
+          <t>birth_milestone</t>
+        </is>
+      </c>
+      <c r="E601" s="2">
+        <v>6</v>
+      </c>
+      <c r="F601" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B602" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C602" s="0" t="inlineStr">
+        <is>
+          <t>wishes</t>
+        </is>
+      </c>
+      <c r="D602" s="0" t="inlineStr">
+        <is>
+          <t>birth_wishes</t>
+        </is>
+      </c>
+      <c r="E602" s="2">
+        <v>6</v>
+      </c>
+      <c r="F602" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B603" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C603" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="D603" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="E603" s="2">
+        <v>6</v>
+      </c>
+      <c r="F603" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B604" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C604" s="0" t="inlineStr">
+        <is>
+          <t>extfamily</t>
+        </is>
+      </c>
+      <c r="D604" s="0" t="inlineStr">
+        <is>
+          <t>birth_extfamily</t>
+        </is>
+      </c>
+      <c r="E604" s="2">
+        <v>5</v>
+      </c>
+      <c r="F604" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B605" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C605" s="0" t="inlineStr">
+        <is>
+          <t>flowers</t>
+        </is>
+      </c>
+      <c r="D605" s="0" t="inlineStr">
+        <is>
+          <t>birth_flowers</t>
+        </is>
+      </c>
+      <c r="E605" s="2">
+        <v>5</v>
+      </c>
+      <c r="F605" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B606" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C606" s="0" t="inlineStr">
+        <is>
+          <t>hubbywife</t>
+        </is>
+      </c>
+      <c r="D606" s="0" t="inlineStr">
+        <is>
+          <t>birth_hubbywife</t>
+        </is>
+      </c>
+      <c r="E606" s="2">
+        <v>5</v>
+      </c>
+      <c r="F606" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B607" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C607" s="0" t="inlineStr">
+        <is>
+          <t>kids</t>
+        </is>
+      </c>
+      <c r="D607" s="0" t="inlineStr">
+        <is>
+          <t>birth_kids</t>
+        </is>
+      </c>
+      <c r="E607" s="2">
+        <v>5</v>
+      </c>
+      <c r="F607" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B608" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C608" s="0" t="inlineStr">
+        <is>
+          <t>sonanddaughter</t>
+        </is>
+      </c>
+      <c r="D608" s="0" t="inlineStr">
+        <is>
+          <t>birth_sonanddaughter</t>
+        </is>
+      </c>
+      <c r="E608" s="2">
+        <v>5</v>
+      </c>
+      <c r="F608" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B609" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C609" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D609" s="0" t="inlineStr">
+        <is>
+          <t>gen_getwell</t>
+        </is>
+      </c>
+      <c r="E609" s="2">
+        <v>5</v>
+      </c>
+      <c r="F609" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B610" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C610" s="0" t="inlineStr">
+        <is>
+          <t>bronsis</t>
+        </is>
+      </c>
+      <c r="D610" s="0" t="inlineStr">
+        <is>
+          <t>birth_bronsis</t>
+        </is>
+      </c>
+      <c r="E610" s="2">
+        <v>4</v>
+      </c>
+      <c r="F610" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B611" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C611" s="0" t="inlineStr">
+        <is>
+          <t>songs</t>
+        </is>
+      </c>
+      <c r="D611" s="0" t="inlineStr">
+        <is>
+          <t>birth_songs</t>
+        </is>
+      </c>
+      <c r="E611" s="2">
+        <v>4</v>
+      </c>
+      <c r="F611" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B612" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C612" s="0" t="inlineStr">
+        <is>
+          <t>newbaby</t>
+        </is>
+      </c>
+      <c r="D612" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newbaby</t>
+        </is>
+      </c>
+      <c r="E612" s="2">
+        <v>4</v>
+      </c>
+      <c r="F612" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B613" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C613" s="0" t="inlineStr">
+        <is>
+          <t>eaug_flwrmonthaug</t>
+        </is>
+      </c>
+      <c r="D613" s="0" t="inlineStr">
+        <is>
+          <t>eaug_flwrmonthaug</t>
+        </is>
+      </c>
+      <c r="E613" s="2">
+        <v>4</v>
+      </c>
+      <c r="F613" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B614" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C614" s="0" t="inlineStr">
+        <is>
+          <t>eaug_happinesshappens_day</t>
+        </is>
+      </c>
+      <c r="D614" s="0" t="inlineStr">
+        <is>
+          <t>eaug_happinesshappens_day</t>
+        </is>
+      </c>
+      <c r="E614" s="2">
+        <v>4</v>
+      </c>
+      <c r="F614" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B615" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C615" s="0" t="inlineStr">
+        <is>
+          <t>bestfriends</t>
+        </is>
+      </c>
+      <c r="D615" s="0" t="inlineStr">
+        <is>
+          <t>friend_bestfriends</t>
+        </is>
+      </c>
+      <c r="E615" s="2">
+        <v>4</v>
+      </c>
+      <c r="F615" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B616" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C616" s="0" t="inlineStr">
+        <is>
+          <t>morning</t>
+        </is>
+      </c>
+      <c r="D616" s="0" t="inlineStr">
+        <is>
+          <t>gen_morning</t>
+        </is>
+      </c>
+      <c r="E616" s="2">
+        <v>4</v>
+      </c>
+      <c r="F616" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B617" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C617" s="0" t="inlineStr">
+        <is>
+          <t>wedding</t>
+        </is>
+      </c>
+      <c r="D617" s="0" t="inlineStr">
+        <is>
+          <t>thank_wedding</t>
+        </is>
+      </c>
+      <c r="E617" s="2">
+        <v>4</v>
+      </c>
+      <c r="F617" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B618" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C618" s="0" t="inlineStr">
+        <is>
+          <t>hugs</t>
+        </is>
+      </c>
+      <c r="D618" s="0" t="inlineStr">
+        <is>
+          <t>cute_hugs</t>
+        </is>
+      </c>
+      <c r="E618" s="2">
+        <v>3</v>
+      </c>
+      <c r="F618" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B619" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C619" s="0" t="inlineStr">
+        <is>
+          <t>eaug_booklover_day</t>
+        </is>
+      </c>
+      <c r="D619" s="0" t="inlineStr">
+        <is>
+          <t>eaug_booklover_day</t>
+        </is>
+      </c>
+      <c r="E619" s="2">
+        <v>3</v>
+      </c>
+      <c r="F619" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B620" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C620" s="0" t="inlineStr">
+        <is>
+          <t>hvgtday</t>
+        </is>
+      </c>
+      <c r="D620" s="0" t="inlineStr">
+        <is>
+          <t>gen_hvgtday</t>
+        </is>
+      </c>
+      <c r="E620" s="2">
+        <v>3</v>
+      </c>
+      <c r="F620" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B621" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C621" s="0" t="inlineStr">
+        <is>
+          <t>sorry</t>
+        </is>
+      </c>
+      <c r="D621" s="0" t="inlineStr">
+        <is>
+          <t>gen_sorry</t>
+        </is>
+      </c>
+      <c r="E621" s="2">
+        <v>3</v>
+      </c>
+      <c r="F621" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B622" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C622" s="0" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="D622" s="0" t="inlineStr">
+        <is>
+          <t>insp_health</t>
+        </is>
+      </c>
+      <c r="E622" s="2">
+        <v>3</v>
+      </c>
+      <c r="F622" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B623" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C623" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="D623" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="E623" s="2">
+        <v>2</v>
+      </c>
+      <c r="F623" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B624" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C624" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugsweetheartday</t>
+        </is>
+      </c>
+      <c r="D624" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugsweetheartday</t>
+        </is>
+      </c>
+      <c r="E624" s="2">
+        <v>2</v>
+      </c>
+      <c r="F624" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B625" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C625" s="0" t="inlineStr">
+        <is>
+          <t>eaug_internationalcat_day</t>
+        </is>
+      </c>
+      <c r="D625" s="0" t="inlineStr">
+        <is>
+          <t>eaug_internationalcat_day</t>
+        </is>
+      </c>
+      <c r="E625" s="2">
+        <v>2</v>
+      </c>
+      <c r="F625" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B626" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C626" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalraspberry_tart_day</t>
+        </is>
+      </c>
+      <c r="D626" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalraspberry_tart_day</t>
+        </is>
+      </c>
+      <c r="E626" s="2">
+        <v>2</v>
+      </c>
+      <c r="F626" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B627" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C627" s="0" t="inlineStr">
+        <is>
+          <t>eaug_thankyouday</t>
+        </is>
+      </c>
+      <c r="D627" s="0" t="inlineStr">
+        <is>
+          <t>eaug_thankyouday</t>
+        </is>
+      </c>
+      <c r="E627" s="2">
+        <v>2</v>
+      </c>
+      <c r="F627" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B628" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C628" s="0" t="inlineStr">
+        <is>
+          <t>goodnight</t>
+        </is>
+      </c>
+      <c r="D628" s="0" t="inlineStr">
+        <is>
+          <t>gen_goodnight</t>
+        </is>
+      </c>
+      <c r="E628" s="2">
+        <v>2</v>
+      </c>
+      <c r="F628" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B629" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C629" s="0" t="inlineStr">
+        <is>
+          <t>monblues</t>
+        </is>
+      </c>
+      <c r="D629" s="0" t="inlineStr">
+        <is>
+          <t>gen_monblues</t>
+        </is>
+      </c>
+      <c r="E629" s="2">
+        <v>2</v>
+      </c>
+      <c r="F629" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B630" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C630" s="0" t="inlineStr">
+        <is>
+          <t>quotesmessages_images_getwell_messages</t>
+        </is>
+      </c>
+      <c r="D630" s="0" t="inlineStr">
+        <is>
+          <t>gen_quotesmessages_images_getwell_messages</t>
+        </is>
+      </c>
+      <c r="E630" s="2">
+        <v>2</v>
+      </c>
+      <c r="F630" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B631" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C631" s="0" t="inlineStr">
+        <is>
+          <t>quotesmessages_images_goodmorning_images</t>
+        </is>
+      </c>
+      <c r="D631" s="0" t="inlineStr">
+        <is>
+          <t>gen_quotesmessages_images_goodmorning_images</t>
+        </is>
+      </c>
+      <c r="E631" s="2">
+        <v>2</v>
+      </c>
+      <c r="F631" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B632" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C632" s="0" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="D632" s="0" t="inlineStr">
+        <is>
+          <t>gen_weekend</t>
+        </is>
+      </c>
+      <c r="E632" s="2">
+        <v>2</v>
+      </c>
+      <c r="F632" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B633" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C633" s="0" t="inlineStr">
+        <is>
+          <t>dating</t>
+        </is>
+      </c>
+      <c r="D633" s="0" t="inlineStr">
+        <is>
+          <t>love_dating</t>
+        </is>
+      </c>
+      <c r="E633" s="2">
+        <v>2</v>
+      </c>
+      <c r="F633" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B634" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C634" s="0" t="inlineStr">
+        <is>
+          <t>sweetheart</t>
+        </is>
+      </c>
+      <c r="D634" s="0" t="inlineStr">
+        <is>
+          <t>love_sweetheart</t>
+        </is>
+      </c>
+      <c r="E634" s="2">
+        <v>2</v>
+      </c>
+      <c r="F634" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B635" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C635" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D635" s="0" t="inlineStr">
+        <is>
+          <t>pet_getwell</t>
+        </is>
+      </c>
+      <c r="E635" s="2">
+        <v>2</v>
+      </c>
+      <c r="F635" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B636" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C636" s="0" t="inlineStr">
+        <is>
+          <t>lossofpet</t>
+        </is>
+      </c>
+      <c r="D636" s="0" t="inlineStr">
+        <is>
+          <t>pet_lossofpet</t>
+        </is>
+      </c>
+      <c r="E636" s="2">
+        <v>2</v>
+      </c>
+      <c r="F636" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B637" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C637" s="0" t="inlineStr">
+        <is>
+          <t>inspirational</t>
+        </is>
+      </c>
+      <c r="D637" s="0" t="inlineStr">
+        <is>
+          <t>thank_inspirational</t>
+        </is>
+      </c>
+      <c r="E637" s="2">
+        <v>2</v>
+      </c>
+      <c r="F637" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B638" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C638" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D638" s="0" t="inlineStr">
+        <is>
+          <t>thank_love</t>
+        </is>
+      </c>
+      <c r="E638" s="2">
+        <v>2</v>
+      </c>
+      <c r="F638" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B639" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C639" s="0" t="inlineStr">
+        <is>
+          <t>forhim</t>
+        </is>
+      </c>
+      <c r="D639" s="0" t="inlineStr">
+        <is>
+          <t>birth_forhim</t>
+        </is>
+      </c>
+      <c r="E639" s="2">
+        <v>1</v>
+      </c>
+      <c r="F639" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B640" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C640" s="0" t="inlineStr">
+        <is>
+          <t>momndad</t>
+        </is>
+      </c>
+      <c r="D640" s="0" t="inlineStr">
+        <is>
+          <t>birth_momndad</t>
+        </is>
+      </c>
+      <c r="E640" s="2">
+        <v>1</v>
+      </c>
+      <c r="F640" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B641" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C641" s="0" t="inlineStr">
+        <is>
+          <t>specials</t>
+        </is>
+      </c>
+      <c r="D641" s="0" t="inlineStr">
+        <is>
+          <t>birth_specials</t>
+        </is>
+      </c>
+      <c r="E641" s="2">
+        <v>1</v>
+      </c>
+      <c r="F641" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B642" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C642" s="0" t="inlineStr">
+        <is>
+          <t>atworketc</t>
+        </is>
+      </c>
+      <c r="D642" s="0" t="inlineStr">
+        <is>
+          <t>bus_atworketc</t>
+        </is>
+      </c>
+      <c r="E642" s="2">
+        <v>1</v>
+      </c>
+      <c r="F642" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B643" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C643" s="0" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="D643" s="0" t="inlineStr">
+        <is>
+          <t>congrats_engagement</t>
+        </is>
+      </c>
+      <c r="E643" s="2">
+        <v>1</v>
+      </c>
+      <c r="F643" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B644" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C644" s="0" t="inlineStr">
+        <is>
+          <t>foreveryone</t>
+        </is>
+      </c>
+      <c r="D644" s="0" t="inlineStr">
+        <is>
+          <t>congrats_foreveryone</t>
+        </is>
+      </c>
+      <c r="E644" s="2">
+        <v>1</v>
+      </c>
+      <c r="F644" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B645" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C645" s="0" t="inlineStr">
+        <is>
+          <t>newcarandlicense</t>
+        </is>
+      </c>
+      <c r="D645" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newcarandlicense</t>
+        </is>
+      </c>
+      <c r="E645" s="2">
+        <v>1</v>
+      </c>
+      <c r="F645" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B646" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C646" s="0" t="inlineStr">
+        <is>
+          <t>newhome</t>
+        </is>
+      </c>
+      <c r="D646" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newhome</t>
+        </is>
+      </c>
+      <c r="E646" s="2">
+        <v>1</v>
+      </c>
+      <c r="F646" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B647" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C647" s="0" t="inlineStr">
+        <is>
+          <t>eaug_girlfriendsday</t>
+        </is>
+      </c>
+      <c r="D647" s="0" t="inlineStr">
+        <is>
+          <t>eaug_girlfriendsday</t>
+        </is>
+      </c>
+      <c r="E647" s="2">
+        <v>1</v>
+      </c>
+      <c r="F647" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B648" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C648" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationallighthouse_day</t>
+        </is>
+      </c>
+      <c r="D648" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationallighthouse_day</t>
+        </is>
+      </c>
+      <c r="E648" s="2">
+        <v>1</v>
+      </c>
+      <c r="F648" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B649" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C649" s="0" t="inlineStr">
+        <is>
+          <t>eaug_romawaremonth</t>
+        </is>
+      </c>
+      <c r="D649" s="0" t="inlineStr">
+        <is>
+          <t>eaug_romawaremonth</t>
+        </is>
+      </c>
+      <c r="E649" s="2">
+        <v>1</v>
+      </c>
+      <c r="F649" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B650" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C650" s="0" t="inlineStr">
+        <is>
+          <t>eaug_smilemonth</t>
+        </is>
+      </c>
+      <c r="D650" s="0" t="inlineStr">
+        <is>
+          <t>eaug_smilemonth</t>
+        </is>
+      </c>
+      <c r="E650" s="2">
+        <v>1</v>
+      </c>
+      <c r="F650" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B651" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C651" s="0" t="inlineStr">
+        <is>
+          <t>eaug_womensequality_day</t>
+        </is>
+      </c>
+      <c r="D651" s="0" t="inlineStr">
+        <is>
+          <t>eaug_womensequality_day</t>
+        </is>
+      </c>
+      <c r="E651" s="2">
+        <v>1</v>
+      </c>
+      <c r="F651" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B652" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C652" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_missingu</t>
+        </is>
+      </c>
+      <c r="D652" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_missingu</t>
+        </is>
+      </c>
+      <c r="E652" s="2">
+        <v>1</v>
+      </c>
+      <c r="F652" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B653" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C653" s="0" t="inlineStr">
+        <is>
+          <t>emay_gethappyweek</t>
+        </is>
+      </c>
+      <c r="D653" s="0" t="inlineStr">
+        <is>
+          <t>emay_gethappyweek</t>
+        </is>
+      </c>
+      <c r="E653" s="2">
+        <v>1</v>
+      </c>
+      <c r="F653" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B654" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C654" s="0" t="inlineStr">
+        <is>
+          <t>eoct_nationalcat_day</t>
+        </is>
+      </c>
+      <c r="D654" s="0" t="inlineStr">
+        <is>
+          <t>eoct_nationalcat_day</t>
+        </is>
+      </c>
+      <c r="E654" s="2">
+        <v>1</v>
+      </c>
+      <c r="F654" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B655" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C655" s="0" t="inlineStr">
+        <is>
+          <t>esep_trueloveforeverday</t>
+        </is>
+      </c>
+      <c r="D655" s="0" t="inlineStr">
+        <is>
+          <t>esep_trueloveforeverday</t>
+        </is>
+      </c>
+      <c r="E655" s="2">
+        <v>1</v>
+      </c>
+      <c r="F655" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B656" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C656" s="0" t="inlineStr">
+        <is>
+          <t>sisters</t>
+        </is>
+      </c>
+      <c r="D656" s="0" t="inlineStr">
+        <is>
+          <t>fkt_sisters</t>
+        </is>
+      </c>
+      <c r="E656" s="2">
+        <v>1</v>
+      </c>
+      <c r="F656" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B657" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C657" s="0" t="inlineStr">
+        <is>
+          <t>roses</t>
+        </is>
+      </c>
+      <c r="D657" s="0" t="inlineStr">
+        <is>
+          <t>flwr_roses</t>
+        </is>
+      </c>
+      <c r="E657" s="2">
+        <v>1</v>
+      </c>
+      <c r="F657" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B658" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C658" s="0" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
+      <c r="D658" s="0" t="inlineStr">
+        <is>
+          <t>friend_thoughts</t>
+        </is>
+      </c>
+      <c r="E658" s="2">
+        <v>1</v>
+      </c>
+      <c r="F658" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B659" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C659" s="0" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="D659" s="0" t="inlineStr">
+        <is>
+          <t>gen_hi</t>
+        </is>
+      </c>
+      <c r="E659" s="2">
+        <v>1</v>
+      </c>
+      <c r="F659" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B660" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C660" s="0" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="D660" s="0" t="inlineStr">
+        <is>
+          <t>gen_luck</t>
+        </is>
+      </c>
+      <c r="E660" s="2">
+        <v>1</v>
+      </c>
+      <c r="F660" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B661" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C661" s="0" t="inlineStr">
+        <is>
+          <t>missyou</t>
+        </is>
+      </c>
+      <c r="D661" s="0" t="inlineStr">
+        <is>
+          <t>gen_missyou</t>
+        </is>
+      </c>
+      <c r="E661" s="2">
+        <v>1</v>
+      </c>
+      <c r="F661" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B662" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C662" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="D662" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="E662" s="2">
+        <v>1</v>
+      </c>
+      <c r="F662" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B663" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C663" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_kisses</t>
+        </is>
+      </c>
+      <c r="D663" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_kisses</t>
+        </is>
+      </c>
+      <c r="E663" s="2">
+        <v>1</v>
+      </c>
+      <c r="F663" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B664" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C664" s="0" t="inlineStr">
+        <is>
+          <t>lovepoems</t>
+        </is>
+      </c>
+      <c r="D664" s="0" t="inlineStr">
+        <is>
+          <t>love_lovepoems</t>
+        </is>
+      </c>
+      <c r="E664" s="2">
+        <v>1</v>
+      </c>
+      <c r="F664" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B665" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C665" s="0" t="inlineStr">
+        <is>
+          <t>lovesongs</t>
+        </is>
+      </c>
+      <c r="D665" s="0" t="inlineStr">
+        <is>
+          <t>love_lovesongs</t>
+        </is>
+      </c>
+      <c r="E665" s="2">
+        <v>1</v>
+      </c>
+      <c r="F665" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B666" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C666" s="0" t="inlineStr">
+        <is>
+          <t>wed_weddingetc</t>
+        </is>
+      </c>
+      <c r="D666" s="0" t="inlineStr">
+        <is>
+          <t>wed_weddingetc</t>
+        </is>
+      </c>
+      <c r="E666" s="2">
+        <v>1</v>
+      </c>
+      <c r="F666" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-08</t>
+        </is>
+      </c>
+      <c r="B667" s="4"/>
+      <c r="C667" s="4"/>
+      <c r="D667" s="4"/>
+      <c r="E667" s="5">
+        <v>776</v>
+      </c>
+      <c r="F667" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -21131,36 +23944,70 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B9" s="2">
+        <v>839</v>
+      </c>
+      <c r="C9" s="2">
+        <v>228</v>
+      </c>
+      <c r="D9" s="2">
+        <v>292</v>
+      </c>
+      <c r="E9" s="2">
+        <v>161</v>
+      </c>
+      <c r="F9" s="2">
+        <v>82</v>
+      </c>
+      <c r="G9" s="2">
+        <v>38</v>
+      </c>
+      <c r="H9" s="2">
+        <v>38</v>
+      </c>
+      <c r="I9" s="2">
+        <v>0</v>
+      </c>
+      <c r="J9" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="5">
-        <v>5868</v>
-      </c>
-      <c r="C9" s="5">
-        <v>1914</v>
-      </c>
-      <c r="D9" s="5">
-        <v>1788</v>
-      </c>
-      <c r="E9" s="5">
-        <v>1132</v>
-      </c>
-      <c r="F9" s="5">
-        <v>616</v>
-      </c>
-      <c r="G9" s="5">
-        <v>216</v>
-      </c>
-      <c r="H9" s="5">
-        <v>173</v>
-      </c>
-      <c r="I9" s="5">
+      <c r="B10" s="5">
+        <v>6707</v>
+      </c>
+      <c r="C10" s="5">
+        <v>2142</v>
+      </c>
+      <c r="D10" s="5">
+        <v>2080</v>
+      </c>
+      <c r="E10" s="5">
+        <v>1293</v>
+      </c>
+      <c r="F10" s="5">
+        <v>698</v>
+      </c>
+      <c r="G10" s="5">
+        <v>254</v>
+      </c>
+      <c r="H10" s="5">
+        <v>211</v>
+      </c>
+      <c r="I10" s="5">
         <v>28</v>
       </c>
-      <c r="J9" s="5">
+      <c r="J10" s="5">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Record 11 August: eleven days, 9,133 sends tracked
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9KsXegBwxB1sWdCzRVLrr
</commit_message>
<xml_diff>
--- a/reports/daily_tracking.xlsx
+++ b/reports/daily_tracking.xlsx
@@ -224,7 +224,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
@@ -247,7 +247,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -591,28 +591,56 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B12" s="2">
+        <v>766</v>
+      </c>
+      <c r="C12" s="2">
+        <v>515</v>
+      </c>
+      <c r="D12" s="2">
+        <v>251</v>
+      </c>
+      <c r="E12" s="2">
+        <v>732</v>
+      </c>
+      <c r="F12" s="2">
+        <v>34</v>
+      </c>
+      <c r="G12" s="2">
+        <v>265</v>
+      </c>
+      <c r="H12" s="2">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="5">
-        <v>8367</v>
-      </c>
-      <c r="C12" s="5">
-        <v>5462</v>
-      </c>
-      <c r="D12" s="5">
-        <v>2905</v>
-      </c>
-      <c r="E12" s="5">
-        <v>7975</v>
-      </c>
-      <c r="F12" s="5">
-        <v>392</v>
-      </c>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
+      <c r="B13" s="5">
+        <v>9133</v>
+      </c>
+      <c r="C13" s="5">
+        <v>5977</v>
+      </c>
+      <c r="D13" s="5">
+        <v>3156</v>
+      </c>
+      <c r="E13" s="5">
+        <v>8707</v>
+      </c>
+      <c r="F13" s="5">
+        <v>426</v>
+      </c>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -636,8 +664,8 @@
     <col min="13" max="13" width="21" customWidth="1"/>
     <col min="14" max="14" width="11" customWidth="1"/>
     <col min="15" max="15" width="11" customWidth="1"/>
-    <col min="16" max="16" width="17" customWidth="1"/>
-    <col min="17" max="17" width="18" customWidth="1"/>
+    <col min="16" max="16" width="18" customWidth="1"/>
+    <col min="17" max="17" width="17" customWidth="1"/>
     <col min="18" max="18" width="17" customWidth="1"/>
     <col min="19" max="19" width="23" customWidth="1"/>
   </cols>
@@ -720,12 +748,12 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>World languages</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Keeping in touch</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
@@ -788,10 +816,10 @@
         <v>4</v>
       </c>
       <c r="P2" s="2">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q2" s="2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="R2" s="2">
         <v>2</v>
@@ -849,10 +877,10 @@
         <v>1</v>
       </c>
       <c r="P3" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q3" s="2">
         <v>10</v>
-      </c>
-      <c r="Q3" s="2">
-        <v>2</v>
       </c>
       <c r="R3" s="2">
         <v>0</v>
@@ -971,10 +999,10 @@
         <v>1</v>
       </c>
       <c r="P5" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q5" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R5" s="2">
         <v>0</v>
@@ -1032,10 +1060,10 @@
         <v>0</v>
       </c>
       <c r="P6" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6" s="2">
         <v>2</v>
@@ -1093,10 +1121,10 @@
         <v>0</v>
       </c>
       <c r="P7" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q7" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R7" s="2">
         <v>3</v>
@@ -1276,10 +1304,10 @@
         <v>5</v>
       </c>
       <c r="P10" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R10" s="2">
         <v>0</v>
@@ -1337,10 +1365,10 @@
         <v>3</v>
       </c>
       <c r="P11" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q11" s="2">
         <v>0</v>
-      </c>
-      <c r="Q11" s="2">
-        <v>2</v>
       </c>
       <c r="R11" s="2">
         <v>0</v>
@@ -1350,63 +1378,124 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B12" s="2">
+        <v>732</v>
+      </c>
+      <c r="C12" s="2">
+        <v>481</v>
+      </c>
+      <c r="D12" s="2">
+        <v>81</v>
+      </c>
+      <c r="E12" s="2">
+        <v>46</v>
+      </c>
+      <c r="F12" s="2">
+        <v>37</v>
+      </c>
+      <c r="G12" s="2">
+        <v>31</v>
+      </c>
+      <c r="H12" s="2">
+        <v>13</v>
+      </c>
+      <c r="I12" s="2">
+        <v>5</v>
+      </c>
+      <c r="J12" s="2">
+        <v>14</v>
+      </c>
+      <c r="K12" s="2">
+        <v>14</v>
+      </c>
+      <c r="L12" s="2">
+        <v>2</v>
+      </c>
+      <c r="M12" s="2">
+        <v>1</v>
+      </c>
+      <c r="N12" s="2">
+        <v>1</v>
+      </c>
+      <c r="O12" s="2">
+        <v>0</v>
+      </c>
+      <c r="P12" s="2">
+        <v>6</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>0</v>
+      </c>
+      <c r="R12" s="2">
+        <v>0</v>
+      </c>
+      <c r="S12" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="5">
-        <v>7975</v>
-      </c>
-      <c r="C12" s="5">
-        <v>5219</v>
-      </c>
-      <c r="D12" s="5">
-        <v>774</v>
-      </c>
-      <c r="E12" s="5">
-        <v>479</v>
-      </c>
-      <c r="F12" s="5">
-        <v>379</v>
-      </c>
-      <c r="G12" s="5">
-        <v>321</v>
-      </c>
-      <c r="H12" s="5">
-        <v>197</v>
-      </c>
-      <c r="I12" s="5">
-        <v>159</v>
-      </c>
-      <c r="J12" s="5">
-        <v>149</v>
-      </c>
-      <c r="K12" s="5">
-        <v>94</v>
-      </c>
-      <c r="L12" s="5">
-        <v>78</v>
-      </c>
-      <c r="M12" s="5">
+      <c r="B13" s="5">
+        <v>8707</v>
+      </c>
+      <c r="C13" s="5">
+        <v>5700</v>
+      </c>
+      <c r="D13" s="5">
+        <v>855</v>
+      </c>
+      <c r="E13" s="5">
+        <v>525</v>
+      </c>
+      <c r="F13" s="5">
+        <v>416</v>
+      </c>
+      <c r="G13" s="5">
+        <v>352</v>
+      </c>
+      <c r="H13" s="5">
+        <v>210</v>
+      </c>
+      <c r="I13" s="5">
+        <v>164</v>
+      </c>
+      <c r="J13" s="5">
+        <v>163</v>
+      </c>
+      <c r="K13" s="5">
+        <v>108</v>
+      </c>
+      <c r="L13" s="5">
+        <v>80</v>
+      </c>
+      <c r="M13" s="5">
+        <v>33</v>
+      </c>
+      <c r="N13" s="5">
         <v>32</v>
       </c>
-      <c r="N12" s="5">
-        <v>31</v>
-      </c>
-      <c r="O12" s="5">
+      <c r="O13" s="5">
         <v>23</v>
       </c>
-      <c r="P12" s="5">
+      <c r="P13" s="5">
         <v>17</v>
       </c>
-      <c r="Q12" s="5">
-        <v>11</v>
-      </c>
-      <c r="R12" s="5">
+      <c r="Q13" s="5">
+        <v>17</v>
+      </c>
+      <c r="R13" s="5">
         <v>9</v>
       </c>
-      <c r="S12" s="5">
+      <c r="S13" s="5">
         <v>3</v>
       </c>
     </row>
@@ -6201,6 +6290,444 @@
       </c>
       <c r="H152" s="4"/>
     </row>
+    <row r="153">
+      <c r="A153" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B153" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C153" s="0" t="inlineStr">
+        <is>
+          <t>birth</t>
+        </is>
+      </c>
+      <c r="D153" s="2">
+        <v>325</v>
+      </c>
+      <c r="E153" s="2">
+        <v>156</v>
+      </c>
+      <c r="F153" s="2">
+        <v>481</v>
+      </c>
+      <c r="G153" s="3">
+        <v>0.657103825136612</v>
+      </c>
+      <c r="H153" s="2">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B154" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C154" s="0" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="D154" s="2">
+        <v>69</v>
+      </c>
+      <c r="E154" s="2">
+        <v>12</v>
+      </c>
+      <c r="F154" s="2">
+        <v>81</v>
+      </c>
+      <c r="G154" s="3">
+        <v>0.11065573770491803</v>
+      </c>
+      <c r="H154" s="2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B155" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C155" s="0" t="inlineStr">
+        <is>
+          <t>anniv</t>
+        </is>
+      </c>
+      <c r="D155" s="2">
+        <v>30</v>
+      </c>
+      <c r="E155" s="2">
+        <v>16</v>
+      </c>
+      <c r="F155" s="2">
+        <v>46</v>
+      </c>
+      <c r="G155" s="3">
+        <v>0.06284153005464481</v>
+      </c>
+      <c r="H155" s="2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B156" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C156" s="0" t="inlineStr">
+        <is>
+          <t>gen</t>
+        </is>
+      </c>
+      <c r="D156" s="2">
+        <v>27</v>
+      </c>
+      <c r="E156" s="2">
+        <v>10</v>
+      </c>
+      <c r="F156" s="2">
+        <v>37</v>
+      </c>
+      <c r="G156" s="3">
+        <v>0.050546448087431695</v>
+      </c>
+      <c r="H156" s="2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B157" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C157" s="0" t="inlineStr">
+        <is>
+          <t>thank</t>
+        </is>
+      </c>
+      <c r="D157" s="2">
+        <v>9</v>
+      </c>
+      <c r="E157" s="2">
+        <v>22</v>
+      </c>
+      <c r="F157" s="2">
+        <v>31</v>
+      </c>
+      <c r="G157" s="3">
+        <v>0.04234972677595628</v>
+      </c>
+      <c r="H157" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B158" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C158" s="0" t="inlineStr">
+        <is>
+          <t>congrats</t>
+        </is>
+      </c>
+      <c r="D158" s="2">
+        <v>6</v>
+      </c>
+      <c r="E158" s="2">
+        <v>8</v>
+      </c>
+      <c r="F158" s="2">
+        <v>14</v>
+      </c>
+      <c r="G158" s="3">
+        <v>0.01912568306010929</v>
+      </c>
+      <c r="H158" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B159" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C159" s="0" t="inlineStr">
+        <is>
+          <t>insp</t>
+        </is>
+      </c>
+      <c r="D159" s="2">
+        <v>14</v>
+      </c>
+      <c r="E159" s="2">
+        <v>0</v>
+      </c>
+      <c r="F159" s="2">
+        <v>14</v>
+      </c>
+      <c r="G159" s="3">
+        <v>0.01912568306010929</v>
+      </c>
+      <c r="H159" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B160" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C160" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D160" s="2">
+        <v>9</v>
+      </c>
+      <c r="E160" s="2">
+        <v>4</v>
+      </c>
+      <c r="F160" s="2">
+        <v>13</v>
+      </c>
+      <c r="G160" s="3">
+        <v>0.017759562841530054</v>
+      </c>
+      <c r="H160" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B161" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C161" s="0" t="inlineStr">
+        <is>
+          <t>intouch</t>
+        </is>
+      </c>
+      <c r="D161" s="2">
+        <v>6</v>
+      </c>
+      <c r="E161" s="2">
+        <v>0</v>
+      </c>
+      <c r="F161" s="2">
+        <v>6</v>
+      </c>
+      <c r="G161" s="3">
+        <v>0.00819672131147541</v>
+      </c>
+      <c r="H161" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B162" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C162" s="0" t="inlineStr">
+        <is>
+          <t>friend</t>
+        </is>
+      </c>
+      <c r="D162" s="2">
+        <v>4</v>
+      </c>
+      <c r="E162" s="2">
+        <v>1</v>
+      </c>
+      <c r="F162" s="2">
+        <v>5</v>
+      </c>
+      <c r="G162" s="3">
+        <v>0.006830601092896175</v>
+      </c>
+      <c r="H162" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B163" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C163" s="0" t="inlineStr">
+        <is>
+          <t>flwr</t>
+        </is>
+      </c>
+      <c r="D163" s="2">
+        <v>2</v>
+      </c>
+      <c r="E163" s="2">
+        <v>0</v>
+      </c>
+      <c r="F163" s="2">
+        <v>2</v>
+      </c>
+      <c r="G163" s="3">
+        <v>0.00273224043715847</v>
+      </c>
+      <c r="H163" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B164" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C164" s="0" t="inlineStr">
+        <is>
+          <t>fkt</t>
+        </is>
+      </c>
+      <c r="D164" s="2">
+        <v>1</v>
+      </c>
+      <c r="E164" s="2">
+        <v>0</v>
+      </c>
+      <c r="F164" s="2">
+        <v>1</v>
+      </c>
+      <c r="G164" s="3">
+        <v>0.001366120218579235</v>
+      </c>
+      <c r="H164" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B165" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C165" s="0" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="D165" s="2">
+        <v>1</v>
+      </c>
+      <c r="E165" s="2">
+        <v>0</v>
+      </c>
+      <c r="F165" s="2">
+        <v>1</v>
+      </c>
+      <c r="G165" s="3">
+        <v>0.001366120218579235</v>
+      </c>
+      <c r="H165" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-11</t>
+        </is>
+      </c>
+      <c r="B166" s="4"/>
+      <c r="C166" s="4"/>
+      <c r="D166" s="5">
+        <v>503</v>
+      </c>
+      <c r="E166" s="5">
+        <v>229</v>
+      </c>
+      <c r="F166" s="5">
+        <v>732</v>
+      </c>
+      <c r="G166" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="H166" s="4"/>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -29823,6 +30350,2344 @@
         <v>897</v>
       </c>
       <c r="F848" s="4"/>
+    </row>
+    <row r="849">
+      <c r="A849" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B849" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C849" s="0" t="inlineStr">
+        <is>
+          <t>happybirthday</t>
+        </is>
+      </c>
+      <c r="D849" s="0" t="inlineStr">
+        <is>
+          <t>birth_happybirthday</t>
+        </is>
+      </c>
+      <c r="E849" s="2">
+        <v>338</v>
+      </c>
+      <c r="F849" s="2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B850" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C850" s="0" t="inlineStr">
+        <is>
+          <t>anniversaryetc</t>
+        </is>
+      </c>
+      <c r="D850" s="0" t="inlineStr">
+        <is>
+          <t>anniv_anniversaryetc</t>
+        </is>
+      </c>
+      <c r="E850" s="2">
+        <v>33</v>
+      </c>
+      <c r="F850" s="2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B851" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C851" s="0" t="inlineStr">
+        <is>
+          <t>fun</t>
+        </is>
+      </c>
+      <c r="D851" s="0" t="inlineStr">
+        <is>
+          <t>birth_fun</t>
+        </is>
+      </c>
+      <c r="E851" s="2">
+        <v>26</v>
+      </c>
+      <c r="F851" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B852" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C852" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="D852" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="E852" s="2">
+        <v>21</v>
+      </c>
+      <c r="F852" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B853" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C853" s="0" t="inlineStr">
+        <is>
+          <t>sonanddaughter</t>
+        </is>
+      </c>
+      <c r="D853" s="0" t="inlineStr">
+        <is>
+          <t>birth_sonanddaughter</t>
+        </is>
+      </c>
+      <c r="E853" s="2">
+        <v>18</v>
+      </c>
+      <c r="F853" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B854" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C854" s="0" t="inlineStr">
+        <is>
+          <t>birthday</t>
+        </is>
+      </c>
+      <c r="D854" s="0" t="inlineStr">
+        <is>
+          <t>thank_birthday</t>
+        </is>
+      </c>
+      <c r="E854" s="2">
+        <v>14</v>
+      </c>
+      <c r="F854" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B855" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C855" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D855" s="0" t="inlineStr">
+        <is>
+          <t>birth_milestone</t>
+        </is>
+      </c>
+      <c r="E855" s="2">
+        <v>13</v>
+      </c>
+      <c r="F855" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B856" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C856" s="0" t="inlineStr">
+        <is>
+          <t>songs</t>
+        </is>
+      </c>
+      <c r="D856" s="0" t="inlineStr">
+        <is>
+          <t>birth_songs</t>
+        </is>
+      </c>
+      <c r="E856" s="2">
+        <v>13</v>
+      </c>
+      <c r="F856" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B857" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C857" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalraspberry_tart_day</t>
+        </is>
+      </c>
+      <c r="D857" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalraspberry_tart_day</t>
+        </is>
+      </c>
+      <c r="E857" s="2">
+        <v>13</v>
+      </c>
+      <c r="F857" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B858" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C858" s="0" t="inlineStr">
+        <is>
+          <t>flowers</t>
+        </is>
+      </c>
+      <c r="D858" s="0" t="inlineStr">
+        <is>
+          <t>birth_flowers</t>
+        </is>
+      </c>
+      <c r="E858" s="2">
+        <v>12</v>
+      </c>
+      <c r="F858" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B859" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C859" s="0" t="inlineStr">
+        <is>
+          <t>eaug_sonand_daughter_day</t>
+        </is>
+      </c>
+      <c r="D859" s="0" t="inlineStr">
+        <is>
+          <t>eaug_sonand_daughter_day</t>
+        </is>
+      </c>
+      <c r="E859" s="2">
+        <v>11</v>
+      </c>
+      <c r="F859" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B860" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C860" s="0" t="inlineStr">
+        <is>
+          <t>extfamily</t>
+        </is>
+      </c>
+      <c r="D860" s="0" t="inlineStr">
+        <is>
+          <t>birth_extfamily</t>
+        </is>
+      </c>
+      <c r="E860" s="2">
+        <v>10</v>
+      </c>
+      <c r="F860" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B861" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C861" s="0" t="inlineStr">
+        <is>
+          <t>friends</t>
+        </is>
+      </c>
+      <c r="D861" s="0" t="inlineStr">
+        <is>
+          <t>birth_friends</t>
+        </is>
+      </c>
+      <c r="E861" s="2">
+        <v>9</v>
+      </c>
+      <c r="F861" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B862" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C862" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D862" s="0" t="inlineStr">
+        <is>
+          <t>gen_getwell</t>
+        </is>
+      </c>
+      <c r="E862" s="2">
+        <v>9</v>
+      </c>
+      <c r="F862" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B863" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C863" s="0" t="inlineStr">
+        <is>
+          <t>blessings</t>
+        </is>
+      </c>
+      <c r="D863" s="0" t="inlineStr">
+        <is>
+          <t>birth_blessings</t>
+        </is>
+      </c>
+      <c r="E863" s="2">
+        <v>8</v>
+      </c>
+      <c r="F863" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B864" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C864" s="0" t="inlineStr">
+        <is>
+          <t>wishes</t>
+        </is>
+      </c>
+      <c r="D864" s="0" t="inlineStr">
+        <is>
+          <t>birth_wishes</t>
+        </is>
+      </c>
+      <c r="E864" s="2">
+        <v>8</v>
+      </c>
+      <c r="F864" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B865" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C865" s="0" t="inlineStr">
+        <is>
+          <t>everyday</t>
+        </is>
+      </c>
+      <c r="D865" s="0" t="inlineStr">
+        <is>
+          <t>thank_everyday</t>
+        </is>
+      </c>
+      <c r="E865" s="2">
+        <v>8</v>
+      </c>
+      <c r="F865" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B866" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C866" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="D866" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="E866" s="2">
+        <v>7</v>
+      </c>
+      <c r="F866" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B867" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C867" s="0" t="inlineStr">
+        <is>
+          <t>belated</t>
+        </is>
+      </c>
+      <c r="D867" s="0" t="inlineStr">
+        <is>
+          <t>birth_belated</t>
+        </is>
+      </c>
+      <c r="E867" s="2">
+        <v>7</v>
+      </c>
+      <c r="F867" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B868" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C868" s="0" t="inlineStr">
+        <is>
+          <t>kids</t>
+        </is>
+      </c>
+      <c r="D868" s="0" t="inlineStr">
+        <is>
+          <t>birth_kids</t>
+        </is>
+      </c>
+      <c r="E868" s="2">
+        <v>7</v>
+      </c>
+      <c r="F868" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B869" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C869" s="0" t="inlineStr">
+        <is>
+          <t>thinkingofyou</t>
+        </is>
+      </c>
+      <c r="D869" s="0" t="inlineStr">
+        <is>
+          <t>gen_thinkingofyou</t>
+        </is>
+      </c>
+      <c r="E869" s="2">
+        <v>7</v>
+      </c>
+      <c r="F869" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B870" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C870" s="0" t="inlineStr">
+        <is>
+          <t>sympathy</t>
+        </is>
+      </c>
+      <c r="D870" s="0" t="inlineStr">
+        <is>
+          <t>insp_sympathy</t>
+        </is>
+      </c>
+      <c r="E870" s="2">
+        <v>7</v>
+      </c>
+      <c r="F870" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B871" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C871" s="0" t="inlineStr">
+        <is>
+          <t>bronsis</t>
+        </is>
+      </c>
+      <c r="D871" s="0" t="inlineStr">
+        <is>
+          <t>birth_bronsis</t>
+        </is>
+      </c>
+      <c r="E871" s="2">
+        <v>6</v>
+      </c>
+      <c r="F871" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B872" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C872" s="0" t="inlineStr">
+        <is>
+          <t>foreveryone</t>
+        </is>
+      </c>
+      <c r="D872" s="0" t="inlineStr">
+        <is>
+          <t>congrats_foreveryone</t>
+        </is>
+      </c>
+      <c r="E872" s="2">
+        <v>6</v>
+      </c>
+      <c r="F872" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B873" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C873" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_general</t>
+        </is>
+      </c>
+      <c r="D873" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_general</t>
+        </is>
+      </c>
+      <c r="E873" s="2">
+        <v>6</v>
+      </c>
+      <c r="F873" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B874" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C874" s="0" t="inlineStr">
+        <is>
+          <t>newbaby</t>
+        </is>
+      </c>
+      <c r="D874" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newbaby</t>
+        </is>
+      </c>
+      <c r="E874" s="2">
+        <v>5</v>
+      </c>
+      <c r="F874" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B875" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C875" s="0" t="inlineStr">
+        <is>
+          <t>eaug_creamsicleday</t>
+        </is>
+      </c>
+      <c r="D875" s="0" t="inlineStr">
+        <is>
+          <t>eaug_creamsicleday</t>
+        </is>
+      </c>
+      <c r="E875" s="2">
+        <v>5</v>
+      </c>
+      <c r="F875" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B876" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C876" s="0" t="inlineStr">
+        <is>
+          <t>eaug_internationalleft_handers_day</t>
+        </is>
+      </c>
+      <c r="D876" s="0" t="inlineStr">
+        <is>
+          <t>eaug_internationalleft_handers_day</t>
+        </is>
+      </c>
+      <c r="E876" s="2">
+        <v>5</v>
+      </c>
+      <c r="F876" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B877" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C877" s="0" t="inlineStr">
+        <is>
+          <t>hvgtday</t>
+        </is>
+      </c>
+      <c r="D877" s="0" t="inlineStr">
+        <is>
+          <t>gen_hvgtday</t>
+        </is>
+      </c>
+      <c r="E877" s="2">
+        <v>5</v>
+      </c>
+      <c r="F877" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B878" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C878" s="0" t="inlineStr">
+        <is>
+          <t>missingyou</t>
+        </is>
+      </c>
+      <c r="D878" s="0" t="inlineStr">
+        <is>
+          <t>intouch_missingyou</t>
+        </is>
+      </c>
+      <c r="E878" s="2">
+        <v>5</v>
+      </c>
+      <c r="F878" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B879" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C879" s="0" t="inlineStr">
+        <is>
+          <t>wed_wed_congrats</t>
+        </is>
+      </c>
+      <c r="D879" s="0" t="inlineStr">
+        <is>
+          <t>wed_wed_congrats</t>
+        </is>
+      </c>
+      <c r="E879" s="2">
+        <v>5</v>
+      </c>
+      <c r="F879" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B880" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C880" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="D880" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="E880" s="2">
+        <v>4</v>
+      </c>
+      <c r="F880" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B881" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C881" s="0" t="inlineStr">
+        <is>
+          <t>forher</t>
+        </is>
+      </c>
+      <c r="D881" s="0" t="inlineStr">
+        <is>
+          <t>birth_forher</t>
+        </is>
+      </c>
+      <c r="E881" s="2">
+        <v>4</v>
+      </c>
+      <c r="F881" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B882" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C882" s="0" t="inlineStr">
+        <is>
+          <t>eaug_thankyouday</t>
+        </is>
+      </c>
+      <c r="D882" s="0" t="inlineStr">
+        <is>
+          <t>eaug_thankyouday</t>
+        </is>
+      </c>
+      <c r="E882" s="2">
+        <v>4</v>
+      </c>
+      <c r="F882" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B883" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C883" s="0" t="inlineStr">
+        <is>
+          <t>recovery</t>
+        </is>
+      </c>
+      <c r="D883" s="0" t="inlineStr">
+        <is>
+          <t>insp_recovery</t>
+        </is>
+      </c>
+      <c r="E883" s="2">
+        <v>4</v>
+      </c>
+      <c r="F883" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B884" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C884" s="0" t="inlineStr">
+        <is>
+          <t>congratulations</t>
+        </is>
+      </c>
+      <c r="D884" s="0" t="inlineStr">
+        <is>
+          <t>thank_congratulations</t>
+        </is>
+      </c>
+      <c r="E884" s="2">
+        <v>4</v>
+      </c>
+      <c r="F884" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B885" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C885" s="0" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="D885" s="0" t="inlineStr">
+        <is>
+          <t>friend_hello</t>
+        </is>
+      </c>
+      <c r="E885" s="2">
+        <v>3</v>
+      </c>
+      <c r="F885" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B886" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C886" s="0" t="inlineStr">
+        <is>
+          <t>morning</t>
+        </is>
+      </c>
+      <c r="D886" s="0" t="inlineStr">
+        <is>
+          <t>gen_morning</t>
+        </is>
+      </c>
+      <c r="E886" s="2">
+        <v>3</v>
+      </c>
+      <c r="F886" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B887" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C887" s="0" t="inlineStr">
+        <is>
+          <t>youarewelcome</t>
+        </is>
+      </c>
+      <c r="D887" s="0" t="inlineStr">
+        <is>
+          <t>gen_youarewelcome</t>
+        </is>
+      </c>
+      <c r="E887" s="2">
+        <v>3</v>
+      </c>
+      <c r="F887" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B888" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C888" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="D888" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="E888" s="2">
+        <v>3</v>
+      </c>
+      <c r="F888" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B889" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C889" s="0" t="inlineStr">
+        <is>
+          <t>inspirational</t>
+        </is>
+      </c>
+      <c r="D889" s="0" t="inlineStr">
+        <is>
+          <t>thank_inspirational</t>
+        </is>
+      </c>
+      <c r="E889" s="2">
+        <v>3</v>
+      </c>
+      <c r="F889" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B890" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C890" s="0" t="inlineStr">
+        <is>
+          <t>eaug_internationalyouth_day</t>
+        </is>
+      </c>
+      <c r="D890" s="0" t="inlineStr">
+        <is>
+          <t>eaug_internationalyouth_day</t>
+        </is>
+      </c>
+      <c r="E890" s="2">
+        <v>2</v>
+      </c>
+      <c r="F890" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B891" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C891" s="0" t="inlineStr">
+        <is>
+          <t>eaug_romanceday</t>
+        </is>
+      </c>
+      <c r="D891" s="0" t="inlineStr">
+        <is>
+          <t>eaug_romanceday</t>
+        </is>
+      </c>
+      <c r="E891" s="2">
+        <v>2</v>
+      </c>
+      <c r="F891" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B892" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C892" s="0" t="inlineStr">
+        <is>
+          <t>youcare</t>
+        </is>
+      </c>
+      <c r="D892" s="0" t="inlineStr">
+        <is>
+          <t>flwr_youcare</t>
+        </is>
+      </c>
+      <c r="E892" s="2">
+        <v>2</v>
+      </c>
+      <c r="F892" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B893" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C893" s="0" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="D893" s="0" t="inlineStr">
+        <is>
+          <t>gen_luck</t>
+        </is>
+      </c>
+      <c r="E893" s="2">
+        <v>2</v>
+      </c>
+      <c r="F893" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B894" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C894" s="0" t="inlineStr">
+        <is>
+          <t>tuestoons</t>
+        </is>
+      </c>
+      <c r="D894" s="0" t="inlineStr">
+        <is>
+          <t>gen_tuestoons</t>
+        </is>
+      </c>
+      <c r="E894" s="2">
+        <v>2</v>
+      </c>
+      <c r="F894" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B895" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C895" s="0" t="inlineStr">
+        <is>
+          <t>voyage</t>
+        </is>
+      </c>
+      <c r="D895" s="0" t="inlineStr">
+        <is>
+          <t>gen_voyage</t>
+        </is>
+      </c>
+      <c r="E895" s="2">
+        <v>2</v>
+      </c>
+      <c r="F895" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B896" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C896" s="0" t="inlineStr">
+        <is>
+          <t>youarespecial</t>
+        </is>
+      </c>
+      <c r="D896" s="0" t="inlineStr">
+        <is>
+          <t>love_youarespecial</t>
+        </is>
+      </c>
+      <c r="E896" s="2">
+        <v>2</v>
+      </c>
+      <c r="F896" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B897" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C897" s="0" t="inlineStr">
+        <is>
+          <t>wedding</t>
+        </is>
+      </c>
+      <c r="D897" s="0" t="inlineStr">
+        <is>
+          <t>thank_wedding</t>
+        </is>
+      </c>
+      <c r="E897" s="2">
+        <v>2</v>
+      </c>
+      <c r="F897" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B898" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C898" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D898" s="0" t="inlineStr">
+        <is>
+          <t>anniv_milestone</t>
+        </is>
+      </c>
+      <c r="E898" s="2">
+        <v>1</v>
+      </c>
+      <c r="F898" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B899" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C899" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_family</t>
+        </is>
+      </c>
+      <c r="D899" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_family</t>
+        </is>
+      </c>
+      <c r="E899" s="2">
+        <v>1</v>
+      </c>
+      <c r="F899" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B900" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C900" s="0" t="inlineStr">
+        <is>
+          <t>hubbywife</t>
+        </is>
+      </c>
+      <c r="D900" s="0" t="inlineStr">
+        <is>
+          <t>birth_hubbywife</t>
+        </is>
+      </c>
+      <c r="E900" s="2">
+        <v>1</v>
+      </c>
+      <c r="F900" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B901" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C901" s="0" t="inlineStr">
+        <is>
+          <t>momndad</t>
+        </is>
+      </c>
+      <c r="D901" s="0" t="inlineStr">
+        <is>
+          <t>birth_momndad</t>
+        </is>
+      </c>
+      <c r="E901" s="2">
+        <v>1</v>
+      </c>
+      <c r="F901" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B902" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C902" s="0" t="inlineStr">
+        <is>
+          <t>newcarandlicense</t>
+        </is>
+      </c>
+      <c r="D902" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newcarandlicense</t>
+        </is>
+      </c>
+      <c r="E902" s="2">
+        <v>1</v>
+      </c>
+      <c r="F902" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B903" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C903" s="0" t="inlineStr">
+        <is>
+          <t>newhome</t>
+        </is>
+      </c>
+      <c r="D903" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newhome</t>
+        </is>
+      </c>
+      <c r="E903" s="2">
+        <v>1</v>
+      </c>
+      <c r="F903" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B904" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C904" s="0" t="inlineStr">
+        <is>
+          <t>newjob</t>
+        </is>
+      </c>
+      <c r="D904" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newjob</t>
+        </is>
+      </c>
+      <c r="E904" s="2">
+        <v>1</v>
+      </c>
+      <c r="F904" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B905" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C905" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugsweetheartday</t>
+        </is>
+      </c>
+      <c r="D905" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugsweetheartday</t>
+        </is>
+      </c>
+      <c r="E905" s="2">
+        <v>1</v>
+      </c>
+      <c r="F905" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B906" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C906" s="0" t="inlineStr">
+        <is>
+          <t>eaug_indindependenceday</t>
+        </is>
+      </c>
+      <c r="D906" s="0" t="inlineStr">
+        <is>
+          <t>eaug_indindependenceday</t>
+        </is>
+      </c>
+      <c r="E906" s="2">
+        <v>1</v>
+      </c>
+      <c r="F906" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B907" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C907" s="0" t="inlineStr">
+        <is>
+          <t>efeb_valen_thanku</t>
+        </is>
+      </c>
+      <c r="D907" s="0" t="inlineStr">
+        <is>
+          <t>efeb_valen_thanku</t>
+        </is>
+      </c>
+      <c r="E907" s="2">
+        <v>1</v>
+      </c>
+      <c r="F907" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B908" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C908" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_happy</t>
+        </is>
+      </c>
+      <c r="D908" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_happy</t>
+        </is>
+      </c>
+      <c r="E908" s="2">
+        <v>1</v>
+      </c>
+      <c r="F908" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B909" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C909" s="0" t="inlineStr">
+        <is>
+          <t>emay_mawlidalnabi</t>
+        </is>
+      </c>
+      <c r="D909" s="0" t="inlineStr">
+        <is>
+          <t>emay_mawlidalnabi</t>
+        </is>
+      </c>
+      <c r="E909" s="2">
+        <v>1</v>
+      </c>
+      <c r="F909" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B910" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C910" s="0" t="inlineStr">
+        <is>
+          <t>emay_mothersday_happy</t>
+        </is>
+      </c>
+      <c r="D910" s="0" t="inlineStr">
+        <is>
+          <t>emay_mothersday_happy</t>
+        </is>
+      </c>
+      <c r="E910" s="2">
+        <v>1</v>
+      </c>
+      <c r="F910" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B911" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C911" s="0" t="inlineStr">
+        <is>
+          <t>emay_mothersday_thanku</t>
+        </is>
+      </c>
+      <c r="D911" s="0" t="inlineStr">
+        <is>
+          <t>emay_mothersday_thanku</t>
+        </is>
+      </c>
+      <c r="E911" s="2">
+        <v>1</v>
+      </c>
+      <c r="F911" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B912" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C912" s="0" t="inlineStr">
+        <is>
+          <t>enov_adventday</t>
+        </is>
+      </c>
+      <c r="D912" s="0" t="inlineStr">
+        <is>
+          <t>enov_adventday</t>
+        </is>
+      </c>
+      <c r="E912" s="2">
+        <v>1</v>
+      </c>
+      <c r="F912" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B913" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C913" s="0" t="inlineStr">
+        <is>
+          <t>enov_allsaintsday</t>
+        </is>
+      </c>
+      <c r="D913" s="0" t="inlineStr">
+        <is>
+          <t>enov_allsaintsday</t>
+        </is>
+      </c>
+      <c r="E913" s="2">
+        <v>1</v>
+      </c>
+      <c r="F913" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B914" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C914" s="0" t="inlineStr">
+        <is>
+          <t>enov_remembranceday</t>
+        </is>
+      </c>
+      <c r="D914" s="0" t="inlineStr">
+        <is>
+          <t>enov_remembranceday</t>
+        </is>
+      </c>
+      <c r="E914" s="2">
+        <v>1</v>
+      </c>
+      <c r="F914" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B915" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C915" s="0" t="inlineStr">
+        <is>
+          <t>enov_thanks_wishes</t>
+        </is>
+      </c>
+      <c r="D915" s="0" t="inlineStr">
+        <is>
+          <t>enov_thanks_wishes</t>
+        </is>
+      </c>
+      <c r="E915" s="2">
+        <v>1</v>
+      </c>
+      <c r="F915" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B916" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C916" s="0" t="inlineStr">
+        <is>
+          <t>esep_roshhashanah_happy</t>
+        </is>
+      </c>
+      <c r="D916" s="0" t="inlineStr">
+        <is>
+          <t>esep_roshhashanah_happy</t>
+        </is>
+      </c>
+      <c r="E916" s="2">
+        <v>1</v>
+      </c>
+      <c r="F916" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B917" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C917" s="0" t="inlineStr">
+        <is>
+          <t>sisters</t>
+        </is>
+      </c>
+      <c r="D917" s="0" t="inlineStr">
+        <is>
+          <t>fkt_sisters</t>
+        </is>
+      </c>
+      <c r="E917" s="2">
+        <v>1</v>
+      </c>
+      <c r="F917" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B918" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C918" s="0" t="inlineStr">
+        <is>
+          <t>friendsforever</t>
+        </is>
+      </c>
+      <c r="D918" s="0" t="inlineStr">
+        <is>
+          <t>friend_friendsforever</t>
+        </is>
+      </c>
+      <c r="E918" s="2">
+        <v>1</v>
+      </c>
+      <c r="F918" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B919" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C919" s="0" t="inlineStr">
+        <is>
+          <t>missingyou</t>
+        </is>
+      </c>
+      <c r="D919" s="0" t="inlineStr">
+        <is>
+          <t>friend_missingyou</t>
+        </is>
+      </c>
+      <c r="E919" s="2">
+        <v>1</v>
+      </c>
+      <c r="F919" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B920" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C920" s="0" t="inlineStr">
+        <is>
+          <t>blessings</t>
+        </is>
+      </c>
+      <c r="D920" s="0" t="inlineStr">
+        <is>
+          <t>gen_blessings</t>
+        </is>
+      </c>
+      <c r="E920" s="2">
+        <v>1</v>
+      </c>
+      <c r="F920" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B921" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C921" s="0" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="D921" s="0" t="inlineStr">
+        <is>
+          <t>gen_hi</t>
+        </is>
+      </c>
+      <c r="E921" s="2">
+        <v>1</v>
+      </c>
+      <c r="F921" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B922" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C922" s="0" t="inlineStr">
+        <is>
+          <t>joke</t>
+        </is>
+      </c>
+      <c r="D922" s="0" t="inlineStr">
+        <is>
+          <t>gen_joke</t>
+        </is>
+      </c>
+      <c r="E922" s="2">
+        <v>1</v>
+      </c>
+      <c r="F922" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B923" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C923" s="0" t="inlineStr">
+        <is>
+          <t>quotesmessages_images_getwell_messages</t>
+        </is>
+      </c>
+      <c r="D923" s="0" t="inlineStr">
+        <is>
+          <t>gen_quotesmessages_images_getwell_messages</t>
+        </is>
+      </c>
+      <c r="E923" s="2">
+        <v>1</v>
+      </c>
+      <c r="F923" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B924" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C924" s="0" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="D924" s="0" t="inlineStr">
+        <is>
+          <t>insp_health</t>
+        </is>
+      </c>
+      <c r="E924" s="2">
+        <v>1</v>
+      </c>
+      <c r="F924" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B925" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C925" s="0" t="inlineStr">
+        <is>
+          <t>poetry</t>
+        </is>
+      </c>
+      <c r="D925" s="0" t="inlineStr">
+        <is>
+          <t>insp_poetry</t>
+        </is>
+      </c>
+      <c r="E925" s="2">
+        <v>1</v>
+      </c>
+      <c r="F925" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B926" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C926" s="0" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="D926" s="0" t="inlineStr">
+        <is>
+          <t>insp_support</t>
+        </is>
+      </c>
+      <c r="E926" s="2">
+        <v>1</v>
+      </c>
+      <c r="F926" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B927" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C927" s="0" t="inlineStr">
+        <is>
+          <t>thinkingofyou</t>
+        </is>
+      </c>
+      <c r="D927" s="0" t="inlineStr">
+        <is>
+          <t>intouch_thinkingofyou</t>
+        </is>
+      </c>
+      <c r="E927" s="2">
+        <v>1</v>
+      </c>
+      <c r="F927" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B928" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C928" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="D928" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="E928" s="2">
+        <v>1</v>
+      </c>
+      <c r="F928" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B929" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C929" s="0" t="inlineStr">
+        <is>
+          <t>lovesongs</t>
+        </is>
+      </c>
+      <c r="D929" s="0" t="inlineStr">
+        <is>
+          <t>love_lovesongs</t>
+        </is>
+      </c>
+      <c r="E929" s="2">
+        <v>1</v>
+      </c>
+      <c r="F929" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B930" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C930" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D930" s="0" t="inlineStr">
+        <is>
+          <t>pet_love</t>
+        </is>
+      </c>
+      <c r="E930" s="2">
+        <v>1</v>
+      </c>
+      <c r="F930" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B931" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C931" s="0" t="inlineStr">
+        <is>
+          <t>wed_wishes</t>
+        </is>
+      </c>
+      <c r="D931" s="0" t="inlineStr">
+        <is>
+          <t>wed_wishes</t>
+        </is>
+      </c>
+      <c r="E931" s="2">
+        <v>1</v>
+      </c>
+      <c r="F931" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-11</t>
+        </is>
+      </c>
+      <c r="B932" s="4"/>
+      <c r="C932" s="4"/>
+      <c r="D932" s="4"/>
+      <c r="E932" s="5">
+        <v>732</v>
+      </c>
+      <c r="F932" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -30236,36 +33101,70 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B12" s="2">
+        <v>766</v>
+      </c>
+      <c r="C12" s="2">
+        <v>226</v>
+      </c>
+      <c r="D12" s="2">
+        <v>237</v>
+      </c>
+      <c r="E12" s="2">
+        <v>155</v>
+      </c>
+      <c r="F12" s="2">
+        <v>95</v>
+      </c>
+      <c r="G12" s="2">
+        <v>28</v>
+      </c>
+      <c r="H12" s="2">
+        <v>25</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0</v>
+      </c>
+      <c r="J12" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="5">
-        <v>8367</v>
-      </c>
-      <c r="C12" s="5">
-        <v>2640</v>
-      </c>
-      <c r="D12" s="5">
-        <v>2595</v>
-      </c>
-      <c r="E12" s="5">
-        <v>1658</v>
-      </c>
-      <c r="F12" s="5">
-        <v>860</v>
-      </c>
-      <c r="G12" s="5">
-        <v>308</v>
-      </c>
-      <c r="H12" s="5">
-        <v>277</v>
-      </c>
-      <c r="I12" s="5">
+      <c r="B13" s="5">
+        <v>9133</v>
+      </c>
+      <c r="C13" s="5">
+        <v>2866</v>
+      </c>
+      <c r="D13" s="5">
+        <v>2832</v>
+      </c>
+      <c r="E13" s="5">
+        <v>1813</v>
+      </c>
+      <c r="F13" s="5">
+        <v>955</v>
+      </c>
+      <c r="G13" s="5">
+        <v>336</v>
+      </c>
+      <c r="H13" s="5">
+        <v>302</v>
+      </c>
+      <c r="I13" s="5">
         <v>28</v>
       </c>
-      <c r="J12" s="5">
+      <c r="J13" s="5">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Record 12 August: twelve days, 9,968 sends tracked
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9KsXegBwxB1sWdCzRVLrr
</commit_message>
<xml_diff>
--- a/reports/daily_tracking.xlsx
+++ b/reports/daily_tracking.xlsx
@@ -224,7 +224,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -247,7 +247,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -619,28 +619,56 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B13" s="2">
+        <v>835</v>
+      </c>
+      <c r="C13" s="2">
+        <v>570</v>
+      </c>
+      <c r="D13" s="2">
+        <v>265</v>
+      </c>
+      <c r="E13" s="2">
+        <v>773</v>
+      </c>
+      <c r="F13" s="2">
+        <v>62</v>
+      </c>
+      <c r="G13" s="2">
+        <v>250</v>
+      </c>
+      <c r="H13" s="2">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B13" s="5">
-        <v>9133</v>
-      </c>
-      <c r="C13" s="5">
-        <v>5977</v>
-      </c>
-      <c r="D13" s="5">
-        <v>3156</v>
-      </c>
-      <c r="E13" s="5">
-        <v>8707</v>
-      </c>
-      <c r="F13" s="5">
-        <v>426</v>
-      </c>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
+      <c r="B14" s="5">
+        <v>9968</v>
+      </c>
+      <c r="C14" s="5">
+        <v>6547</v>
+      </c>
+      <c r="D14" s="5">
+        <v>3421</v>
+      </c>
+      <c r="E14" s="5">
+        <v>9480</v>
+      </c>
+      <c r="F14" s="5">
+        <v>488</v>
+      </c>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -657,15 +685,15 @@
     <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="9" max="9" width="24" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="17" customWidth="1"/>
     <col min="12" max="12" width="11" customWidth="1"/>
     <col min="13" max="13" width="21" customWidth="1"/>
     <col min="14" max="14" width="11" customWidth="1"/>
     <col min="15" max="15" width="11" customWidth="1"/>
-    <col min="16" max="16" width="18" customWidth="1"/>
-    <col min="17" max="17" width="17" customWidth="1"/>
+    <col min="16" max="16" width="17" customWidth="1"/>
+    <col min="17" max="17" width="18" customWidth="1"/>
     <col min="18" max="18" width="17" customWidth="1"/>
     <col min="19" max="19" width="23" customWidth="1"/>
   </cols>
@@ -713,14 +741,14 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Friendship</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Inspirational &amp; sympathy</t>
-        </is>
-      </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Congratulations</t>
@@ -748,12 +776,12 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>Keeping in touch</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>World languages</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
@@ -795,10 +823,10 @@
         <v>19</v>
       </c>
       <c r="I2" s="2">
+        <v>10</v>
+      </c>
+      <c r="J2" s="2">
         <v>28</v>
-      </c>
-      <c r="J2" s="2">
-        <v>10</v>
       </c>
       <c r="K2" s="2">
         <v>12</v>
@@ -816,10 +844,10 @@
         <v>4</v>
       </c>
       <c r="P2" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q2" s="2">
         <v>6</v>
-      </c>
-      <c r="Q2" s="2">
-        <v>2</v>
       </c>
       <c r="R2" s="2">
         <v>2</v>
@@ -856,10 +884,10 @@
         <v>24</v>
       </c>
       <c r="I3" s="2">
+        <v>19</v>
+      </c>
+      <c r="J3" s="2">
         <v>41</v>
-      </c>
-      <c r="J3" s="2">
-        <v>19</v>
       </c>
       <c r="K3" s="2">
         <v>11</v>
@@ -877,10 +905,10 @@
         <v>1</v>
       </c>
       <c r="P3" s="2">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="Q3" s="2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="R3" s="2">
         <v>0</v>
@@ -917,10 +945,10 @@
         <v>18</v>
       </c>
       <c r="I4" s="2">
+        <v>16</v>
+      </c>
+      <c r="J4" s="2">
         <v>11</v>
-      </c>
-      <c r="J4" s="2">
-        <v>16</v>
       </c>
       <c r="K4" s="2">
         <v>17</v>
@@ -978,10 +1006,10 @@
         <v>26</v>
       </c>
       <c r="I5" s="2">
+        <v>15</v>
+      </c>
+      <c r="J5" s="2">
         <v>22</v>
-      </c>
-      <c r="J5" s="2">
-        <v>15</v>
       </c>
       <c r="K5" s="2">
         <v>4</v>
@@ -999,10 +1027,10 @@
         <v>1</v>
       </c>
       <c r="P5" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q5" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R5" s="2">
         <v>0</v>
@@ -1039,10 +1067,10 @@
         <v>13</v>
       </c>
       <c r="I6" s="2">
+        <v>15</v>
+      </c>
+      <c r="J6" s="2">
         <v>11</v>
-      </c>
-      <c r="J6" s="2">
-        <v>15</v>
       </c>
       <c r="K6" s="2">
         <v>8</v>
@@ -1060,10 +1088,10 @@
         <v>0</v>
       </c>
       <c r="P6" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="2">
         <v>0</v>
-      </c>
-      <c r="Q6" s="2">
-        <v>1</v>
       </c>
       <c r="R6" s="2">
         <v>2</v>
@@ -1100,10 +1128,10 @@
         <v>11</v>
       </c>
       <c r="I7" s="2">
+        <v>12</v>
+      </c>
+      <c r="J7" s="2">
         <v>16</v>
-      </c>
-      <c r="J7" s="2">
-        <v>12</v>
       </c>
       <c r="K7" s="2">
         <v>10</v>
@@ -1121,10 +1149,10 @@
         <v>0</v>
       </c>
       <c r="P7" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="2">
         <v>0</v>
-      </c>
-      <c r="Q7" s="2">
-        <v>1</v>
       </c>
       <c r="R7" s="2">
         <v>3</v>
@@ -1161,10 +1189,10 @@
         <v>17</v>
       </c>
       <c r="I8" s="2">
+        <v>14</v>
+      </c>
+      <c r="J8" s="2">
         <v>7</v>
-      </c>
-      <c r="J8" s="2">
-        <v>14</v>
       </c>
       <c r="K8" s="2">
         <v>8</v>
@@ -1222,10 +1250,10 @@
         <v>20</v>
       </c>
       <c r="I9" s="2">
+        <v>12</v>
+      </c>
+      <c r="J9" s="2">
         <v>5</v>
-      </c>
-      <c r="J9" s="2">
-        <v>12</v>
       </c>
       <c r="K9" s="2">
         <v>8</v>
@@ -1283,10 +1311,10 @@
         <v>35</v>
       </c>
       <c r="I10" s="2">
+        <v>20</v>
+      </c>
+      <c r="J10" s="2">
         <v>7</v>
-      </c>
-      <c r="J10" s="2">
-        <v>20</v>
       </c>
       <c r="K10" s="2">
         <v>6</v>
@@ -1304,10 +1332,10 @@
         <v>5</v>
       </c>
       <c r="P10" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="2">
         <v>0</v>
-      </c>
-      <c r="Q10" s="2">
-        <v>1</v>
       </c>
       <c r="R10" s="2">
         <v>0</v>
@@ -1344,10 +1372,10 @@
         <v>14</v>
       </c>
       <c r="I11" s="2">
+        <v>16</v>
+      </c>
+      <c r="J11" s="2">
         <v>11</v>
-      </c>
-      <c r="J11" s="2">
-        <v>16</v>
       </c>
       <c r="K11" s="2">
         <v>10</v>
@@ -1365,10 +1393,10 @@
         <v>3</v>
       </c>
       <c r="P11" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R11" s="2">
         <v>0</v>
@@ -1405,10 +1433,10 @@
         <v>13</v>
       </c>
       <c r="I12" s="2">
+        <v>14</v>
+      </c>
+      <c r="J12" s="2">
         <v>5</v>
-      </c>
-      <c r="J12" s="2">
-        <v>14</v>
       </c>
       <c r="K12" s="2">
         <v>14</v>
@@ -1426,10 +1454,10 @@
         <v>0</v>
       </c>
       <c r="P12" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="2">
         <v>6</v>
-      </c>
-      <c r="Q12" s="2">
-        <v>0</v>
       </c>
       <c r="R12" s="2">
         <v>0</v>
@@ -1439,63 +1467,124 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B13" s="2">
+        <v>773</v>
+      </c>
+      <c r="C13" s="2">
+        <v>567</v>
+      </c>
+      <c r="D13" s="2">
+        <v>42</v>
+      </c>
+      <c r="E13" s="2">
+        <v>46</v>
+      </c>
+      <c r="F13" s="2">
+        <v>38</v>
+      </c>
+      <c r="G13" s="2">
+        <v>24</v>
+      </c>
+      <c r="H13" s="2">
+        <v>16</v>
+      </c>
+      <c r="I13" s="2">
+        <v>16</v>
+      </c>
+      <c r="J13" s="2">
+        <v>7</v>
+      </c>
+      <c r="K13" s="2">
+        <v>5</v>
+      </c>
+      <c r="L13" s="2">
+        <v>2</v>
+      </c>
+      <c r="M13" s="2">
+        <v>2</v>
+      </c>
+      <c r="N13" s="2">
+        <v>1</v>
+      </c>
+      <c r="O13" s="2">
+        <v>2</v>
+      </c>
+      <c r="P13" s="2">
+        <v>3</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>2</v>
+      </c>
+      <c r="R13" s="2">
+        <v>0</v>
+      </c>
+      <c r="S13" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B13" s="5">
-        <v>8707</v>
-      </c>
-      <c r="C13" s="5">
-        <v>5700</v>
-      </c>
-      <c r="D13" s="5">
-        <v>855</v>
-      </c>
-      <c r="E13" s="5">
-        <v>525</v>
-      </c>
-      <c r="F13" s="5">
-        <v>416</v>
-      </c>
-      <c r="G13" s="5">
-        <v>352</v>
-      </c>
-      <c r="H13" s="5">
-        <v>210</v>
-      </c>
-      <c r="I13" s="5">
-        <v>164</v>
-      </c>
-      <c r="J13" s="5">
-        <v>163</v>
-      </c>
-      <c r="K13" s="5">
-        <v>108</v>
-      </c>
-      <c r="L13" s="5">
-        <v>80</v>
-      </c>
-      <c r="M13" s="5">
+      <c r="B14" s="5">
+        <v>9480</v>
+      </c>
+      <c r="C14" s="5">
+        <v>6267</v>
+      </c>
+      <c r="D14" s="5">
+        <v>897</v>
+      </c>
+      <c r="E14" s="5">
+        <v>571</v>
+      </c>
+      <c r="F14" s="5">
+        <v>454</v>
+      </c>
+      <c r="G14" s="5">
+        <v>376</v>
+      </c>
+      <c r="H14" s="5">
+        <v>226</v>
+      </c>
+      <c r="I14" s="5">
+        <v>179</v>
+      </c>
+      <c r="J14" s="5">
+        <v>171</v>
+      </c>
+      <c r="K14" s="5">
+        <v>113</v>
+      </c>
+      <c r="L14" s="5">
+        <v>82</v>
+      </c>
+      <c r="M14" s="5">
+        <v>35</v>
+      </c>
+      <c r="N14" s="5">
         <v>33</v>
       </c>
-      <c r="N13" s="5">
-        <v>32</v>
-      </c>
-      <c r="O13" s="5">
-        <v>23</v>
-      </c>
-      <c r="P13" s="5">
-        <v>17</v>
-      </c>
-      <c r="Q13" s="5">
-        <v>17</v>
-      </c>
-      <c r="R13" s="5">
+      <c r="O14" s="5">
+        <v>25</v>
+      </c>
+      <c r="P14" s="5">
+        <v>20</v>
+      </c>
+      <c r="Q14" s="5">
+        <v>19</v>
+      </c>
+      <c r="R14" s="5">
         <v>9</v>
       </c>
-      <c r="S13" s="5">
+      <c r="S14" s="5">
         <v>3</v>
       </c>
     </row>
@@ -6728,6 +6817,508 @@
       </c>
       <c r="H166" s="4"/>
     </row>
+    <row r="167">
+      <c r="A167" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B167" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C167" s="0" t="inlineStr">
+        <is>
+          <t>birth</t>
+        </is>
+      </c>
+      <c r="D167" s="2">
+        <v>414</v>
+      </c>
+      <c r="E167" s="2">
+        <v>153</v>
+      </c>
+      <c r="F167" s="2">
+        <v>567</v>
+      </c>
+      <c r="G167" s="3">
+        <v>0.7335058214747736</v>
+      </c>
+      <c r="H167" s="2">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B168" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C168" s="0" t="inlineStr">
+        <is>
+          <t>anniv</t>
+        </is>
+      </c>
+      <c r="D168" s="2">
+        <v>33</v>
+      </c>
+      <c r="E168" s="2">
+        <v>13</v>
+      </c>
+      <c r="F168" s="2">
+        <v>46</v>
+      </c>
+      <c r="G168" s="3">
+        <v>0.059508408796895215</v>
+      </c>
+      <c r="H168" s="2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B169" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C169" s="0" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="D169" s="2">
+        <v>36</v>
+      </c>
+      <c r="E169" s="2">
+        <v>6</v>
+      </c>
+      <c r="F169" s="2">
+        <v>42</v>
+      </c>
+      <c r="G169" s="3">
+        <v>0.054333764553686936</v>
+      </c>
+      <c r="H169" s="2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B170" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C170" s="0" t="inlineStr">
+        <is>
+          <t>gen</t>
+        </is>
+      </c>
+      <c r="D170" s="2">
+        <v>26</v>
+      </c>
+      <c r="E170" s="2">
+        <v>12</v>
+      </c>
+      <c r="F170" s="2">
+        <v>38</v>
+      </c>
+      <c r="G170" s="3">
+        <v>0.04915912031047866</v>
+      </c>
+      <c r="H170" s="2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B171" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C171" s="0" t="inlineStr">
+        <is>
+          <t>thank</t>
+        </is>
+      </c>
+      <c r="D171" s="2">
+        <v>5</v>
+      </c>
+      <c r="E171" s="2">
+        <v>19</v>
+      </c>
+      <c r="F171" s="2">
+        <v>24</v>
+      </c>
+      <c r="G171" s="3">
+        <v>0.031047865459249677</v>
+      </c>
+      <c r="H171" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B172" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C172" s="0" t="inlineStr">
+        <is>
+          <t>insp</t>
+        </is>
+      </c>
+      <c r="D172" s="2">
+        <v>14</v>
+      </c>
+      <c r="E172" s="2">
+        <v>2</v>
+      </c>
+      <c r="F172" s="2">
+        <v>16</v>
+      </c>
+      <c r="G172" s="3">
+        <v>0.02069857697283312</v>
+      </c>
+      <c r="H172" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B173" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C173" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D173" s="2">
+        <v>11</v>
+      </c>
+      <c r="E173" s="2">
+        <v>5</v>
+      </c>
+      <c r="F173" s="2">
+        <v>16</v>
+      </c>
+      <c r="G173" s="3">
+        <v>0.02069857697283312</v>
+      </c>
+      <c r="H173" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B174" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C174" s="0" t="inlineStr">
+        <is>
+          <t>friend</t>
+        </is>
+      </c>
+      <c r="D174" s="2">
+        <v>3</v>
+      </c>
+      <c r="E174" s="2">
+        <v>4</v>
+      </c>
+      <c r="F174" s="2">
+        <v>7</v>
+      </c>
+      <c r="G174" s="3">
+        <v>0.009055627425614488</v>
+      </c>
+      <c r="H174" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B175" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C175" s="0" t="inlineStr">
+        <is>
+          <t>congrats</t>
+        </is>
+      </c>
+      <c r="D175" s="2">
+        <v>1</v>
+      </c>
+      <c r="E175" s="2">
+        <v>4</v>
+      </c>
+      <c r="F175" s="2">
+        <v>5</v>
+      </c>
+      <c r="G175" s="3">
+        <v>0.00646830530401035</v>
+      </c>
+      <c r="H175" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B176" s="0" t="inlineStr">
+        <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="C176" s="0" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="D176" s="2">
+        <v>0</v>
+      </c>
+      <c r="E176" s="2">
+        <v>3</v>
+      </c>
+      <c r="F176" s="2">
+        <v>3</v>
+      </c>
+      <c r="G176" s="3">
+        <v>0.0038809831824062097</v>
+      </c>
+      <c r="H176" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B177" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C177" s="0" t="inlineStr">
+        <is>
+          <t>cute</t>
+        </is>
+      </c>
+      <c r="D177" s="2">
+        <v>2</v>
+      </c>
+      <c r="E177" s="2">
+        <v>0</v>
+      </c>
+      <c r="F177" s="2">
+        <v>2</v>
+      </c>
+      <c r="G177" s="3">
+        <v>0.00258732212160414</v>
+      </c>
+      <c r="H177" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B178" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C178" s="0" t="inlineStr">
+        <is>
+          <t>fkt</t>
+        </is>
+      </c>
+      <c r="D178" s="2">
+        <v>1</v>
+      </c>
+      <c r="E178" s="2">
+        <v>1</v>
+      </c>
+      <c r="F178" s="2">
+        <v>2</v>
+      </c>
+      <c r="G178" s="3">
+        <v>0.00258732212160414</v>
+      </c>
+      <c r="H178" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B179" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C179" s="0" t="inlineStr">
+        <is>
+          <t>flwr</t>
+        </is>
+      </c>
+      <c r="D179" s="2">
+        <v>2</v>
+      </c>
+      <c r="E179" s="2">
+        <v>0</v>
+      </c>
+      <c r="F179" s="2">
+        <v>2</v>
+      </c>
+      <c r="G179" s="3">
+        <v>0.00258732212160414</v>
+      </c>
+      <c r="H179" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B180" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C180" s="0" t="inlineStr">
+        <is>
+          <t>intouch</t>
+        </is>
+      </c>
+      <c r="D180" s="2">
+        <v>2</v>
+      </c>
+      <c r="E180" s="2">
+        <v>0</v>
+      </c>
+      <c r="F180" s="2">
+        <v>2</v>
+      </c>
+      <c r="G180" s="3">
+        <v>0.00258732212160414</v>
+      </c>
+      <c r="H180" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B181" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C181" s="0" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="D181" s="2">
+        <v>1</v>
+      </c>
+      <c r="E181" s="2">
+        <v>0</v>
+      </c>
+      <c r="F181" s="2">
+        <v>1</v>
+      </c>
+      <c r="G181" s="3">
+        <v>0.00129366106080207</v>
+      </c>
+      <c r="H181" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-12</t>
+        </is>
+      </c>
+      <c r="B182" s="4"/>
+      <c r="C182" s="4"/>
+      <c r="D182" s="5">
+        <v>551</v>
+      </c>
+      <c r="E182" s="5">
+        <v>222</v>
+      </c>
+      <c r="F182" s="5">
+        <v>773</v>
+      </c>
+      <c r="G182" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="H182" s="4"/>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -32688,6 +33279,2344 @@
         <v>732</v>
       </c>
       <c r="F932" s="4"/>
+    </row>
+    <row r="933">
+      <c r="A933" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B933" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C933" s="0" t="inlineStr">
+        <is>
+          <t>happybirthday</t>
+        </is>
+      </c>
+      <c r="D933" s="0" t="inlineStr">
+        <is>
+          <t>birth_happybirthday</t>
+        </is>
+      </c>
+      <c r="E933" s="2">
+        <v>458</v>
+      </c>
+      <c r="F933" s="2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B934" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C934" s="0" t="inlineStr">
+        <is>
+          <t>anniversaryetc</t>
+        </is>
+      </c>
+      <c r="D934" s="0" t="inlineStr">
+        <is>
+          <t>anniv_anniversaryetc</t>
+        </is>
+      </c>
+      <c r="E934" s="2">
+        <v>29</v>
+      </c>
+      <c r="F934" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B935" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C935" s="0" t="inlineStr">
+        <is>
+          <t>fun</t>
+        </is>
+      </c>
+      <c r="D935" s="0" t="inlineStr">
+        <is>
+          <t>birth_fun</t>
+        </is>
+      </c>
+      <c r="E935" s="2">
+        <v>22</v>
+      </c>
+      <c r="F935" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B936" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C936" s="0" t="inlineStr">
+        <is>
+          <t>sympathy</t>
+        </is>
+      </c>
+      <c r="D936" s="0" t="inlineStr">
+        <is>
+          <t>insp_sympathy</t>
+        </is>
+      </c>
+      <c r="E936" s="2">
+        <v>13</v>
+      </c>
+      <c r="F936" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B937" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C937" s="0" t="inlineStr">
+        <is>
+          <t>flowers</t>
+        </is>
+      </c>
+      <c r="D937" s="0" t="inlineStr">
+        <is>
+          <t>birth_flowers</t>
+        </is>
+      </c>
+      <c r="E937" s="2">
+        <v>11</v>
+      </c>
+      <c r="F937" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B938" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C938" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D938" s="0" t="inlineStr">
+        <is>
+          <t>gen_getwell</t>
+        </is>
+      </c>
+      <c r="E938" s="2">
+        <v>11</v>
+      </c>
+      <c r="F938" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B939" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C939" s="0" t="inlineStr">
+        <is>
+          <t>birthday</t>
+        </is>
+      </c>
+      <c r="D939" s="0" t="inlineStr">
+        <is>
+          <t>thank_birthday</t>
+        </is>
+      </c>
+      <c r="E939" s="2">
+        <v>11</v>
+      </c>
+      <c r="F939" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B940" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C940" s="0" t="inlineStr">
+        <is>
+          <t>bronsis</t>
+        </is>
+      </c>
+      <c r="D940" s="0" t="inlineStr">
+        <is>
+          <t>birth_bronsis</t>
+        </is>
+      </c>
+      <c r="E940" s="2">
+        <v>10</v>
+      </c>
+      <c r="F940" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B941" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C941" s="0" t="inlineStr">
+        <is>
+          <t>eaug_juliennefries_day</t>
+        </is>
+      </c>
+      <c r="D941" s="0" t="inlineStr">
+        <is>
+          <t>eaug_juliennefries_day</t>
+        </is>
+      </c>
+      <c r="E941" s="2">
+        <v>10</v>
+      </c>
+      <c r="F941" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B942" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C942" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_general</t>
+        </is>
+      </c>
+      <c r="D942" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_general</t>
+        </is>
+      </c>
+      <c r="E942" s="2">
+        <v>10</v>
+      </c>
+      <c r="F942" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B943" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C943" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="D943" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="E943" s="2">
+        <v>9</v>
+      </c>
+      <c r="F943" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B944" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C944" s="0" t="inlineStr">
+        <is>
+          <t>sonanddaughter</t>
+        </is>
+      </c>
+      <c r="D944" s="0" t="inlineStr">
+        <is>
+          <t>birth_sonanddaughter</t>
+        </is>
+      </c>
+      <c r="E944" s="2">
+        <v>9</v>
+      </c>
+      <c r="F944" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B945" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C945" s="0" t="inlineStr">
+        <is>
+          <t>songs</t>
+        </is>
+      </c>
+      <c r="D945" s="0" t="inlineStr">
+        <is>
+          <t>birth_songs</t>
+        </is>
+      </c>
+      <c r="E945" s="2">
+        <v>9</v>
+      </c>
+      <c r="F945" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B946" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C946" s="0" t="inlineStr">
+        <is>
+          <t>wishes</t>
+        </is>
+      </c>
+      <c r="D946" s="0" t="inlineStr">
+        <is>
+          <t>birth_wishes</t>
+        </is>
+      </c>
+      <c r="E946" s="2">
+        <v>9</v>
+      </c>
+      <c r="F946" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B947" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C947" s="0" t="inlineStr">
+        <is>
+          <t>morning</t>
+        </is>
+      </c>
+      <c r="D947" s="0" t="inlineStr">
+        <is>
+          <t>gen_morning</t>
+        </is>
+      </c>
+      <c r="E947" s="2">
+        <v>8</v>
+      </c>
+      <c r="F947" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B948" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C948" s="0" t="inlineStr">
+        <is>
+          <t>everyday</t>
+        </is>
+      </c>
+      <c r="D948" s="0" t="inlineStr">
+        <is>
+          <t>thank_everyday</t>
+        </is>
+      </c>
+      <c r="E948" s="2">
+        <v>8</v>
+      </c>
+      <c r="F948" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B949" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C949" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D949" s="0" t="inlineStr">
+        <is>
+          <t>birth_milestone</t>
+        </is>
+      </c>
+      <c r="E949" s="2">
+        <v>7</v>
+      </c>
+      <c r="F949" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B950" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C950" s="0" t="inlineStr">
+        <is>
+          <t>eaug_romanceday</t>
+        </is>
+      </c>
+      <c r="D950" s="0" t="inlineStr">
+        <is>
+          <t>eaug_romanceday</t>
+        </is>
+      </c>
+      <c r="E950" s="2">
+        <v>7</v>
+      </c>
+      <c r="F950" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B951" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C951" s="0" t="inlineStr">
+        <is>
+          <t>friends</t>
+        </is>
+      </c>
+      <c r="D951" s="0" t="inlineStr">
+        <is>
+          <t>birth_friends</t>
+        </is>
+      </c>
+      <c r="E951" s="2">
+        <v>6</v>
+      </c>
+      <c r="F951" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B952" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C952" s="0" t="inlineStr">
+        <is>
+          <t>hubbywife</t>
+        </is>
+      </c>
+      <c r="D952" s="0" t="inlineStr">
+        <is>
+          <t>birth_hubbywife</t>
+        </is>
+      </c>
+      <c r="E952" s="2">
+        <v>6</v>
+      </c>
+      <c r="F952" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B953" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C953" s="0" t="inlineStr">
+        <is>
+          <t>specials</t>
+        </is>
+      </c>
+      <c r="D953" s="0" t="inlineStr">
+        <is>
+          <t>birth_specials</t>
+        </is>
+      </c>
+      <c r="E953" s="2">
+        <v>5</v>
+      </c>
+      <c r="F953" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B954" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C954" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D954" s="0" t="inlineStr">
+        <is>
+          <t>anniv_milestone</t>
+        </is>
+      </c>
+      <c r="E954" s="2">
+        <v>4</v>
+      </c>
+      <c r="F954" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B955" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C955" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="D955" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="E955" s="2">
+        <v>4</v>
+      </c>
+      <c r="F955" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B956" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C956" s="0" t="inlineStr">
+        <is>
+          <t>belated</t>
+        </is>
+      </c>
+      <c r="D956" s="0" t="inlineStr">
+        <is>
+          <t>birth_belated</t>
+        </is>
+      </c>
+      <c r="E956" s="2">
+        <v>4</v>
+      </c>
+      <c r="F956" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B957" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C957" s="0" t="inlineStr">
+        <is>
+          <t>blessings</t>
+        </is>
+      </c>
+      <c r="D957" s="0" t="inlineStr">
+        <is>
+          <t>birth_blessings</t>
+        </is>
+      </c>
+      <c r="E957" s="2">
+        <v>4</v>
+      </c>
+      <c r="F957" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B958" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C958" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="D958" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="E958" s="2">
+        <v>4</v>
+      </c>
+      <c r="F958" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B959" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C959" s="0" t="inlineStr">
+        <is>
+          <t>bestfriends</t>
+        </is>
+      </c>
+      <c r="D959" s="0" t="inlineStr">
+        <is>
+          <t>friend_bestfriends</t>
+        </is>
+      </c>
+      <c r="E959" s="2">
+        <v>4</v>
+      </c>
+      <c r="F959" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B960" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C960" s="0" t="inlineStr">
+        <is>
+          <t>thinkingofyou</t>
+        </is>
+      </c>
+      <c r="D960" s="0" t="inlineStr">
+        <is>
+          <t>gen_thinkingofyou</t>
+        </is>
+      </c>
+      <c r="E960" s="2">
+        <v>4</v>
+      </c>
+      <c r="F960" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B961" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C961" s="0" t="inlineStr">
+        <is>
+          <t>eaug_vanillacustard_day</t>
+        </is>
+      </c>
+      <c r="D961" s="0" t="inlineStr">
+        <is>
+          <t>eaug_vanillacustard_day</t>
+        </is>
+      </c>
+      <c r="E961" s="2">
+        <v>3</v>
+      </c>
+      <c r="F961" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B962" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C962" s="0" t="inlineStr">
+        <is>
+          <t>hvgtday</t>
+        </is>
+      </c>
+      <c r="D962" s="0" t="inlineStr">
+        <is>
+          <t>gen_hvgtday</t>
+        </is>
+      </c>
+      <c r="E962" s="2">
+        <v>3</v>
+      </c>
+      <c r="F962" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B963" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C963" s="0" t="inlineStr">
+        <is>
+          <t>voyage</t>
+        </is>
+      </c>
+      <c r="D963" s="0" t="inlineStr">
+        <is>
+          <t>gen_voyage</t>
+        </is>
+      </c>
+      <c r="E963" s="2">
+        <v>3</v>
+      </c>
+      <c r="F963" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B964" s="0" t="inlineStr">
+        <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="C964" s="0" t="inlineStr">
+        <is>
+          <t>russian_birthday</t>
+        </is>
+      </c>
+      <c r="D964" s="0" t="inlineStr">
+        <is>
+          <t>w_russian_birthday</t>
+        </is>
+      </c>
+      <c r="E964" s="2">
+        <v>3</v>
+      </c>
+      <c r="F964" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B965" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C965" s="0" t="inlineStr">
+        <is>
+          <t>extfamily</t>
+        </is>
+      </c>
+      <c r="D965" s="0" t="inlineStr">
+        <is>
+          <t>birth_extfamily</t>
+        </is>
+      </c>
+      <c r="E965" s="2">
+        <v>2</v>
+      </c>
+      <c r="F965" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B966" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C966" s="0" t="inlineStr">
+        <is>
+          <t>momndad</t>
+        </is>
+      </c>
+      <c r="D966" s="0" t="inlineStr">
+        <is>
+          <t>birth_momndad</t>
+        </is>
+      </c>
+      <c r="E966" s="2">
+        <v>2</v>
+      </c>
+      <c r="F966" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B967" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C967" s="0" t="inlineStr">
+        <is>
+          <t>newbaby</t>
+        </is>
+      </c>
+      <c r="D967" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newbaby</t>
+        </is>
+      </c>
+      <c r="E967" s="2">
+        <v>2</v>
+      </c>
+      <c r="F967" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B968" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C968" s="0" t="inlineStr">
+        <is>
+          <t>newhome</t>
+        </is>
+      </c>
+      <c r="D968" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newhome</t>
+        </is>
+      </c>
+      <c r="E968" s="2">
+        <v>2</v>
+      </c>
+      <c r="F968" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B969" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C969" s="0" t="inlineStr">
+        <is>
+          <t>hugs</t>
+        </is>
+      </c>
+      <c r="D969" s="0" t="inlineStr">
+        <is>
+          <t>cute_hugs</t>
+        </is>
+      </c>
+      <c r="E969" s="2">
+        <v>2</v>
+      </c>
+      <c r="F969" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B970" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C970" s="0" t="inlineStr">
+        <is>
+          <t>eaug_internationalleft_handers_day</t>
+        </is>
+      </c>
+      <c r="D970" s="0" t="inlineStr">
+        <is>
+          <t>eaug_internationalleft_handers_day</t>
+        </is>
+      </c>
+      <c r="E970" s="2">
+        <v>2</v>
+      </c>
+      <c r="F970" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B971" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C971" s="0" t="inlineStr">
+        <is>
+          <t>eaug_justbecauseday</t>
+        </is>
+      </c>
+      <c r="D971" s="0" t="inlineStr">
+        <is>
+          <t>eaug_justbecauseday</t>
+        </is>
+      </c>
+      <c r="E971" s="2">
+        <v>2</v>
+      </c>
+      <c r="F971" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B972" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C972" s="0" t="inlineStr">
+        <is>
+          <t>eaug_smilemonth</t>
+        </is>
+      </c>
+      <c r="D972" s="0" t="inlineStr">
+        <is>
+          <t>eaug_smilemonth</t>
+        </is>
+      </c>
+      <c r="E972" s="2">
+        <v>2</v>
+      </c>
+      <c r="F972" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B973" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C973" s="0" t="inlineStr">
+        <is>
+          <t>esep_wifeappreciation_day</t>
+        </is>
+      </c>
+      <c r="D973" s="0" t="inlineStr">
+        <is>
+          <t>esep_wifeappreciation_day</t>
+        </is>
+      </c>
+      <c r="E973" s="2">
+        <v>2</v>
+      </c>
+      <c r="F973" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B974" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C974" s="0" t="inlineStr">
+        <is>
+          <t>goodnight</t>
+        </is>
+      </c>
+      <c r="D974" s="0" t="inlineStr">
+        <is>
+          <t>gen_goodnight</t>
+        </is>
+      </c>
+      <c r="E974" s="2">
+        <v>2</v>
+      </c>
+      <c r="F974" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B975" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C975" s="0" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="D975" s="0" t="inlineStr">
+        <is>
+          <t>gen_hi</t>
+        </is>
+      </c>
+      <c r="E975" s="2">
+        <v>2</v>
+      </c>
+      <c r="F975" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B976" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C976" s="0" t="inlineStr">
+        <is>
+          <t>justbecause</t>
+        </is>
+      </c>
+      <c r="D976" s="0" t="inlineStr">
+        <is>
+          <t>intouch_justbecause</t>
+        </is>
+      </c>
+      <c r="E976" s="2">
+        <v>2</v>
+      </c>
+      <c r="F976" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B977" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C977" s="0" t="inlineStr">
+        <is>
+          <t>lovepoems</t>
+        </is>
+      </c>
+      <c r="D977" s="0" t="inlineStr">
+        <is>
+          <t>love_lovepoems</t>
+        </is>
+      </c>
+      <c r="E977" s="2">
+        <v>2</v>
+      </c>
+      <c r="F977" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B978" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C978" s="0" t="inlineStr">
+        <is>
+          <t>wedding</t>
+        </is>
+      </c>
+      <c r="D978" s="0" t="inlineStr">
+        <is>
+          <t>thank_wedding</t>
+        </is>
+      </c>
+      <c r="E978" s="2">
+        <v>2</v>
+      </c>
+      <c r="F978" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B979" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C979" s="0" t="inlineStr">
+        <is>
+          <t>balloons</t>
+        </is>
+      </c>
+      <c r="D979" s="0" t="inlineStr">
+        <is>
+          <t>birth_balloons</t>
+        </is>
+      </c>
+      <c r="E979" s="2">
+        <v>1</v>
+      </c>
+      <c r="F979" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B980" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C980" s="0" t="inlineStr">
+        <is>
+          <t>grandparents</t>
+        </is>
+      </c>
+      <c r="D980" s="0" t="inlineStr">
+        <is>
+          <t>birth_grandparents</t>
+        </is>
+      </c>
+      <c r="E980" s="2">
+        <v>1</v>
+      </c>
+      <c r="F980" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B981" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C981" s="0" t="inlineStr">
+        <is>
+          <t>pets</t>
+        </is>
+      </c>
+      <c r="D981" s="0" t="inlineStr">
+        <is>
+          <t>birth_pets</t>
+        </is>
+      </c>
+      <c r="E981" s="2">
+        <v>1</v>
+      </c>
+      <c r="F981" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B982" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C982" s="0" t="inlineStr">
+        <is>
+          <t>studentsandnewgrads</t>
+        </is>
+      </c>
+      <c r="D982" s="0" t="inlineStr">
+        <is>
+          <t>congrats_studentsandnewgrads</t>
+        </is>
+      </c>
+      <c r="E982" s="2">
+        <v>1</v>
+      </c>
+      <c r="F982" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B983" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C983" s="0" t="inlineStr">
+        <is>
+          <t>eapr_easter_humor</t>
+        </is>
+      </c>
+      <c r="D983" s="0" t="inlineStr">
+        <is>
+          <t>eapr_easter_humor</t>
+        </is>
+      </c>
+      <c r="E983" s="2">
+        <v>1</v>
+      </c>
+      <c r="F983" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B984" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C984" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalrelaxation_day</t>
+        </is>
+      </c>
+      <c r="D984" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalrelaxation_day</t>
+        </is>
+      </c>
+      <c r="E984" s="2">
+        <v>1</v>
+      </c>
+      <c r="F984" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B985" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C985" s="0" t="inlineStr">
+        <is>
+          <t>eaug_rakshabandhan_happy</t>
+        </is>
+      </c>
+      <c r="D985" s="0" t="inlineStr">
+        <is>
+          <t>eaug_rakshabandhan_happy</t>
+        </is>
+      </c>
+      <c r="E985" s="2">
+        <v>1</v>
+      </c>
+      <c r="F985" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B986" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C986" s="0" t="inlineStr">
+        <is>
+          <t>eaug_thankyouday</t>
+        </is>
+      </c>
+      <c r="D986" s="0" t="inlineStr">
+        <is>
+          <t>eaug_thankyouday</t>
+        </is>
+      </c>
+      <c r="E986" s="2">
+        <v>1</v>
+      </c>
+      <c r="F986" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B987" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C987" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_birthday</t>
+        </is>
+      </c>
+      <c r="D987" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_birthday</t>
+        </is>
+      </c>
+      <c r="E987" s="2">
+        <v>1</v>
+      </c>
+      <c r="F987" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B988" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C988" s="0" t="inlineStr">
+        <is>
+          <t>emay_graduation_wishes</t>
+        </is>
+      </c>
+      <c r="D988" s="0" t="inlineStr">
+        <is>
+          <t>emay_graduation_wishes</t>
+        </is>
+      </c>
+      <c r="E988" s="2">
+        <v>1</v>
+      </c>
+      <c r="F988" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B989" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C989" s="0" t="inlineStr">
+        <is>
+          <t>enov_adventday</t>
+        </is>
+      </c>
+      <c r="D989" s="0" t="inlineStr">
+        <is>
+          <t>enov_adventday</t>
+        </is>
+      </c>
+      <c r="E989" s="2">
+        <v>1</v>
+      </c>
+      <c r="F989" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B990" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C990" s="0" t="inlineStr">
+        <is>
+          <t>eoct_sweetday_specials</t>
+        </is>
+      </c>
+      <c r="D990" s="0" t="inlineStr">
+        <is>
+          <t>eoct_sweetday_specials</t>
+        </is>
+      </c>
+      <c r="E990" s="2">
+        <v>1</v>
+      </c>
+      <c r="F990" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B991" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C991" s="0" t="inlineStr">
+        <is>
+          <t>esep_fall_specials</t>
+        </is>
+      </c>
+      <c r="D991" s="0" t="inlineStr">
+        <is>
+          <t>esep_fall_specials</t>
+        </is>
+      </c>
+      <c r="E991" s="2">
+        <v>1</v>
+      </c>
+      <c r="F991" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B992" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C992" s="0" t="inlineStr">
+        <is>
+          <t>esep_longestkissday</t>
+        </is>
+      </c>
+      <c r="D992" s="0" t="inlineStr">
+        <is>
+          <t>esep_longestkissday</t>
+        </is>
+      </c>
+      <c r="E992" s="2">
+        <v>1</v>
+      </c>
+      <c r="F992" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B993" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C993" s="0" t="inlineStr">
+        <is>
+          <t>sisters</t>
+        </is>
+      </c>
+      <c r="D993" s="0" t="inlineStr">
+        <is>
+          <t>fkt_sisters</t>
+        </is>
+      </c>
+      <c r="E993" s="2">
+        <v>1</v>
+      </c>
+      <c r="F993" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B994" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C994" s="0" t="inlineStr">
+        <is>
+          <t>sonsdaughter</t>
+        </is>
+      </c>
+      <c r="D994" s="0" t="inlineStr">
+        <is>
+          <t>fkt_sonsdaughter</t>
+        </is>
+      </c>
+      <c r="E994" s="2">
+        <v>1</v>
+      </c>
+      <c r="F994" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B995" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C995" s="0" t="inlineStr">
+        <is>
+          <t>roses</t>
+        </is>
+      </c>
+      <c r="D995" s="0" t="inlineStr">
+        <is>
+          <t>flwr_roses</t>
+        </is>
+      </c>
+      <c r="E995" s="2">
+        <v>1</v>
+      </c>
+      <c r="F995" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B996" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C996" s="0" t="inlineStr">
+        <is>
+          <t>youcare</t>
+        </is>
+      </c>
+      <c r="D996" s="0" t="inlineStr">
+        <is>
+          <t>flwr_youcare</t>
+        </is>
+      </c>
+      <c r="E996" s="2">
+        <v>1</v>
+      </c>
+      <c r="F996" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B997" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C997" s="0" t="inlineStr">
+        <is>
+          <t>foryou</t>
+        </is>
+      </c>
+      <c r="D997" s="0" t="inlineStr">
+        <is>
+          <t>friend_foryou</t>
+        </is>
+      </c>
+      <c r="E997" s="2">
+        <v>1</v>
+      </c>
+      <c r="F997" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B998" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C998" s="0" t="inlineStr">
+        <is>
+          <t>friendsforever</t>
+        </is>
+      </c>
+      <c r="D998" s="0" t="inlineStr">
+        <is>
+          <t>friend_friendsforever</t>
+        </is>
+      </c>
+      <c r="E998" s="2">
+        <v>1</v>
+      </c>
+      <c r="F998" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B999" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C999" s="0" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="D999" s="0" t="inlineStr">
+        <is>
+          <t>friend_hello</t>
+        </is>
+      </c>
+      <c r="E999" s="2">
+        <v>1</v>
+      </c>
+      <c r="F999" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1000" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1000" s="0" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="D1000" s="0" t="inlineStr">
+        <is>
+          <t>gen_luck</t>
+        </is>
+      </c>
+      <c r="E1000" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1000" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1001" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1001" s="0" t="inlineStr">
+        <is>
+          <t>midcrisis</t>
+        </is>
+      </c>
+      <c r="D1001" s="0" t="inlineStr">
+        <is>
+          <t>gen_midcrisis</t>
+        </is>
+      </c>
+      <c r="E1001" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1001" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1002" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1002" s="0" t="inlineStr">
+        <is>
+          <t>missyou</t>
+        </is>
+      </c>
+      <c r="D1002" s="0" t="inlineStr">
+        <is>
+          <t>gen_missyou</t>
+        </is>
+      </c>
+      <c r="E1002" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1002" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1003" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1003" s="0" t="inlineStr">
+        <is>
+          <t>sorry</t>
+        </is>
+      </c>
+      <c r="D1003" s="0" t="inlineStr">
+        <is>
+          <t>gen_sorry</t>
+        </is>
+      </c>
+      <c r="E1003" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1003" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1004" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1004" s="0" t="inlineStr">
+        <is>
+          <t>youarewelcome</t>
+        </is>
+      </c>
+      <c r="D1004" s="0" t="inlineStr">
+        <is>
+          <t>gen_youarewelcome</t>
+        </is>
+      </c>
+      <c r="E1004" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1004" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1005" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1005" s="0" t="inlineStr">
+        <is>
+          <t>poetry</t>
+        </is>
+      </c>
+      <c r="D1005" s="0" t="inlineStr">
+        <is>
+          <t>insp_poetry</t>
+        </is>
+      </c>
+      <c r="E1005" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1005" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1006" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1006" s="0" t="inlineStr">
+        <is>
+          <t>quotes</t>
+        </is>
+      </c>
+      <c r="D1006" s="0" t="inlineStr">
+        <is>
+          <t>insp_quotes</t>
+        </is>
+      </c>
+      <c r="E1006" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1006" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1007" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1007" s="0" t="inlineStr">
+        <is>
+          <t>recovery</t>
+        </is>
+      </c>
+      <c r="D1007" s="0" t="inlineStr">
+        <is>
+          <t>insp_recovery</t>
+        </is>
+      </c>
+      <c r="E1007" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1007" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1008" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1008" s="0" t="inlineStr">
+        <is>
+          <t>dating</t>
+        </is>
+      </c>
+      <c r="D1008" s="0" t="inlineStr">
+        <is>
+          <t>love_dating</t>
+        </is>
+      </c>
+      <c r="E1008" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1008" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1009" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1009" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="D1009" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="E1009" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1009" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1010" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1010" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="D1010" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="E1010" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1010" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1011" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1011" s="0" t="inlineStr">
+        <is>
+          <t>newlove</t>
+        </is>
+      </c>
+      <c r="D1011" s="0" t="inlineStr">
+        <is>
+          <t>love_newlove</t>
+        </is>
+      </c>
+      <c r="E1011" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1011" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1012" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C1012" s="0" t="inlineStr">
+        <is>
+          <t>lossofpet</t>
+        </is>
+      </c>
+      <c r="D1012" s="0" t="inlineStr">
+        <is>
+          <t>pet_lossofpet</t>
+        </is>
+      </c>
+      <c r="E1012" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1012" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1013" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1013" s="0" t="inlineStr">
+        <is>
+          <t>congratulations</t>
+        </is>
+      </c>
+      <c r="D1013" s="0" t="inlineStr">
+        <is>
+          <t>thank_congratulations</t>
+        </is>
+      </c>
+      <c r="E1013" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1013" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1014" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1014" s="0" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="D1014" s="0" t="inlineStr">
+        <is>
+          <t>thank_family</t>
+        </is>
+      </c>
+      <c r="E1014" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1014" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1015" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1015" s="0" t="inlineStr">
+        <is>
+          <t>stayintouch</t>
+        </is>
+      </c>
+      <c r="D1015" s="0" t="inlineStr">
+        <is>
+          <t>thank_stayintouch</t>
+        </is>
+      </c>
+      <c r="E1015" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1015" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1016" s="4"/>
+      <c r="C1016" s="4"/>
+      <c r="D1016" s="4"/>
+      <c r="E1016" s="5">
+        <v>773</v>
+      </c>
+      <c r="F1016" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -32721,12 +35650,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Whatsapp</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Text</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -32770,10 +35699,10 @@
         <v>1059</v>
       </c>
       <c r="C2" s="2">
+        <v>280</v>
+      </c>
+      <c r="D2" s="2">
         <v>404</v>
-      </c>
-      <c r="D2" s="2">
-        <v>280</v>
       </c>
       <c r="E2" s="2">
         <v>177</v>
@@ -32804,10 +35733,10 @@
         <v>999</v>
       </c>
       <c r="C3" s="2">
+        <v>266</v>
+      </c>
+      <c r="D3" s="2">
         <v>355</v>
-      </c>
-      <c r="D3" s="2">
-        <v>266</v>
       </c>
       <c r="E3" s="2">
         <v>174</v>
@@ -32838,10 +35767,10 @@
         <v>765</v>
       </c>
       <c r="C4" s="2">
+        <v>238</v>
+      </c>
+      <c r="D4" s="2">
         <v>242</v>
-      </c>
-      <c r="D4" s="2">
-        <v>238</v>
       </c>
       <c r="E4" s="2">
         <v>148</v>
@@ -32872,10 +35801,10 @@
         <v>805</v>
       </c>
       <c r="C5" s="2">
+        <v>268</v>
+      </c>
+      <c r="D5" s="2">
         <v>247</v>
-      </c>
-      <c r="D5" s="2">
-        <v>268</v>
       </c>
       <c r="E5" s="2">
         <v>160</v>
@@ -32906,10 +35835,10 @@
         <v>742</v>
       </c>
       <c r="C6" s="2">
+        <v>247</v>
+      </c>
+      <c r="D6" s="2">
         <v>224</v>
-      </c>
-      <c r="D6" s="2">
-        <v>247</v>
       </c>
       <c r="E6" s="2">
         <v>131</v>
@@ -32940,10 +35869,10 @@
         <v>738</v>
       </c>
       <c r="C7" s="2">
+        <v>245</v>
+      </c>
+      <c r="D7" s="2">
         <v>224</v>
-      </c>
-      <c r="D7" s="2">
-        <v>245</v>
       </c>
       <c r="E7" s="2">
         <v>163</v>
@@ -32974,10 +35903,10 @@
         <v>760</v>
       </c>
       <c r="C8" s="2">
+        <v>244</v>
+      </c>
+      <c r="D8" s="2">
         <v>218</v>
-      </c>
-      <c r="D8" s="2">
-        <v>244</v>
       </c>
       <c r="E8" s="2">
         <v>179</v>
@@ -33008,10 +35937,10 @@
         <v>839</v>
       </c>
       <c r="C9" s="2">
+        <v>292</v>
+      </c>
+      <c r="D9" s="2">
         <v>228</v>
-      </c>
-      <c r="D9" s="2">
-        <v>292</v>
       </c>
       <c r="E9" s="2">
         <v>161</v>
@@ -33042,10 +35971,10 @@
         <v>711</v>
       </c>
       <c r="C10" s="2">
+        <v>225</v>
+      </c>
+      <c r="D10" s="2">
         <v>210</v>
-      </c>
-      <c r="D10" s="2">
-        <v>225</v>
       </c>
       <c r="E10" s="2">
         <v>165</v>
@@ -33076,10 +36005,10 @@
         <v>949</v>
       </c>
       <c r="C11" s="2">
+        <v>290</v>
+      </c>
+      <c r="D11" s="2">
         <v>288</v>
-      </c>
-      <c r="D11" s="2">
-        <v>290</v>
       </c>
       <c r="E11" s="2">
         <v>200</v>
@@ -33110,10 +36039,10 @@
         <v>766</v>
       </c>
       <c r="C12" s="2">
+        <v>237</v>
+      </c>
+      <c r="D12" s="2">
         <v>226</v>
-      </c>
-      <c r="D12" s="2">
-        <v>237</v>
       </c>
       <c r="E12" s="2">
         <v>155</v>
@@ -33135,36 +36064,70 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B13" s="2">
+        <v>835</v>
+      </c>
+      <c r="C13" s="2">
+        <v>312</v>
+      </c>
+      <c r="D13" s="2">
+        <v>211</v>
+      </c>
+      <c r="E13" s="2">
+        <v>162</v>
+      </c>
+      <c r="F13" s="2">
+        <v>88</v>
+      </c>
+      <c r="G13" s="2">
+        <v>41</v>
+      </c>
+      <c r="H13" s="2">
+        <v>21</v>
+      </c>
+      <c r="I13" s="2">
+        <v>0</v>
+      </c>
+      <c r="J13" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B13" s="5">
-        <v>9133</v>
-      </c>
-      <c r="C13" s="5">
-        <v>2866</v>
-      </c>
-      <c r="D13" s="5">
-        <v>2832</v>
-      </c>
-      <c r="E13" s="5">
-        <v>1813</v>
-      </c>
-      <c r="F13" s="5">
-        <v>955</v>
-      </c>
-      <c r="G13" s="5">
-        <v>336</v>
-      </c>
-      <c r="H13" s="5">
-        <v>302</v>
-      </c>
-      <c r="I13" s="5">
+      <c r="B14" s="5">
+        <v>9968</v>
+      </c>
+      <c r="C14" s="5">
+        <v>3144</v>
+      </c>
+      <c r="D14" s="5">
+        <v>3077</v>
+      </c>
+      <c r="E14" s="5">
+        <v>1975</v>
+      </c>
+      <c r="F14" s="5">
+        <v>1043</v>
+      </c>
+      <c r="G14" s="5">
+        <v>377</v>
+      </c>
+      <c r="H14" s="5">
+        <v>323</v>
+      </c>
+      <c r="I14" s="5">
         <v>28</v>
       </c>
-      <c r="J13" s="5">
+      <c r="J14" s="5">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Record 13 August: thirteen days, 10,776 sends tracked
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9KsXegBwxB1sWdCzRVLrr
</commit_message>
<xml_diff>
--- a/reports/daily_tracking.xlsx
+++ b/reports/daily_tracking.xlsx
@@ -224,7 +224,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13">
@@ -247,7 +247,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -647,28 +647,56 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B14" s="2">
+        <v>808</v>
+      </c>
+      <c r="C14" s="2">
+        <v>548</v>
+      </c>
+      <c r="D14" s="2">
+        <v>260</v>
+      </c>
+      <c r="E14" s="2">
+        <v>710</v>
+      </c>
+      <c r="F14" s="2">
+        <v>98</v>
+      </c>
+      <c r="G14" s="2">
+        <v>253</v>
+      </c>
+      <c r="H14" s="2">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="5">
-        <v>9968</v>
-      </c>
-      <c r="C14" s="5">
-        <v>6547</v>
-      </c>
-      <c r="D14" s="5">
-        <v>3421</v>
-      </c>
-      <c r="E14" s="5">
-        <v>9480</v>
-      </c>
-      <c r="F14" s="5">
-        <v>488</v>
-      </c>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
+      <c r="B15" s="5">
+        <v>10776</v>
+      </c>
+      <c r="C15" s="5">
+        <v>7095</v>
+      </c>
+      <c r="D15" s="5">
+        <v>3681</v>
+      </c>
+      <c r="E15" s="5">
+        <v>10190</v>
+      </c>
+      <c r="F15" s="5">
+        <v>586</v>
+      </c>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -689,8 +717,8 @@
     <col min="10" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="17" customWidth="1"/>
     <col min="12" max="12" width="11" customWidth="1"/>
-    <col min="13" max="13" width="21" customWidth="1"/>
-    <col min="14" max="14" width="11" customWidth="1"/>
+    <col min="13" max="13" width="11" customWidth="1"/>
+    <col min="14" max="14" width="21" customWidth="1"/>
     <col min="15" max="15" width="11" customWidth="1"/>
     <col min="16" max="16" width="17" customWidth="1"/>
     <col min="17" max="17" width="18" customWidth="1"/>
@@ -761,12 +789,12 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Family &amp; loved ones</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Pets</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
@@ -896,10 +924,10 @@
         <v>8</v>
       </c>
       <c r="M3" s="2">
+        <v>1</v>
+      </c>
+      <c r="N3" s="2">
         <v>3</v>
-      </c>
-      <c r="N3" s="2">
-        <v>1</v>
       </c>
       <c r="O3" s="2">
         <v>1</v>
@@ -1018,10 +1046,10 @@
         <v>0</v>
       </c>
       <c r="M5" s="2">
+        <v>2</v>
+      </c>
+      <c r="N5" s="2">
         <v>5</v>
-      </c>
-      <c r="N5" s="2">
-        <v>2</v>
       </c>
       <c r="O5" s="2">
         <v>1</v>
@@ -1079,10 +1107,10 @@
         <v>17</v>
       </c>
       <c r="M6" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N6" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O6" s="2">
         <v>0</v>
@@ -1140,10 +1168,10 @@
         <v>0</v>
       </c>
       <c r="M7" s="2">
+        <v>2</v>
+      </c>
+      <c r="N7" s="2">
         <v>8</v>
-      </c>
-      <c r="N7" s="2">
-        <v>2</v>
       </c>
       <c r="O7" s="2">
         <v>0</v>
@@ -1201,10 +1229,10 @@
         <v>6</v>
       </c>
       <c r="M8" s="2">
+        <v>3</v>
+      </c>
+      <c r="N8" s="2">
         <v>6</v>
-      </c>
-      <c r="N8" s="2">
-        <v>3</v>
       </c>
       <c r="O8" s="2">
         <v>1</v>
@@ -1262,10 +1290,10 @@
         <v>39</v>
       </c>
       <c r="M9" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N9" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O9" s="2">
         <v>3</v>
@@ -1323,10 +1351,10 @@
         <v>4</v>
       </c>
       <c r="M10" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N10" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O10" s="2">
         <v>5</v>
@@ -1384,10 +1412,10 @@
         <v>3</v>
       </c>
       <c r="M11" s="2">
+        <v>8</v>
+      </c>
+      <c r="N11" s="2">
         <v>4</v>
-      </c>
-      <c r="N11" s="2">
-        <v>8</v>
       </c>
       <c r="O11" s="2">
         <v>3</v>
@@ -1506,10 +1534,10 @@
         <v>2</v>
       </c>
       <c r="M13" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N13" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O13" s="2">
         <v>2</v>
@@ -1528,64 +1556,125 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B14" s="2">
+        <v>710</v>
+      </c>
+      <c r="C14" s="2">
+        <v>481</v>
+      </c>
+      <c r="D14" s="2">
+        <v>52</v>
+      </c>
+      <c r="E14" s="2">
+        <v>55</v>
+      </c>
+      <c r="F14" s="2">
+        <v>38</v>
+      </c>
+      <c r="G14" s="2">
+        <v>30</v>
+      </c>
+      <c r="H14" s="2">
+        <v>18</v>
+      </c>
+      <c r="I14" s="2">
+        <v>12</v>
+      </c>
+      <c r="J14" s="2">
+        <v>2</v>
+      </c>
+      <c r="K14" s="2">
+        <v>5</v>
+      </c>
+      <c r="L14" s="2">
+        <v>3</v>
+      </c>
+      <c r="M14" s="2">
+        <v>5</v>
+      </c>
+      <c r="N14" s="2">
+        <v>1</v>
+      </c>
+      <c r="O14" s="2">
+        <v>0</v>
+      </c>
+      <c r="P14" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>0</v>
+      </c>
+      <c r="R14" s="2">
+        <v>3</v>
+      </c>
+      <c r="S14" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="5">
-        <v>9480</v>
-      </c>
-      <c r="C14" s="5">
-        <v>6267</v>
-      </c>
-      <c r="D14" s="5">
-        <v>897</v>
-      </c>
-      <c r="E14" s="5">
-        <v>571</v>
-      </c>
-      <c r="F14" s="5">
-        <v>454</v>
-      </c>
-      <c r="G14" s="5">
-        <v>376</v>
-      </c>
-      <c r="H14" s="5">
-        <v>226</v>
-      </c>
-      <c r="I14" s="5">
-        <v>179</v>
-      </c>
-      <c r="J14" s="5">
-        <v>171</v>
-      </c>
-      <c r="K14" s="5">
-        <v>113</v>
-      </c>
-      <c r="L14" s="5">
-        <v>82</v>
-      </c>
-      <c r="M14" s="5">
-        <v>35</v>
-      </c>
-      <c r="N14" s="5">
-        <v>33</v>
-      </c>
-      <c r="O14" s="5">
+      <c r="B15" s="5">
+        <v>10190</v>
+      </c>
+      <c r="C15" s="5">
+        <v>6748</v>
+      </c>
+      <c r="D15" s="5">
+        <v>949</v>
+      </c>
+      <c r="E15" s="5">
+        <v>626</v>
+      </c>
+      <c r="F15" s="5">
+        <v>492</v>
+      </c>
+      <c r="G15" s="5">
+        <v>406</v>
+      </c>
+      <c r="H15" s="5">
+        <v>244</v>
+      </c>
+      <c r="I15" s="5">
+        <v>191</v>
+      </c>
+      <c r="J15" s="5">
+        <v>173</v>
+      </c>
+      <c r="K15" s="5">
+        <v>118</v>
+      </c>
+      <c r="L15" s="5">
+        <v>85</v>
+      </c>
+      <c r="M15" s="5">
+        <v>38</v>
+      </c>
+      <c r="N15" s="5">
+        <v>36</v>
+      </c>
+      <c r="O15" s="5">
         <v>25</v>
       </c>
-      <c r="P14" s="5">
-        <v>20</v>
-      </c>
-      <c r="Q14" s="5">
+      <c r="P15" s="5">
+        <v>22</v>
+      </c>
+      <c r="Q15" s="5">
         <v>19</v>
       </c>
-      <c r="R14" s="5">
-        <v>9</v>
-      </c>
-      <c r="S14" s="5">
-        <v>3</v>
+      <c r="R15" s="5">
+        <v>12</v>
+      </c>
+      <c r="S15" s="5">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -7319,6 +7408,508 @@
       </c>
       <c r="H182" s="4"/>
     </row>
+    <row r="183">
+      <c r="A183" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B183" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C183" s="0" t="inlineStr">
+        <is>
+          <t>birth</t>
+        </is>
+      </c>
+      <c r="D183" s="2">
+        <v>334</v>
+      </c>
+      <c r="E183" s="2">
+        <v>147</v>
+      </c>
+      <c r="F183" s="2">
+        <v>481</v>
+      </c>
+      <c r="G183" s="3">
+        <v>0.6774647887323944</v>
+      </c>
+      <c r="H183" s="2">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B184" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C184" s="0" t="inlineStr">
+        <is>
+          <t>anniv</t>
+        </is>
+      </c>
+      <c r="D184" s="2">
+        <v>47</v>
+      </c>
+      <c r="E184" s="2">
+        <v>8</v>
+      </c>
+      <c r="F184" s="2">
+        <v>55</v>
+      </c>
+      <c r="G184" s="3">
+        <v>0.07746478873239436</v>
+      </c>
+      <c r="H184" s="2">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B185" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C185" s="0" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="D185" s="2">
+        <v>36</v>
+      </c>
+      <c r="E185" s="2">
+        <v>16</v>
+      </c>
+      <c r="F185" s="2">
+        <v>52</v>
+      </c>
+      <c r="G185" s="3">
+        <v>0.07323943661971831</v>
+      </c>
+      <c r="H185" s="2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B186" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C186" s="0" t="inlineStr">
+        <is>
+          <t>gen</t>
+        </is>
+      </c>
+      <c r="D186" s="2">
+        <v>28</v>
+      </c>
+      <c r="E186" s="2">
+        <v>10</v>
+      </c>
+      <c r="F186" s="2">
+        <v>38</v>
+      </c>
+      <c r="G186" s="3">
+        <v>0.05352112676056338</v>
+      </c>
+      <c r="H186" s="2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B187" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C187" s="0" t="inlineStr">
+        <is>
+          <t>thank</t>
+        </is>
+      </c>
+      <c r="D187" s="2">
+        <v>9</v>
+      </c>
+      <c r="E187" s="2">
+        <v>21</v>
+      </c>
+      <c r="F187" s="2">
+        <v>30</v>
+      </c>
+      <c r="G187" s="3">
+        <v>0.04225352112676056</v>
+      </c>
+      <c r="H187" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B188" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C188" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D188" s="2">
+        <v>13</v>
+      </c>
+      <c r="E188" s="2">
+        <v>5</v>
+      </c>
+      <c r="F188" s="2">
+        <v>18</v>
+      </c>
+      <c r="G188" s="3">
+        <v>0.02535211267605634</v>
+      </c>
+      <c r="H188" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B189" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C189" s="0" t="inlineStr">
+        <is>
+          <t>insp</t>
+        </is>
+      </c>
+      <c r="D189" s="2">
+        <v>12</v>
+      </c>
+      <c r="E189" s="2">
+        <v>0</v>
+      </c>
+      <c r="F189" s="2">
+        <v>12</v>
+      </c>
+      <c r="G189" s="3">
+        <v>0.016901408450704224</v>
+      </c>
+      <c r="H189" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B190" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C190" s="0" t="inlineStr">
+        <is>
+          <t>congrats</t>
+        </is>
+      </c>
+      <c r="D190" s="2">
+        <v>2</v>
+      </c>
+      <c r="E190" s="2">
+        <v>3</v>
+      </c>
+      <c r="F190" s="2">
+        <v>5</v>
+      </c>
+      <c r="G190" s="3">
+        <v>0.007042253521126761</v>
+      </c>
+      <c r="H190" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B191" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C191" s="0" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="D191" s="2">
+        <v>4</v>
+      </c>
+      <c r="E191" s="2">
+        <v>1</v>
+      </c>
+      <c r="F191" s="2">
+        <v>5</v>
+      </c>
+      <c r="G191" s="3">
+        <v>0.007042253521126761</v>
+      </c>
+      <c r="H191" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B192" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C192" s="0" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+      <c r="D192" s="2">
+        <v>3</v>
+      </c>
+      <c r="E192" s="2">
+        <v>0</v>
+      </c>
+      <c r="F192" s="2">
+        <v>3</v>
+      </c>
+      <c r="G192" s="3">
+        <v>0.004225352112676056</v>
+      </c>
+      <c r="H192" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B193" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C193" s="0" t="inlineStr">
+        <is>
+          <t>flwr</t>
+        </is>
+      </c>
+      <c r="D193" s="2">
+        <v>3</v>
+      </c>
+      <c r="E193" s="2">
+        <v>0</v>
+      </c>
+      <c r="F193" s="2">
+        <v>3</v>
+      </c>
+      <c r="G193" s="3">
+        <v>0.004225352112676056</v>
+      </c>
+      <c r="H193" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B194" s="0" t="inlineStr">
+        <is>
+          <t>Invitations &amp; parties</t>
+        </is>
+      </c>
+      <c r="C194" s="0" t="inlineStr">
+        <is>
+          <t>invp</t>
+        </is>
+      </c>
+      <c r="D194" s="2">
+        <v>3</v>
+      </c>
+      <c r="E194" s="2">
+        <v>0</v>
+      </c>
+      <c r="F194" s="2">
+        <v>3</v>
+      </c>
+      <c r="G194" s="3">
+        <v>0.004225352112676056</v>
+      </c>
+      <c r="H194" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B195" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C195" s="0" t="inlineStr">
+        <is>
+          <t>friend</t>
+        </is>
+      </c>
+      <c r="D195" s="2">
+        <v>2</v>
+      </c>
+      <c r="E195" s="2">
+        <v>0</v>
+      </c>
+      <c r="F195" s="2">
+        <v>2</v>
+      </c>
+      <c r="G195" s="3">
+        <v>0.0028169014084507044</v>
+      </c>
+      <c r="H195" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B196" s="0" t="inlineStr">
+        <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="C196" s="0" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="D196" s="2">
+        <v>1</v>
+      </c>
+      <c r="E196" s="2">
+        <v>1</v>
+      </c>
+      <c r="F196" s="2">
+        <v>2</v>
+      </c>
+      <c r="G196" s="3">
+        <v>0.0028169014084507044</v>
+      </c>
+      <c r="H196" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B197" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C197" s="0" t="inlineStr">
+        <is>
+          <t>fkt</t>
+        </is>
+      </c>
+      <c r="D197" s="2">
+        <v>1</v>
+      </c>
+      <c r="E197" s="2">
+        <v>0</v>
+      </c>
+      <c r="F197" s="2">
+        <v>1</v>
+      </c>
+      <c r="G197" s="3">
+        <v>0.0014084507042253522</v>
+      </c>
+      <c r="H197" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-13</t>
+        </is>
+      </c>
+      <c r="B198" s="4"/>
+      <c r="C198" s="4"/>
+      <c r="D198" s="5">
+        <v>498</v>
+      </c>
+      <c r="E198" s="5">
+        <v>212</v>
+      </c>
+      <c r="F198" s="5">
+        <v>710</v>
+      </c>
+      <c r="G198" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="H198" s="4"/>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -35617,6 +36208,2176 @@
         <v>773</v>
       </c>
       <c r="F1016" s="4"/>
+    </row>
+    <row r="1017">
+      <c r="A1017" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1017" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1017" s="0" t="inlineStr">
+        <is>
+          <t>happybirthday</t>
+        </is>
+      </c>
+      <c r="D1017" s="0" t="inlineStr">
+        <is>
+          <t>birth_happybirthday</t>
+        </is>
+      </c>
+      <c r="E1017" s="2">
+        <v>363</v>
+      </c>
+      <c r="F1017" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1018" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1018" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="D1018" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="E1018" s="2">
+        <v>32</v>
+      </c>
+      <c r="F1018" s="2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1019" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1019" s="0" t="inlineStr">
+        <is>
+          <t>morning</t>
+        </is>
+      </c>
+      <c r="D1019" s="0" t="inlineStr">
+        <is>
+          <t>gen_morning</t>
+        </is>
+      </c>
+      <c r="E1019" s="2">
+        <v>22</v>
+      </c>
+      <c r="F1019" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1020" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1020" s="0" t="inlineStr">
+        <is>
+          <t>fun</t>
+        </is>
+      </c>
+      <c r="D1020" s="0" t="inlineStr">
+        <is>
+          <t>birth_fun</t>
+        </is>
+      </c>
+      <c r="E1020" s="2">
+        <v>16</v>
+      </c>
+      <c r="F1020" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1021" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1021" s="0" t="inlineStr">
+        <is>
+          <t>eaug_smilemonth</t>
+        </is>
+      </c>
+      <c r="D1021" s="0" t="inlineStr">
+        <is>
+          <t>eaug_smilemonth</t>
+        </is>
+      </c>
+      <c r="E1021" s="2">
+        <v>15</v>
+      </c>
+      <c r="F1021" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1022" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1022" s="0" t="inlineStr">
+        <is>
+          <t>eaug_internationalleft_handers_day</t>
+        </is>
+      </c>
+      <c r="D1022" s="0" t="inlineStr">
+        <is>
+          <t>eaug_internationalleft_handers_day</t>
+        </is>
+      </c>
+      <c r="E1022" s="2">
+        <v>14</v>
+      </c>
+      <c r="F1022" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1023" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1023" s="0" t="inlineStr">
+        <is>
+          <t>birthday</t>
+        </is>
+      </c>
+      <c r="D1023" s="0" t="inlineStr">
+        <is>
+          <t>thank_birthday</t>
+        </is>
+      </c>
+      <c r="E1023" s="2">
+        <v>14</v>
+      </c>
+      <c r="F1023" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1024" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1024" s="0" t="inlineStr">
+        <is>
+          <t>anniversaryetc</t>
+        </is>
+      </c>
+      <c r="D1024" s="0" t="inlineStr">
+        <is>
+          <t>anniv_anniversaryetc</t>
+        </is>
+      </c>
+      <c r="E1024" s="2">
+        <v>12</v>
+      </c>
+      <c r="F1024" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1025" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1025" s="0" t="inlineStr">
+        <is>
+          <t>flowers</t>
+        </is>
+      </c>
+      <c r="D1025" s="0" t="inlineStr">
+        <is>
+          <t>birth_flowers</t>
+        </is>
+      </c>
+      <c r="E1025" s="2">
+        <v>12</v>
+      </c>
+      <c r="F1025" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1026" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1026" s="0" t="inlineStr">
+        <is>
+          <t>bronsis</t>
+        </is>
+      </c>
+      <c r="D1026" s="0" t="inlineStr">
+        <is>
+          <t>birth_bronsis</t>
+        </is>
+      </c>
+      <c r="E1026" s="2">
+        <v>11</v>
+      </c>
+      <c r="F1026" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1027" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1027" s="0" t="inlineStr">
+        <is>
+          <t>wishes</t>
+        </is>
+      </c>
+      <c r="D1027" s="0" t="inlineStr">
+        <is>
+          <t>birth_wishes</t>
+        </is>
+      </c>
+      <c r="E1027" s="2">
+        <v>11</v>
+      </c>
+      <c r="F1027" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1028" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1028" s="0" t="inlineStr">
+        <is>
+          <t>sonanddaughter</t>
+        </is>
+      </c>
+      <c r="D1028" s="0" t="inlineStr">
+        <is>
+          <t>birth_sonanddaughter</t>
+        </is>
+      </c>
+      <c r="E1028" s="2">
+        <v>10</v>
+      </c>
+      <c r="F1028" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1029" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1029" s="0" t="inlineStr">
+        <is>
+          <t>belated</t>
+        </is>
+      </c>
+      <c r="D1029" s="0" t="inlineStr">
+        <is>
+          <t>birth_belated</t>
+        </is>
+      </c>
+      <c r="E1029" s="2">
+        <v>9</v>
+      </c>
+      <c r="F1029" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1030" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1030" s="0" t="inlineStr">
+        <is>
+          <t>extfamily</t>
+        </is>
+      </c>
+      <c r="D1030" s="0" t="inlineStr">
+        <is>
+          <t>birth_extfamily</t>
+        </is>
+      </c>
+      <c r="E1030" s="2">
+        <v>9</v>
+      </c>
+      <c r="F1030" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1031" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1031" s="0" t="inlineStr">
+        <is>
+          <t>sympathy</t>
+        </is>
+      </c>
+      <c r="D1031" s="0" t="inlineStr">
+        <is>
+          <t>insp_sympathy</t>
+        </is>
+      </c>
+      <c r="E1031" s="2">
+        <v>9</v>
+      </c>
+      <c r="F1031" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1032" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1032" s="0" t="inlineStr">
+        <is>
+          <t>kids</t>
+        </is>
+      </c>
+      <c r="D1032" s="0" t="inlineStr">
+        <is>
+          <t>birth_kids</t>
+        </is>
+      </c>
+      <c r="E1032" s="2">
+        <v>8</v>
+      </c>
+      <c r="F1032" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1033" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1033" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D1033" s="0" t="inlineStr">
+        <is>
+          <t>gen_getwell</t>
+        </is>
+      </c>
+      <c r="E1033" s="2">
+        <v>8</v>
+      </c>
+      <c r="F1033" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1034" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1034" s="0" t="inlineStr">
+        <is>
+          <t>blessings</t>
+        </is>
+      </c>
+      <c r="D1034" s="0" t="inlineStr">
+        <is>
+          <t>birth_blessings</t>
+        </is>
+      </c>
+      <c r="E1034" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1034" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1035" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1035" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D1035" s="0" t="inlineStr">
+        <is>
+          <t>birth_milestone</t>
+        </is>
+      </c>
+      <c r="E1035" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1035" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1036" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1036" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_general</t>
+        </is>
+      </c>
+      <c r="D1036" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_general</t>
+        </is>
+      </c>
+      <c r="E1036" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1036" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1037" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1037" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="D1037" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="E1037" s="2">
+        <v>6</v>
+      </c>
+      <c r="F1037" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1038" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1038" s="0" t="inlineStr">
+        <is>
+          <t>songs</t>
+        </is>
+      </c>
+      <c r="D1038" s="0" t="inlineStr">
+        <is>
+          <t>birth_songs</t>
+        </is>
+      </c>
+      <c r="E1038" s="2">
+        <v>6</v>
+      </c>
+      <c r="F1038" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1039" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1039" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D1039" s="0" t="inlineStr">
+        <is>
+          <t>thank_love</t>
+        </is>
+      </c>
+      <c r="E1039" s="2">
+        <v>6</v>
+      </c>
+      <c r="F1039" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1040" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1040" s="0" t="inlineStr">
+        <is>
+          <t>thinkingofyou</t>
+        </is>
+      </c>
+      <c r="D1040" s="0" t="inlineStr">
+        <is>
+          <t>gen_thinkingofyou</t>
+        </is>
+      </c>
+      <c r="E1040" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1040" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1041" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1041" s="0" t="inlineStr">
+        <is>
+          <t>everyday</t>
+        </is>
+      </c>
+      <c r="D1041" s="0" t="inlineStr">
+        <is>
+          <t>thank_everyday</t>
+        </is>
+      </c>
+      <c r="E1041" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1041" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1042" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1042" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_birthday</t>
+        </is>
+      </c>
+      <c r="D1042" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_birthday</t>
+        </is>
+      </c>
+      <c r="E1042" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1042" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1043" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1043" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="D1043" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="E1043" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1043" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1044" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1044" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="D1044" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="E1044" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1044" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1045" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1045" s="0" t="inlineStr">
+        <is>
+          <t>friends</t>
+        </is>
+      </c>
+      <c r="D1045" s="0" t="inlineStr">
+        <is>
+          <t>birth_friends</t>
+        </is>
+      </c>
+      <c r="E1045" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1045" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1046" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1046" s="0" t="inlineStr">
+        <is>
+          <t>hubbywife</t>
+        </is>
+      </c>
+      <c r="D1046" s="0" t="inlineStr">
+        <is>
+          <t>birth_hubbywife</t>
+        </is>
+      </c>
+      <c r="E1046" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1046" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1047" s="0" t="inlineStr">
+        <is>
+          <t>Invitations &amp; parties</t>
+        </is>
+      </c>
+      <c r="C1047" s="0" t="inlineStr">
+        <is>
+          <t>birth_gen</t>
+        </is>
+      </c>
+      <c r="D1047" s="0" t="inlineStr">
+        <is>
+          <t>invp_birth_gen</t>
+        </is>
+      </c>
+      <c r="E1047" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1047" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1048" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C1048" s="0" t="inlineStr">
+        <is>
+          <t>lossofpet</t>
+        </is>
+      </c>
+      <c r="D1048" s="0" t="inlineStr">
+        <is>
+          <t>pet_lossofpet</t>
+        </is>
+      </c>
+      <c r="E1048" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1048" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1049" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1049" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D1049" s="0" t="inlineStr">
+        <is>
+          <t>anniv_milestone</t>
+        </is>
+      </c>
+      <c r="E1049" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1049" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1050" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1050" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="D1050" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="E1050" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1050" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1051" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1051" s="0" t="inlineStr">
+        <is>
+          <t>forher</t>
+        </is>
+      </c>
+      <c r="D1051" s="0" t="inlineStr">
+        <is>
+          <t>birth_forher</t>
+        </is>
+      </c>
+      <c r="E1051" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1051" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1052" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1052" s="0" t="inlineStr">
+        <is>
+          <t>momndad</t>
+        </is>
+      </c>
+      <c r="D1052" s="0" t="inlineStr">
+        <is>
+          <t>birth_momndad</t>
+        </is>
+      </c>
+      <c r="E1052" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1052" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1053" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1053" s="0" t="inlineStr">
+        <is>
+          <t>onotheroccasions</t>
+        </is>
+      </c>
+      <c r="D1053" s="0" t="inlineStr">
+        <is>
+          <t>congrats_onotheroccasions</t>
+        </is>
+      </c>
+      <c r="E1053" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1053" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1054" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1054" s="0" t="inlineStr">
+        <is>
+          <t>studentsandnewgrads</t>
+        </is>
+      </c>
+      <c r="D1054" s="0" t="inlineStr">
+        <is>
+          <t>congrats_studentsandnewgrads</t>
+        </is>
+      </c>
+      <c r="E1054" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1054" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1055" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1055" s="0" t="inlineStr">
+        <is>
+          <t>eaug_creamsicleday</t>
+        </is>
+      </c>
+      <c r="D1055" s="0" t="inlineStr">
+        <is>
+          <t>eaug_creamsicleday</t>
+        </is>
+      </c>
+      <c r="E1055" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1055" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1056" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1056" s="0" t="inlineStr">
+        <is>
+          <t>eaug_flwrmonthaug</t>
+        </is>
+      </c>
+      <c r="D1056" s="0" t="inlineStr">
+        <is>
+          <t>eaug_flwrmonthaug</t>
+        </is>
+      </c>
+      <c r="E1056" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1056" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1057" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1057" s="0" t="inlineStr">
+        <is>
+          <t>eaug_romanceday</t>
+        </is>
+      </c>
+      <c r="D1057" s="0" t="inlineStr">
+        <is>
+          <t>eaug_romanceday</t>
+        </is>
+      </c>
+      <c r="E1057" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1057" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1058" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1058" s="0" t="inlineStr">
+        <is>
+          <t>eaug_zorastriannewyear</t>
+        </is>
+      </c>
+      <c r="D1058" s="0" t="inlineStr">
+        <is>
+          <t>eaug_zorastriannewyear</t>
+        </is>
+      </c>
+      <c r="E1058" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1058" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1059" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1059" s="0" t="inlineStr">
+        <is>
+          <t>eoct_nationaliloveyou_day</t>
+        </is>
+      </c>
+      <c r="D1059" s="0" t="inlineStr">
+        <is>
+          <t>eoct_nationaliloveyou_day</t>
+        </is>
+      </c>
+      <c r="E1059" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1059" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1060" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C1060" s="0" t="inlineStr">
+        <is>
+          <t>roses</t>
+        </is>
+      </c>
+      <c r="D1060" s="0" t="inlineStr">
+        <is>
+          <t>flwr_roses</t>
+        </is>
+      </c>
+      <c r="E1060" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1060" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1061" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1061" s="0" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="D1061" s="0" t="inlineStr">
+        <is>
+          <t>insp_support</t>
+        </is>
+      </c>
+      <c r="E1061" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1061" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1062" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C1062" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D1062" s="0" t="inlineStr">
+        <is>
+          <t>pet_getwell</t>
+        </is>
+      </c>
+      <c r="E1062" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1062" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1063" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1063" s="0" t="inlineStr">
+        <is>
+          <t>congratulations</t>
+        </is>
+      </c>
+      <c r="D1063" s="0" t="inlineStr">
+        <is>
+          <t>thank_congratulations</t>
+        </is>
+      </c>
+      <c r="E1063" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1063" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1064" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1064" s="0" t="inlineStr">
+        <is>
+          <t>inspirational</t>
+        </is>
+      </c>
+      <c r="D1064" s="0" t="inlineStr">
+        <is>
+          <t>thank_inspirational</t>
+        </is>
+      </c>
+      <c r="E1064" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1064" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1065" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1065" s="0" t="inlineStr">
+        <is>
+          <t>wed_wed_congrats</t>
+        </is>
+      </c>
+      <c r="D1065" s="0" t="inlineStr">
+        <is>
+          <t>wed_wed_congrats</t>
+        </is>
+      </c>
+      <c r="E1065" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1065" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1066" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1066" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_family</t>
+        </is>
+      </c>
+      <c r="D1066" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_family</t>
+        </is>
+      </c>
+      <c r="E1066" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1066" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1067" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1067" s="0" t="inlineStr">
+        <is>
+          <t>forhim</t>
+        </is>
+      </c>
+      <c r="D1067" s="0" t="inlineStr">
+        <is>
+          <t>birth_forhim</t>
+        </is>
+      </c>
+      <c r="E1067" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1067" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1068" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1068" s="0" t="inlineStr">
+        <is>
+          <t>pets</t>
+        </is>
+      </c>
+      <c r="D1068" s="0" t="inlineStr">
+        <is>
+          <t>birth_pets</t>
+        </is>
+      </c>
+      <c r="E1068" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1068" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1069" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C1069" s="0" t="inlineStr">
+        <is>
+          <t>accolades</t>
+        </is>
+      </c>
+      <c r="D1069" s="0" t="inlineStr">
+        <is>
+          <t>bus_accolades</t>
+        </is>
+      </c>
+      <c r="E1069" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1069" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1070" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C1070" s="0" t="inlineStr">
+        <is>
+          <t>apologies</t>
+        </is>
+      </c>
+      <c r="D1070" s="0" t="inlineStr">
+        <is>
+          <t>bus_apologies</t>
+        </is>
+      </c>
+      <c r="E1070" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1070" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1071" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C1071" s="0" t="inlineStr">
+        <is>
+          <t>farewell</t>
+        </is>
+      </c>
+      <c r="D1071" s="0" t="inlineStr">
+        <is>
+          <t>bus_farewell</t>
+        </is>
+      </c>
+      <c r="E1071" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1071" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1072" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1072" s="0" t="inlineStr">
+        <is>
+          <t>newjob</t>
+        </is>
+      </c>
+      <c r="D1072" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newjob</t>
+        </is>
+      </c>
+      <c r="E1072" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1072" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1073" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1073" s="0" t="inlineStr">
+        <is>
+          <t>eaug_indindependenceday</t>
+        </is>
+      </c>
+      <c r="D1073" s="0" t="inlineStr">
+        <is>
+          <t>eaug_indindependenceday</t>
+        </is>
+      </c>
+      <c r="E1073" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1073" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1074" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1074" s="0" t="inlineStr">
+        <is>
+          <t>efeb_lent</t>
+        </is>
+      </c>
+      <c r="D1074" s="0" t="inlineStr">
+        <is>
+          <t>efeb_lent</t>
+        </is>
+      </c>
+      <c r="E1074" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1074" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1075" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1075" s="0" t="inlineStr">
+        <is>
+          <t>emar_stjosephs_day</t>
+        </is>
+      </c>
+      <c r="D1075" s="0" t="inlineStr">
+        <is>
+          <t>emar_stjosephs_day</t>
+        </is>
+      </c>
+      <c r="E1075" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1075" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1076" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1076" s="0" t="inlineStr">
+        <is>
+          <t>esep_fall_specials</t>
+        </is>
+      </c>
+      <c r="D1076" s="0" t="inlineStr">
+        <is>
+          <t>esep_fall_specials</t>
+        </is>
+      </c>
+      <c r="E1076" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1076" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1077" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1077" s="0" t="inlineStr">
+        <is>
+          <t>esep_longestkissday</t>
+        </is>
+      </c>
+      <c r="D1077" s="0" t="inlineStr">
+        <is>
+          <t>esep_longestkissday</t>
+        </is>
+      </c>
+      <c r="E1077" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1077" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1078" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1078" s="0" t="inlineStr">
+        <is>
+          <t>esep_wifeappreciation_day</t>
+        </is>
+      </c>
+      <c r="D1078" s="0" t="inlineStr">
+        <is>
+          <t>esep_wifeappreciation_day</t>
+        </is>
+      </c>
+      <c r="E1078" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1078" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1079" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C1079" s="0" t="inlineStr">
+        <is>
+          <t>sonsdaughter</t>
+        </is>
+      </c>
+      <c r="D1079" s="0" t="inlineStr">
+        <is>
+          <t>fkt_sonsdaughter</t>
+        </is>
+      </c>
+      <c r="E1079" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1079" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1080" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C1080" s="0" t="inlineStr">
+        <is>
+          <t>youcare</t>
+        </is>
+      </c>
+      <c r="D1080" s="0" t="inlineStr">
+        <is>
+          <t>flwr_youcare</t>
+        </is>
+      </c>
+      <c r="E1080" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1080" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1081" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C1081" s="0" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="D1081" s="0" t="inlineStr">
+        <is>
+          <t>friend_hello</t>
+        </is>
+      </c>
+      <c r="E1081" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1081" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1082" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C1082" s="0" t="inlineStr">
+        <is>
+          <t>justpals</t>
+        </is>
+      </c>
+      <c r="D1082" s="0" t="inlineStr">
+        <is>
+          <t>friend_justpals</t>
+        </is>
+      </c>
+      <c r="E1082" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1082" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1083" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1083" s="0" t="inlineStr">
+        <is>
+          <t>hvgtday</t>
+        </is>
+      </c>
+      <c r="D1083" s="0" t="inlineStr">
+        <is>
+          <t>gen_hvgtday</t>
+        </is>
+      </c>
+      <c r="E1083" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1083" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1084" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1084" s="0" t="inlineStr">
+        <is>
+          <t>quotesmessages_images_getwell_images</t>
+        </is>
+      </c>
+      <c r="D1084" s="0" t="inlineStr">
+        <is>
+          <t>gen_quotesmessages_images_getwell_images</t>
+        </is>
+      </c>
+      <c r="E1084" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1084" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1085" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1085" s="0" t="inlineStr">
+        <is>
+          <t>voyage</t>
+        </is>
+      </c>
+      <c r="D1085" s="0" t="inlineStr">
+        <is>
+          <t>gen_voyage</t>
+        </is>
+      </c>
+      <c r="E1085" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1085" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1086" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1086" s="0" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="D1086" s="0" t="inlineStr">
+        <is>
+          <t>insp_health</t>
+        </is>
+      </c>
+      <c r="E1086" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1086" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1087" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1087" s="0" t="inlineStr">
+        <is>
+          <t>iamsorry</t>
+        </is>
+      </c>
+      <c r="D1087" s="0" t="inlineStr">
+        <is>
+          <t>love_iamsorry</t>
+        </is>
+      </c>
+      <c r="E1087" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1087" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1088" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1088" s="0" t="inlineStr">
+        <is>
+          <t>lovepoems</t>
+        </is>
+      </c>
+      <c r="D1088" s="0" t="inlineStr">
+        <is>
+          <t>love_lovepoems</t>
+        </is>
+      </c>
+      <c r="E1088" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1088" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1089" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1089" s="0" t="inlineStr">
+        <is>
+          <t>youarespecial</t>
+        </is>
+      </c>
+      <c r="D1089" s="0" t="inlineStr">
+        <is>
+          <t>love_youarespecial</t>
+        </is>
+      </c>
+      <c r="E1089" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1089" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1090" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1090" s="0" t="inlineStr">
+        <is>
+          <t>wedding</t>
+        </is>
+      </c>
+      <c r="D1090" s="0" t="inlineStr">
+        <is>
+          <t>thank_wedding</t>
+        </is>
+      </c>
+      <c r="E1090" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1090" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1091" s="0" t="inlineStr">
+        <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="C1091" s="0" t="inlineStr">
+        <is>
+          <t>hindi_rakshabandhan</t>
+        </is>
+      </c>
+      <c r="D1091" s="0" t="inlineStr">
+        <is>
+          <t>w_hindi_rakshabandhan</t>
+        </is>
+      </c>
+      <c r="E1091" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1091" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1092" s="0" t="inlineStr">
+        <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="C1092" s="0" t="inlineStr">
+        <is>
+          <t>mandarin_birthday</t>
+        </is>
+      </c>
+      <c r="D1092" s="0" t="inlineStr">
+        <is>
+          <t>w_mandarin_birthday</t>
+        </is>
+      </c>
+      <c r="E1092" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1092" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1093" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1093" s="0" t="inlineStr">
+        <is>
+          <t>wed_foreachother</t>
+        </is>
+      </c>
+      <c r="D1093" s="0" t="inlineStr">
+        <is>
+          <t>wed_foreachother</t>
+        </is>
+      </c>
+      <c r="E1093" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1093" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1094" s="4"/>
+      <c r="C1094" s="4"/>
+      <c r="D1094" s="4"/>
+      <c r="E1094" s="5">
+        <v>710</v>
+      </c>
+      <c r="F1094" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -36098,36 +38859,70 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B14" s="2">
+        <v>808</v>
+      </c>
+      <c r="C14" s="2">
+        <v>296</v>
+      </c>
+      <c r="D14" s="2">
+        <v>216</v>
+      </c>
+      <c r="E14" s="2">
+        <v>156</v>
+      </c>
+      <c r="F14" s="2">
+        <v>76</v>
+      </c>
+      <c r="G14" s="2">
+        <v>37</v>
+      </c>
+      <c r="H14" s="2">
+        <v>27</v>
+      </c>
+      <c r="I14" s="2">
+        <v>0</v>
+      </c>
+      <c r="J14" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="5">
-        <v>9968</v>
-      </c>
-      <c r="C14" s="5">
-        <v>3144</v>
-      </c>
-      <c r="D14" s="5">
-        <v>3077</v>
-      </c>
-      <c r="E14" s="5">
-        <v>1975</v>
-      </c>
-      <c r="F14" s="5">
-        <v>1043</v>
-      </c>
-      <c r="G14" s="5">
-        <v>377</v>
-      </c>
-      <c r="H14" s="5">
-        <v>323</v>
-      </c>
-      <c r="I14" s="5">
+      <c r="B15" s="5">
+        <v>10776</v>
+      </c>
+      <c r="C15" s="5">
+        <v>3440</v>
+      </c>
+      <c r="D15" s="5">
+        <v>3293</v>
+      </c>
+      <c r="E15" s="5">
+        <v>2131</v>
+      </c>
+      <c r="F15" s="5">
+        <v>1119</v>
+      </c>
+      <c r="G15" s="5">
+        <v>414</v>
+      </c>
+      <c r="H15" s="5">
+        <v>350</v>
+      </c>
+      <c r="I15" s="5">
         <v>28</v>
       </c>
-      <c r="J14" s="5">
+      <c r="J15" s="5">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Record 14 August: fourteen days, 11,690 sends tracked
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9KsXegBwxB1sWdCzRVLrr
</commit_message>
<xml_diff>
--- a/reports/daily_tracking.xlsx
+++ b/reports/daily_tracking.xlsx
@@ -224,7 +224,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
@@ -247,7 +247,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -675,28 +675,56 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B15" s="2">
+        <v>914</v>
+      </c>
+      <c r="C15" s="2">
+        <v>603</v>
+      </c>
+      <c r="D15" s="2">
+        <v>311</v>
+      </c>
+      <c r="E15" s="2">
+        <v>811</v>
+      </c>
+      <c r="F15" s="2">
+        <v>103</v>
+      </c>
+      <c r="G15" s="2">
+        <v>272</v>
+      </c>
+      <c r="H15" s="2">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B15" s="5">
-        <v>10776</v>
-      </c>
-      <c r="C15" s="5">
-        <v>7095</v>
-      </c>
-      <c r="D15" s="5">
-        <v>3681</v>
-      </c>
-      <c r="E15" s="5">
-        <v>10190</v>
-      </c>
-      <c r="F15" s="5">
-        <v>586</v>
-      </c>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
+      <c r="B16" s="5">
+        <v>11690</v>
+      </c>
+      <c r="C16" s="5">
+        <v>7698</v>
+      </c>
+      <c r="D16" s="5">
+        <v>3992</v>
+      </c>
+      <c r="E16" s="5">
+        <v>11001</v>
+      </c>
+      <c r="F16" s="5">
+        <v>689</v>
+      </c>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -717,8 +745,8 @@
     <col min="10" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="17" customWidth="1"/>
     <col min="12" max="12" width="11" customWidth="1"/>
-    <col min="13" max="13" width="11" customWidth="1"/>
-    <col min="14" max="14" width="21" customWidth="1"/>
+    <col min="13" max="13" width="21" customWidth="1"/>
+    <col min="14" max="14" width="11" customWidth="1"/>
     <col min="15" max="15" width="11" customWidth="1"/>
     <col min="16" max="16" width="17" customWidth="1"/>
     <col min="17" max="17" width="18" customWidth="1"/>
@@ -789,12 +817,12 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Pets</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Family &amp; loved ones</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
@@ -924,10 +952,10 @@
         <v>8</v>
       </c>
       <c r="M3" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N3" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O3" s="2">
         <v>1</v>
@@ -1046,10 +1074,10 @@
         <v>0</v>
       </c>
       <c r="M5" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N5" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O5" s="2">
         <v>1</v>
@@ -1107,10 +1135,10 @@
         <v>17</v>
       </c>
       <c r="M6" s="2">
+        <v>1</v>
+      </c>
+      <c r="N6" s="2">
         <v>4</v>
-      </c>
-      <c r="N6" s="2">
-        <v>1</v>
       </c>
       <c r="O6" s="2">
         <v>0</v>
@@ -1168,10 +1196,10 @@
         <v>0</v>
       </c>
       <c r="M7" s="2">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="N7" s="2">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="O7" s="2">
         <v>0</v>
@@ -1229,10 +1257,10 @@
         <v>6</v>
       </c>
       <c r="M8" s="2">
+        <v>6</v>
+      </c>
+      <c r="N8" s="2">
         <v>3</v>
-      </c>
-      <c r="N8" s="2">
-        <v>6</v>
       </c>
       <c r="O8" s="2">
         <v>1</v>
@@ -1290,10 +1318,10 @@
         <v>39</v>
       </c>
       <c r="M9" s="2">
+        <v>1</v>
+      </c>
+      <c r="N9" s="2">
         <v>4</v>
-      </c>
-      <c r="N9" s="2">
-        <v>1</v>
       </c>
       <c r="O9" s="2">
         <v>3</v>
@@ -1351,10 +1379,10 @@
         <v>4</v>
       </c>
       <c r="M10" s="2">
+        <v>1</v>
+      </c>
+      <c r="N10" s="2">
         <v>4</v>
-      </c>
-      <c r="N10" s="2">
-        <v>1</v>
       </c>
       <c r="O10" s="2">
         <v>5</v>
@@ -1412,10 +1440,10 @@
         <v>3</v>
       </c>
       <c r="M11" s="2">
+        <v>4</v>
+      </c>
+      <c r="N11" s="2">
         <v>8</v>
-      </c>
-      <c r="N11" s="2">
-        <v>4</v>
       </c>
       <c r="O11" s="2">
         <v>3</v>
@@ -1534,10 +1562,10 @@
         <v>2</v>
       </c>
       <c r="M13" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N13" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O13" s="2">
         <v>2</v>
@@ -1595,10 +1623,10 @@
         <v>3</v>
       </c>
       <c r="M14" s="2">
+        <v>1</v>
+      </c>
+      <c r="N14" s="2">
         <v>5</v>
-      </c>
-      <c r="N14" s="2">
-        <v>1</v>
       </c>
       <c r="O14" s="2">
         <v>0</v>
@@ -1617,63 +1645,124 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B15" s="2">
+        <v>811</v>
+      </c>
+      <c r="C15" s="2">
+        <v>441</v>
+      </c>
+      <c r="D15" s="2">
+        <v>187</v>
+      </c>
+      <c r="E15" s="2">
+        <v>47</v>
+      </c>
+      <c r="F15" s="2">
+        <v>50</v>
+      </c>
+      <c r="G15" s="2">
+        <v>22</v>
+      </c>
+      <c r="H15" s="2">
+        <v>10</v>
+      </c>
+      <c r="I15" s="2">
+        <v>28</v>
+      </c>
+      <c r="J15" s="2">
+        <v>2</v>
+      </c>
+      <c r="K15" s="2">
+        <v>14</v>
+      </c>
+      <c r="L15" s="2">
+        <v>3</v>
+      </c>
+      <c r="M15" s="2">
+        <v>3</v>
+      </c>
+      <c r="N15" s="2">
+        <v>0</v>
+      </c>
+      <c r="O15" s="2">
+        <v>0</v>
+      </c>
+      <c r="P15" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>1</v>
+      </c>
+      <c r="R15" s="2">
+        <v>3</v>
+      </c>
+      <c r="S15" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B15" s="5">
-        <v>10190</v>
-      </c>
-      <c r="C15" s="5">
-        <v>6748</v>
-      </c>
-      <c r="D15" s="5">
-        <v>949</v>
-      </c>
-      <c r="E15" s="5">
-        <v>626</v>
-      </c>
-      <c r="F15" s="5">
-        <v>492</v>
-      </c>
-      <c r="G15" s="5">
-        <v>406</v>
-      </c>
-      <c r="H15" s="5">
-        <v>244</v>
-      </c>
-      <c r="I15" s="5">
-        <v>191</v>
-      </c>
-      <c r="J15" s="5">
-        <v>173</v>
-      </c>
-      <c r="K15" s="5">
-        <v>118</v>
-      </c>
-      <c r="L15" s="5">
-        <v>85</v>
-      </c>
-      <c r="M15" s="5">
+      <c r="B16" s="5">
+        <v>11001</v>
+      </c>
+      <c r="C16" s="5">
+        <v>7189</v>
+      </c>
+      <c r="D16" s="5">
+        <v>1136</v>
+      </c>
+      <c r="E16" s="5">
+        <v>673</v>
+      </c>
+      <c r="F16" s="5">
+        <v>542</v>
+      </c>
+      <c r="G16" s="5">
+        <v>428</v>
+      </c>
+      <c r="H16" s="5">
+        <v>254</v>
+      </c>
+      <c r="I16" s="5">
+        <v>219</v>
+      </c>
+      <c r="J16" s="5">
+        <v>175</v>
+      </c>
+      <c r="K16" s="5">
+        <v>132</v>
+      </c>
+      <c r="L16" s="5">
+        <v>88</v>
+      </c>
+      <c r="M16" s="5">
+        <v>39</v>
+      </c>
+      <c r="N16" s="5">
         <v>38</v>
       </c>
-      <c r="N15" s="5">
-        <v>36</v>
-      </c>
-      <c r="O15" s="5">
+      <c r="O16" s="5">
         <v>25</v>
       </c>
-      <c r="P15" s="5">
+      <c r="P16" s="5">
         <v>22</v>
       </c>
-      <c r="Q15" s="5">
-        <v>19</v>
-      </c>
-      <c r="R15" s="5">
-        <v>12</v>
-      </c>
-      <c r="S15" s="5">
+      <c r="Q16" s="5">
+        <v>20</v>
+      </c>
+      <c r="R16" s="5">
+        <v>15</v>
+      </c>
+      <c r="S16" s="5">
         <v>6</v>
       </c>
     </row>
@@ -7910,6 +7999,444 @@
       </c>
       <c r="H198" s="4"/>
     </row>
+    <row r="199">
+      <c r="A199" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B199" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C199" s="0" t="inlineStr">
+        <is>
+          <t>birth</t>
+        </is>
+      </c>
+      <c r="D199" s="2">
+        <v>302</v>
+      </c>
+      <c r="E199" s="2">
+        <v>139</v>
+      </c>
+      <c r="F199" s="2">
+        <v>441</v>
+      </c>
+      <c r="G199" s="3">
+        <v>0.5437731196054254</v>
+      </c>
+      <c r="H199" s="2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B200" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C200" s="0" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="D200" s="2">
+        <v>127</v>
+      </c>
+      <c r="E200" s="2">
+        <v>60</v>
+      </c>
+      <c r="F200" s="2">
+        <v>187</v>
+      </c>
+      <c r="G200" s="3">
+        <v>0.23057953144266338</v>
+      </c>
+      <c r="H200" s="2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B201" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C201" s="0" t="inlineStr">
+        <is>
+          <t>gen</t>
+        </is>
+      </c>
+      <c r="D201" s="2">
+        <v>41</v>
+      </c>
+      <c r="E201" s="2">
+        <v>9</v>
+      </c>
+      <c r="F201" s="2">
+        <v>50</v>
+      </c>
+      <c r="G201" s="3">
+        <v>0.06165228113440197</v>
+      </c>
+      <c r="H201" s="2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B202" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C202" s="0" t="inlineStr">
+        <is>
+          <t>anniv</t>
+        </is>
+      </c>
+      <c r="D202" s="2">
+        <v>33</v>
+      </c>
+      <c r="E202" s="2">
+        <v>14</v>
+      </c>
+      <c r="F202" s="2">
+        <v>47</v>
+      </c>
+      <c r="G202" s="3">
+        <v>0.05795314426633785</v>
+      </c>
+      <c r="H202" s="2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B203" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C203" s="0" t="inlineStr">
+        <is>
+          <t>insp</t>
+        </is>
+      </c>
+      <c r="D203" s="2">
+        <v>22</v>
+      </c>
+      <c r="E203" s="2">
+        <v>6</v>
+      </c>
+      <c r="F203" s="2">
+        <v>28</v>
+      </c>
+      <c r="G203" s="3">
+        <v>0.0345252774352651</v>
+      </c>
+      <c r="H203" s="2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B204" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C204" s="0" t="inlineStr">
+        <is>
+          <t>thank</t>
+        </is>
+      </c>
+      <c r="D204" s="2">
+        <v>2</v>
+      </c>
+      <c r="E204" s="2">
+        <v>20</v>
+      </c>
+      <c r="F204" s="2">
+        <v>22</v>
+      </c>
+      <c r="G204" s="3">
+        <v>0.027127003699136867</v>
+      </c>
+      <c r="H204" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B205" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C205" s="0" t="inlineStr">
+        <is>
+          <t>congrats</t>
+        </is>
+      </c>
+      <c r="D205" s="2">
+        <v>10</v>
+      </c>
+      <c r="E205" s="2">
+        <v>4</v>
+      </c>
+      <c r="F205" s="2">
+        <v>14</v>
+      </c>
+      <c r="G205" s="3">
+        <v>0.01726263871763255</v>
+      </c>
+      <c r="H205" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B206" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C206" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D206" s="2">
+        <v>7</v>
+      </c>
+      <c r="E206" s="2">
+        <v>3</v>
+      </c>
+      <c r="F206" s="2">
+        <v>10</v>
+      </c>
+      <c r="G206" s="3">
+        <v>0.012330456226880395</v>
+      </c>
+      <c r="H206" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B207" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C207" s="0" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+      <c r="D207" s="2">
+        <v>3</v>
+      </c>
+      <c r="E207" s="2">
+        <v>0</v>
+      </c>
+      <c r="F207" s="2">
+        <v>3</v>
+      </c>
+      <c r="G207" s="3">
+        <v>0.0036991368680641184</v>
+      </c>
+      <c r="H207" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B208" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C208" s="0" t="inlineStr">
+        <is>
+          <t>fkt</t>
+        </is>
+      </c>
+      <c r="D208" s="2">
+        <v>1</v>
+      </c>
+      <c r="E208" s="2">
+        <v>2</v>
+      </c>
+      <c r="F208" s="2">
+        <v>3</v>
+      </c>
+      <c r="G208" s="3">
+        <v>0.0036991368680641184</v>
+      </c>
+      <c r="H208" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B209" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C209" s="0" t="inlineStr">
+        <is>
+          <t>flwr</t>
+        </is>
+      </c>
+      <c r="D209" s="2">
+        <v>2</v>
+      </c>
+      <c r="E209" s="2">
+        <v>1</v>
+      </c>
+      <c r="F209" s="2">
+        <v>3</v>
+      </c>
+      <c r="G209" s="3">
+        <v>0.0036991368680641184</v>
+      </c>
+      <c r="H209" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B210" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C210" s="0" t="inlineStr">
+        <is>
+          <t>friend</t>
+        </is>
+      </c>
+      <c r="D210" s="2">
+        <v>1</v>
+      </c>
+      <c r="E210" s="2">
+        <v>1</v>
+      </c>
+      <c r="F210" s="2">
+        <v>2</v>
+      </c>
+      <c r="G210" s="3">
+        <v>0.002466091245376079</v>
+      </c>
+      <c r="H210" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B211" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C211" s="0" t="inlineStr">
+        <is>
+          <t>intouch</t>
+        </is>
+      </c>
+      <c r="D211" s="2">
+        <v>1</v>
+      </c>
+      <c r="E211" s="2">
+        <v>0</v>
+      </c>
+      <c r="F211" s="2">
+        <v>1</v>
+      </c>
+      <c r="G211" s="3">
+        <v>0.0012330456226880395</v>
+      </c>
+      <c r="H211" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-14</t>
+        </is>
+      </c>
+      <c r="B212" s="4"/>
+      <c r="C212" s="4"/>
+      <c r="D212" s="5">
+        <v>552</v>
+      </c>
+      <c r="E212" s="5">
+        <v>259</v>
+      </c>
+      <c r="F212" s="5">
+        <v>811</v>
+      </c>
+      <c r="G212" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="H212" s="4"/>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -38378,6 +38905,2260 @@
         <v>710</v>
       </c>
       <c r="F1094" s="4"/>
+    </row>
+    <row r="1095">
+      <c r="A1095" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1095" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1095" s="0" t="inlineStr">
+        <is>
+          <t>happybirthday</t>
+        </is>
+      </c>
+      <c r="D1095" s="0" t="inlineStr">
+        <is>
+          <t>birth_happybirthday</t>
+        </is>
+      </c>
+      <c r="E1095" s="2">
+        <v>326</v>
+      </c>
+      <c r="F1095" s="2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1096" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1096" s="0" t="inlineStr">
+        <is>
+          <t>eaug_indindependenceday</t>
+        </is>
+      </c>
+      <c r="D1096" s="0" t="inlineStr">
+        <is>
+          <t>eaug_indindependenceday</t>
+        </is>
+      </c>
+      <c r="E1096" s="2">
+        <v>114</v>
+      </c>
+      <c r="F1096" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1097" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1097" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="D1097" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="E1097" s="2">
+        <v>29</v>
+      </c>
+      <c r="F1097" s="2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1098" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1098" s="0" t="inlineStr">
+        <is>
+          <t>eaug_creamsicleday</t>
+        </is>
+      </c>
+      <c r="D1098" s="0" t="inlineStr">
+        <is>
+          <t>eaug_creamsicleday</t>
+        </is>
+      </c>
+      <c r="E1098" s="2">
+        <v>24</v>
+      </c>
+      <c r="F1098" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1099" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1099" s="0" t="inlineStr">
+        <is>
+          <t>eaug_zorastriannewyear</t>
+        </is>
+      </c>
+      <c r="D1099" s="0" t="inlineStr">
+        <is>
+          <t>eaug_zorastriannewyear</t>
+        </is>
+      </c>
+      <c r="E1099" s="2">
+        <v>19</v>
+      </c>
+      <c r="F1099" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1100" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1100" s="0" t="inlineStr">
+        <is>
+          <t>sympathy</t>
+        </is>
+      </c>
+      <c r="D1100" s="0" t="inlineStr">
+        <is>
+          <t>insp_sympathy</t>
+        </is>
+      </c>
+      <c r="E1100" s="2">
+        <v>19</v>
+      </c>
+      <c r="F1100" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1101" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1101" s="0" t="inlineStr">
+        <is>
+          <t>sonanddaughter</t>
+        </is>
+      </c>
+      <c r="D1101" s="0" t="inlineStr">
+        <is>
+          <t>birth_sonanddaughter</t>
+        </is>
+      </c>
+      <c r="E1101" s="2">
+        <v>18</v>
+      </c>
+      <c r="F1101" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1102" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1102" s="0" t="inlineStr">
+        <is>
+          <t>birthday</t>
+        </is>
+      </c>
+      <c r="D1102" s="0" t="inlineStr">
+        <is>
+          <t>thank_birthday</t>
+        </is>
+      </c>
+      <c r="E1102" s="2">
+        <v>16</v>
+      </c>
+      <c r="F1102" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1103" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1103" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D1103" s="0" t="inlineStr">
+        <is>
+          <t>birth_milestone</t>
+        </is>
+      </c>
+      <c r="E1103" s="2">
+        <v>15</v>
+      </c>
+      <c r="F1103" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1104" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1104" s="0" t="inlineStr">
+        <is>
+          <t>fun</t>
+        </is>
+      </c>
+      <c r="D1104" s="0" t="inlineStr">
+        <is>
+          <t>birth_fun</t>
+        </is>
+      </c>
+      <c r="E1104" s="2">
+        <v>14</v>
+      </c>
+      <c r="F1104" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1105" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1105" s="0" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="D1105" s="0" t="inlineStr">
+        <is>
+          <t>gen_weekend</t>
+        </is>
+      </c>
+      <c r="E1105" s="2">
+        <v>13</v>
+      </c>
+      <c r="F1105" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1106" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1106" s="0" t="inlineStr">
+        <is>
+          <t>thinkingofyou</t>
+        </is>
+      </c>
+      <c r="D1106" s="0" t="inlineStr">
+        <is>
+          <t>gen_thinkingofyou</t>
+        </is>
+      </c>
+      <c r="E1106" s="2">
+        <v>12</v>
+      </c>
+      <c r="F1106" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1107" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1107" s="0" t="inlineStr">
+        <is>
+          <t>extfamily</t>
+        </is>
+      </c>
+      <c r="D1107" s="0" t="inlineStr">
+        <is>
+          <t>birth_extfamily</t>
+        </is>
+      </c>
+      <c r="E1107" s="2">
+        <v>11</v>
+      </c>
+      <c r="F1107" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1108" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1108" s="0" t="inlineStr">
+        <is>
+          <t>anniversaryetc</t>
+        </is>
+      </c>
+      <c r="D1108" s="0" t="inlineStr">
+        <is>
+          <t>anniv_anniversaryetc</t>
+        </is>
+      </c>
+      <c r="E1108" s="2">
+        <v>10</v>
+      </c>
+      <c r="F1108" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1109" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1109" s="0" t="inlineStr">
+        <is>
+          <t>bronsis</t>
+        </is>
+      </c>
+      <c r="D1109" s="0" t="inlineStr">
+        <is>
+          <t>birth_bronsis</t>
+        </is>
+      </c>
+      <c r="E1109" s="2">
+        <v>10</v>
+      </c>
+      <c r="F1109" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1110" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1110" s="0" t="inlineStr">
+        <is>
+          <t>songs</t>
+        </is>
+      </c>
+      <c r="D1110" s="0" t="inlineStr">
+        <is>
+          <t>birth_songs</t>
+        </is>
+      </c>
+      <c r="E1110" s="2">
+        <v>9</v>
+      </c>
+      <c r="F1110" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1111" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1111" s="0" t="inlineStr">
+        <is>
+          <t>morning</t>
+        </is>
+      </c>
+      <c r="D1111" s="0" t="inlineStr">
+        <is>
+          <t>gen_morning</t>
+        </is>
+      </c>
+      <c r="E1111" s="2">
+        <v>8</v>
+      </c>
+      <c r="F1111" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1112" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1112" s="0" t="inlineStr">
+        <is>
+          <t>newbaby</t>
+        </is>
+      </c>
+      <c r="D1112" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newbaby</t>
+        </is>
+      </c>
+      <c r="E1112" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1112" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1113" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1113" s="0" t="inlineStr">
+        <is>
+          <t>encour</t>
+        </is>
+      </c>
+      <c r="D1113" s="0" t="inlineStr">
+        <is>
+          <t>insp_encour</t>
+        </is>
+      </c>
+      <c r="E1113" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1113" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1114" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1114" s="0" t="inlineStr">
+        <is>
+          <t>belated</t>
+        </is>
+      </c>
+      <c r="D1114" s="0" t="inlineStr">
+        <is>
+          <t>birth_belated</t>
+        </is>
+      </c>
+      <c r="E1114" s="2">
+        <v>6</v>
+      </c>
+      <c r="F1114" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1115" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1115" s="0" t="inlineStr">
+        <is>
+          <t>friends</t>
+        </is>
+      </c>
+      <c r="D1115" s="0" t="inlineStr">
+        <is>
+          <t>birth_friends</t>
+        </is>
+      </c>
+      <c r="E1115" s="2">
+        <v>6</v>
+      </c>
+      <c r="F1115" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1116" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1116" s="0" t="inlineStr">
+        <is>
+          <t>hvgtday</t>
+        </is>
+      </c>
+      <c r="D1116" s="0" t="inlineStr">
+        <is>
+          <t>gen_hvgtday</t>
+        </is>
+      </c>
+      <c r="E1116" s="2">
+        <v>6</v>
+      </c>
+      <c r="F1116" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1117" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1117" s="0" t="inlineStr">
+        <is>
+          <t>everyday</t>
+        </is>
+      </c>
+      <c r="D1117" s="0" t="inlineStr">
+        <is>
+          <t>thank_everyday</t>
+        </is>
+      </c>
+      <c r="E1117" s="2">
+        <v>6</v>
+      </c>
+      <c r="F1117" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1118" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1118" s="0" t="inlineStr">
+        <is>
+          <t>blessings</t>
+        </is>
+      </c>
+      <c r="D1118" s="0" t="inlineStr">
+        <is>
+          <t>birth_blessings</t>
+        </is>
+      </c>
+      <c r="E1118" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1118" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1119" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1119" s="0" t="inlineStr">
+        <is>
+          <t>kids</t>
+        </is>
+      </c>
+      <c r="D1119" s="0" t="inlineStr">
+        <is>
+          <t>birth_kids</t>
+        </is>
+      </c>
+      <c r="E1119" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1119" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1120" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1120" s="0" t="inlineStr">
+        <is>
+          <t>wishes</t>
+        </is>
+      </c>
+      <c r="D1120" s="0" t="inlineStr">
+        <is>
+          <t>birth_wishes</t>
+        </is>
+      </c>
+      <c r="E1120" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1120" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1121" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1121" s="0" t="inlineStr">
+        <is>
+          <t>eaug_flwrmonthaug</t>
+        </is>
+      </c>
+      <c r="D1121" s="0" t="inlineStr">
+        <is>
+          <t>eaug_flwrmonthaug</t>
+        </is>
+      </c>
+      <c r="E1121" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1121" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1122" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1122" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="D1122" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="E1122" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1122" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1123" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1123" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D1123" s="0" t="inlineStr">
+        <is>
+          <t>anniv_milestone</t>
+        </is>
+      </c>
+      <c r="E1123" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1123" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1124" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1124" s="0" t="inlineStr">
+        <is>
+          <t>flowers</t>
+        </is>
+      </c>
+      <c r="D1124" s="0" t="inlineStr">
+        <is>
+          <t>birth_flowers</t>
+        </is>
+      </c>
+      <c r="E1124" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1124" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1125" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1125" s="0" t="inlineStr">
+        <is>
+          <t>zodiac</t>
+        </is>
+      </c>
+      <c r="D1125" s="0" t="inlineStr">
+        <is>
+          <t>birth_zodiac</t>
+        </is>
+      </c>
+      <c r="E1125" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1125" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1126" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1126" s="0" t="inlineStr">
+        <is>
+          <t>eapr_goodfriday</t>
+        </is>
+      </c>
+      <c r="D1126" s="0" t="inlineStr">
+        <is>
+          <t>eapr_goodfriday</t>
+        </is>
+      </c>
+      <c r="E1126" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1126" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1127" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1127" s="0" t="inlineStr">
+        <is>
+          <t>enov_cappuccinoday</t>
+        </is>
+      </c>
+      <c r="D1127" s="0" t="inlineStr">
+        <is>
+          <t>enov_cappuccinoday</t>
+        </is>
+      </c>
+      <c r="E1127" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1127" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1128" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1128" s="0" t="inlineStr">
+        <is>
+          <t>sweetheart</t>
+        </is>
+      </c>
+      <c r="D1128" s="0" t="inlineStr">
+        <is>
+          <t>love_sweetheart</t>
+        </is>
+      </c>
+      <c r="E1128" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1128" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1129" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1129" s="0" t="inlineStr">
+        <is>
+          <t>forher</t>
+        </is>
+      </c>
+      <c r="D1129" s="0" t="inlineStr">
+        <is>
+          <t>birth_forher</t>
+        </is>
+      </c>
+      <c r="E1129" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1129" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1130" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1130" s="0" t="inlineStr">
+        <is>
+          <t>momndad</t>
+        </is>
+      </c>
+      <c r="D1130" s="0" t="inlineStr">
+        <is>
+          <t>birth_momndad</t>
+        </is>
+      </c>
+      <c r="E1130" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1130" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1131" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C1131" s="0" t="inlineStr">
+        <is>
+          <t>atworketc</t>
+        </is>
+      </c>
+      <c r="D1131" s="0" t="inlineStr">
+        <is>
+          <t>bus_atworketc</t>
+        </is>
+      </c>
+      <c r="E1131" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1131" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1132" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1132" s="0" t="inlineStr">
+        <is>
+          <t>foreveryone</t>
+        </is>
+      </c>
+      <c r="D1132" s="0" t="inlineStr">
+        <is>
+          <t>congrats_foreveryone</t>
+        </is>
+      </c>
+      <c r="E1132" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1132" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1133" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1133" s="0" t="inlineStr">
+        <is>
+          <t>newhome</t>
+        </is>
+      </c>
+      <c r="D1133" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newhome</t>
+        </is>
+      </c>
+      <c r="E1133" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1133" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1134" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1134" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_happy</t>
+        </is>
+      </c>
+      <c r="D1134" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipday_happy</t>
+        </is>
+      </c>
+      <c r="E1134" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1134" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1135" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1135" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="D1135" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="E1135" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1135" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1136" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1136" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalrelaxation_day</t>
+        </is>
+      </c>
+      <c r="D1136" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalrelaxation_day</t>
+        </is>
+      </c>
+      <c r="E1136" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1136" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1137" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1137" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_happy</t>
+        </is>
+      </c>
+      <c r="D1137" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_happy</t>
+        </is>
+      </c>
+      <c r="E1137" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1137" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1138" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C1138" s="0" t="inlineStr">
+        <is>
+          <t>sisters</t>
+        </is>
+      </c>
+      <c r="D1138" s="0" t="inlineStr">
+        <is>
+          <t>fkt_sisters</t>
+        </is>
+      </c>
+      <c r="E1138" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1138" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1139" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C1139" s="0" t="inlineStr">
+        <is>
+          <t>flrwishes</t>
+        </is>
+      </c>
+      <c r="D1139" s="0" t="inlineStr">
+        <is>
+          <t>flwr_flrwishes</t>
+        </is>
+      </c>
+      <c r="E1139" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1139" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1140" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1140" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D1140" s="0" t="inlineStr">
+        <is>
+          <t>gen_getwell</t>
+        </is>
+      </c>
+      <c r="E1140" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1140" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1141" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1141" s="0" t="inlineStr">
+        <is>
+          <t>nameday</t>
+        </is>
+      </c>
+      <c r="D1141" s="0" t="inlineStr">
+        <is>
+          <t>gen_nameday</t>
+        </is>
+      </c>
+      <c r="E1141" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1141" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1142" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1142" s="0" t="inlineStr">
+        <is>
+          <t>quotesmessages_images_getwell_images</t>
+        </is>
+      </c>
+      <c r="D1142" s="0" t="inlineStr">
+        <is>
+          <t>gen_quotesmessages_images_getwell_images</t>
+        </is>
+      </c>
+      <c r="E1142" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1142" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1143" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1143" s="0" t="inlineStr">
+        <is>
+          <t>quotesmessages_images_getwell_quotes</t>
+        </is>
+      </c>
+      <c r="D1143" s="0" t="inlineStr">
+        <is>
+          <t>gen_quotesmessages_images_getwell_quotes</t>
+        </is>
+      </c>
+      <c r="E1143" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1143" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1144" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1144" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="D1144" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="E1144" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1144" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1145" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1145" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_general</t>
+        </is>
+      </c>
+      <c r="D1145" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_general</t>
+        </is>
+      </c>
+      <c r="E1145" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1145" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1146" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1146" s="0" t="inlineStr">
+        <is>
+          <t>wed_arndworld</t>
+        </is>
+      </c>
+      <c r="D1146" s="0" t="inlineStr">
+        <is>
+          <t>wed_arndworld</t>
+        </is>
+      </c>
+      <c r="E1146" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1146" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1147" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1147" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="D1147" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="E1147" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1147" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1148" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1148" s="0" t="inlineStr">
+        <is>
+          <t>collassociates</t>
+        </is>
+      </c>
+      <c r="D1148" s="0" t="inlineStr">
+        <is>
+          <t>birth_collassociates</t>
+        </is>
+      </c>
+      <c r="E1148" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1148" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1149" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C1149" s="0" t="inlineStr">
+        <is>
+          <t>retirement</t>
+        </is>
+      </c>
+      <c r="D1149" s="0" t="inlineStr">
+        <is>
+          <t>bus_retirement</t>
+        </is>
+      </c>
+      <c r="E1149" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1149" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1150" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1150" s="0" t="inlineStr">
+        <is>
+          <t>businessandworkplace</t>
+        </is>
+      </c>
+      <c r="D1150" s="0" t="inlineStr">
+        <is>
+          <t>congrats_businessandworkplace</t>
+        </is>
+      </c>
+      <c r="E1150" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1150" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1151" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1151" s="0" t="inlineStr">
+        <is>
+          <t>retirement</t>
+        </is>
+      </c>
+      <c r="D1151" s="0" t="inlineStr">
+        <is>
+          <t>congrats_retirement</t>
+        </is>
+      </c>
+      <c r="E1151" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1151" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1152" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1152" s="0" t="inlineStr">
+        <is>
+          <t>studentsandnewgrads</t>
+        </is>
+      </c>
+      <c r="D1152" s="0" t="inlineStr">
+        <is>
+          <t>congrats_studentsandnewgrads</t>
+        </is>
+      </c>
+      <c r="E1152" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1152" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1153" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1153" s="0" t="inlineStr">
+        <is>
+          <t>eaug_lemonmeringue_pie_day</t>
+        </is>
+      </c>
+      <c r="D1153" s="0" t="inlineStr">
+        <is>
+          <t>eaug_lemonmeringue_pie_day</t>
+        </is>
+      </c>
+      <c r="E1153" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1153" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1154" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1154" s="0" t="inlineStr">
+        <is>
+          <t>eaug_thankyouday</t>
+        </is>
+      </c>
+      <c r="D1154" s="0" t="inlineStr">
+        <is>
+          <t>eaug_thankyouday</t>
+        </is>
+      </c>
+      <c r="E1154" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1154" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1155" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1155" s="0" t="inlineStr">
+        <is>
+          <t>edec_c_thankyou</t>
+        </is>
+      </c>
+      <c r="D1155" s="0" t="inlineStr">
+        <is>
+          <t>edec_c_thankyou</t>
+        </is>
+      </c>
+      <c r="E1155" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1155" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1156" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1156" s="0" t="inlineStr">
+        <is>
+          <t>edec_feastof_immaculate_conception</t>
+        </is>
+      </c>
+      <c r="D1156" s="0" t="inlineStr">
+        <is>
+          <t>edec_feastof_immaculate_conception</t>
+        </is>
+      </c>
+      <c r="E1156" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1156" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1157" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1157" s="0" t="inlineStr">
+        <is>
+          <t>ejan_danceday</t>
+        </is>
+      </c>
+      <c r="D1157" s="0" t="inlineStr">
+        <is>
+          <t>ejan_danceday</t>
+        </is>
+      </c>
+      <c r="E1157" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1157" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1158" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1158" s="0" t="inlineStr">
+        <is>
+          <t>ejan_thankyoucards</t>
+        </is>
+      </c>
+      <c r="D1158" s="0" t="inlineStr">
+        <is>
+          <t>ejan_thankyoucards</t>
+        </is>
+      </c>
+      <c r="E1158" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1158" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1159" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1159" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_missingu</t>
+        </is>
+      </c>
+      <c r="D1159" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_missingu</t>
+        </is>
+      </c>
+      <c r="E1159" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1159" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1160" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1160" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_thank</t>
+        </is>
+      </c>
+      <c r="D1160" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_thank</t>
+        </is>
+      </c>
+      <c r="E1160" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1160" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1161" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1161" s="0" t="inlineStr">
+        <is>
+          <t>eoct_sweetday_thanku</t>
+        </is>
+      </c>
+      <c r="D1161" s="0" t="inlineStr">
+        <is>
+          <t>eoct_sweetday_thanku</t>
+        </is>
+      </c>
+      <c r="E1161" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1161" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1162" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C1162" s="0" t="inlineStr">
+        <is>
+          <t>familyoccasions</t>
+        </is>
+      </c>
+      <c r="D1162" s="0" t="inlineStr">
+        <is>
+          <t>fkt_familyoccasions</t>
+        </is>
+      </c>
+      <c r="E1162" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1162" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1163" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C1163" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D1163" s="0" t="inlineStr">
+        <is>
+          <t>flwr_love</t>
+        </is>
+      </c>
+      <c r="E1163" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1163" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1164" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C1164" s="0" t="inlineStr">
+        <is>
+          <t>friendsforever</t>
+        </is>
+      </c>
+      <c r="D1164" s="0" t="inlineStr">
+        <is>
+          <t>friend_friendsforever</t>
+        </is>
+      </c>
+      <c r="E1164" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1164" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1165" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C1165" s="0" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
+      <c r="D1165" s="0" t="inlineStr">
+        <is>
+          <t>friend_thoughts</t>
+        </is>
+      </c>
+      <c r="E1165" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1165" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1166" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1166" s="0" t="inlineStr">
+        <is>
+          <t>goodnight</t>
+        </is>
+      </c>
+      <c r="D1166" s="0" t="inlineStr">
+        <is>
+          <t>gen_goodnight</t>
+        </is>
+      </c>
+      <c r="E1166" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1166" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1167" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1167" s="0" t="inlineStr">
+        <is>
+          <t>quotesmessages_images_getwell_messages</t>
+        </is>
+      </c>
+      <c r="D1167" s="0" t="inlineStr">
+        <is>
+          <t>gen_quotesmessages_images_getwell_messages</t>
+        </is>
+      </c>
+      <c r="E1167" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1167" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1168" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1168" s="0" t="inlineStr">
+        <is>
+          <t>sorry</t>
+        </is>
+      </c>
+      <c r="D1168" s="0" t="inlineStr">
+        <is>
+          <t>gen_sorry</t>
+        </is>
+      </c>
+      <c r="E1168" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1168" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1169" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1169" s="0" t="inlineStr">
+        <is>
+          <t>angels</t>
+        </is>
+      </c>
+      <c r="D1169" s="0" t="inlineStr">
+        <is>
+          <t>insp_angels</t>
+        </is>
+      </c>
+      <c r="E1169" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1169" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1170" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1170" s="0" t="inlineStr">
+        <is>
+          <t>recovery</t>
+        </is>
+      </c>
+      <c r="D1170" s="0" t="inlineStr">
+        <is>
+          <t>insp_recovery</t>
+        </is>
+      </c>
+      <c r="E1170" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1170" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1171" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C1171" s="0" t="inlineStr">
+        <is>
+          <t>justbecause</t>
+        </is>
+      </c>
+      <c r="D1171" s="0" t="inlineStr">
+        <is>
+          <t>intouch_justbecause</t>
+        </is>
+      </c>
+      <c r="E1171" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1171" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1172" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1172" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="D1172" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="E1172" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1172" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1173" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1173" s="0" t="inlineStr">
+        <is>
+          <t>missing_forher</t>
+        </is>
+      </c>
+      <c r="D1173" s="0" t="inlineStr">
+        <is>
+          <t>love_missing_forher</t>
+        </is>
+      </c>
+      <c r="E1173" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1173" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1174" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1174" s="0" t="inlineStr">
+        <is>
+          <t>newlove</t>
+        </is>
+      </c>
+      <c r="D1174" s="0" t="inlineStr">
+        <is>
+          <t>love_newlove</t>
+        </is>
+      </c>
+      <c r="E1174" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1174" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1175" s="4"/>
+      <c r="C1175" s="4"/>
+      <c r="D1175" s="4"/>
+      <c r="E1175" s="5">
+        <v>811</v>
+      </c>
+      <c r="F1175" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -38893,36 +41674,70 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B15" s="2">
+        <v>914</v>
+      </c>
+      <c r="C15" s="2">
+        <v>233</v>
+      </c>
+      <c r="D15" s="2">
+        <v>363</v>
+      </c>
+      <c r="E15" s="2">
+        <v>183</v>
+      </c>
+      <c r="F15" s="2">
+        <v>71</v>
+      </c>
+      <c r="G15" s="2">
+        <v>34</v>
+      </c>
+      <c r="H15" s="2">
+        <v>30</v>
+      </c>
+      <c r="I15" s="2">
+        <v>0</v>
+      </c>
+      <c r="J15" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B15" s="5">
-        <v>10776</v>
-      </c>
-      <c r="C15" s="5">
-        <v>3440</v>
-      </c>
-      <c r="D15" s="5">
-        <v>3293</v>
-      </c>
-      <c r="E15" s="5">
-        <v>2131</v>
-      </c>
-      <c r="F15" s="5">
-        <v>1119</v>
-      </c>
-      <c r="G15" s="5">
-        <v>414</v>
-      </c>
-      <c r="H15" s="5">
-        <v>350</v>
-      </c>
-      <c r="I15" s="5">
+      <c r="B16" s="5">
+        <v>11690</v>
+      </c>
+      <c r="C16" s="5">
+        <v>3673</v>
+      </c>
+      <c r="D16" s="5">
+        <v>3656</v>
+      </c>
+      <c r="E16" s="5">
+        <v>2314</v>
+      </c>
+      <c r="F16" s="5">
+        <v>1190</v>
+      </c>
+      <c r="G16" s="5">
+        <v>448</v>
+      </c>
+      <c r="H16" s="5">
+        <v>380</v>
+      </c>
+      <c r="I16" s="5">
         <v>28</v>
       </c>
-      <c r="J15" s="5">
+      <c r="J16" s="5">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Record 15 August: fifteen days, 12,518 sends tracked
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9KsXegBwxB1sWdCzRVLrr
</commit_message>
<xml_diff>
--- a/reports/daily_tracking.xlsx
+++ b/reports/daily_tracking.xlsx
@@ -224,7 +224,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
@@ -247,7 +247,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
@@ -703,28 +703,56 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <v>828</v>
+      </c>
+      <c r="C16" s="2">
+        <v>594</v>
+      </c>
+      <c r="D16" s="2">
+        <v>234</v>
+      </c>
+      <c r="E16" s="2">
+        <v>797</v>
+      </c>
+      <c r="F16" s="2">
+        <v>31</v>
+      </c>
+      <c r="G16" s="2">
+        <v>247</v>
+      </c>
+      <c r="H16" s="2">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B16" s="5">
-        <v>11690</v>
-      </c>
-      <c r="C16" s="5">
-        <v>7698</v>
-      </c>
-      <c r="D16" s="5">
-        <v>3992</v>
-      </c>
-      <c r="E16" s="5">
-        <v>11241</v>
-      </c>
-      <c r="F16" s="5">
-        <v>449</v>
-      </c>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
+      <c r="B17" s="5">
+        <v>12518</v>
+      </c>
+      <c r="C17" s="5">
+        <v>8292</v>
+      </c>
+      <c r="D17" s="5">
+        <v>4226</v>
+      </c>
+      <c r="E17" s="5">
+        <v>12038</v>
+      </c>
+      <c r="F17" s="5">
+        <v>480</v>
+      </c>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -1706,64 +1734,125 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <v>797</v>
+      </c>
+      <c r="C16" s="2">
+        <v>485</v>
+      </c>
+      <c r="D16" s="2">
+        <v>140</v>
+      </c>
+      <c r="E16" s="2">
+        <v>58</v>
+      </c>
+      <c r="F16" s="2">
+        <v>27</v>
+      </c>
+      <c r="G16" s="2">
+        <v>34</v>
+      </c>
+      <c r="H16" s="2">
+        <v>19</v>
+      </c>
+      <c r="I16" s="2">
+        <v>18</v>
+      </c>
+      <c r="J16" s="2">
+        <v>3</v>
+      </c>
+      <c r="K16" s="2">
+        <v>7</v>
+      </c>
+      <c r="L16" s="2">
+        <v>1</v>
+      </c>
+      <c r="M16" s="2">
+        <v>1</v>
+      </c>
+      <c r="N16" s="2">
+        <v>1</v>
+      </c>
+      <c r="O16" s="2">
+        <v>1</v>
+      </c>
+      <c r="P16" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>0</v>
+      </c>
+      <c r="R16" s="2">
+        <v>1</v>
+      </c>
+      <c r="S16" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B16" s="5">
-        <v>11241</v>
-      </c>
-      <c r="C16" s="5">
-        <v>7356</v>
-      </c>
-      <c r="D16" s="5">
-        <v>1145</v>
-      </c>
-      <c r="E16" s="5">
-        <v>685</v>
-      </c>
-      <c r="F16" s="5">
-        <v>542</v>
-      </c>
-      <c r="G16" s="5">
-        <v>428</v>
-      </c>
-      <c r="H16" s="5">
-        <v>262</v>
-      </c>
-      <c r="I16" s="5">
-        <v>219</v>
-      </c>
-      <c r="J16" s="5">
-        <v>175</v>
-      </c>
-      <c r="K16" s="5">
-        <v>133</v>
-      </c>
-      <c r="L16" s="5">
-        <v>88</v>
-      </c>
-      <c r="M16" s="5">
-        <v>58</v>
-      </c>
-      <c r="N16" s="5">
-        <v>49</v>
-      </c>
-      <c r="O16" s="5">
-        <v>38</v>
-      </c>
-      <c r="P16" s="5">
+      <c r="B17" s="5">
+        <v>12038</v>
+      </c>
+      <c r="C17" s="5">
+        <v>7841</v>
+      </c>
+      <c r="D17" s="5">
+        <v>1285</v>
+      </c>
+      <c r="E17" s="5">
+        <v>743</v>
+      </c>
+      <c r="F17" s="5">
+        <v>569</v>
+      </c>
+      <c r="G17" s="5">
+        <v>462</v>
+      </c>
+      <c r="H17" s="5">
+        <v>281</v>
+      </c>
+      <c r="I17" s="5">
+        <v>237</v>
+      </c>
+      <c r="J17" s="5">
+        <v>178</v>
+      </c>
+      <c r="K17" s="5">
+        <v>140</v>
+      </c>
+      <c r="L17" s="5">
+        <v>89</v>
+      </c>
+      <c r="M17" s="5">
+        <v>59</v>
+      </c>
+      <c r="N17" s="5">
+        <v>50</v>
+      </c>
+      <c r="O17" s="5">
+        <v>39</v>
+      </c>
+      <c r="P17" s="5">
         <v>22</v>
       </c>
-      <c r="Q16" s="5">
+      <c r="Q17" s="5">
         <v>20</v>
       </c>
-      <c r="R16" s="5">
-        <v>15</v>
-      </c>
-      <c r="S16" s="5">
-        <v>6</v>
+      <c r="R17" s="5">
+        <v>16</v>
+      </c>
+      <c r="S17" s="5">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -8501,6 +8590,508 @@
       </c>
       <c r="H214" s="4"/>
     </row>
+    <row r="215">
+      <c r="A215" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B215" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C215" s="0" t="inlineStr">
+        <is>
+          <t>birth</t>
+        </is>
+      </c>
+      <c r="D215" s="2">
+        <v>363</v>
+      </c>
+      <c r="E215" s="2">
+        <v>122</v>
+      </c>
+      <c r="F215" s="2">
+        <v>485</v>
+      </c>
+      <c r="G215" s="3">
+        <v>0.6085319949811794</v>
+      </c>
+      <c r="H215" s="2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B216" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C216" s="0" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="D216" s="2">
+        <v>114</v>
+      </c>
+      <c r="E216" s="2">
+        <v>26</v>
+      </c>
+      <c r="F216" s="2">
+        <v>140</v>
+      </c>
+      <c r="G216" s="3">
+        <v>0.17565872020075282</v>
+      </c>
+      <c r="H216" s="2">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B217" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C217" s="0" t="inlineStr">
+        <is>
+          <t>anniv</t>
+        </is>
+      </c>
+      <c r="D217" s="2">
+        <v>48</v>
+      </c>
+      <c r="E217" s="2">
+        <v>10</v>
+      </c>
+      <c r="F217" s="2">
+        <v>58</v>
+      </c>
+      <c r="G217" s="3">
+        <v>0.07277289836888332</v>
+      </c>
+      <c r="H217" s="2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B218" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C218" s="0" t="inlineStr">
+        <is>
+          <t>thank</t>
+        </is>
+      </c>
+      <c r="D218" s="2">
+        <v>16</v>
+      </c>
+      <c r="E218" s="2">
+        <v>18</v>
+      </c>
+      <c r="F218" s="2">
+        <v>34</v>
+      </c>
+      <c r="G218" s="3">
+        <v>0.04265997490589712</v>
+      </c>
+      <c r="H218" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B219" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C219" s="0" t="inlineStr">
+        <is>
+          <t>gen</t>
+        </is>
+      </c>
+      <c r="D219" s="2">
+        <v>19</v>
+      </c>
+      <c r="E219" s="2">
+        <v>8</v>
+      </c>
+      <c r="F219" s="2">
+        <v>27</v>
+      </c>
+      <c r="G219" s="3">
+        <v>0.033877038895859475</v>
+      </c>
+      <c r="H219" s="2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B220" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C220" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D220" s="2">
+        <v>10</v>
+      </c>
+      <c r="E220" s="2">
+        <v>9</v>
+      </c>
+      <c r="F220" s="2">
+        <v>19</v>
+      </c>
+      <c r="G220" s="3">
+        <v>0.02383939774153074</v>
+      </c>
+      <c r="H220" s="2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B221" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C221" s="0" t="inlineStr">
+        <is>
+          <t>insp</t>
+        </is>
+      </c>
+      <c r="D221" s="2">
+        <v>15</v>
+      </c>
+      <c r="E221" s="2">
+        <v>3</v>
+      </c>
+      <c r="F221" s="2">
+        <v>18</v>
+      </c>
+      <c r="G221" s="3">
+        <v>0.02258469259723965</v>
+      </c>
+      <c r="H221" s="2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B222" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C222" s="0" t="inlineStr">
+        <is>
+          <t>congrats</t>
+        </is>
+      </c>
+      <c r="D222" s="2">
+        <v>3</v>
+      </c>
+      <c r="E222" s="2">
+        <v>4</v>
+      </c>
+      <c r="F222" s="2">
+        <v>7</v>
+      </c>
+      <c r="G222" s="3">
+        <v>0.00878293601003764</v>
+      </c>
+      <c r="H222" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B223" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C223" s="0" t="inlineStr">
+        <is>
+          <t>friend</t>
+        </is>
+      </c>
+      <c r="D223" s="2">
+        <v>2</v>
+      </c>
+      <c r="E223" s="2">
+        <v>1</v>
+      </c>
+      <c r="F223" s="2">
+        <v>3</v>
+      </c>
+      <c r="G223" s="3">
+        <v>0.0037641154328732747</v>
+      </c>
+      <c r="H223" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B224" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C224" s="0" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+      <c r="D224" s="2">
+        <v>1</v>
+      </c>
+      <c r="E224" s="2">
+        <v>0</v>
+      </c>
+      <c r="F224" s="2">
+        <v>1</v>
+      </c>
+      <c r="G224" s="3">
+        <v>0.0012547051442910915</v>
+      </c>
+      <c r="H224" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B225" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C225" s="0" t="inlineStr">
+        <is>
+          <t>cute</t>
+        </is>
+      </c>
+      <c r="D225" s="2">
+        <v>1</v>
+      </c>
+      <c r="E225" s="2">
+        <v>0</v>
+      </c>
+      <c r="F225" s="2">
+        <v>1</v>
+      </c>
+      <c r="G225" s="3">
+        <v>0.0012547051442910915</v>
+      </c>
+      <c r="H225" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B226" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C226" s="0" t="inlineStr">
+        <is>
+          <t>fkt</t>
+        </is>
+      </c>
+      <c r="D226" s="2">
+        <v>1</v>
+      </c>
+      <c r="E226" s="2">
+        <v>0</v>
+      </c>
+      <c r="F226" s="2">
+        <v>1</v>
+      </c>
+      <c r="G226" s="3">
+        <v>0.0012547051442910915</v>
+      </c>
+      <c r="H226" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B227" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C227" s="0" t="inlineStr">
+        <is>
+          <t>flwr</t>
+        </is>
+      </c>
+      <c r="D227" s="2">
+        <v>0</v>
+      </c>
+      <c r="E227" s="2">
+        <v>1</v>
+      </c>
+      <c r="F227" s="2">
+        <v>1</v>
+      </c>
+      <c r="G227" s="3">
+        <v>0.0012547051442910915</v>
+      </c>
+      <c r="H227" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B228" s="0" t="inlineStr">
+        <is>
+          <t>Invitations &amp; parties</t>
+        </is>
+      </c>
+      <c r="C228" s="0" t="inlineStr">
+        <is>
+          <t>invp</t>
+        </is>
+      </c>
+      <c r="D228" s="2">
+        <v>0</v>
+      </c>
+      <c r="E228" s="2">
+        <v>1</v>
+      </c>
+      <c r="F228" s="2">
+        <v>1</v>
+      </c>
+      <c r="G228" s="3">
+        <v>0.0012547051442910915</v>
+      </c>
+      <c r="H228" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B229" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C229" s="0" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="D229" s="2">
+        <v>1</v>
+      </c>
+      <c r="E229" s="2">
+        <v>0</v>
+      </c>
+      <c r="F229" s="2">
+        <v>1</v>
+      </c>
+      <c r="G229" s="3">
+        <v>0.0012547051442910915</v>
+      </c>
+      <c r="H229" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-15</t>
+        </is>
+      </c>
+      <c r="B230" s="4"/>
+      <c r="C230" s="4"/>
+      <c r="D230" s="5">
+        <v>594</v>
+      </c>
+      <c r="E230" s="5">
+        <v>203</v>
+      </c>
+      <c r="F230" s="5">
+        <v>797</v>
+      </c>
+      <c r="G230" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="H230" s="4"/>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -41391,6 +41982,2344 @@
         <v>884</v>
       </c>
       <c r="F1181" s="4"/>
+    </row>
+    <row r="1182">
+      <c r="A1182" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1182" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1182" s="0" t="inlineStr">
+        <is>
+          <t>happybirthday</t>
+        </is>
+      </c>
+      <c r="D1182" s="0" t="inlineStr">
+        <is>
+          <t>birth_happybirthday</t>
+        </is>
+      </c>
+      <c r="E1182" s="2">
+        <v>388</v>
+      </c>
+      <c r="F1182" s="2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1183" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1183" s="0" t="inlineStr">
+        <is>
+          <t>eaug_indindependenceday</t>
+        </is>
+      </c>
+      <c r="D1183" s="0" t="inlineStr">
+        <is>
+          <t>eaug_indindependenceday</t>
+        </is>
+      </c>
+      <c r="E1183" s="2">
+        <v>62</v>
+      </c>
+      <c r="F1183" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1184" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1184" s="0" t="inlineStr">
+        <is>
+          <t>anniversaryetc</t>
+        </is>
+      </c>
+      <c r="D1184" s="0" t="inlineStr">
+        <is>
+          <t>anniv_anniversaryetc</t>
+        </is>
+      </c>
+      <c r="E1184" s="2">
+        <v>37</v>
+      </c>
+      <c r="F1184" s="2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1185" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1185" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalrelaxation_day</t>
+        </is>
+      </c>
+      <c r="D1185" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalrelaxation_day</t>
+        </is>
+      </c>
+      <c r="E1185" s="2">
+        <v>29</v>
+      </c>
+      <c r="F1185" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1186" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1186" s="0" t="inlineStr">
+        <is>
+          <t>sympathy</t>
+        </is>
+      </c>
+      <c r="D1186" s="0" t="inlineStr">
+        <is>
+          <t>insp_sympathy</t>
+        </is>
+      </c>
+      <c r="E1186" s="2">
+        <v>17</v>
+      </c>
+      <c r="F1186" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1187" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1187" s="0" t="inlineStr">
+        <is>
+          <t>everyday</t>
+        </is>
+      </c>
+      <c r="D1187" s="0" t="inlineStr">
+        <is>
+          <t>thank_everyday</t>
+        </is>
+      </c>
+      <c r="E1187" s="2">
+        <v>16</v>
+      </c>
+      <c r="F1187" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1188" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1188" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="D1188" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="E1188" s="2">
+        <v>15</v>
+      </c>
+      <c r="F1188" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1189" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1189" s="0" t="inlineStr">
+        <is>
+          <t>sonanddaughter</t>
+        </is>
+      </c>
+      <c r="D1189" s="0" t="inlineStr">
+        <is>
+          <t>birth_sonanddaughter</t>
+        </is>
+      </c>
+      <c r="E1189" s="2">
+        <v>15</v>
+      </c>
+      <c r="F1189" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1190" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1190" s="0" t="inlineStr">
+        <is>
+          <t>fun</t>
+        </is>
+      </c>
+      <c r="D1190" s="0" t="inlineStr">
+        <is>
+          <t>birth_fun</t>
+        </is>
+      </c>
+      <c r="E1190" s="2">
+        <v>14</v>
+      </c>
+      <c r="F1190" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1191" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1191" s="0" t="inlineStr">
+        <is>
+          <t>birthday</t>
+        </is>
+      </c>
+      <c r="D1191" s="0" t="inlineStr">
+        <is>
+          <t>thank_birthday</t>
+        </is>
+      </c>
+      <c r="E1191" s="2">
+        <v>11</v>
+      </c>
+      <c r="F1191" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1192" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1192" s="0" t="inlineStr">
+        <is>
+          <t>belated</t>
+        </is>
+      </c>
+      <c r="D1192" s="0" t="inlineStr">
+        <is>
+          <t>birth_belated</t>
+        </is>
+      </c>
+      <c r="E1192" s="2">
+        <v>10</v>
+      </c>
+      <c r="F1192" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1193" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1193" s="0" t="inlineStr">
+        <is>
+          <t>songs</t>
+        </is>
+      </c>
+      <c r="D1193" s="0" t="inlineStr">
+        <is>
+          <t>birth_songs</t>
+        </is>
+      </c>
+      <c r="E1193" s="2">
+        <v>10</v>
+      </c>
+      <c r="F1193" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1194" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1194" s="0" t="inlineStr">
+        <is>
+          <t>thinkingofyou</t>
+        </is>
+      </c>
+      <c r="D1194" s="0" t="inlineStr">
+        <is>
+          <t>gen_thinkingofyou</t>
+        </is>
+      </c>
+      <c r="E1194" s="2">
+        <v>10</v>
+      </c>
+      <c r="F1194" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1195" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1195" s="0" t="inlineStr">
+        <is>
+          <t>flowers</t>
+        </is>
+      </c>
+      <c r="D1195" s="0" t="inlineStr">
+        <is>
+          <t>birth_flowers</t>
+        </is>
+      </c>
+      <c r="E1195" s="2">
+        <v>8</v>
+      </c>
+      <c r="F1195" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1196" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1196" s="0" t="inlineStr">
+        <is>
+          <t>sweetheart</t>
+        </is>
+      </c>
+      <c r="D1196" s="0" t="inlineStr">
+        <is>
+          <t>love_sweetheart</t>
+        </is>
+      </c>
+      <c r="E1196" s="2">
+        <v>8</v>
+      </c>
+      <c r="F1196" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1197" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1197" s="0" t="inlineStr">
+        <is>
+          <t>bronsis</t>
+        </is>
+      </c>
+      <c r="D1197" s="0" t="inlineStr">
+        <is>
+          <t>birth_bronsis</t>
+        </is>
+      </c>
+      <c r="E1197" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1197" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1198" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1198" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D1198" s="0" t="inlineStr">
+        <is>
+          <t>birth_milestone</t>
+        </is>
+      </c>
+      <c r="E1198" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1198" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1199" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1199" s="0" t="inlineStr">
+        <is>
+          <t>eaug_zorastriannewyear</t>
+        </is>
+      </c>
+      <c r="D1199" s="0" t="inlineStr">
+        <is>
+          <t>eaug_zorastriannewyear</t>
+        </is>
+      </c>
+      <c r="E1199" s="2">
+        <v>6</v>
+      </c>
+      <c r="F1199" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1200" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1200" s="0" t="inlineStr">
+        <is>
+          <t>wedding</t>
+        </is>
+      </c>
+      <c r="D1200" s="0" t="inlineStr">
+        <is>
+          <t>thank_wedding</t>
+        </is>
+      </c>
+      <c r="E1200" s="2">
+        <v>6</v>
+      </c>
+      <c r="F1200" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1201" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1201" s="0" t="inlineStr">
+        <is>
+          <t>blessings</t>
+        </is>
+      </c>
+      <c r="D1201" s="0" t="inlineStr">
+        <is>
+          <t>birth_blessings</t>
+        </is>
+      </c>
+      <c r="E1201" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1201" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1202" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1202" s="0" t="inlineStr">
+        <is>
+          <t>kids</t>
+        </is>
+      </c>
+      <c r="D1202" s="0" t="inlineStr">
+        <is>
+          <t>birth_kids</t>
+        </is>
+      </c>
+      <c r="E1202" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1202" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1203" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1203" s="0" t="inlineStr">
+        <is>
+          <t>eaug_lemonmeringue_pie_day</t>
+        </is>
+      </c>
+      <c r="D1203" s="0" t="inlineStr">
+        <is>
+          <t>eaug_lemonmeringue_pie_day</t>
+        </is>
+      </c>
+      <c r="E1203" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1203" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1204" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1204" s="0" t="inlineStr">
+        <is>
+          <t>nameday</t>
+        </is>
+      </c>
+      <c r="D1204" s="0" t="inlineStr">
+        <is>
+          <t>gen_nameday</t>
+        </is>
+      </c>
+      <c r="E1204" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1204" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1205" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1205" s="0" t="inlineStr">
+        <is>
+          <t>extfamily</t>
+        </is>
+      </c>
+      <c r="D1205" s="0" t="inlineStr">
+        <is>
+          <t>birth_extfamily</t>
+        </is>
+      </c>
+      <c r="E1205" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1205" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1206" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1206" s="0" t="inlineStr">
+        <is>
+          <t>hubbywife</t>
+        </is>
+      </c>
+      <c r="D1206" s="0" t="inlineStr">
+        <is>
+          <t>birth_hubbywife</t>
+        </is>
+      </c>
+      <c r="E1206" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1206" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1207" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1207" s="0" t="inlineStr">
+        <is>
+          <t>eaug_smilemonth</t>
+        </is>
+      </c>
+      <c r="D1207" s="0" t="inlineStr">
+        <is>
+          <t>eaug_smilemonth</t>
+        </is>
+      </c>
+      <c r="E1207" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1207" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1208" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1208" s="0" t="inlineStr">
+        <is>
+          <t>esep_trueloveforeverday</t>
+        </is>
+      </c>
+      <c r="D1208" s="0" t="inlineStr">
+        <is>
+          <t>esep_trueloveforeverday</t>
+        </is>
+      </c>
+      <c r="E1208" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1208" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1209" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1209" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_general</t>
+        </is>
+      </c>
+      <c r="D1209" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_general</t>
+        </is>
+      </c>
+      <c r="E1209" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1209" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1210" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1210" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="D1210" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="E1210" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1210" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1211" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1211" s="0" t="inlineStr">
+        <is>
+          <t>friends</t>
+        </is>
+      </c>
+      <c r="D1211" s="0" t="inlineStr">
+        <is>
+          <t>birth_friends</t>
+        </is>
+      </c>
+      <c r="E1211" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1211" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1212" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1212" s="0" t="inlineStr">
+        <is>
+          <t>eaug_rakshabandhan_happy</t>
+        </is>
+      </c>
+      <c r="D1212" s="0" t="inlineStr">
+        <is>
+          <t>eaug_rakshabandhan_happy</t>
+        </is>
+      </c>
+      <c r="E1212" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1212" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1213" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1213" s="0" t="inlineStr">
+        <is>
+          <t>edec_feastof_immaculate_conception</t>
+        </is>
+      </c>
+      <c r="D1213" s="0" t="inlineStr">
+        <is>
+          <t>edec_feastof_immaculate_conception</t>
+        </is>
+      </c>
+      <c r="E1213" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1213" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1214" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1214" s="0" t="inlineStr">
+        <is>
+          <t>emay_mothersday_happy</t>
+        </is>
+      </c>
+      <c r="D1214" s="0" t="inlineStr">
+        <is>
+          <t>emay_mothersday_happy</t>
+        </is>
+      </c>
+      <c r="E1214" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1214" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1215" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1215" s="0" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="D1215" s="0" t="inlineStr">
+        <is>
+          <t>gen_luck</t>
+        </is>
+      </c>
+      <c r="E1215" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1215" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1216" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1216" s="0" t="inlineStr">
+        <is>
+          <t>morning</t>
+        </is>
+      </c>
+      <c r="D1216" s="0" t="inlineStr">
+        <is>
+          <t>gen_morning</t>
+        </is>
+      </c>
+      <c r="E1216" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1216" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1217" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1217" s="0" t="inlineStr">
+        <is>
+          <t>wed_wishes</t>
+        </is>
+      </c>
+      <c r="D1217" s="0" t="inlineStr">
+        <is>
+          <t>wed_wishes</t>
+        </is>
+      </c>
+      <c r="E1217" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1217" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1218" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1218" s="0" t="inlineStr">
+        <is>
+          <t>wishes</t>
+        </is>
+      </c>
+      <c r="D1218" s="0" t="inlineStr">
+        <is>
+          <t>birth_wishes</t>
+        </is>
+      </c>
+      <c r="E1218" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1218" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1219" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1219" s="0" t="inlineStr">
+        <is>
+          <t>foreveryone</t>
+        </is>
+      </c>
+      <c r="D1219" s="0" t="inlineStr">
+        <is>
+          <t>congrats_foreveryone</t>
+        </is>
+      </c>
+      <c r="E1219" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1219" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1220" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1220" s="0" t="inlineStr">
+        <is>
+          <t>newbaby</t>
+        </is>
+      </c>
+      <c r="D1220" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newbaby</t>
+        </is>
+      </c>
+      <c r="E1220" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1220" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1221" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1221" s="0" t="inlineStr">
+        <is>
+          <t>newjob</t>
+        </is>
+      </c>
+      <c r="D1221" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newjob</t>
+        </is>
+      </c>
+      <c r="E1221" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1221" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1222" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1222" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalrum_day</t>
+        </is>
+      </c>
+      <c r="D1222" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalrum_day</t>
+        </is>
+      </c>
+      <c r="E1222" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1222" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1223" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1223" s="0" t="inlineStr">
+        <is>
+          <t>ejan_thankyoucards</t>
+        </is>
+      </c>
+      <c r="D1223" s="0" t="inlineStr">
+        <is>
+          <t>ejan_thankyoucards</t>
+        </is>
+      </c>
+      <c r="E1223" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1223" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1224" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1224" s="0" t="inlineStr">
+        <is>
+          <t>emay_mothersday_fnd</t>
+        </is>
+      </c>
+      <c r="D1224" s="0" t="inlineStr">
+        <is>
+          <t>emay_mothersday_fnd</t>
+        </is>
+      </c>
+      <c r="E1224" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1224" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1225" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C1225" s="0" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
+      <c r="D1225" s="0" t="inlineStr">
+        <is>
+          <t>friend_thoughts</t>
+        </is>
+      </c>
+      <c r="E1225" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1225" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1226" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1226" s="0" t="inlineStr">
+        <is>
+          <t>goodnight</t>
+        </is>
+      </c>
+      <c r="D1226" s="0" t="inlineStr">
+        <is>
+          <t>gen_goodnight</t>
+        </is>
+      </c>
+      <c r="E1226" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1226" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1227" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1227" s="0" t="inlineStr">
+        <is>
+          <t>hvgtday</t>
+        </is>
+      </c>
+      <c r="D1227" s="0" t="inlineStr">
+        <is>
+          <t>gen_hvgtday</t>
+        </is>
+      </c>
+      <c r="E1227" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1227" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1228" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1228" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D1228" s="0" t="inlineStr">
+        <is>
+          <t>anniv_milestone</t>
+        </is>
+      </c>
+      <c r="E1228" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1228" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1229" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1229" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="D1229" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="E1229" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1229" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1230" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1230" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_family</t>
+        </is>
+      </c>
+      <c r="D1230" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_family</t>
+        </is>
+      </c>
+      <c r="E1230" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1230" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1231" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1231" s="0" t="inlineStr">
+        <is>
+          <t>momndad</t>
+        </is>
+      </c>
+      <c r="D1231" s="0" t="inlineStr">
+        <is>
+          <t>birth_momndad</t>
+        </is>
+      </c>
+      <c r="E1231" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1231" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1232" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1232" s="0" t="inlineStr">
+        <is>
+          <t>pets</t>
+        </is>
+      </c>
+      <c r="D1232" s="0" t="inlineStr">
+        <is>
+          <t>birth_pets</t>
+        </is>
+      </c>
+      <c r="E1232" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1232" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1233" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1233" s="0" t="inlineStr">
+        <is>
+          <t>specials</t>
+        </is>
+      </c>
+      <c r="D1233" s="0" t="inlineStr">
+        <is>
+          <t>birth_specials</t>
+        </is>
+      </c>
+      <c r="E1233" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1233" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1234" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C1234" s="0" t="inlineStr">
+        <is>
+          <t>retirement</t>
+        </is>
+      </c>
+      <c r="D1234" s="0" t="inlineStr">
+        <is>
+          <t>bus_retirement</t>
+        </is>
+      </c>
+      <c r="E1234" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1234" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1235" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1235" s="0" t="inlineStr">
+        <is>
+          <t>newhome</t>
+        </is>
+      </c>
+      <c r="D1235" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newhome</t>
+        </is>
+      </c>
+      <c r="E1235" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1235" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1236" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C1236" s="0" t="inlineStr">
+        <is>
+          <t>hugs</t>
+        </is>
+      </c>
+      <c r="D1236" s="0" t="inlineStr">
+        <is>
+          <t>cute_hugs</t>
+        </is>
+      </c>
+      <c r="E1236" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1236" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1237" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1237" s="0" t="inlineStr">
+        <is>
+          <t>eaug_flwrmonthaug</t>
+        </is>
+      </c>
+      <c r="D1237" s="0" t="inlineStr">
+        <is>
+          <t>eaug_flwrmonthaug</t>
+        </is>
+      </c>
+      <c r="E1237" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1237" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1238" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1238" s="0" t="inlineStr">
+        <is>
+          <t>ejul_livebetterday</t>
+        </is>
+      </c>
+      <c r="D1238" s="0" t="inlineStr">
+        <is>
+          <t>ejul_livebetterday</t>
+        </is>
+      </c>
+      <c r="E1238" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1238" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1239" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1239" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_birthday</t>
+        </is>
+      </c>
+      <c r="D1239" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_birthday</t>
+        </is>
+      </c>
+      <c r="E1239" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1239" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1240" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1240" s="0" t="inlineStr">
+        <is>
+          <t>emar_mothersdayuk</t>
+        </is>
+      </c>
+      <c r="D1240" s="0" t="inlineStr">
+        <is>
+          <t>emar_mothersdayuk</t>
+        </is>
+      </c>
+      <c r="E1240" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1240" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1241" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1241" s="0" t="inlineStr">
+        <is>
+          <t>emar_rollercoaster_day</t>
+        </is>
+      </c>
+      <c r="D1241" s="0" t="inlineStr">
+        <is>
+          <t>emar_rollercoaster_day</t>
+        </is>
+      </c>
+      <c r="E1241" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1241" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1242" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1242" s="0" t="inlineStr">
+        <is>
+          <t>emay_mothersday_friends</t>
+        </is>
+      </c>
+      <c r="D1242" s="0" t="inlineStr">
+        <is>
+          <t>emay_mothersday_friends</t>
+        </is>
+      </c>
+      <c r="E1242" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1242" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1243" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1243" s="0" t="inlineStr">
+        <is>
+          <t>eoct_sweetday_romance</t>
+        </is>
+      </c>
+      <c r="D1243" s="0" t="inlineStr">
+        <is>
+          <t>eoct_sweetday_romance</t>
+        </is>
+      </c>
+      <c r="E1243" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1243" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1244" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1244" s="0" t="inlineStr">
+        <is>
+          <t>eoct_yomkippur</t>
+        </is>
+      </c>
+      <c r="D1244" s="0" t="inlineStr">
+        <is>
+          <t>eoct_yomkippur</t>
+        </is>
+      </c>
+      <c r="E1244" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1244" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1245" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1245" s="0" t="inlineStr">
+        <is>
+          <t>esep_beerlovers_day</t>
+        </is>
+      </c>
+      <c r="D1245" s="0" t="inlineStr">
+        <is>
+          <t>esep_beerlovers_day</t>
+        </is>
+      </c>
+      <c r="E1245" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1245" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1246" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1246" s="0" t="inlineStr">
+        <is>
+          <t>esep_durgapuja_blessings</t>
+        </is>
+      </c>
+      <c r="D1246" s="0" t="inlineStr">
+        <is>
+          <t>esep_durgapuja_blessings</t>
+        </is>
+      </c>
+      <c r="E1246" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1246" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1247" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1247" s="0" t="inlineStr">
+        <is>
+          <t>esep_longestkissday</t>
+        </is>
+      </c>
+      <c r="D1247" s="0" t="inlineStr">
+        <is>
+          <t>esep_longestkissday</t>
+        </is>
+      </c>
+      <c r="E1247" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1247" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1248" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C1248" s="0" t="inlineStr">
+        <is>
+          <t>sisters</t>
+        </is>
+      </c>
+      <c r="D1248" s="0" t="inlineStr">
+        <is>
+          <t>fkt_sisters</t>
+        </is>
+      </c>
+      <c r="E1248" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1248" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1249" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C1249" s="0" t="inlineStr">
+        <is>
+          <t>youcare</t>
+        </is>
+      </c>
+      <c r="D1249" s="0" t="inlineStr">
+        <is>
+          <t>flwr_youcare</t>
+        </is>
+      </c>
+      <c r="E1249" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1249" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1250" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C1250" s="0" t="inlineStr">
+        <is>
+          <t>foryou</t>
+        </is>
+      </c>
+      <c r="D1250" s="0" t="inlineStr">
+        <is>
+          <t>friend_foryou</t>
+        </is>
+      </c>
+      <c r="E1250" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1250" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1251" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1251" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D1251" s="0" t="inlineStr">
+        <is>
+          <t>gen_getwell</t>
+        </is>
+      </c>
+      <c r="E1251" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1251" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1252" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1252" s="0" t="inlineStr">
+        <is>
+          <t>quotesmessages_images_goodmorning_images</t>
+        </is>
+      </c>
+      <c r="D1252" s="0" t="inlineStr">
+        <is>
+          <t>gen_quotesmessages_images_goodmorning_images</t>
+        </is>
+      </c>
+      <c r="E1252" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1252" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1253" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1253" s="0" t="inlineStr">
+        <is>
+          <t>recovery</t>
+        </is>
+      </c>
+      <c r="D1253" s="0" t="inlineStr">
+        <is>
+          <t>insp_recovery</t>
+        </is>
+      </c>
+      <c r="E1253" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1253" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1254" s="0" t="inlineStr">
+        <is>
+          <t>Invitations &amp; parties</t>
+        </is>
+      </c>
+      <c r="C1254" s="0" t="inlineStr">
+        <is>
+          <t>birth_gen</t>
+        </is>
+      </c>
+      <c r="D1254" s="0" t="inlineStr">
+        <is>
+          <t>invp_birth_gen</t>
+        </is>
+      </c>
+      <c r="E1254" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1254" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1255" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1255" s="0" t="inlineStr">
+        <is>
+          <t>cute</t>
+        </is>
+      </c>
+      <c r="D1255" s="0" t="inlineStr">
+        <is>
+          <t>love_cute</t>
+        </is>
+      </c>
+      <c r="E1255" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1255" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1256" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1256" s="0" t="inlineStr">
+        <is>
+          <t>hugs</t>
+        </is>
+      </c>
+      <c r="D1256" s="0" t="inlineStr">
+        <is>
+          <t>love_hugs</t>
+        </is>
+      </c>
+      <c r="E1256" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1256" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1257" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1257" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="D1257" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="E1257" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1257" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1258" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1258" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_kisses</t>
+        </is>
+      </c>
+      <c r="D1258" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_kisses</t>
+        </is>
+      </c>
+      <c r="E1258" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1258" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1259" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1259" s="0" t="inlineStr">
+        <is>
+          <t>missing_forher</t>
+        </is>
+      </c>
+      <c r="D1259" s="0" t="inlineStr">
+        <is>
+          <t>love_missing_forher</t>
+        </is>
+      </c>
+      <c r="E1259" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1259" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1260" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1260" s="0" t="inlineStr">
+        <is>
+          <t>thinkingyou</t>
+        </is>
+      </c>
+      <c r="D1260" s="0" t="inlineStr">
+        <is>
+          <t>love_thinkingyou</t>
+        </is>
+      </c>
+      <c r="E1260" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1260" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1261" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1261" s="0" t="inlineStr">
+        <is>
+          <t>youarespecial</t>
+        </is>
+      </c>
+      <c r="D1261" s="0" t="inlineStr">
+        <is>
+          <t>love_youarespecial</t>
+        </is>
+      </c>
+      <c r="E1261" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1261" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1262" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C1262" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D1262" s="0" t="inlineStr">
+        <is>
+          <t>pet_getwell</t>
+        </is>
+      </c>
+      <c r="E1262" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1262" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1263" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1263" s="0" t="inlineStr">
+        <is>
+          <t>inspirational</t>
+        </is>
+      </c>
+      <c r="D1263" s="0" t="inlineStr">
+        <is>
+          <t>thank_inspirational</t>
+        </is>
+      </c>
+      <c r="E1263" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1263" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1264" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1264" s="0" t="inlineStr">
+        <is>
+          <t>wed_wed_congrats</t>
+        </is>
+      </c>
+      <c r="D1264" s="0" t="inlineStr">
+        <is>
+          <t>wed_wed_congrats</t>
+        </is>
+      </c>
+      <c r="E1264" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1264" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-15</t>
+        </is>
+      </c>
+      <c r="B1265" s="4"/>
+      <c r="C1265" s="4"/>
+      <c r="D1265" s="4"/>
+      <c r="E1265" s="5">
+        <v>797</v>
+      </c>
+      <c r="F1265" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -41940,36 +44869,70 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <v>828</v>
+      </c>
+      <c r="C16" s="2">
+        <v>249</v>
+      </c>
+      <c r="D16" s="2">
+        <v>266</v>
+      </c>
+      <c r="E16" s="2">
+        <v>208</v>
+      </c>
+      <c r="F16" s="2">
+        <v>61</v>
+      </c>
+      <c r="G16" s="2">
+        <v>28</v>
+      </c>
+      <c r="H16" s="2">
+        <v>16</v>
+      </c>
+      <c r="I16" s="2">
+        <v>0</v>
+      </c>
+      <c r="J16" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B16" s="5">
-        <v>11690</v>
-      </c>
-      <c r="C16" s="5">
-        <v>3673</v>
-      </c>
-      <c r="D16" s="5">
-        <v>3656</v>
-      </c>
-      <c r="E16" s="5">
-        <v>2314</v>
-      </c>
-      <c r="F16" s="5">
-        <v>1190</v>
-      </c>
-      <c r="G16" s="5">
-        <v>448</v>
-      </c>
-      <c r="H16" s="5">
-        <v>380</v>
-      </c>
-      <c r="I16" s="5">
+      <c r="B17" s="5">
+        <v>12518</v>
+      </c>
+      <c r="C17" s="5">
+        <v>3922</v>
+      </c>
+      <c r="D17" s="5">
+        <v>3922</v>
+      </c>
+      <c r="E17" s="5">
+        <v>2522</v>
+      </c>
+      <c r="F17" s="5">
+        <v>1251</v>
+      </c>
+      <c r="G17" s="5">
+        <v>476</v>
+      </c>
+      <c r="H17" s="5">
+        <v>396</v>
+      </c>
+      <c r="I17" s="5">
         <v>28</v>
       </c>
-      <c r="J16" s="5">
+      <c r="J17" s="5">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Record 16 August: sixteen days, 13,279 sends tracked
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9KsXegBwxB1sWdCzRVLrr
</commit_message>
<xml_diff>
--- a/reports/daily_tracking.xlsx
+++ b/reports/daily_tracking.xlsx
@@ -224,7 +224,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
@@ -247,7 +247,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
@@ -731,28 +731,56 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B17" s="2">
+        <v>761</v>
+      </c>
+      <c r="C17" s="2">
+        <v>518</v>
+      </c>
+      <c r="D17" s="2">
+        <v>243</v>
+      </c>
+      <c r="E17" s="2">
+        <v>720</v>
+      </c>
+      <c r="F17" s="2">
+        <v>41</v>
+      </c>
+      <c r="G17" s="2">
+        <v>263</v>
+      </c>
+      <c r="H17" s="2">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B17" s="5">
-        <v>12518</v>
-      </c>
-      <c r="C17" s="5">
-        <v>8292</v>
-      </c>
-      <c r="D17" s="5">
-        <v>4226</v>
-      </c>
-      <c r="E17" s="5">
-        <v>12038</v>
-      </c>
-      <c r="F17" s="5">
-        <v>480</v>
-      </c>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
+      <c r="B18" s="5">
+        <v>13279</v>
+      </c>
+      <c r="C18" s="5">
+        <v>8810</v>
+      </c>
+      <c r="D18" s="5">
+        <v>4469</v>
+      </c>
+      <c r="E18" s="5">
+        <v>12758</v>
+      </c>
+      <c r="F18" s="5">
+        <v>521</v>
+      </c>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -776,8 +804,8 @@
     <col min="13" max="13" width="21" customWidth="1"/>
     <col min="14" max="14" width="11" customWidth="1"/>
     <col min="15" max="15" width="11" customWidth="1"/>
-    <col min="16" max="16" width="17" customWidth="1"/>
-    <col min="17" max="17" width="18" customWidth="1"/>
+    <col min="16" max="16" width="18" customWidth="1"/>
+    <col min="17" max="17" width="17" customWidth="1"/>
     <col min="18" max="18" width="17" customWidth="1"/>
     <col min="19" max="19" width="23" customWidth="1"/>
   </cols>
@@ -860,12 +888,12 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>World languages</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Keeping in touch</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
@@ -928,10 +956,10 @@
         <v>3</v>
       </c>
       <c r="P2" s="2">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q2" s="2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="R2" s="2">
         <v>2</v>
@@ -989,10 +1017,10 @@
         <v>1</v>
       </c>
       <c r="P3" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q3" s="2">
         <v>10</v>
-      </c>
-      <c r="Q3" s="2">
-        <v>2</v>
       </c>
       <c r="R3" s="2">
         <v>0</v>
@@ -1111,10 +1139,10 @@
         <v>2</v>
       </c>
       <c r="P5" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q5" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R5" s="2">
         <v>0</v>
@@ -1172,10 +1200,10 @@
         <v>4</v>
       </c>
       <c r="P6" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6" s="2">
         <v>2</v>
@@ -1233,10 +1261,10 @@
         <v>2</v>
       </c>
       <c r="P7" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q7" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R7" s="2">
         <v>3</v>
@@ -1416,10 +1444,10 @@
         <v>4</v>
       </c>
       <c r="P10" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R10" s="2">
         <v>0</v>
@@ -1477,10 +1505,10 @@
         <v>8</v>
       </c>
       <c r="P11" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q11" s="2">
         <v>0</v>
-      </c>
-      <c r="Q11" s="2">
-        <v>2</v>
       </c>
       <c r="R11" s="2">
         <v>0</v>
@@ -1538,10 +1566,10 @@
         <v>1</v>
       </c>
       <c r="P12" s="2">
+        <v>6</v>
+      </c>
+      <c r="Q12" s="2">
         <v>0</v>
-      </c>
-      <c r="Q12" s="2">
-        <v>6</v>
       </c>
       <c r="R12" s="2">
         <v>0</v>
@@ -1599,10 +1627,10 @@
         <v>1</v>
       </c>
       <c r="P13" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q13" s="2">
         <v>3</v>
-      </c>
-      <c r="Q13" s="2">
-        <v>2</v>
       </c>
       <c r="R13" s="2">
         <v>0</v>
@@ -1660,10 +1688,10 @@
         <v>5</v>
       </c>
       <c r="P14" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q14" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R14" s="2">
         <v>3</v>
@@ -1721,10 +1749,10 @@
         <v>0</v>
       </c>
       <c r="P15" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q15" s="2">
         <v>0</v>
-      </c>
-      <c r="Q15" s="2">
-        <v>1</v>
       </c>
       <c r="R15" s="2">
         <v>3</v>
@@ -1795,64 +1823,125 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B17" s="2">
+        <v>720</v>
+      </c>
+      <c r="C17" s="2">
+        <v>482</v>
+      </c>
+      <c r="D17" s="2">
+        <v>36</v>
+      </c>
+      <c r="E17" s="2">
+        <v>56</v>
+      </c>
+      <c r="F17" s="2">
+        <v>46</v>
+      </c>
+      <c r="G17" s="2">
+        <v>23</v>
+      </c>
+      <c r="H17" s="2">
+        <v>19</v>
+      </c>
+      <c r="I17" s="2">
+        <v>14</v>
+      </c>
+      <c r="J17" s="2">
+        <v>3</v>
+      </c>
+      <c r="K17" s="2">
+        <v>17</v>
+      </c>
+      <c r="L17" s="2">
+        <v>1</v>
+      </c>
+      <c r="M17" s="2">
+        <v>4</v>
+      </c>
+      <c r="N17" s="2">
+        <v>12</v>
+      </c>
+      <c r="O17" s="2">
+        <v>1</v>
+      </c>
+      <c r="P17" s="2">
+        <v>4</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>0</v>
+      </c>
+      <c r="R17" s="2">
+        <v>1</v>
+      </c>
+      <c r="S17" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B17" s="5">
-        <v>12038</v>
-      </c>
-      <c r="C17" s="5">
-        <v>7841</v>
-      </c>
-      <c r="D17" s="5">
-        <v>1285</v>
-      </c>
-      <c r="E17" s="5">
-        <v>743</v>
-      </c>
-      <c r="F17" s="5">
-        <v>569</v>
-      </c>
-      <c r="G17" s="5">
-        <v>462</v>
-      </c>
-      <c r="H17" s="5">
-        <v>281</v>
-      </c>
-      <c r="I17" s="5">
-        <v>237</v>
-      </c>
-      <c r="J17" s="5">
-        <v>178</v>
-      </c>
-      <c r="K17" s="5">
-        <v>140</v>
-      </c>
-      <c r="L17" s="5">
-        <v>89</v>
-      </c>
-      <c r="M17" s="5">
-        <v>59</v>
-      </c>
-      <c r="N17" s="5">
-        <v>50</v>
-      </c>
-      <c r="O17" s="5">
-        <v>39</v>
-      </c>
-      <c r="P17" s="5">
+      <c r="B18" s="5">
+        <v>12758</v>
+      </c>
+      <c r="C18" s="5">
+        <v>8323</v>
+      </c>
+      <c r="D18" s="5">
+        <v>1321</v>
+      </c>
+      <c r="E18" s="5">
+        <v>799</v>
+      </c>
+      <c r="F18" s="5">
+        <v>615</v>
+      </c>
+      <c r="G18" s="5">
+        <v>485</v>
+      </c>
+      <c r="H18" s="5">
+        <v>300</v>
+      </c>
+      <c r="I18" s="5">
+        <v>251</v>
+      </c>
+      <c r="J18" s="5">
+        <v>181</v>
+      </c>
+      <c r="K18" s="5">
+        <v>157</v>
+      </c>
+      <c r="L18" s="5">
+        <v>90</v>
+      </c>
+      <c r="M18" s="5">
+        <v>63</v>
+      </c>
+      <c r="N18" s="5">
+        <v>62</v>
+      </c>
+      <c r="O18" s="5">
+        <v>40</v>
+      </c>
+      <c r="P18" s="5">
+        <v>24</v>
+      </c>
+      <c r="Q18" s="5">
         <v>22</v>
       </c>
-      <c r="Q17" s="5">
-        <v>20</v>
-      </c>
-      <c r="R17" s="5">
-        <v>16</v>
-      </c>
-      <c r="S17" s="5">
-        <v>7</v>
+      <c r="R18" s="5">
+        <v>17</v>
+      </c>
+      <c r="S18" s="5">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -9092,6 +9181,540 @@
       </c>
       <c r="H230" s="4"/>
     </row>
+    <row r="231">
+      <c r="A231" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B231" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C231" s="0" t="inlineStr">
+        <is>
+          <t>birth</t>
+        </is>
+      </c>
+      <c r="D231" s="2">
+        <v>352</v>
+      </c>
+      <c r="E231" s="2">
+        <v>130</v>
+      </c>
+      <c r="F231" s="2">
+        <v>482</v>
+      </c>
+      <c r="G231" s="3">
+        <v>0.6694444444444444</v>
+      </c>
+      <c r="H231" s="2">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B232" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C232" s="0" t="inlineStr">
+        <is>
+          <t>anniv</t>
+        </is>
+      </c>
+      <c r="D232" s="2">
+        <v>43</v>
+      </c>
+      <c r="E232" s="2">
+        <v>13</v>
+      </c>
+      <c r="F232" s="2">
+        <v>56</v>
+      </c>
+      <c r="G232" s="3">
+        <v>0.07777777777777778</v>
+      </c>
+      <c r="H232" s="2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B233" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C233" s="0" t="inlineStr">
+        <is>
+          <t>gen</t>
+        </is>
+      </c>
+      <c r="D233" s="2">
+        <v>34</v>
+      </c>
+      <c r="E233" s="2">
+        <v>12</v>
+      </c>
+      <c r="F233" s="2">
+        <v>46</v>
+      </c>
+      <c r="G233" s="3">
+        <v>0.06388888888888888</v>
+      </c>
+      <c r="H233" s="2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B234" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C234" s="0" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="D234" s="2">
+        <v>24</v>
+      </c>
+      <c r="E234" s="2">
+        <v>12</v>
+      </c>
+      <c r="F234" s="2">
+        <v>36</v>
+      </c>
+      <c r="G234" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="H234" s="2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B235" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C235" s="0" t="inlineStr">
+        <is>
+          <t>thank</t>
+        </is>
+      </c>
+      <c r="D235" s="2">
+        <v>6</v>
+      </c>
+      <c r="E235" s="2">
+        <v>17</v>
+      </c>
+      <c r="F235" s="2">
+        <v>23</v>
+      </c>
+      <c r="G235" s="3">
+        <v>0.03194444444444444</v>
+      </c>
+      <c r="H235" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B236" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C236" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D236" s="2">
+        <v>15</v>
+      </c>
+      <c r="E236" s="2">
+        <v>4</v>
+      </c>
+      <c r="F236" s="2">
+        <v>19</v>
+      </c>
+      <c r="G236" s="3">
+        <v>0.02638888888888889</v>
+      </c>
+      <c r="H236" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B237" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C237" s="0" t="inlineStr">
+        <is>
+          <t>congrats</t>
+        </is>
+      </c>
+      <c r="D237" s="2">
+        <v>12</v>
+      </c>
+      <c r="E237" s="2">
+        <v>5</v>
+      </c>
+      <c r="F237" s="2">
+        <v>17</v>
+      </c>
+      <c r="G237" s="3">
+        <v>0.02361111111111111</v>
+      </c>
+      <c r="H237" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B238" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C238" s="0" t="inlineStr">
+        <is>
+          <t>insp</t>
+        </is>
+      </c>
+      <c r="D238" s="2">
+        <v>12</v>
+      </c>
+      <c r="E238" s="2">
+        <v>2</v>
+      </c>
+      <c r="F238" s="2">
+        <v>14</v>
+      </c>
+      <c r="G238" s="3">
+        <v>0.019444444444444445</v>
+      </c>
+      <c r="H238" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B239" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C239" s="0" t="inlineStr">
+        <is>
+          <t>cute</t>
+        </is>
+      </c>
+      <c r="D239" s="2">
+        <v>12</v>
+      </c>
+      <c r="E239" s="2">
+        <v>0</v>
+      </c>
+      <c r="F239" s="2">
+        <v>12</v>
+      </c>
+      <c r="G239" s="3">
+        <v>0.016666666666666666</v>
+      </c>
+      <c r="H239" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B240" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C240" s="0" t="inlineStr">
+        <is>
+          <t>fkt</t>
+        </is>
+      </c>
+      <c r="D240" s="2">
+        <v>2</v>
+      </c>
+      <c r="E240" s="2">
+        <v>2</v>
+      </c>
+      <c r="F240" s="2">
+        <v>4</v>
+      </c>
+      <c r="G240" s="3">
+        <v>0.005555555555555556</v>
+      </c>
+      <c r="H240" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B241" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C241" s="0" t="inlineStr">
+        <is>
+          <t>intouch</t>
+        </is>
+      </c>
+      <c r="D241" s="2">
+        <v>2</v>
+      </c>
+      <c r="E241" s="2">
+        <v>2</v>
+      </c>
+      <c r="F241" s="2">
+        <v>4</v>
+      </c>
+      <c r="G241" s="3">
+        <v>0.005555555555555556</v>
+      </c>
+      <c r="H241" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B242" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C242" s="0" t="inlineStr">
+        <is>
+          <t>friend</t>
+        </is>
+      </c>
+      <c r="D242" s="2">
+        <v>2</v>
+      </c>
+      <c r="E242" s="2">
+        <v>1</v>
+      </c>
+      <c r="F242" s="2">
+        <v>3</v>
+      </c>
+      <c r="G242" s="3">
+        <v>0.004166666666666667</v>
+      </c>
+      <c r="H242" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B243" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C243" s="0" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+      <c r="D243" s="2">
+        <v>0</v>
+      </c>
+      <c r="E243" s="2">
+        <v>1</v>
+      </c>
+      <c r="F243" s="2">
+        <v>1</v>
+      </c>
+      <c r="G243" s="3">
+        <v>0.001388888888888889</v>
+      </c>
+      <c r="H243" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B244" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C244" s="0" t="inlineStr">
+        <is>
+          <t>flwr</t>
+        </is>
+      </c>
+      <c r="D244" s="2">
+        <v>1</v>
+      </c>
+      <c r="E244" s="2">
+        <v>0</v>
+      </c>
+      <c r="F244" s="2">
+        <v>1</v>
+      </c>
+      <c r="G244" s="3">
+        <v>0.001388888888888889</v>
+      </c>
+      <c r="H244" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B245" s="0" t="inlineStr">
+        <is>
+          <t>Invitations &amp; parties</t>
+        </is>
+      </c>
+      <c r="C245" s="0" t="inlineStr">
+        <is>
+          <t>invp</t>
+        </is>
+      </c>
+      <c r="D245" s="2">
+        <v>0</v>
+      </c>
+      <c r="E245" s="2">
+        <v>1</v>
+      </c>
+      <c r="F245" s="2">
+        <v>1</v>
+      </c>
+      <c r="G245" s="3">
+        <v>0.001388888888888889</v>
+      </c>
+      <c r="H245" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B246" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C246" s="0" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="D246" s="2">
+        <v>1</v>
+      </c>
+      <c r="E246" s="2">
+        <v>0</v>
+      </c>
+      <c r="F246" s="2">
+        <v>1</v>
+      </c>
+      <c r="G246" s="3">
+        <v>0.001388888888888889</v>
+      </c>
+      <c r="H246" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-16</t>
+        </is>
+      </c>
+      <c r="B247" s="4"/>
+      <c r="C247" s="4"/>
+      <c r="D247" s="5">
+        <v>518</v>
+      </c>
+      <c r="E247" s="5">
+        <v>202</v>
+      </c>
+      <c r="F247" s="5">
+        <v>720</v>
+      </c>
+      <c r="G247" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="H247" s="4"/>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -44320,6 +44943,2540 @@
         <v>797</v>
       </c>
       <c r="F1265" s="4"/>
+    </row>
+    <row r="1266">
+      <c r="A1266" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1266" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1266" s="0" t="inlineStr">
+        <is>
+          <t>happybirthday</t>
+        </is>
+      </c>
+      <c r="D1266" s="0" t="inlineStr">
+        <is>
+          <t>birth_happybirthday</t>
+        </is>
+      </c>
+      <c r="E1266" s="2">
+        <v>367</v>
+      </c>
+      <c r="F1266" s="2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1267" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1267" s="0" t="inlineStr">
+        <is>
+          <t>anniversaryetc</t>
+        </is>
+      </c>
+      <c r="D1267" s="0" t="inlineStr">
+        <is>
+          <t>anniv_anniversaryetc</t>
+        </is>
+      </c>
+      <c r="E1267" s="2">
+        <v>38</v>
+      </c>
+      <c r="F1267" s="2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1268" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1268" s="0" t="inlineStr">
+        <is>
+          <t>fun</t>
+        </is>
+      </c>
+      <c r="D1268" s="0" t="inlineStr">
+        <is>
+          <t>birth_fun</t>
+        </is>
+      </c>
+      <c r="E1268" s="2">
+        <v>20</v>
+      </c>
+      <c r="F1268" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1269" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1269" s="0" t="inlineStr">
+        <is>
+          <t>blessings</t>
+        </is>
+      </c>
+      <c r="D1269" s="0" t="inlineStr">
+        <is>
+          <t>birth_blessings</t>
+        </is>
+      </c>
+      <c r="E1269" s="2">
+        <v>13</v>
+      </c>
+      <c r="F1269" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1270" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1270" s="0" t="inlineStr">
+        <is>
+          <t>sonanddaughter</t>
+        </is>
+      </c>
+      <c r="D1270" s="0" t="inlineStr">
+        <is>
+          <t>birth_sonanddaughter</t>
+        </is>
+      </c>
+      <c r="E1270" s="2">
+        <v>12</v>
+      </c>
+      <c r="F1270" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1271" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1271" s="0" t="inlineStr">
+        <is>
+          <t>birthday</t>
+        </is>
+      </c>
+      <c r="D1271" s="0" t="inlineStr">
+        <is>
+          <t>thank_birthday</t>
+        </is>
+      </c>
+      <c r="E1271" s="2">
+        <v>11</v>
+      </c>
+      <c r="F1271" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1272" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1272" s="0" t="inlineStr">
+        <is>
+          <t>songs</t>
+        </is>
+      </c>
+      <c r="D1272" s="0" t="inlineStr">
+        <is>
+          <t>birth_songs</t>
+        </is>
+      </c>
+      <c r="E1272" s="2">
+        <v>10</v>
+      </c>
+      <c r="F1272" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1273" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C1273" s="0" t="inlineStr">
+        <is>
+          <t>cuteetc</t>
+        </is>
+      </c>
+      <c r="D1273" s="0" t="inlineStr">
+        <is>
+          <t>cute_cuteetc</t>
+        </is>
+      </c>
+      <c r="E1273" s="2">
+        <v>10</v>
+      </c>
+      <c r="F1273" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1274" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1274" s="0" t="inlineStr">
+        <is>
+          <t>belated</t>
+        </is>
+      </c>
+      <c r="D1274" s="0" t="inlineStr">
+        <is>
+          <t>birth_belated</t>
+        </is>
+      </c>
+      <c r="E1274" s="2">
+        <v>9</v>
+      </c>
+      <c r="F1274" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1275" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1275" s="0" t="inlineStr">
+        <is>
+          <t>newbaby</t>
+        </is>
+      </c>
+      <c r="D1275" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newbaby</t>
+        </is>
+      </c>
+      <c r="E1275" s="2">
+        <v>9</v>
+      </c>
+      <c r="F1275" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1276" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1276" s="0" t="inlineStr">
+        <is>
+          <t>morning</t>
+        </is>
+      </c>
+      <c r="D1276" s="0" t="inlineStr">
+        <is>
+          <t>gen_morning</t>
+        </is>
+      </c>
+      <c r="E1276" s="2">
+        <v>8</v>
+      </c>
+      <c r="F1276" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1277" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1277" s="0" t="inlineStr">
+        <is>
+          <t>sympathy</t>
+        </is>
+      </c>
+      <c r="D1277" s="0" t="inlineStr">
+        <is>
+          <t>insp_sympathy</t>
+        </is>
+      </c>
+      <c r="E1277" s="2">
+        <v>8</v>
+      </c>
+      <c r="F1277" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1278" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1278" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="D1278" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="E1278" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1278" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1279" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1279" s="0" t="inlineStr">
+        <is>
+          <t>bronsis</t>
+        </is>
+      </c>
+      <c r="D1279" s="0" t="inlineStr">
+        <is>
+          <t>birth_bronsis</t>
+        </is>
+      </c>
+      <c r="E1279" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1279" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1280" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1280" s="0" t="inlineStr">
+        <is>
+          <t>hubbywife</t>
+        </is>
+      </c>
+      <c r="D1280" s="0" t="inlineStr">
+        <is>
+          <t>birth_hubbywife</t>
+        </is>
+      </c>
+      <c r="E1280" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1280" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1281" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1281" s="0" t="inlineStr">
+        <is>
+          <t>wishes</t>
+        </is>
+      </c>
+      <c r="D1281" s="0" t="inlineStr">
+        <is>
+          <t>birth_wishes</t>
+        </is>
+      </c>
+      <c r="E1281" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1281" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1282" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1282" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipweek</t>
+        </is>
+      </c>
+      <c r="D1282" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipweek</t>
+        </is>
+      </c>
+      <c r="E1282" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1282" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1283" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1283" s="0" t="inlineStr">
+        <is>
+          <t>missyou</t>
+        </is>
+      </c>
+      <c r="D1283" s="0" t="inlineStr">
+        <is>
+          <t>gen_missyou</t>
+        </is>
+      </c>
+      <c r="E1283" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1283" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1284" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1284" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="D1284" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="E1284" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1284" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1285" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1285" s="0" t="inlineStr">
+        <is>
+          <t>flowers</t>
+        </is>
+      </c>
+      <c r="D1285" s="0" t="inlineStr">
+        <is>
+          <t>birth_flowers</t>
+        </is>
+      </c>
+      <c r="E1285" s="2">
+        <v>6</v>
+      </c>
+      <c r="F1285" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1286" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1286" s="0" t="inlineStr">
+        <is>
+          <t>kids</t>
+        </is>
+      </c>
+      <c r="D1286" s="0" t="inlineStr">
+        <is>
+          <t>birth_kids</t>
+        </is>
+      </c>
+      <c r="E1286" s="2">
+        <v>6</v>
+      </c>
+      <c r="F1286" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1287" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1287" s="0" t="inlineStr">
+        <is>
+          <t>hvgtday</t>
+        </is>
+      </c>
+      <c r="D1287" s="0" t="inlineStr">
+        <is>
+          <t>gen_hvgtday</t>
+        </is>
+      </c>
+      <c r="E1287" s="2">
+        <v>6</v>
+      </c>
+      <c r="F1287" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1288" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1288" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_family</t>
+        </is>
+      </c>
+      <c r="D1288" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_family</t>
+        </is>
+      </c>
+      <c r="E1288" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1288" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1289" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1289" s="0" t="inlineStr">
+        <is>
+          <t>extfamily</t>
+        </is>
+      </c>
+      <c r="D1289" s="0" t="inlineStr">
+        <is>
+          <t>birth_extfamily</t>
+        </is>
+      </c>
+      <c r="E1289" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1289" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1290" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1290" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalrum_day</t>
+        </is>
+      </c>
+      <c r="D1290" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalrum_day</t>
+        </is>
+      </c>
+      <c r="E1290" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1290" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1291" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1291" s="0" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="D1291" s="0" t="inlineStr">
+        <is>
+          <t>gen_hi</t>
+        </is>
+      </c>
+      <c r="E1291" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1291" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1292" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1292" s="0" t="inlineStr">
+        <is>
+          <t>thinkingofyou</t>
+        </is>
+      </c>
+      <c r="D1292" s="0" t="inlineStr">
+        <is>
+          <t>gen_thinkingofyou</t>
+        </is>
+      </c>
+      <c r="E1292" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1292" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1293" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1293" s="0" t="inlineStr">
+        <is>
+          <t>sweetheart</t>
+        </is>
+      </c>
+      <c r="D1293" s="0" t="inlineStr">
+        <is>
+          <t>love_sweetheart</t>
+        </is>
+      </c>
+      <c r="E1293" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1293" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1294" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1294" s="0" t="inlineStr">
+        <is>
+          <t>everyday</t>
+        </is>
+      </c>
+      <c r="D1294" s="0" t="inlineStr">
+        <is>
+          <t>thank_everyday</t>
+        </is>
+      </c>
+      <c r="E1294" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1294" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1295" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1295" s="0" t="inlineStr">
+        <is>
+          <t>eaug_rakshabandhan_happy</t>
+        </is>
+      </c>
+      <c r="D1295" s="0" t="inlineStr">
+        <is>
+          <t>eaug_rakshabandhan_happy</t>
+        </is>
+      </c>
+      <c r="E1295" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1295" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1296" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1296" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="D1296" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="E1296" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1296" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1297" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1297" s="0" t="inlineStr">
+        <is>
+          <t>friends</t>
+        </is>
+      </c>
+      <c r="D1297" s="0" t="inlineStr">
+        <is>
+          <t>birth_friends</t>
+        </is>
+      </c>
+      <c r="E1297" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1297" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1298" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1298" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D1298" s="0" t="inlineStr">
+        <is>
+          <t>birth_milestone</t>
+        </is>
+      </c>
+      <c r="E1298" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1298" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1299" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1299" s="0" t="inlineStr">
+        <is>
+          <t>foreveryone</t>
+        </is>
+      </c>
+      <c r="D1299" s="0" t="inlineStr">
+        <is>
+          <t>congrats_foreveryone</t>
+        </is>
+      </c>
+      <c r="E1299" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1299" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1300" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1300" s="0" t="inlineStr">
+        <is>
+          <t>newcarandlicense</t>
+        </is>
+      </c>
+      <c r="D1300" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newcarandlicense</t>
+        </is>
+      </c>
+      <c r="E1300" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1300" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1301" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C1301" s="0" t="inlineStr">
+        <is>
+          <t>sisters</t>
+        </is>
+      </c>
+      <c r="D1301" s="0" t="inlineStr">
+        <is>
+          <t>fkt_sisters</t>
+        </is>
+      </c>
+      <c r="E1301" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1301" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1302" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1302" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D1302" s="0" t="inlineStr">
+        <is>
+          <t>gen_getwell</t>
+        </is>
+      </c>
+      <c r="E1302" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1302" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1303" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1303" s="0" t="inlineStr">
+        <is>
+          <t>voyage</t>
+        </is>
+      </c>
+      <c r="D1303" s="0" t="inlineStr">
+        <is>
+          <t>gen_voyage</t>
+        </is>
+      </c>
+      <c r="E1303" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1303" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1304" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1304" s="0" t="inlineStr">
+        <is>
+          <t>recovery</t>
+        </is>
+      </c>
+      <c r="D1304" s="0" t="inlineStr">
+        <is>
+          <t>insp_recovery</t>
+        </is>
+      </c>
+      <c r="E1304" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1304" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1305" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1305" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_general</t>
+        </is>
+      </c>
+      <c r="D1305" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_general</t>
+        </is>
+      </c>
+      <c r="E1305" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1305" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1306" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1306" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D1306" s="0" t="inlineStr">
+        <is>
+          <t>thank_love</t>
+        </is>
+      </c>
+      <c r="E1306" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1306" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1307" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1307" s="0" t="inlineStr">
+        <is>
+          <t>belated</t>
+        </is>
+      </c>
+      <c r="D1307" s="0" t="inlineStr">
+        <is>
+          <t>anniv_belated</t>
+        </is>
+      </c>
+      <c r="E1307" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1307" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1308" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1308" s="0" t="inlineStr">
+        <is>
+          <t>forher</t>
+        </is>
+      </c>
+      <c r="D1308" s="0" t="inlineStr">
+        <is>
+          <t>birth_forher</t>
+        </is>
+      </c>
+      <c r="E1308" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1308" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1309" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1309" s="0" t="inlineStr">
+        <is>
+          <t>forhim</t>
+        </is>
+      </c>
+      <c r="D1309" s="0" t="inlineStr">
+        <is>
+          <t>birth_forhim</t>
+        </is>
+      </c>
+      <c r="E1309" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1309" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1310" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1310" s="0" t="inlineStr">
+        <is>
+          <t>momndad</t>
+        </is>
+      </c>
+      <c r="D1310" s="0" t="inlineStr">
+        <is>
+          <t>birth_momndad</t>
+        </is>
+      </c>
+      <c r="E1310" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1310" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1311" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C1311" s="0" t="inlineStr">
+        <is>
+          <t>hugs</t>
+        </is>
+      </c>
+      <c r="D1311" s="0" t="inlineStr">
+        <is>
+          <t>cute_hugs</t>
+        </is>
+      </c>
+      <c r="E1311" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1311" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1312" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1312" s="0" t="inlineStr">
+        <is>
+          <t>eaug_zorastriannewyear</t>
+        </is>
+      </c>
+      <c r="D1312" s="0" t="inlineStr">
+        <is>
+          <t>eaug_zorastriannewyear</t>
+        </is>
+      </c>
+      <c r="E1312" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1312" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1313" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1313" s="0" t="inlineStr">
+        <is>
+          <t>ejun_internationalchildrens_day</t>
+        </is>
+      </c>
+      <c r="D1313" s="0" t="inlineStr">
+        <is>
+          <t>ejun_internationalchildrens_day</t>
+        </is>
+      </c>
+      <c r="E1313" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1313" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1314" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1314" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_thank</t>
+        </is>
+      </c>
+      <c r="D1314" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_thank</t>
+        </is>
+      </c>
+      <c r="E1314" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1314" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1315" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1315" s="0" t="inlineStr">
+        <is>
+          <t>emar_rollercoaster_day</t>
+        </is>
+      </c>
+      <c r="D1315" s="0" t="inlineStr">
+        <is>
+          <t>emar_rollercoaster_day</t>
+        </is>
+      </c>
+      <c r="E1315" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1315" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1316" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1316" s="0" t="inlineStr">
+        <is>
+          <t>esep_trueloveforeverday</t>
+        </is>
+      </c>
+      <c r="D1316" s="0" t="inlineStr">
+        <is>
+          <t>esep_trueloveforeverday</t>
+        </is>
+      </c>
+      <c r="E1316" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1316" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1317" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C1317" s="0" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="D1317" s="0" t="inlineStr">
+        <is>
+          <t>friend_hello</t>
+        </is>
+      </c>
+      <c r="E1317" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1317" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1318" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1318" s="0" t="inlineStr">
+        <is>
+          <t>goodnight</t>
+        </is>
+      </c>
+      <c r="D1318" s="0" t="inlineStr">
+        <is>
+          <t>gen_goodnight</t>
+        </is>
+      </c>
+      <c r="E1318" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1318" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1319" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1319" s="0" t="inlineStr">
+        <is>
+          <t>quotesmessages_images_getwell_messages</t>
+        </is>
+      </c>
+      <c r="D1319" s="0" t="inlineStr">
+        <is>
+          <t>gen_quotesmessages_images_getwell_messages</t>
+        </is>
+      </c>
+      <c r="E1319" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1319" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1320" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1320" s="0" t="inlineStr">
+        <is>
+          <t>quotesmessages_images_thankyou_quotes</t>
+        </is>
+      </c>
+      <c r="D1320" s="0" t="inlineStr">
+        <is>
+          <t>gen_quotesmessages_images_thankyou_quotes</t>
+        </is>
+      </c>
+      <c r="E1320" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1320" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1321" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1321" s="0" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="D1321" s="0" t="inlineStr">
+        <is>
+          <t>insp_health</t>
+        </is>
+      </c>
+      <c r="E1321" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1321" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1322" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C1322" s="0" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="D1322" s="0" t="inlineStr">
+        <is>
+          <t>intouch_hi</t>
+        </is>
+      </c>
+      <c r="E1322" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1322" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1323" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1323" s="0" t="inlineStr">
+        <is>
+          <t>wedding</t>
+        </is>
+      </c>
+      <c r="D1323" s="0" t="inlineStr">
+        <is>
+          <t>thank_wedding</t>
+        </is>
+      </c>
+      <c r="E1323" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1323" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1324" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1324" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="D1324" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="E1324" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1324" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1325" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1325" s="0" t="inlineStr">
+        <is>
+          <t>pets</t>
+        </is>
+      </c>
+      <c r="D1325" s="0" t="inlineStr">
+        <is>
+          <t>birth_pets</t>
+        </is>
+      </c>
+      <c r="E1325" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1325" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1326" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C1326" s="0" t="inlineStr">
+        <is>
+          <t>accolades</t>
+        </is>
+      </c>
+      <c r="D1326" s="0" t="inlineStr">
+        <is>
+          <t>bus_accolades</t>
+        </is>
+      </c>
+      <c r="E1326" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1326" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1327" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1327" s="0" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="D1327" s="0" t="inlineStr">
+        <is>
+          <t>congrats_engagement</t>
+        </is>
+      </c>
+      <c r="E1327" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1327" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1328" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1328" s="0" t="inlineStr">
+        <is>
+          <t>newjob</t>
+        </is>
+      </c>
+      <c r="D1328" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newjob</t>
+        </is>
+      </c>
+      <c r="E1328" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1328" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1329" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1329" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="D1329" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="E1329" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1329" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1330" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1330" s="0" t="inlineStr">
+        <is>
+          <t>eaug_indindependenceday</t>
+        </is>
+      </c>
+      <c r="D1330" s="0" t="inlineStr">
+        <is>
+          <t>eaug_indindependenceday</t>
+        </is>
+      </c>
+      <c r="E1330" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1330" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1331" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1331" s="0" t="inlineStr">
+        <is>
+          <t>eaug_jokeday</t>
+        </is>
+      </c>
+      <c r="D1331" s="0" t="inlineStr">
+        <is>
+          <t>eaug_jokeday</t>
+        </is>
+      </c>
+      <c r="E1331" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1331" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1332" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1332" s="0" t="inlineStr">
+        <is>
+          <t>eaug_thankyouday</t>
+        </is>
+      </c>
+      <c r="D1332" s="0" t="inlineStr">
+        <is>
+          <t>eaug_thankyouday</t>
+        </is>
+      </c>
+      <c r="E1332" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1332" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1333" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1333" s="0" t="inlineStr">
+        <is>
+          <t>eaug_vanillacustard_day</t>
+        </is>
+      </c>
+      <c r="D1333" s="0" t="inlineStr">
+        <is>
+          <t>eaug_vanillacustard_day</t>
+        </is>
+      </c>
+      <c r="E1333" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1333" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1334" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1334" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_love</t>
+        </is>
+      </c>
+      <c r="D1334" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_love</t>
+        </is>
+      </c>
+      <c r="E1334" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1334" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1335" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1335" s="0" t="inlineStr">
+        <is>
+          <t>eoct_sweetday_thanku</t>
+        </is>
+      </c>
+      <c r="D1335" s="0" t="inlineStr">
+        <is>
+          <t>eoct_sweetday_thanku</t>
+        </is>
+      </c>
+      <c r="E1335" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1335" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1336" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1336" s="0" t="inlineStr">
+        <is>
+          <t>esep_nationalcoffee_day</t>
+        </is>
+      </c>
+      <c r="D1336" s="0" t="inlineStr">
+        <is>
+          <t>esep_nationalcoffee_day</t>
+        </is>
+      </c>
+      <c r="E1336" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1336" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1337" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C1337" s="0" t="inlineStr">
+        <is>
+          <t>huswife</t>
+        </is>
+      </c>
+      <c r="D1337" s="0" t="inlineStr">
+        <is>
+          <t>fkt_huswife</t>
+        </is>
+      </c>
+      <c r="E1337" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1337" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1338" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C1338" s="0" t="inlineStr">
+        <is>
+          <t>youcare</t>
+        </is>
+      </c>
+      <c r="D1338" s="0" t="inlineStr">
+        <is>
+          <t>flwr_youcare</t>
+        </is>
+      </c>
+      <c r="E1338" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1338" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1339" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C1339" s="0" t="inlineStr">
+        <is>
+          <t>bestfriends</t>
+        </is>
+      </c>
+      <c r="D1339" s="0" t="inlineStr">
+        <is>
+          <t>friend_bestfriends</t>
+        </is>
+      </c>
+      <c r="E1339" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1339" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1340" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1340" s="0" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="D1340" s="0" t="inlineStr">
+        <is>
+          <t>gen_luck</t>
+        </is>
+      </c>
+      <c r="E1340" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1340" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1341" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1341" s="0" t="inlineStr">
+        <is>
+          <t>morningquotes</t>
+        </is>
+      </c>
+      <c r="D1341" s="0" t="inlineStr">
+        <is>
+          <t>gen_morningquotes</t>
+        </is>
+      </c>
+      <c r="E1341" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1341" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1342" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1342" s="0" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="D1342" s="0" t="inlineStr">
+        <is>
+          <t>gen_weekend</t>
+        </is>
+      </c>
+      <c r="E1342" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1342" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1343" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1343" s="0" t="inlineStr">
+        <is>
+          <t>encour</t>
+        </is>
+      </c>
+      <c r="D1343" s="0" t="inlineStr">
+        <is>
+          <t>insp_encour</t>
+        </is>
+      </c>
+      <c r="E1343" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1343" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1344" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C1344" s="0" t="inlineStr">
+        <is>
+          <t>missingyou</t>
+        </is>
+      </c>
+      <c r="D1344" s="0" t="inlineStr">
+        <is>
+          <t>intouch_missingyou</t>
+        </is>
+      </c>
+      <c r="E1344" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1344" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1345" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C1345" s="0" t="inlineStr">
+        <is>
+          <t>sendsmile</t>
+        </is>
+      </c>
+      <c r="D1345" s="0" t="inlineStr">
+        <is>
+          <t>intouch_sendsmile</t>
+        </is>
+      </c>
+      <c r="E1345" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1345" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1346" s="0" t="inlineStr">
+        <is>
+          <t>Invitations &amp; parties</t>
+        </is>
+      </c>
+      <c r="C1346" s="0" t="inlineStr">
+        <is>
+          <t>otherinvitations</t>
+        </is>
+      </c>
+      <c r="D1346" s="0" t="inlineStr">
+        <is>
+          <t>invp_otherinvitations</t>
+        </is>
+      </c>
+      <c r="E1346" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1346" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1347" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1347" s="0" t="inlineStr">
+        <is>
+          <t>foreverlove</t>
+        </is>
+      </c>
+      <c r="D1347" s="0" t="inlineStr">
+        <is>
+          <t>love_foreverlove</t>
+        </is>
+      </c>
+      <c r="E1347" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1347" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1348" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1348" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="D1348" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="E1348" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1348" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1349" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1349" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_kisses</t>
+        </is>
+      </c>
+      <c r="D1349" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_kisses</t>
+        </is>
+      </c>
+      <c r="E1349" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1349" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1350" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1350" s="0" t="inlineStr">
+        <is>
+          <t>youarespecial</t>
+        </is>
+      </c>
+      <c r="D1350" s="0" t="inlineStr">
+        <is>
+          <t>love_youarespecial</t>
+        </is>
+      </c>
+      <c r="E1350" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1350" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1351" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C1351" s="0" t="inlineStr">
+        <is>
+          <t>lossofpet</t>
+        </is>
+      </c>
+      <c r="D1351" s="0" t="inlineStr">
+        <is>
+          <t>pet_lossofpet</t>
+        </is>
+      </c>
+      <c r="E1351" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1351" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1352" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1352" s="0" t="inlineStr">
+        <is>
+          <t>congratulations</t>
+        </is>
+      </c>
+      <c r="D1352" s="0" t="inlineStr">
+        <is>
+          <t>thank_congratulations</t>
+        </is>
+      </c>
+      <c r="E1352" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1352" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1353" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1353" s="0" t="inlineStr">
+        <is>
+          <t>friendship</t>
+        </is>
+      </c>
+      <c r="D1353" s="0" t="inlineStr">
+        <is>
+          <t>thank_friendship</t>
+        </is>
+      </c>
+      <c r="E1353" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1353" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1354" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1354" s="0" t="inlineStr">
+        <is>
+          <t>wed_wed_congrats</t>
+        </is>
+      </c>
+      <c r="D1354" s="0" t="inlineStr">
+        <is>
+          <t>wed_wed_congrats</t>
+        </is>
+      </c>
+      <c r="E1354" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1354" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1355" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1355" s="0" t="inlineStr">
+        <is>
+          <t>wed_wishes</t>
+        </is>
+      </c>
+      <c r="D1355" s="0" t="inlineStr">
+        <is>
+          <t>wed_wishes</t>
+        </is>
+      </c>
+      <c r="E1355" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1355" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-16</t>
+        </is>
+      </c>
+      <c r="B1356" s="4"/>
+      <c r="C1356" s="4"/>
+      <c r="D1356" s="4"/>
+      <c r="E1356" s="5">
+        <v>720</v>
+      </c>
+      <c r="F1356" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -44903,36 +48060,70 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B17" s="2">
+        <v>761</v>
+      </c>
+      <c r="C17" s="2">
+        <v>267</v>
+      </c>
+      <c r="D17" s="2">
+        <v>207</v>
+      </c>
+      <c r="E17" s="2">
+        <v>150</v>
+      </c>
+      <c r="F17" s="2">
+        <v>76</v>
+      </c>
+      <c r="G17" s="2">
+        <v>41</v>
+      </c>
+      <c r="H17" s="2">
+        <v>20</v>
+      </c>
+      <c r="I17" s="2">
+        <v>0</v>
+      </c>
+      <c r="J17" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B17" s="5">
-        <v>12518</v>
-      </c>
-      <c r="C17" s="5">
-        <v>3922</v>
-      </c>
-      <c r="D17" s="5">
-        <v>3922</v>
-      </c>
-      <c r="E17" s="5">
-        <v>2522</v>
-      </c>
-      <c r="F17" s="5">
-        <v>1251</v>
-      </c>
-      <c r="G17" s="5">
-        <v>476</v>
-      </c>
-      <c r="H17" s="5">
-        <v>396</v>
-      </c>
-      <c r="I17" s="5">
+      <c r="B18" s="5">
+        <v>13279</v>
+      </c>
+      <c r="C18" s="5">
+        <v>4189</v>
+      </c>
+      <c r="D18" s="5">
+        <v>4129</v>
+      </c>
+      <c r="E18" s="5">
+        <v>2672</v>
+      </c>
+      <c r="F18" s="5">
+        <v>1327</v>
+      </c>
+      <c r="G18" s="5">
+        <v>517</v>
+      </c>
+      <c r="H18" s="5">
+        <v>416</v>
+      </c>
+      <c r="I18" s="5">
         <v>28</v>
       </c>
-      <c r="J17" s="5">
+      <c r="J18" s="5">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Record 18 August: eighteen days, 14,795 sends tracked
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9KsXegBwxB1sWdCzRVLrr
</commit_message>
<xml_diff>
--- a/reports/daily_tracking.xlsx
+++ b/reports/daily_tracking.xlsx
@@ -224,7 +224,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13">
@@ -247,7 +247,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
@@ -787,28 +787,56 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B19" s="2">
+        <v>822</v>
+      </c>
+      <c r="C19" s="2">
+        <v>520</v>
+      </c>
+      <c r="D19" s="2">
+        <v>302</v>
+      </c>
+      <c r="E19" s="2">
+        <v>771</v>
+      </c>
+      <c r="F19" s="2">
+        <v>51</v>
+      </c>
+      <c r="G19" s="2">
+        <v>264</v>
+      </c>
+      <c r="H19" s="2">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B19" s="5">
-        <v>13973</v>
-      </c>
-      <c r="C19" s="5">
-        <v>9311</v>
-      </c>
-      <c r="D19" s="5">
-        <v>4662</v>
-      </c>
-      <c r="E19" s="5">
-        <v>13426</v>
-      </c>
-      <c r="F19" s="5">
-        <v>547</v>
-      </c>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
+      <c r="B20" s="5">
+        <v>14795</v>
+      </c>
+      <c r="C20" s="5">
+        <v>9831</v>
+      </c>
+      <c r="D20" s="5">
+        <v>4964</v>
+      </c>
+      <c r="E20" s="5">
+        <v>14197</v>
+      </c>
+      <c r="F20" s="5">
+        <v>598</v>
+      </c>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -1973,64 +2001,125 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B19" s="2">
+        <v>771</v>
+      </c>
+      <c r="C19" s="2">
+        <v>523</v>
+      </c>
+      <c r="D19" s="2">
+        <v>38</v>
+      </c>
+      <c r="E19" s="2">
+        <v>63</v>
+      </c>
+      <c r="F19" s="2">
+        <v>44</v>
+      </c>
+      <c r="G19" s="2">
+        <v>23</v>
+      </c>
+      <c r="H19" s="2">
+        <v>20</v>
+      </c>
+      <c r="I19" s="2">
+        <v>20</v>
+      </c>
+      <c r="J19" s="2">
+        <v>1</v>
+      </c>
+      <c r="K19" s="2">
+        <v>13</v>
+      </c>
+      <c r="L19" s="2">
+        <v>5</v>
+      </c>
+      <c r="M19" s="2">
+        <v>6</v>
+      </c>
+      <c r="N19" s="2">
+        <v>6</v>
+      </c>
+      <c r="O19" s="2">
+        <v>2</v>
+      </c>
+      <c r="P19" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q19" s="2">
+        <v>1</v>
+      </c>
+      <c r="R19" s="2">
+        <v>1</v>
+      </c>
+      <c r="S19" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B19" s="5">
-        <v>13426</v>
-      </c>
-      <c r="C19" s="5">
-        <v>8742</v>
-      </c>
-      <c r="D19" s="5">
-        <v>1365</v>
-      </c>
-      <c r="E19" s="5">
-        <v>837</v>
-      </c>
-      <c r="F19" s="5">
-        <v>680</v>
-      </c>
-      <c r="G19" s="5">
-        <v>502</v>
-      </c>
-      <c r="H19" s="5">
-        <v>323</v>
-      </c>
-      <c r="I19" s="5">
-        <v>264</v>
-      </c>
-      <c r="J19" s="5">
-        <v>194</v>
-      </c>
-      <c r="K19" s="5">
-        <v>174</v>
-      </c>
-      <c r="L19" s="5">
-        <v>97</v>
-      </c>
-      <c r="M19" s="5">
-        <v>70</v>
-      </c>
-      <c r="N19" s="5">
-        <v>66</v>
-      </c>
-      <c r="O19" s="5">
-        <v>40</v>
-      </c>
-      <c r="P19" s="5">
-        <v>24</v>
-      </c>
-      <c r="Q19" s="5">
-        <v>22</v>
-      </c>
-      <c r="R19" s="5">
-        <v>17</v>
-      </c>
-      <c r="S19" s="5">
-        <v>9</v>
+      <c r="B20" s="5">
+        <v>14197</v>
+      </c>
+      <c r="C20" s="5">
+        <v>9265</v>
+      </c>
+      <c r="D20" s="5">
+        <v>1403</v>
+      </c>
+      <c r="E20" s="5">
+        <v>900</v>
+      </c>
+      <c r="F20" s="5">
+        <v>724</v>
+      </c>
+      <c r="G20" s="5">
+        <v>525</v>
+      </c>
+      <c r="H20" s="5">
+        <v>343</v>
+      </c>
+      <c r="I20" s="5">
+        <v>284</v>
+      </c>
+      <c r="J20" s="5">
+        <v>195</v>
+      </c>
+      <c r="K20" s="5">
+        <v>187</v>
+      </c>
+      <c r="L20" s="5">
+        <v>102</v>
+      </c>
+      <c r="M20" s="5">
+        <v>76</v>
+      </c>
+      <c r="N20" s="5">
+        <v>72</v>
+      </c>
+      <c r="O20" s="5">
+        <v>42</v>
+      </c>
+      <c r="P20" s="5">
+        <v>26</v>
+      </c>
+      <c r="Q20" s="5">
+        <v>23</v>
+      </c>
+      <c r="R20" s="5">
+        <v>18</v>
+      </c>
+      <c r="S20" s="5">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -10242,6 +10331,572 @@
       </c>
       <c r="H261" s="4"/>
     </row>
+    <row r="262">
+      <c r="A262" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B262" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C262" s="0" t="inlineStr">
+        <is>
+          <t>birth</t>
+        </is>
+      </c>
+      <c r="D262" s="2">
+        <v>359</v>
+      </c>
+      <c r="E262" s="2">
+        <v>164</v>
+      </c>
+      <c r="F262" s="2">
+        <v>523</v>
+      </c>
+      <c r="G262" s="3">
+        <v>0.6783398184176395</v>
+      </c>
+      <c r="H262" s="2">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B263" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C263" s="0" t="inlineStr">
+        <is>
+          <t>anniv</t>
+        </is>
+      </c>
+      <c r="D263" s="2">
+        <v>34</v>
+      </c>
+      <c r="E263" s="2">
+        <v>29</v>
+      </c>
+      <c r="F263" s="2">
+        <v>63</v>
+      </c>
+      <c r="G263" s="3">
+        <v>0.08171206225680934</v>
+      </c>
+      <c r="H263" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B264" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C264" s="0" t="inlineStr">
+        <is>
+          <t>gen</t>
+        </is>
+      </c>
+      <c r="D264" s="2">
+        <v>29</v>
+      </c>
+      <c r="E264" s="2">
+        <v>15</v>
+      </c>
+      <c r="F264" s="2">
+        <v>44</v>
+      </c>
+      <c r="G264" s="3">
+        <v>0.057068741893644616</v>
+      </c>
+      <c r="H264" s="2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B265" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C265" s="0" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="D265" s="2">
+        <v>28</v>
+      </c>
+      <c r="E265" s="2">
+        <v>10</v>
+      </c>
+      <c r="F265" s="2">
+        <v>38</v>
+      </c>
+      <c r="G265" s="3">
+        <v>0.04928664072632944</v>
+      </c>
+      <c r="H265" s="2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B266" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C266" s="0" t="inlineStr">
+        <is>
+          <t>thank</t>
+        </is>
+      </c>
+      <c r="D266" s="2">
+        <v>5</v>
+      </c>
+      <c r="E266" s="2">
+        <v>18</v>
+      </c>
+      <c r="F266" s="2">
+        <v>23</v>
+      </c>
+      <c r="G266" s="3">
+        <v>0.029831387808041506</v>
+      </c>
+      <c r="H266" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B267" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C267" s="0" t="inlineStr">
+        <is>
+          <t>insp</t>
+        </is>
+      </c>
+      <c r="D267" s="2">
+        <v>15</v>
+      </c>
+      <c r="E267" s="2">
+        <v>5</v>
+      </c>
+      <c r="F267" s="2">
+        <v>20</v>
+      </c>
+      <c r="G267" s="3">
+        <v>0.02594033722438392</v>
+      </c>
+      <c r="H267" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B268" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C268" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D268" s="2">
+        <v>12</v>
+      </c>
+      <c r="E268" s="2">
+        <v>8</v>
+      </c>
+      <c r="F268" s="2">
+        <v>20</v>
+      </c>
+      <c r="G268" s="3">
+        <v>0.02594033722438392</v>
+      </c>
+      <c r="H268" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B269" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C269" s="0" t="inlineStr">
+        <is>
+          <t>congrats</t>
+        </is>
+      </c>
+      <c r="D269" s="2">
+        <v>13</v>
+      </c>
+      <c r="E269" s="2">
+        <v>0</v>
+      </c>
+      <c r="F269" s="2">
+        <v>13</v>
+      </c>
+      <c r="G269" s="3">
+        <v>0.016861219195849545</v>
+      </c>
+      <c r="H269" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B270" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C270" s="0" t="inlineStr">
+        <is>
+          <t>cute</t>
+        </is>
+      </c>
+      <c r="D270" s="2">
+        <v>6</v>
+      </c>
+      <c r="E270" s="2">
+        <v>0</v>
+      </c>
+      <c r="F270" s="2">
+        <v>6</v>
+      </c>
+      <c r="G270" s="3">
+        <v>0.007782101167315175</v>
+      </c>
+      <c r="H270" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B271" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C271" s="0" t="inlineStr">
+        <is>
+          <t>fkt</t>
+        </is>
+      </c>
+      <c r="D271" s="2">
+        <v>6</v>
+      </c>
+      <c r="E271" s="2">
+        <v>0</v>
+      </c>
+      <c r="F271" s="2">
+        <v>6</v>
+      </c>
+      <c r="G271" s="3">
+        <v>0.007782101167315175</v>
+      </c>
+      <c r="H271" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B272" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C272" s="0" t="inlineStr">
+        <is>
+          <t>flwr</t>
+        </is>
+      </c>
+      <c r="D272" s="2">
+        <v>4</v>
+      </c>
+      <c r="E272" s="2">
+        <v>1</v>
+      </c>
+      <c r="F272" s="2">
+        <v>5</v>
+      </c>
+      <c r="G272" s="3">
+        <v>0.00648508430609598</v>
+      </c>
+      <c r="H272" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B273" s="0" t="inlineStr">
+        <is>
+          <t>Invitations &amp; parties</t>
+        </is>
+      </c>
+      <c r="C273" s="0" t="inlineStr">
+        <is>
+          <t>invp</t>
+        </is>
+      </c>
+      <c r="D273" s="2">
+        <v>3</v>
+      </c>
+      <c r="E273" s="2">
+        <v>0</v>
+      </c>
+      <c r="F273" s="2">
+        <v>3</v>
+      </c>
+      <c r="G273" s="3">
+        <v>0.0038910505836575876</v>
+      </c>
+      <c r="H273" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B274" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C274" s="0" t="inlineStr">
+        <is>
+          <t>intouch</t>
+        </is>
+      </c>
+      <c r="D274" s="2">
+        <v>2</v>
+      </c>
+      <c r="E274" s="2">
+        <v>0</v>
+      </c>
+      <c r="F274" s="2">
+        <v>2</v>
+      </c>
+      <c r="G274" s="3">
+        <v>0.0025940337224383916</v>
+      </c>
+      <c r="H274" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B275" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C275" s="0" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="D275" s="2">
+        <v>2</v>
+      </c>
+      <c r="E275" s="2">
+        <v>0</v>
+      </c>
+      <c r="F275" s="2">
+        <v>2</v>
+      </c>
+      <c r="G275" s="3">
+        <v>0.0025940337224383916</v>
+      </c>
+      <c r="H275" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B276" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C276" s="0" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+      <c r="D276" s="2">
+        <v>1</v>
+      </c>
+      <c r="E276" s="2">
+        <v>0</v>
+      </c>
+      <c r="F276" s="2">
+        <v>1</v>
+      </c>
+      <c r="G276" s="3">
+        <v>0.0012970168612191958</v>
+      </c>
+      <c r="H276" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B277" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C277" s="0" t="inlineStr">
+        <is>
+          <t>friend</t>
+        </is>
+      </c>
+      <c r="D277" s="2">
+        <v>1</v>
+      </c>
+      <c r="E277" s="2">
+        <v>0</v>
+      </c>
+      <c r="F277" s="2">
+        <v>1</v>
+      </c>
+      <c r="G277" s="3">
+        <v>0.0012970168612191958</v>
+      </c>
+      <c r="H277" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B278" s="0" t="inlineStr">
+        <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="C278" s="0" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="D278" s="2">
+        <v>0</v>
+      </c>
+      <c r="E278" s="2">
+        <v>1</v>
+      </c>
+      <c r="F278" s="2">
+        <v>1</v>
+      </c>
+      <c r="G278" s="3">
+        <v>0.0012970168612191958</v>
+      </c>
+      <c r="H278" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-18</t>
+        </is>
+      </c>
+      <c r="B279" s="4"/>
+      <c r="C279" s="4"/>
+      <c r="D279" s="5">
+        <v>520</v>
+      </c>
+      <c r="E279" s="5">
+        <v>251</v>
+      </c>
+      <c r="F279" s="5">
+        <v>771</v>
+      </c>
+      <c r="G279" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="H279" s="4"/>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -50370,6 +51025,2540 @@
         <v>730</v>
       </c>
       <c r="F1441" s="4"/>
+    </row>
+    <row r="1442">
+      <c r="A1442" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1442" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1442" s="0" t="inlineStr">
+        <is>
+          <t>happybirthday</t>
+        </is>
+      </c>
+      <c r="D1442" s="0" t="inlineStr">
+        <is>
+          <t>birth_happybirthday</t>
+        </is>
+      </c>
+      <c r="E1442" s="2">
+        <v>421</v>
+      </c>
+      <c r="F1442" s="2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1443">
+      <c r="A1443" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1443" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1443" s="0" t="inlineStr">
+        <is>
+          <t>anniversaryetc</t>
+        </is>
+      </c>
+      <c r="D1443" s="0" t="inlineStr">
+        <is>
+          <t>anniv_anniversaryetc</t>
+        </is>
+      </c>
+      <c r="E1443" s="2">
+        <v>41</v>
+      </c>
+      <c r="F1443" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1444">
+      <c r="A1444" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1444" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1444" s="0" t="inlineStr">
+        <is>
+          <t>fun</t>
+        </is>
+      </c>
+      <c r="D1444" s="0" t="inlineStr">
+        <is>
+          <t>birth_fun</t>
+        </is>
+      </c>
+      <c r="E1444" s="2">
+        <v>17</v>
+      </c>
+      <c r="F1444" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1445">
+      <c r="A1445" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1445" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1445" s="0" t="inlineStr">
+        <is>
+          <t>thinkingofyou</t>
+        </is>
+      </c>
+      <c r="D1445" s="0" t="inlineStr">
+        <is>
+          <t>gen_thinkingofyou</t>
+        </is>
+      </c>
+      <c r="E1445" s="2">
+        <v>16</v>
+      </c>
+      <c r="F1445" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1446">
+      <c r="A1446" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1446" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1446" s="0" t="inlineStr">
+        <is>
+          <t>flowers</t>
+        </is>
+      </c>
+      <c r="D1446" s="0" t="inlineStr">
+        <is>
+          <t>birth_flowers</t>
+        </is>
+      </c>
+      <c r="E1446" s="2">
+        <v>15</v>
+      </c>
+      <c r="F1446" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1447">
+      <c r="A1447" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1447" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1447" s="0" t="inlineStr">
+        <is>
+          <t>sympathy</t>
+        </is>
+      </c>
+      <c r="D1447" s="0" t="inlineStr">
+        <is>
+          <t>insp_sympathy</t>
+        </is>
+      </c>
+      <c r="E1447" s="2">
+        <v>15</v>
+      </c>
+      <c r="F1447" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1448">
+      <c r="A1448" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1448" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1448" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="D1448" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="E1448" s="2">
+        <v>13</v>
+      </c>
+      <c r="F1448" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1449">
+      <c r="A1449" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1449" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1449" s="0" t="inlineStr">
+        <is>
+          <t>birthday</t>
+        </is>
+      </c>
+      <c r="D1449" s="0" t="inlineStr">
+        <is>
+          <t>thank_birthday</t>
+        </is>
+      </c>
+      <c r="E1449" s="2">
+        <v>13</v>
+      </c>
+      <c r="F1449" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1450">
+      <c r="A1450" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1450" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1450" s="0" t="inlineStr">
+        <is>
+          <t>bronsis</t>
+        </is>
+      </c>
+      <c r="D1450" s="0" t="inlineStr">
+        <is>
+          <t>birth_bronsis</t>
+        </is>
+      </c>
+      <c r="E1450" s="2">
+        <v>10</v>
+      </c>
+      <c r="F1450" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1451">
+      <c r="A1451" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1451" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1451" s="0" t="inlineStr">
+        <is>
+          <t>songs</t>
+        </is>
+      </c>
+      <c r="D1451" s="0" t="inlineStr">
+        <is>
+          <t>birth_songs</t>
+        </is>
+      </c>
+      <c r="E1451" s="2">
+        <v>9</v>
+      </c>
+      <c r="F1451" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1452">
+      <c r="A1452" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1452" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1452" s="0" t="inlineStr">
+        <is>
+          <t>sweetheart</t>
+        </is>
+      </c>
+      <c r="D1452" s="0" t="inlineStr">
+        <is>
+          <t>love_sweetheart</t>
+        </is>
+      </c>
+      <c r="E1452" s="2">
+        <v>9</v>
+      </c>
+      <c r="F1452" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1453">
+      <c r="A1453" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1453" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1453" s="0" t="inlineStr">
+        <is>
+          <t>belated</t>
+        </is>
+      </c>
+      <c r="D1453" s="0" t="inlineStr">
+        <is>
+          <t>birth_belated</t>
+        </is>
+      </c>
+      <c r="E1453" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1453" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1454">
+      <c r="A1454" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1454" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1454" s="0" t="inlineStr">
+        <is>
+          <t>wishes</t>
+        </is>
+      </c>
+      <c r="D1454" s="0" t="inlineStr">
+        <is>
+          <t>birth_wishes</t>
+        </is>
+      </c>
+      <c r="E1454" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1454" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1455">
+      <c r="A1455" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1455" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1455" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugsweetheartday</t>
+        </is>
+      </c>
+      <c r="D1455" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugsweetheartday</t>
+        </is>
+      </c>
+      <c r="E1455" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1455" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1456">
+      <c r="A1456" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1456" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1456" s="0" t="inlineStr">
+        <is>
+          <t>morning</t>
+        </is>
+      </c>
+      <c r="D1456" s="0" t="inlineStr">
+        <is>
+          <t>gen_morning</t>
+        </is>
+      </c>
+      <c r="E1456" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1456" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1457">
+      <c r="A1457" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1457" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1457" s="0" t="inlineStr">
+        <is>
+          <t>blessings</t>
+        </is>
+      </c>
+      <c r="D1457" s="0" t="inlineStr">
+        <is>
+          <t>birth_blessings</t>
+        </is>
+      </c>
+      <c r="E1457" s="2">
+        <v>6</v>
+      </c>
+      <c r="F1457" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1458">
+      <c r="A1458" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1458" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1458" s="0" t="inlineStr">
+        <is>
+          <t>friends</t>
+        </is>
+      </c>
+      <c r="D1458" s="0" t="inlineStr">
+        <is>
+          <t>birth_friends</t>
+        </is>
+      </c>
+      <c r="E1458" s="2">
+        <v>6</v>
+      </c>
+      <c r="F1458" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1459">
+      <c r="A1459" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1459" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1459" s="0" t="inlineStr">
+        <is>
+          <t>foreveryone</t>
+        </is>
+      </c>
+      <c r="D1459" s="0" t="inlineStr">
+        <is>
+          <t>congrats_foreveryone</t>
+        </is>
+      </c>
+      <c r="E1459" s="2">
+        <v>6</v>
+      </c>
+      <c r="F1459" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1460">
+      <c r="A1460" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1460" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1460" s="0" t="inlineStr">
+        <is>
+          <t>everyday</t>
+        </is>
+      </c>
+      <c r="D1460" s="0" t="inlineStr">
+        <is>
+          <t>thank_everyday</t>
+        </is>
+      </c>
+      <c r="E1460" s="2">
+        <v>6</v>
+      </c>
+      <c r="F1460" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1461">
+      <c r="A1461" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1461" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1461" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="D1461" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forher</t>
+        </is>
+      </c>
+      <c r="E1461" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1461" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1462" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1462" s="0" t="inlineStr">
+        <is>
+          <t>hubbywife</t>
+        </is>
+      </c>
+      <c r="D1462" s="0" t="inlineStr">
+        <is>
+          <t>birth_hubbywife</t>
+        </is>
+      </c>
+      <c r="E1462" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1462" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1463">
+      <c r="A1463" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1463" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1463" s="0" t="inlineStr">
+        <is>
+          <t>sonanddaughter</t>
+        </is>
+      </c>
+      <c r="D1463" s="0" t="inlineStr">
+        <is>
+          <t>birth_sonanddaughter</t>
+        </is>
+      </c>
+      <c r="E1463" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1463" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1464">
+      <c r="A1464" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1464" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C1464" s="0" t="inlineStr">
+        <is>
+          <t>hugs</t>
+        </is>
+      </c>
+      <c r="D1464" s="0" t="inlineStr">
+        <is>
+          <t>cute_hugs</t>
+        </is>
+      </c>
+      <c r="E1464" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1464" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1465">
+      <c r="A1465" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1465" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1465" s="0" t="inlineStr">
+        <is>
+          <t>eaug_icecream_pie_day</t>
+        </is>
+      </c>
+      <c r="D1465" s="0" t="inlineStr">
+        <is>
+          <t>eaug_icecream_pie_day</t>
+        </is>
+      </c>
+      <c r="E1465" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1465" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1466">
+      <c r="A1466" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1466" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1466" s="0" t="inlineStr">
+        <is>
+          <t>hvgtday</t>
+        </is>
+      </c>
+      <c r="D1466" s="0" t="inlineStr">
+        <is>
+          <t>gen_hvgtday</t>
+        </is>
+      </c>
+      <c r="E1466" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1466" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1467">
+      <c r="A1467" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1467" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1467" s="0" t="inlineStr">
+        <is>
+          <t>balloons</t>
+        </is>
+      </c>
+      <c r="D1467" s="0" t="inlineStr">
+        <is>
+          <t>birth_balloons</t>
+        </is>
+      </c>
+      <c r="E1467" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1467" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1468">
+      <c r="A1468" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1468" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1468" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D1468" s="0" t="inlineStr">
+        <is>
+          <t>birth_milestone</t>
+        </is>
+      </c>
+      <c r="E1468" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1468" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1469">
+      <c r="A1469" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1469" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1469" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D1469" s="0" t="inlineStr">
+        <is>
+          <t>gen_getwell</t>
+        </is>
+      </c>
+      <c r="E1469" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1469" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1470">
+      <c r="A1470" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1470" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1470" s="0" t="inlineStr">
+        <is>
+          <t>extfamily</t>
+        </is>
+      </c>
+      <c r="D1470" s="0" t="inlineStr">
+        <is>
+          <t>birth_extfamily</t>
+        </is>
+      </c>
+      <c r="E1470" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1470" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1471">
+      <c r="A1471" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1471" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1471" s="0" t="inlineStr">
+        <is>
+          <t>newbaby</t>
+        </is>
+      </c>
+      <c r="D1471" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newbaby</t>
+        </is>
+      </c>
+      <c r="E1471" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1471" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1472">
+      <c r="A1472" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1472" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1472" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="D1472" s="0" t="inlineStr">
+        <is>
+          <t>eaug_hugmonth</t>
+        </is>
+      </c>
+      <c r="E1472" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1472" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1473">
+      <c r="A1473" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1473" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1473" s="0" t="inlineStr">
+        <is>
+          <t>ejul_kissingday</t>
+        </is>
+      </c>
+      <c r="D1473" s="0" t="inlineStr">
+        <is>
+          <t>ejul_kissingday</t>
+        </is>
+      </c>
+      <c r="E1473" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1473" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1474">
+      <c r="A1474" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1474" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1474" s="0" t="inlineStr">
+        <is>
+          <t>esep_fall_specials</t>
+        </is>
+      </c>
+      <c r="D1474" s="0" t="inlineStr">
+        <is>
+          <t>esep_fall_specials</t>
+        </is>
+      </c>
+      <c r="E1474" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1474" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1475">
+      <c r="A1475" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1475" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C1475" s="0" t="inlineStr">
+        <is>
+          <t>sisters</t>
+        </is>
+      </c>
+      <c r="D1475" s="0" t="inlineStr">
+        <is>
+          <t>fkt_sisters</t>
+        </is>
+      </c>
+      <c r="E1475" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1475" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1476">
+      <c r="A1476" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1476" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C1476" s="0" t="inlineStr">
+        <is>
+          <t>sonsdaughter</t>
+        </is>
+      </c>
+      <c r="D1476" s="0" t="inlineStr">
+        <is>
+          <t>fkt_sonsdaughter</t>
+        </is>
+      </c>
+      <c r="E1476" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1476" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1477">
+      <c r="A1477" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1477" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C1477" s="0" t="inlineStr">
+        <is>
+          <t>flrwishes</t>
+        </is>
+      </c>
+      <c r="D1477" s="0" t="inlineStr">
+        <is>
+          <t>flwr_flrwishes</t>
+        </is>
+      </c>
+      <c r="E1477" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1477" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1478">
+      <c r="A1478" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1478" s="0" t="inlineStr">
+        <is>
+          <t>Invitations &amp; parties</t>
+        </is>
+      </c>
+      <c r="C1478" s="0" t="inlineStr">
+        <is>
+          <t>birth_gen</t>
+        </is>
+      </c>
+      <c r="D1478" s="0" t="inlineStr">
+        <is>
+          <t>invp_birth_gen</t>
+        </is>
+      </c>
+      <c r="E1478" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1478" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1479">
+      <c r="A1479" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1479" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1479" s="0" t="inlineStr">
+        <is>
+          <t>loveetc</t>
+        </is>
+      </c>
+      <c r="D1479" s="0" t="inlineStr">
+        <is>
+          <t>love_loveetc</t>
+        </is>
+      </c>
+      <c r="E1479" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1479" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1480">
+      <c r="A1480" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1480" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1480" s="0" t="inlineStr">
+        <is>
+          <t>ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="D1480" s="0" t="inlineStr">
+        <is>
+          <t>anniv_ouranniversary_forhim</t>
+        </is>
+      </c>
+      <c r="E1480" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1480" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1481">
+      <c r="A1481" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1481" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1481" s="0" t="inlineStr">
+        <is>
+          <t>kids</t>
+        </is>
+      </c>
+      <c r="D1481" s="0" t="inlineStr">
+        <is>
+          <t>birth_kids</t>
+        </is>
+      </c>
+      <c r="E1481" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1481" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1482">
+      <c r="A1482" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1482" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1482" s="0" t="inlineStr">
+        <is>
+          <t>momndad</t>
+        </is>
+      </c>
+      <c r="D1482" s="0" t="inlineStr">
+        <is>
+          <t>birth_momndad</t>
+        </is>
+      </c>
+      <c r="E1482" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1482" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1483">
+      <c r="A1483" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1483" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1483" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalaviation_day</t>
+        </is>
+      </c>
+      <c r="D1483" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalaviation_day</t>
+        </is>
+      </c>
+      <c r="E1483" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1483" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1484">
+      <c r="A1484" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1484" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1484" s="0" t="inlineStr">
+        <is>
+          <t>eaug_rakshabandhan_happy</t>
+        </is>
+      </c>
+      <c r="D1484" s="0" t="inlineStr">
+        <is>
+          <t>eaug_rakshabandhan_happy</t>
+        </is>
+      </c>
+      <c r="E1484" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1484" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1485">
+      <c r="A1485" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1485" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1485" s="0" t="inlineStr">
+        <is>
+          <t>esep_janmashtami</t>
+        </is>
+      </c>
+      <c r="D1485" s="0" t="inlineStr">
+        <is>
+          <t>esep_janmashtami</t>
+        </is>
+      </c>
+      <c r="E1485" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1485" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1486">
+      <c r="A1486" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1486" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1486" s="0" t="inlineStr">
+        <is>
+          <t>esep_longestkissday</t>
+        </is>
+      </c>
+      <c r="D1486" s="0" t="inlineStr">
+        <is>
+          <t>esep_longestkissday</t>
+        </is>
+      </c>
+      <c r="E1486" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1486" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1487">
+      <c r="A1487" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1487" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C1487" s="0" t="inlineStr">
+        <is>
+          <t>roses</t>
+        </is>
+      </c>
+      <c r="D1487" s="0" t="inlineStr">
+        <is>
+          <t>flwr_roses</t>
+        </is>
+      </c>
+      <c r="E1487" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1487" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1488">
+      <c r="A1488" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1488" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1488" s="0" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="D1488" s="0" t="inlineStr">
+        <is>
+          <t>gen_luck</t>
+        </is>
+      </c>
+      <c r="E1488" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1488" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1489">
+      <c r="A1489" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1489" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1489" s="0" t="inlineStr">
+        <is>
+          <t>quotesmessages_images_getwell_messages</t>
+        </is>
+      </c>
+      <c r="D1489" s="0" t="inlineStr">
+        <is>
+          <t>gen_quotesmessages_images_getwell_messages</t>
+        </is>
+      </c>
+      <c r="E1489" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1489" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1490">
+      <c r="A1490" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1490" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1490" s="0" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="D1490" s="0" t="inlineStr">
+        <is>
+          <t>insp_health</t>
+        </is>
+      </c>
+      <c r="E1490" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1490" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1491">
+      <c r="A1491" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1491" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1491" s="0" t="inlineStr">
+        <is>
+          <t>recovery</t>
+        </is>
+      </c>
+      <c r="D1491" s="0" t="inlineStr">
+        <is>
+          <t>insp_recovery</t>
+        </is>
+      </c>
+      <c r="E1491" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1491" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1492">
+      <c r="A1492" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1492" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1492" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="D1492" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="E1492" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1492" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1493">
+      <c r="A1493" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1493" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1493" s="0" t="inlineStr">
+        <is>
+          <t>missing_forhim</t>
+        </is>
+      </c>
+      <c r="D1493" s="0" t="inlineStr">
+        <is>
+          <t>love_missing_forhim</t>
+        </is>
+      </c>
+      <c r="E1493" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1493" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1494">
+      <c r="A1494" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1494" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C1494" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D1494" s="0" t="inlineStr">
+        <is>
+          <t>pet_getwell</t>
+        </is>
+      </c>
+      <c r="E1494" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1494" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1495">
+      <c r="A1495" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1495" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1495" s="0" t="inlineStr">
+        <is>
+          <t>wedding</t>
+        </is>
+      </c>
+      <c r="D1495" s="0" t="inlineStr">
+        <is>
+          <t>thank_wedding</t>
+        </is>
+      </c>
+      <c r="E1495" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1495" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1496">
+      <c r="A1496" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1496" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1496" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D1496" s="0" t="inlineStr">
+        <is>
+          <t>anniv_milestone</t>
+        </is>
+      </c>
+      <c r="E1496" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1496" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1497">
+      <c r="A1497" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1497" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1497" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_family</t>
+        </is>
+      </c>
+      <c r="D1497" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_family</t>
+        </is>
+      </c>
+      <c r="E1497" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1497" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1498">
+      <c r="A1498" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1498" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C1498" s="0" t="inlineStr">
+        <is>
+          <t>retirement</t>
+        </is>
+      </c>
+      <c r="D1498" s="0" t="inlineStr">
+        <is>
+          <t>bus_retirement</t>
+        </is>
+      </c>
+      <c r="E1498" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1498" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1499">
+      <c r="A1499" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1499" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1499" s="0" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="D1499" s="0" t="inlineStr">
+        <is>
+          <t>congrats_engagement</t>
+        </is>
+      </c>
+      <c r="E1499" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1499" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1500">
+      <c r="A1500" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1500" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1500" s="0" t="inlineStr">
+        <is>
+          <t>newcarandlicense</t>
+        </is>
+      </c>
+      <c r="D1500" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newcarandlicense</t>
+        </is>
+      </c>
+      <c r="E1500" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1500" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1501">
+      <c r="A1501" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1501" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1501" s="0" t="inlineStr">
+        <is>
+          <t>onotheroccasions</t>
+        </is>
+      </c>
+      <c r="D1501" s="0" t="inlineStr">
+        <is>
+          <t>congrats_onotheroccasions</t>
+        </is>
+      </c>
+      <c r="E1501" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1501" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1502">
+      <c r="A1502" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1502" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1502" s="0" t="inlineStr">
+        <is>
+          <t>studentsandnewgrads</t>
+        </is>
+      </c>
+      <c r="D1502" s="0" t="inlineStr">
+        <is>
+          <t>congrats_studentsandnewgrads</t>
+        </is>
+      </c>
+      <c r="E1502" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1502" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1503">
+      <c r="A1503" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1503" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C1503" s="0" t="inlineStr">
+        <is>
+          <t>heart</t>
+        </is>
+      </c>
+      <c r="D1503" s="0" t="inlineStr">
+        <is>
+          <t>cute_heart</t>
+        </is>
+      </c>
+      <c r="E1503" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1503" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1504">
+      <c r="A1504" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1504" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1504" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipweek</t>
+        </is>
+      </c>
+      <c r="D1504" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipweek</t>
+        </is>
+      </c>
+      <c r="E1504" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1504" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1505">
+      <c r="A1505" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1505" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1505" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalpotato_day</t>
+        </is>
+      </c>
+      <c r="D1505" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalpotato_day</t>
+        </is>
+      </c>
+      <c r="E1505" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1505" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1506">
+      <c r="A1506" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1506" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1506" s="0" t="inlineStr">
+        <is>
+          <t>eaug_rakshabandhan_interactive</t>
+        </is>
+      </c>
+      <c r="D1506" s="0" t="inlineStr">
+        <is>
+          <t>eaug_rakshabandhan_interactive</t>
+        </is>
+      </c>
+      <c r="E1506" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1506" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1507">
+      <c r="A1507" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1507" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1507" s="0" t="inlineStr">
+        <is>
+          <t>eaug_seniorcitizen_day</t>
+        </is>
+      </c>
+      <c r="D1507" s="0" t="inlineStr">
+        <is>
+          <t>eaug_seniorcitizen_day</t>
+        </is>
+      </c>
+      <c r="E1507" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1507" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1508">
+      <c r="A1508" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1508" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1508" s="0" t="inlineStr">
+        <is>
+          <t>ejul_summerleisure_day</t>
+        </is>
+      </c>
+      <c r="D1508" s="0" t="inlineStr">
+        <is>
+          <t>ejul_summerleisure_day</t>
+        </is>
+      </c>
+      <c r="E1508" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1508" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1509">
+      <c r="A1509" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1509" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1509" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_love</t>
+        </is>
+      </c>
+      <c r="D1509" s="0" t="inlineStr">
+        <is>
+          <t>ejun_summer_love</t>
+        </is>
+      </c>
+      <c r="E1509" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1509" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1510">
+      <c r="A1510" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1510" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1510" s="0" t="inlineStr">
+        <is>
+          <t>emay_graduation_happy</t>
+        </is>
+      </c>
+      <c r="D1510" s="0" t="inlineStr">
+        <is>
+          <t>emay_graduation_happy</t>
+        </is>
+      </c>
+      <c r="E1510" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1510" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1511">
+      <c r="A1511" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1511" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1511" s="0" t="inlineStr">
+        <is>
+          <t>emay_graduation_wishes</t>
+        </is>
+      </c>
+      <c r="D1511" s="0" t="inlineStr">
+        <is>
+          <t>emay_graduation_wishes</t>
+        </is>
+      </c>
+      <c r="E1511" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1511" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1512">
+      <c r="A1512" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1512" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1512" s="0" t="inlineStr">
+        <is>
+          <t>eoct_sweetday_missyou</t>
+        </is>
+      </c>
+      <c r="D1512" s="0" t="inlineStr">
+        <is>
+          <t>eoct_sweetday_missyou</t>
+        </is>
+      </c>
+      <c r="E1512" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1512" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1513">
+      <c r="A1513" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1513" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C1513" s="0" t="inlineStr">
+        <is>
+          <t>missingyou</t>
+        </is>
+      </c>
+      <c r="D1513" s="0" t="inlineStr">
+        <is>
+          <t>friend_missingyou</t>
+        </is>
+      </c>
+      <c r="E1513" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1513" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1514">
+      <c r="A1514" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1514" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1514" s="0" t="inlineStr">
+        <is>
+          <t>goodnight</t>
+        </is>
+      </c>
+      <c r="D1514" s="0" t="inlineStr">
+        <is>
+          <t>gen_goodnight</t>
+        </is>
+      </c>
+      <c r="E1514" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1514" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1515">
+      <c r="A1515" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1515" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1515" s="0" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="D1515" s="0" t="inlineStr">
+        <is>
+          <t>gen_hi</t>
+        </is>
+      </c>
+      <c r="E1515" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1515" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1516">
+      <c r="A1516" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1516" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1516" s="0" t="inlineStr">
+        <is>
+          <t>morningquotes</t>
+        </is>
+      </c>
+      <c r="D1516" s="0" t="inlineStr">
+        <is>
+          <t>gen_morningquotes</t>
+        </is>
+      </c>
+      <c r="E1516" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1516" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1517">
+      <c r="A1517" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1517" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1517" s="0" t="inlineStr">
+        <is>
+          <t>quotesmessages_images_getwell_images</t>
+        </is>
+      </c>
+      <c r="D1517" s="0" t="inlineStr">
+        <is>
+          <t>gen_quotesmessages_images_getwell_images</t>
+        </is>
+      </c>
+      <c r="E1517" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1517" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1518">
+      <c r="A1518" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1518" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1518" s="0" t="inlineStr">
+        <is>
+          <t>quotesmessages_images_missyou_messages</t>
+        </is>
+      </c>
+      <c r="D1518" s="0" t="inlineStr">
+        <is>
+          <t>gen_quotesmessages_images_missyou_messages</t>
+        </is>
+      </c>
+      <c r="E1518" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1518" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1519">
+      <c r="A1519" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1519" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1519" s="0" t="inlineStr">
+        <is>
+          <t>sorry</t>
+        </is>
+      </c>
+      <c r="D1519" s="0" t="inlineStr">
+        <is>
+          <t>gen_sorry</t>
+        </is>
+      </c>
+      <c r="E1519" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1519" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1520">
+      <c r="A1520" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1520" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1520" s="0" t="inlineStr">
+        <is>
+          <t>tuestoons</t>
+        </is>
+      </c>
+      <c r="D1520" s="0" t="inlineStr">
+        <is>
+          <t>gen_tuestoons</t>
+        </is>
+      </c>
+      <c r="E1520" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1520" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1521">
+      <c r="A1521" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1521" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1521" s="0" t="inlineStr">
+        <is>
+          <t>youarewelcome</t>
+        </is>
+      </c>
+      <c r="D1521" s="0" t="inlineStr">
+        <is>
+          <t>gen_youarewelcome</t>
+        </is>
+      </c>
+      <c r="E1521" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1521" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1522">
+      <c r="A1522" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1522" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1522" s="0" t="inlineStr">
+        <is>
+          <t>encour</t>
+        </is>
+      </c>
+      <c r="D1522" s="0" t="inlineStr">
+        <is>
+          <t>insp_encour</t>
+        </is>
+      </c>
+      <c r="E1522" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1522" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1523">
+      <c r="A1523" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1523" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C1523" s="0" t="inlineStr">
+        <is>
+          <t>keepintouch</t>
+        </is>
+      </c>
+      <c r="D1523" s="0" t="inlineStr">
+        <is>
+          <t>intouch_keepintouch</t>
+        </is>
+      </c>
+      <c r="E1523" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1523" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1524">
+      <c r="A1524" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1524" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C1524" s="0" t="inlineStr">
+        <is>
+          <t>missingyou</t>
+        </is>
+      </c>
+      <c r="D1524" s="0" t="inlineStr">
+        <is>
+          <t>intouch_missingyou</t>
+        </is>
+      </c>
+      <c r="E1524" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1524" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1525">
+      <c r="A1525" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1525" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1525" s="0" t="inlineStr">
+        <is>
+          <t>cute</t>
+        </is>
+      </c>
+      <c r="D1525" s="0" t="inlineStr">
+        <is>
+          <t>love_cute</t>
+        </is>
+      </c>
+      <c r="E1525" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1525" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1526">
+      <c r="A1526" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1526" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1526" s="0" t="inlineStr">
+        <is>
+          <t>dating</t>
+        </is>
+      </c>
+      <c r="D1526" s="0" t="inlineStr">
+        <is>
+          <t>love_dating</t>
+        </is>
+      </c>
+      <c r="E1526" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1526" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1527">
+      <c r="A1527" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1527" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1527" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_general</t>
+        </is>
+      </c>
+      <c r="D1527" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_general</t>
+        </is>
+      </c>
+      <c r="E1527" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1527" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1528">
+      <c r="A1528" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1528" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1528" s="0" t="inlineStr">
+        <is>
+          <t>missing_forher</t>
+        </is>
+      </c>
+      <c r="D1528" s="0" t="inlineStr">
+        <is>
+          <t>love_missing_forher</t>
+        </is>
+      </c>
+      <c r="E1528" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1528" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1529">
+      <c r="A1529" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1529" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1529" s="0" t="inlineStr">
+        <is>
+          <t>congratulations</t>
+        </is>
+      </c>
+      <c r="D1529" s="0" t="inlineStr">
+        <is>
+          <t>thank_congratulations</t>
+        </is>
+      </c>
+      <c r="E1529" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1529" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1530">
+      <c r="A1530" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1530" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1530" s="0" t="inlineStr">
+        <is>
+          <t>inspirational</t>
+        </is>
+      </c>
+      <c r="D1530" s="0" t="inlineStr">
+        <is>
+          <t>thank_inspirational</t>
+        </is>
+      </c>
+      <c r="E1530" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1530" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1531">
+      <c r="A1531" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1531" s="0" t="inlineStr">
+        <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="C1531" s="0" t="inlineStr">
+        <is>
+          <t>hindi_birthday</t>
+        </is>
+      </c>
+      <c r="D1531" s="0" t="inlineStr">
+        <is>
+          <t>w_hindi_birthday</t>
+        </is>
+      </c>
+      <c r="E1531" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1531" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1532">
+      <c r="A1532" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1532" s="4"/>
+      <c r="C1532" s="4"/>
+      <c r="D1532" s="4"/>
+      <c r="E1532" s="5">
+        <v>771</v>
+      </c>
+      <c r="F1532" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -51021,36 +54210,70 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B19" s="2">
+        <v>822</v>
+      </c>
+      <c r="C19" s="2">
+        <v>264</v>
+      </c>
+      <c r="D19" s="2">
+        <v>275</v>
+      </c>
+      <c r="E19" s="2">
+        <v>126</v>
+      </c>
+      <c r="F19" s="2">
+        <v>77</v>
+      </c>
+      <c r="G19" s="2">
+        <v>55</v>
+      </c>
+      <c r="H19" s="2">
+        <v>25</v>
+      </c>
+      <c r="I19" s="2">
+        <v>0</v>
+      </c>
+      <c r="J19" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B19" s="5">
-        <v>13973</v>
-      </c>
-      <c r="C19" s="5">
-        <v>4439</v>
-      </c>
-      <c r="D19" s="5">
-        <v>4339</v>
-      </c>
-      <c r="E19" s="5">
-        <v>2800</v>
-      </c>
-      <c r="F19" s="5">
-        <v>1390</v>
-      </c>
-      <c r="G19" s="5">
-        <v>536</v>
-      </c>
-      <c r="H19" s="5">
-        <v>440</v>
-      </c>
-      <c r="I19" s="5">
+      <c r="B20" s="5">
+        <v>14795</v>
+      </c>
+      <c r="C20" s="5">
+        <v>4703</v>
+      </c>
+      <c r="D20" s="5">
+        <v>4614</v>
+      </c>
+      <c r="E20" s="5">
+        <v>2926</v>
+      </c>
+      <c r="F20" s="5">
+        <v>1467</v>
+      </c>
+      <c r="G20" s="5">
+        <v>591</v>
+      </c>
+      <c r="H20" s="5">
+        <v>465</v>
+      </c>
+      <c r="I20" s="5">
         <v>28</v>
       </c>
-      <c r="J19" s="5">
+      <c r="J20" s="5">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Record 19 August: nineteen days, 15,568 sends tracked
App 505 sends across 186 cards, all categorised. Web and mobile web 268
sends across 105 cards, 225 categorised - the 43 uncategorised are the
'desktop' row again, which is the surface total rather than a card.

Pivot verified against its own SUM row: columns 7/0/16/12/35/58/0/8/132,
grand 268, every row's cells agreeing with its own Total, no duplicate card
rows, and not a repeat of any pivot already recorded. App log single-dated
with 505 unique ids in 1-520; the 15 gaps are failed sends, which are not
exported.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9KsXegBwxB1sWdCzRVLrr
</commit_message>
<xml_diff>
--- a/reports/daily_tracking.xlsx
+++ b/reports/daily_tracking.xlsx
@@ -224,7 +224,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13">
@@ -247,7 +247,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
@@ -815,28 +815,56 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B20" s="2">
+        <v>773</v>
+      </c>
+      <c r="C20" s="2">
+        <v>505</v>
+      </c>
+      <c r="D20" s="2">
+        <v>268</v>
+      </c>
+      <c r="E20" s="2">
+        <v>730</v>
+      </c>
+      <c r="F20" s="2">
+        <v>43</v>
+      </c>
+      <c r="G20" s="2">
+        <v>236</v>
+      </c>
+      <c r="H20" s="2">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B20" s="5">
-        <v>14795</v>
-      </c>
-      <c r="C20" s="5">
-        <v>9831</v>
-      </c>
-      <c r="D20" s="5">
-        <v>4964</v>
-      </c>
-      <c r="E20" s="5">
-        <v>14205</v>
-      </c>
-      <c r="F20" s="5">
-        <v>590</v>
-      </c>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
+      <c r="B21" s="5">
+        <v>15568</v>
+      </c>
+      <c r="C21" s="5">
+        <v>10336</v>
+      </c>
+      <c r="D21" s="5">
+        <v>5232</v>
+      </c>
+      <c r="E21" s="5">
+        <v>14935</v>
+      </c>
+      <c r="F21" s="5">
+        <v>633</v>
+      </c>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -2062,63 +2090,124 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B20" s="2">
+        <v>730</v>
+      </c>
+      <c r="C20" s="2">
+        <v>532</v>
+      </c>
+      <c r="D20" s="2">
+        <v>26</v>
+      </c>
+      <c r="E20" s="2">
+        <v>31</v>
+      </c>
+      <c r="F20" s="2">
+        <v>44</v>
+      </c>
+      <c r="G20" s="2">
+        <v>32</v>
+      </c>
+      <c r="H20" s="2">
+        <v>14</v>
+      </c>
+      <c r="I20" s="2">
+        <v>22</v>
+      </c>
+      <c r="J20" s="2">
+        <v>2</v>
+      </c>
+      <c r="K20" s="2">
+        <v>8</v>
+      </c>
+      <c r="L20" s="2">
+        <v>2</v>
+      </c>
+      <c r="M20" s="2">
+        <v>4</v>
+      </c>
+      <c r="N20" s="2">
+        <v>5</v>
+      </c>
+      <c r="O20" s="2">
+        <v>1</v>
+      </c>
+      <c r="P20" s="2">
+        <v>4</v>
+      </c>
+      <c r="Q20" s="2">
+        <v>1</v>
+      </c>
+      <c r="R20" s="2">
+        <v>2</v>
+      </c>
+      <c r="S20" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B20" s="5">
-        <v>14205</v>
-      </c>
-      <c r="C20" s="5">
-        <v>9271</v>
-      </c>
-      <c r="D20" s="5">
-        <v>1405</v>
-      </c>
-      <c r="E20" s="5">
-        <v>900</v>
-      </c>
-      <c r="F20" s="5">
-        <v>724</v>
-      </c>
-      <c r="G20" s="5">
-        <v>525</v>
-      </c>
-      <c r="H20" s="5">
-        <v>343</v>
-      </c>
-      <c r="I20" s="5">
-        <v>284</v>
-      </c>
-      <c r="J20" s="5">
+      <c r="B21" s="5">
+        <v>14935</v>
+      </c>
+      <c r="C21" s="5">
+        <v>9803</v>
+      </c>
+      <c r="D21" s="5">
+        <v>1431</v>
+      </c>
+      <c r="E21" s="5">
+        <v>931</v>
+      </c>
+      <c r="F21" s="5">
+        <v>768</v>
+      </c>
+      <c r="G21" s="5">
+        <v>557</v>
+      </c>
+      <c r="H21" s="5">
+        <v>357</v>
+      </c>
+      <c r="I21" s="5">
+        <v>306</v>
+      </c>
+      <c r="J21" s="5">
+        <v>197</v>
+      </c>
+      <c r="K21" s="5">
         <v>195</v>
       </c>
-      <c r="K20" s="5">
-        <v>187</v>
-      </c>
-      <c r="L20" s="5">
-        <v>102</v>
-      </c>
-      <c r="M20" s="5">
-        <v>76</v>
-      </c>
-      <c r="N20" s="5">
-        <v>72</v>
-      </c>
-      <c r="O20" s="5">
-        <v>42</v>
-      </c>
-      <c r="P20" s="5">
-        <v>26</v>
-      </c>
-      <c r="Q20" s="5">
-        <v>23</v>
-      </c>
-      <c r="R20" s="5">
-        <v>18</v>
-      </c>
-      <c r="S20" s="5">
+      <c r="L21" s="5">
+        <v>104</v>
+      </c>
+      <c r="M21" s="5">
+        <v>80</v>
+      </c>
+      <c r="N21" s="5">
+        <v>77</v>
+      </c>
+      <c r="O21" s="5">
+        <v>43</v>
+      </c>
+      <c r="P21" s="5">
+        <v>30</v>
+      </c>
+      <c r="Q21" s="5">
+        <v>24</v>
+      </c>
+      <c r="R21" s="5">
+        <v>20</v>
+      </c>
+      <c r="S21" s="5">
         <v>12</v>
       </c>
     </row>
@@ -10897,6 +10986,540 @@
       </c>
       <c r="H279" s="4"/>
     </row>
+    <row r="280">
+      <c r="A280" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B280" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C280" s="0" t="inlineStr">
+        <is>
+          <t>birth</t>
+        </is>
+      </c>
+      <c r="D280" s="2">
+        <v>362</v>
+      </c>
+      <c r="E280" s="2">
+        <v>170</v>
+      </c>
+      <c r="F280" s="2">
+        <v>532</v>
+      </c>
+      <c r="G280" s="3">
+        <v>0.7287671232876712</v>
+      </c>
+      <c r="H280" s="2">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B281" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C281" s="0" t="inlineStr">
+        <is>
+          <t>gen</t>
+        </is>
+      </c>
+      <c r="D281" s="2">
+        <v>33</v>
+      </c>
+      <c r="E281" s="2">
+        <v>11</v>
+      </c>
+      <c r="F281" s="2">
+        <v>44</v>
+      </c>
+      <c r="G281" s="3">
+        <v>0.06027397260273973</v>
+      </c>
+      <c r="H281" s="2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B282" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C282" s="0" t="inlineStr">
+        <is>
+          <t>thank</t>
+        </is>
+      </c>
+      <c r="D282" s="2">
+        <v>9</v>
+      </c>
+      <c r="E282" s="2">
+        <v>23</v>
+      </c>
+      <c r="F282" s="2">
+        <v>32</v>
+      </c>
+      <c r="G282" s="3">
+        <v>0.043835616438356165</v>
+      </c>
+      <c r="H282" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B283" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C283" s="0" t="inlineStr">
+        <is>
+          <t>anniv</t>
+        </is>
+      </c>
+      <c r="D283" s="2">
+        <v>26</v>
+      </c>
+      <c r="E283" s="2">
+        <v>5</v>
+      </c>
+      <c r="F283" s="2">
+        <v>31</v>
+      </c>
+      <c r="G283" s="3">
+        <v>0.04246575342465753</v>
+      </c>
+      <c r="H283" s="2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B284" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C284" s="0" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="D284" s="2">
+        <v>24</v>
+      </c>
+      <c r="E284" s="2">
+        <v>2</v>
+      </c>
+      <c r="F284" s="2">
+        <v>26</v>
+      </c>
+      <c r="G284" s="3">
+        <v>0.03561643835616438</v>
+      </c>
+      <c r="H284" s="2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B285" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C285" s="0" t="inlineStr">
+        <is>
+          <t>insp</t>
+        </is>
+      </c>
+      <c r="D285" s="2">
+        <v>20</v>
+      </c>
+      <c r="E285" s="2">
+        <v>2</v>
+      </c>
+      <c r="F285" s="2">
+        <v>22</v>
+      </c>
+      <c r="G285" s="3">
+        <v>0.030136986301369864</v>
+      </c>
+      <c r="H285" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B286" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C286" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D286" s="2">
+        <v>9</v>
+      </c>
+      <c r="E286" s="2">
+        <v>5</v>
+      </c>
+      <c r="F286" s="2">
+        <v>14</v>
+      </c>
+      <c r="G286" s="3">
+        <v>0.019178082191780823</v>
+      </c>
+      <c r="H286" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B287" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C287" s="0" t="inlineStr">
+        <is>
+          <t>congrats</t>
+        </is>
+      </c>
+      <c r="D287" s="2">
+        <v>3</v>
+      </c>
+      <c r="E287" s="2">
+        <v>5</v>
+      </c>
+      <c r="F287" s="2">
+        <v>8</v>
+      </c>
+      <c r="G287" s="3">
+        <v>0.010958904109589041</v>
+      </c>
+      <c r="H287" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B288" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C288" s="0" t="inlineStr">
+        <is>
+          <t>cute</t>
+        </is>
+      </c>
+      <c r="D288" s="2">
+        <v>4</v>
+      </c>
+      <c r="E288" s="2">
+        <v>1</v>
+      </c>
+      <c r="F288" s="2">
+        <v>5</v>
+      </c>
+      <c r="G288" s="3">
+        <v>0.00684931506849315</v>
+      </c>
+      <c r="H288" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B289" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C289" s="0" t="inlineStr">
+        <is>
+          <t>fkt</t>
+        </is>
+      </c>
+      <c r="D289" s="2">
+        <v>4</v>
+      </c>
+      <c r="E289" s="2">
+        <v>0</v>
+      </c>
+      <c r="F289" s="2">
+        <v>4</v>
+      </c>
+      <c r="G289" s="3">
+        <v>0.005479452054794521</v>
+      </c>
+      <c r="H289" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B290" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C290" s="0" t="inlineStr">
+        <is>
+          <t>intouch</t>
+        </is>
+      </c>
+      <c r="D290" s="2">
+        <v>4</v>
+      </c>
+      <c r="E290" s="2">
+        <v>0</v>
+      </c>
+      <c r="F290" s="2">
+        <v>4</v>
+      </c>
+      <c r="G290" s="3">
+        <v>0.005479452054794521</v>
+      </c>
+      <c r="H290" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B291" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C291" s="0" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+      <c r="D291" s="2">
+        <v>2</v>
+      </c>
+      <c r="E291" s="2">
+        <v>0</v>
+      </c>
+      <c r="F291" s="2">
+        <v>2</v>
+      </c>
+      <c r="G291" s="3">
+        <v>0.0027397260273972603</v>
+      </c>
+      <c r="H291" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B292" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C292" s="0" t="inlineStr">
+        <is>
+          <t>flwr</t>
+        </is>
+      </c>
+      <c r="D292" s="2">
+        <v>2</v>
+      </c>
+      <c r="E292" s="2">
+        <v>0</v>
+      </c>
+      <c r="F292" s="2">
+        <v>2</v>
+      </c>
+      <c r="G292" s="3">
+        <v>0.0027397260273972603</v>
+      </c>
+      <c r="H292" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B293" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C293" s="0" t="inlineStr">
+        <is>
+          <t>friend</t>
+        </is>
+      </c>
+      <c r="D293" s="2">
+        <v>2</v>
+      </c>
+      <c r="E293" s="2">
+        <v>0</v>
+      </c>
+      <c r="F293" s="2">
+        <v>2</v>
+      </c>
+      <c r="G293" s="3">
+        <v>0.0027397260273972603</v>
+      </c>
+      <c r="H293" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B294" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C294" s="0" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="D294" s="2">
+        <v>1</v>
+      </c>
+      <c r="E294" s="2">
+        <v>0</v>
+      </c>
+      <c r="F294" s="2">
+        <v>1</v>
+      </c>
+      <c r="G294" s="3">
+        <v>0.0013698630136986301</v>
+      </c>
+      <c r="H294" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B295" s="0" t="inlineStr">
+        <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="C295" s="0" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="D295" s="2">
+        <v>0</v>
+      </c>
+      <c r="E295" s="2">
+        <v>1</v>
+      </c>
+      <c r="F295" s="2">
+        <v>1</v>
+      </c>
+      <c r="G295" s="3">
+        <v>0.0013698630136986301</v>
+      </c>
+      <c r="H295" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-19</t>
+        </is>
+      </c>
+      <c r="B296" s="4"/>
+      <c r="C296" s="4"/>
+      <c r="D296" s="5">
+        <v>505</v>
+      </c>
+      <c r="E296" s="5">
+        <v>225</v>
+      </c>
+      <c r="F296" s="5">
+        <v>730</v>
+      </c>
+      <c r="G296" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="H296" s="4"/>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -53615,6 +54238,2036 @@
         <v>771</v>
       </c>
       <c r="F1534" s="4"/>
+    </row>
+    <row r="1535">
+      <c r="A1535" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1535" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1535" s="0" t="inlineStr">
+        <is>
+          <t>happybirthday</t>
+        </is>
+      </c>
+      <c r="D1535" s="0" t="inlineStr">
+        <is>
+          <t>birth_happybirthday</t>
+        </is>
+      </c>
+      <c r="E1535" s="2">
+        <v>413</v>
+      </c>
+      <c r="F1535" s="2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1536">
+      <c r="A1536" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1536" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1536" s="0" t="inlineStr">
+        <is>
+          <t>wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="D1536" s="0" t="inlineStr">
+        <is>
+          <t>anniv_wedanniv_couple</t>
+        </is>
+      </c>
+      <c r="E1536" s="2">
+        <v>26</v>
+      </c>
+      <c r="F1536" s="2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1537">
+      <c r="A1537" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1537" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1537" s="0" t="inlineStr">
+        <is>
+          <t>fun</t>
+        </is>
+      </c>
+      <c r="D1537" s="0" t="inlineStr">
+        <is>
+          <t>birth_fun</t>
+        </is>
+      </c>
+      <c r="E1537" s="2">
+        <v>18</v>
+      </c>
+      <c r="F1537" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1538">
+      <c r="A1538" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1538" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1538" s="0" t="inlineStr">
+        <is>
+          <t>sonanddaughter</t>
+        </is>
+      </c>
+      <c r="D1538" s="0" t="inlineStr">
+        <is>
+          <t>birth_sonanddaughter</t>
+        </is>
+      </c>
+      <c r="E1538" s="2">
+        <v>15</v>
+      </c>
+      <c r="F1538" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1539">
+      <c r="A1539" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1539" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1539" s="0" t="inlineStr">
+        <is>
+          <t>sympathy</t>
+        </is>
+      </c>
+      <c r="D1539" s="0" t="inlineStr">
+        <is>
+          <t>insp_sympathy</t>
+        </is>
+      </c>
+      <c r="E1539" s="2">
+        <v>15</v>
+      </c>
+      <c r="F1539" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1540">
+      <c r="A1540" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1540" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1540" s="0" t="inlineStr">
+        <is>
+          <t>bronsis</t>
+        </is>
+      </c>
+      <c r="D1540" s="0" t="inlineStr">
+        <is>
+          <t>birth_bronsis</t>
+        </is>
+      </c>
+      <c r="E1540" s="2">
+        <v>14</v>
+      </c>
+      <c r="F1540" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1541">
+      <c r="A1541" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1541" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1541" s="0" t="inlineStr">
+        <is>
+          <t>songs</t>
+        </is>
+      </c>
+      <c r="D1541" s="0" t="inlineStr">
+        <is>
+          <t>birth_songs</t>
+        </is>
+      </c>
+      <c r="E1541" s="2">
+        <v>13</v>
+      </c>
+      <c r="F1541" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1542">
+      <c r="A1542" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1542" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1542" s="0" t="inlineStr">
+        <is>
+          <t>birthday</t>
+        </is>
+      </c>
+      <c r="D1542" s="0" t="inlineStr">
+        <is>
+          <t>thank_birthday</t>
+        </is>
+      </c>
+      <c r="E1542" s="2">
+        <v>13</v>
+      </c>
+      <c r="F1542" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1543">
+      <c r="A1543" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1543" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1543" s="0" t="inlineStr">
+        <is>
+          <t>extfamily</t>
+        </is>
+      </c>
+      <c r="D1543" s="0" t="inlineStr">
+        <is>
+          <t>birth_extfamily</t>
+        </is>
+      </c>
+      <c r="E1543" s="2">
+        <v>11</v>
+      </c>
+      <c r="F1543" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1544">
+      <c r="A1544" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1544" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1544" s="0" t="inlineStr">
+        <is>
+          <t>everyday</t>
+        </is>
+      </c>
+      <c r="D1544" s="0" t="inlineStr">
+        <is>
+          <t>thank_everyday</t>
+        </is>
+      </c>
+      <c r="E1544" s="2">
+        <v>10</v>
+      </c>
+      <c r="F1544" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1545">
+      <c r="A1545" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1545" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1545" s="0" t="inlineStr">
+        <is>
+          <t>wishes</t>
+        </is>
+      </c>
+      <c r="D1545" s="0" t="inlineStr">
+        <is>
+          <t>birth_wishes</t>
+        </is>
+      </c>
+      <c r="E1545" s="2">
+        <v>9</v>
+      </c>
+      <c r="F1545" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1546">
+      <c r="A1546" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1546" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1546" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D1546" s="0" t="inlineStr">
+        <is>
+          <t>gen_getwell</t>
+        </is>
+      </c>
+      <c r="E1546" s="2">
+        <v>9</v>
+      </c>
+      <c r="F1546" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1547">
+      <c r="A1547" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1547" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1547" s="0" t="inlineStr">
+        <is>
+          <t>thinkingofyou</t>
+        </is>
+      </c>
+      <c r="D1547" s="0" t="inlineStr">
+        <is>
+          <t>gen_thinkingofyou</t>
+        </is>
+      </c>
+      <c r="E1547" s="2">
+        <v>9</v>
+      </c>
+      <c r="F1547" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1548">
+      <c r="A1548" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1548" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1548" s="0" t="inlineStr">
+        <is>
+          <t>blessings</t>
+        </is>
+      </c>
+      <c r="D1548" s="0" t="inlineStr">
+        <is>
+          <t>birth_blessings</t>
+        </is>
+      </c>
+      <c r="E1548" s="2">
+        <v>8</v>
+      </c>
+      <c r="F1548" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1549">
+      <c r="A1549" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1549" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1549" s="0" t="inlineStr">
+        <is>
+          <t>kids</t>
+        </is>
+      </c>
+      <c r="D1549" s="0" t="inlineStr">
+        <is>
+          <t>birth_kids</t>
+        </is>
+      </c>
+      <c r="E1549" s="2">
+        <v>8</v>
+      </c>
+      <c r="F1549" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1550">
+      <c r="A1550" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1550" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1550" s="0" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D1550" s="0" t="inlineStr">
+        <is>
+          <t>birth_milestone</t>
+        </is>
+      </c>
+      <c r="E1550" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1550" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1551">
+      <c r="A1551" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1551" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1551" s="0" t="inlineStr">
+        <is>
+          <t>morning</t>
+        </is>
+      </c>
+      <c r="D1551" s="0" t="inlineStr">
+        <is>
+          <t>gen_morning</t>
+        </is>
+      </c>
+      <c r="E1551" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1551" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1552">
+      <c r="A1552" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1552" s="0" t="inlineStr">
+        <is>
+          <t>Anniversary</t>
+        </is>
+      </c>
+      <c r="C1552" s="0" t="inlineStr">
+        <is>
+          <t>anniversaryetc</t>
+        </is>
+      </c>
+      <c r="D1552" s="0" t="inlineStr">
+        <is>
+          <t>anniv_anniversaryetc</t>
+        </is>
+      </c>
+      <c r="E1552" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1552" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1553">
+      <c r="A1553" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1553" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1553" s="0" t="inlineStr">
+        <is>
+          <t>belated</t>
+        </is>
+      </c>
+      <c r="D1553" s="0" t="inlineStr">
+        <is>
+          <t>birth_belated</t>
+        </is>
+      </c>
+      <c r="E1553" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1553" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1554">
+      <c r="A1554" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1554" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1554" s="0" t="inlineStr">
+        <is>
+          <t>flowers</t>
+        </is>
+      </c>
+      <c r="D1554" s="0" t="inlineStr">
+        <is>
+          <t>birth_flowers</t>
+        </is>
+      </c>
+      <c r="E1554" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1554" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1555">
+      <c r="A1555" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1555" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1555" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalpotato_day</t>
+        </is>
+      </c>
+      <c r="D1555" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalpotato_day</t>
+        </is>
+      </c>
+      <c r="E1555" s="2">
+        <v>5</v>
+      </c>
+      <c r="F1555" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1556">
+      <c r="A1556" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1556" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1556" s="0" t="inlineStr">
+        <is>
+          <t>foreveryone</t>
+        </is>
+      </c>
+      <c r="D1556" s="0" t="inlineStr">
+        <is>
+          <t>congrats_foreveryone</t>
+        </is>
+      </c>
+      <c r="E1556" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1556" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1557">
+      <c r="A1557" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1557" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C1557" s="0" t="inlineStr">
+        <is>
+          <t>hugs</t>
+        </is>
+      </c>
+      <c r="D1557" s="0" t="inlineStr">
+        <is>
+          <t>cute_hugs</t>
+        </is>
+      </c>
+      <c r="E1557" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1557" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1558">
+      <c r="A1558" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1558" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1558" s="0" t="inlineStr">
+        <is>
+          <t>eaug_romawaremonth</t>
+        </is>
+      </c>
+      <c r="D1558" s="0" t="inlineStr">
+        <is>
+          <t>eaug_romawaremonth</t>
+        </is>
+      </c>
+      <c r="E1558" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1558" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1559">
+      <c r="A1559" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1559" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1559" s="0" t="inlineStr">
+        <is>
+          <t>eaug_softice_cream_day</t>
+        </is>
+      </c>
+      <c r="D1559" s="0" t="inlineStr">
+        <is>
+          <t>eaug_softice_cream_day</t>
+        </is>
+      </c>
+      <c r="E1559" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1559" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1560">
+      <c r="A1560" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1560" s="0" t="inlineStr">
+        <is>
+          <t>Family &amp; loved ones</t>
+        </is>
+      </c>
+      <c r="C1560" s="0" t="inlineStr">
+        <is>
+          <t>lovedones</t>
+        </is>
+      </c>
+      <c r="D1560" s="0" t="inlineStr">
+        <is>
+          <t>fkt_lovedones</t>
+        </is>
+      </c>
+      <c r="E1560" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1560" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1561">
+      <c r="A1561" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1561" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1561" s="0" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="D1561" s="0" t="inlineStr">
+        <is>
+          <t>gen_hi</t>
+        </is>
+      </c>
+      <c r="E1561" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1561" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1562">
+      <c r="A1562" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1562" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1562" s="0" t="inlineStr">
+        <is>
+          <t>hvgtday</t>
+        </is>
+      </c>
+      <c r="D1562" s="0" t="inlineStr">
+        <is>
+          <t>gen_hvgtday</t>
+        </is>
+      </c>
+      <c r="E1562" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1562" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1563">
+      <c r="A1563" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1563" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1563" s="0" t="inlineStr">
+        <is>
+          <t>quotesmessages_images_getwell_images</t>
+        </is>
+      </c>
+      <c r="D1563" s="0" t="inlineStr">
+        <is>
+          <t>gen_quotesmessages_images_getwell_images</t>
+        </is>
+      </c>
+      <c r="E1563" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1563" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1564">
+      <c r="A1564" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1564" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1564" s="0" t="inlineStr">
+        <is>
+          <t>stressbusters</t>
+        </is>
+      </c>
+      <c r="D1564" s="0" t="inlineStr">
+        <is>
+          <t>insp_stressbusters</t>
+        </is>
+      </c>
+      <c r="E1564" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1564" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1565">
+      <c r="A1565" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1565" s="0" t="inlineStr">
+        <is>
+          <t>Keeping in touch</t>
+        </is>
+      </c>
+      <c r="C1565" s="0" t="inlineStr">
+        <is>
+          <t>thinkingofyou</t>
+        </is>
+      </c>
+      <c r="D1565" s="0" t="inlineStr">
+        <is>
+          <t>intouch_thinkingofyou</t>
+        </is>
+      </c>
+      <c r="E1565" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1565" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1566">
+      <c r="A1566" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1566" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1566" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_general</t>
+        </is>
+      </c>
+      <c r="D1566" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_general</t>
+        </is>
+      </c>
+      <c r="E1566" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1566" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1567">
+      <c r="A1567" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1567" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1567" s="0" t="inlineStr">
+        <is>
+          <t>wedding</t>
+        </is>
+      </c>
+      <c r="D1567" s="0" t="inlineStr">
+        <is>
+          <t>thank_wedding</t>
+        </is>
+      </c>
+      <c r="E1567" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1567" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1568">
+      <c r="A1568" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1568" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1568" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalaviation_day</t>
+        </is>
+      </c>
+      <c r="D1568" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalaviation_day</t>
+        </is>
+      </c>
+      <c r="E1568" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1568" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1569">
+      <c r="A1569" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1569" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1569" s="0" t="inlineStr">
+        <is>
+          <t>voyage</t>
+        </is>
+      </c>
+      <c r="D1569" s="0" t="inlineStr">
+        <is>
+          <t>gen_voyage</t>
+        </is>
+      </c>
+      <c r="E1569" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1569" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1570">
+      <c r="A1570" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1570" s="0" t="inlineStr">
+        <is>
+          <t>Inspirational &amp; sympathy</t>
+        </is>
+      </c>
+      <c r="C1570" s="0" t="inlineStr">
+        <is>
+          <t>recovery</t>
+        </is>
+      </c>
+      <c r="D1570" s="0" t="inlineStr">
+        <is>
+          <t>insp_recovery</t>
+        </is>
+      </c>
+      <c r="E1570" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1570" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1571">
+      <c r="A1571" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1571" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1571" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="D1571" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_couples</t>
+        </is>
+      </c>
+      <c r="E1571" s="2">
+        <v>3</v>
+      </c>
+      <c r="F1571" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1572">
+      <c r="A1572" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1572" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1572" s="0" t="inlineStr">
+        <is>
+          <t>hubbywife</t>
+        </is>
+      </c>
+      <c r="D1572" s="0" t="inlineStr">
+        <is>
+          <t>birth_hubbywife</t>
+        </is>
+      </c>
+      <c r="E1572" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1572" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1573">
+      <c r="A1573" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1573" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1573" s="0" t="inlineStr">
+        <is>
+          <t>specials</t>
+        </is>
+      </c>
+      <c r="D1573" s="0" t="inlineStr">
+        <is>
+          <t>birth_specials</t>
+        </is>
+      </c>
+      <c r="E1573" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1573" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1574">
+      <c r="A1574" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1574" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1574" s="0" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="D1574" s="0" t="inlineStr">
+        <is>
+          <t>congrats_engagement</t>
+        </is>
+      </c>
+      <c r="E1574" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1574" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1575">
+      <c r="A1575" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1575" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1575" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalwaffle_day</t>
+        </is>
+      </c>
+      <c r="D1575" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalwaffle_day</t>
+        </is>
+      </c>
+      <c r="E1575" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1575" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1576">
+      <c r="A1576" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1576" s="0" t="inlineStr">
+        <is>
+          <t>Flowers</t>
+        </is>
+      </c>
+      <c r="C1576" s="0" t="inlineStr">
+        <is>
+          <t>roses</t>
+        </is>
+      </c>
+      <c r="D1576" s="0" t="inlineStr">
+        <is>
+          <t>flwr_roses</t>
+        </is>
+      </c>
+      <c r="E1576" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1576" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1577">
+      <c r="A1577" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1577" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1577" s="0" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="D1577" s="0" t="inlineStr">
+        <is>
+          <t>gen_luck</t>
+        </is>
+      </c>
+      <c r="E1577" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1577" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1578">
+      <c r="A1578" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1578" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1578" s="0" t="inlineStr">
+        <is>
+          <t>iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="D1578" s="0" t="inlineStr">
+        <is>
+          <t>love_iloveyou_crazy</t>
+        </is>
+      </c>
+      <c r="E1578" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1578" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1579">
+      <c r="A1579" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1579" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1579" s="0" t="inlineStr">
+        <is>
+          <t>sweetheart</t>
+        </is>
+      </c>
+      <c r="D1579" s="0" t="inlineStr">
+        <is>
+          <t>love_sweetheart</t>
+        </is>
+      </c>
+      <c r="E1579" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1579" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1580">
+      <c r="A1580" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1580" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1580" s="0" t="inlineStr">
+        <is>
+          <t>inspirational</t>
+        </is>
+      </c>
+      <c r="D1580" s="0" t="inlineStr">
+        <is>
+          <t>thank_inspirational</t>
+        </is>
+      </c>
+      <c r="E1580" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1580" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1581">
+      <c r="A1581" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1581" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1581" s="0" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="D1581" s="0" t="inlineStr">
+        <is>
+          <t>thank_love</t>
+        </is>
+      </c>
+      <c r="E1581" s="2">
+        <v>2</v>
+      </c>
+      <c r="F1581" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1582">
+      <c r="A1582" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1582" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1582" s="0" t="inlineStr">
+        <is>
+          <t>friends</t>
+        </is>
+      </c>
+      <c r="D1582" s="0" t="inlineStr">
+        <is>
+          <t>birth_friends</t>
+        </is>
+      </c>
+      <c r="E1582" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1582" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1583">
+      <c r="A1583" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1583" s="0" t="inlineStr">
+        <is>
+          <t>Birthday</t>
+        </is>
+      </c>
+      <c r="C1583" s="0" t="inlineStr">
+        <is>
+          <t>momndad</t>
+        </is>
+      </c>
+      <c r="D1583" s="0" t="inlineStr">
+        <is>
+          <t>birth_momndad</t>
+        </is>
+      </c>
+      <c r="E1583" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1583" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1584">
+      <c r="A1584" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1584" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C1584" s="0" t="inlineStr">
+        <is>
+          <t>apologies</t>
+        </is>
+      </c>
+      <c r="D1584" s="0" t="inlineStr">
+        <is>
+          <t>bus_apologies</t>
+        </is>
+      </c>
+      <c r="E1584" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1584" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1585">
+      <c r="A1585" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1585" s="0" t="inlineStr">
+        <is>
+          <t>Business &amp; work</t>
+        </is>
+      </c>
+      <c r="C1585" s="0" t="inlineStr">
+        <is>
+          <t>appreciate</t>
+        </is>
+      </c>
+      <c r="D1585" s="0" t="inlineStr">
+        <is>
+          <t>bus_appreciate</t>
+        </is>
+      </c>
+      <c r="E1585" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1585" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1586">
+      <c r="A1586" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1586" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1586" s="0" t="inlineStr">
+        <is>
+          <t>newbaby</t>
+        </is>
+      </c>
+      <c r="D1586" s="0" t="inlineStr">
+        <is>
+          <t>congrats_newbaby</t>
+        </is>
+      </c>
+      <c r="E1586" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1586" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1587">
+      <c r="A1587" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1587" s="0" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="C1587" s="0" t="inlineStr">
+        <is>
+          <t>studentsandnewgrads</t>
+        </is>
+      </c>
+      <c r="D1587" s="0" t="inlineStr">
+        <is>
+          <t>congrats_studentsandnewgrads</t>
+        </is>
+      </c>
+      <c r="E1587" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1587" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1588">
+      <c r="A1588" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1588" s="0" t="inlineStr">
+        <is>
+          <t>Cute</t>
+        </is>
+      </c>
+      <c r="C1588" s="0" t="inlineStr">
+        <is>
+          <t>smile</t>
+        </is>
+      </c>
+      <c r="D1588" s="0" t="inlineStr">
+        <is>
+          <t>cute_smile</t>
+        </is>
+      </c>
+      <c r="E1588" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1588" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1589">
+      <c r="A1589" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1589" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1589" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipweek</t>
+        </is>
+      </c>
+      <c r="D1589" s="0" t="inlineStr">
+        <is>
+          <t>eaug_friendshipweek</t>
+        </is>
+      </c>
+      <c r="E1589" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1589" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1590">
+      <c r="A1590" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1590" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1590" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalradio_day</t>
+        </is>
+      </c>
+      <c r="D1590" s="0" t="inlineStr">
+        <is>
+          <t>eaug_nationalradio_day</t>
+        </is>
+      </c>
+      <c r="E1590" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1590" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1591">
+      <c r="A1591" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1591" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1591" s="0" t="inlineStr">
+        <is>
+          <t>ejan_danceday</t>
+        </is>
+      </c>
+      <c r="D1591" s="0" t="inlineStr">
+        <is>
+          <t>ejan_danceday</t>
+        </is>
+      </c>
+      <c r="E1591" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1591" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1592">
+      <c r="A1592" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1592" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1592" s="0" t="inlineStr">
+        <is>
+          <t>emay_graduation_wishes</t>
+        </is>
+      </c>
+      <c r="D1592" s="0" t="inlineStr">
+        <is>
+          <t>emay_graduation_wishes</t>
+        </is>
+      </c>
+      <c r="E1592" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1592" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1593">
+      <c r="A1593" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1593" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1593" s="0" t="inlineStr">
+        <is>
+          <t>eoct_sweetday_missyou</t>
+        </is>
+      </c>
+      <c r="D1593" s="0" t="inlineStr">
+        <is>
+          <t>eoct_sweetday_missyou</t>
+        </is>
+      </c>
+      <c r="E1593" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1593" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1594">
+      <c r="A1594" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1594" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1594" s="0" t="inlineStr">
+        <is>
+          <t>eoct_sweetday_romance</t>
+        </is>
+      </c>
+      <c r="D1594" s="0" t="inlineStr">
+        <is>
+          <t>eoct_sweetday_romance</t>
+        </is>
+      </c>
+      <c r="E1594" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1594" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1595">
+      <c r="A1595" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1595" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1595" s="0" t="inlineStr">
+        <is>
+          <t>esep_fall_specials</t>
+        </is>
+      </c>
+      <c r="D1595" s="0" t="inlineStr">
+        <is>
+          <t>esep_fall_specials</t>
+        </is>
+      </c>
+      <c r="E1595" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1595" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1596">
+      <c r="A1596" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1596" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C1596" s="0" t="inlineStr">
+        <is>
+          <t>teenfriends</t>
+        </is>
+      </c>
+      <c r="D1596" s="0" t="inlineStr">
+        <is>
+          <t>friend_teenfriends</t>
+        </is>
+      </c>
+      <c r="E1596" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1596" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1597">
+      <c r="A1597" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1597" s="0" t="inlineStr">
+        <is>
+          <t>Friendship</t>
+        </is>
+      </c>
+      <c r="C1597" s="0" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
+      <c r="D1597" s="0" t="inlineStr">
+        <is>
+          <t>friend_thoughts</t>
+        </is>
+      </c>
+      <c r="E1597" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1597" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1598">
+      <c r="A1598" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1598" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1598" s="0" t="inlineStr">
+        <is>
+          <t>midcrisis</t>
+        </is>
+      </c>
+      <c r="D1598" s="0" t="inlineStr">
+        <is>
+          <t>gen_midcrisis</t>
+        </is>
+      </c>
+      <c r="E1598" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1598" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1599">
+      <c r="A1599" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1599" s="0" t="inlineStr">
+        <is>
+          <t>Everyday greetings</t>
+        </is>
+      </c>
+      <c r="C1599" s="0" t="inlineStr">
+        <is>
+          <t>quotesmessages_images_getwell_quotes</t>
+        </is>
+      </c>
+      <c r="D1599" s="0" t="inlineStr">
+        <is>
+          <t>gen_quotesmessages_images_getwell_quotes</t>
+        </is>
+      </c>
+      <c r="E1599" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1599" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1600">
+      <c r="A1600" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1600" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1600" s="0" t="inlineStr">
+        <is>
+          <t>loveetc</t>
+        </is>
+      </c>
+      <c r="D1600" s="0" t="inlineStr">
+        <is>
+          <t>love_loveetc</t>
+        </is>
+      </c>
+      <c r="E1600" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1600" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1601">
+      <c r="A1601" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1601" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1601" s="0" t="inlineStr">
+        <is>
+          <t>missing_forher</t>
+        </is>
+      </c>
+      <c r="D1601" s="0" t="inlineStr">
+        <is>
+          <t>love_missing_forher</t>
+        </is>
+      </c>
+      <c r="E1601" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1601" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1602">
+      <c r="A1602" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1602" s="0" t="inlineStr">
+        <is>
+          <t>Love &amp; romance</t>
+        </is>
+      </c>
+      <c r="C1602" s="0" t="inlineStr">
+        <is>
+          <t>newlove</t>
+        </is>
+      </c>
+      <c r="D1602" s="0" t="inlineStr">
+        <is>
+          <t>love_newlove</t>
+        </is>
+      </c>
+      <c r="E1602" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1602" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1603">
+      <c r="A1603" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1603" s="0" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="C1603" s="0" t="inlineStr">
+        <is>
+          <t>getwell</t>
+        </is>
+      </c>
+      <c r="D1603" s="0" t="inlineStr">
+        <is>
+          <t>pet_getwell</t>
+        </is>
+      </c>
+      <c r="E1603" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1603" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1604">
+      <c r="A1604" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1604" s="0" t="inlineStr">
+        <is>
+          <t>Thank you</t>
+        </is>
+      </c>
+      <c r="C1604" s="0" t="inlineStr">
+        <is>
+          <t>flower</t>
+        </is>
+      </c>
+      <c r="D1604" s="0" t="inlineStr">
+        <is>
+          <t>thank_flower</t>
+        </is>
+      </c>
+      <c r="E1604" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1604" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1605">
+      <c r="A1605" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1605" s="0" t="inlineStr">
+        <is>
+          <t>World languages</t>
+        </is>
+      </c>
+      <c r="C1605" s="0" t="inlineStr">
+        <is>
+          <t>german_birthday</t>
+        </is>
+      </c>
+      <c r="D1605" s="0" t="inlineStr">
+        <is>
+          <t>w_german_birthday</t>
+        </is>
+      </c>
+      <c r="E1605" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1605" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1606">
+      <c r="A1606" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1606" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1606" s="0" t="inlineStr">
+        <is>
+          <t>wed_wed_congrats</t>
+        </is>
+      </c>
+      <c r="D1606" s="0" t="inlineStr">
+        <is>
+          <t>wed_wed_congrats</t>
+        </is>
+      </c>
+      <c r="E1606" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1606" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1607">
+      <c r="A1607" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL 2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1607" s="4"/>
+      <c r="C1607" s="4"/>
+      <c r="D1607" s="4"/>
+      <c r="E1607" s="5">
+        <v>730</v>
+      </c>
+      <c r="F1607" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -54300,36 +56953,70 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B20" s="2">
+        <v>773</v>
+      </c>
+      <c r="C20" s="2">
+        <v>237</v>
+      </c>
+      <c r="D20" s="2">
+        <v>242</v>
+      </c>
+      <c r="E20" s="2">
+        <v>148</v>
+      </c>
+      <c r="F20" s="2">
+        <v>82</v>
+      </c>
+      <c r="G20" s="2">
+        <v>42</v>
+      </c>
+      <c r="H20" s="2">
+        <v>22</v>
+      </c>
+      <c r="I20" s="2">
+        <v>0</v>
+      </c>
+      <c r="J20" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B20" s="5">
-        <v>14795</v>
-      </c>
-      <c r="C20" s="5">
-        <v>4703</v>
-      </c>
-      <c r="D20" s="5">
-        <v>4614</v>
-      </c>
-      <c r="E20" s="5">
-        <v>2926</v>
-      </c>
-      <c r="F20" s="5">
-        <v>1467</v>
-      </c>
-      <c r="G20" s="5">
-        <v>591</v>
-      </c>
-      <c r="H20" s="5">
-        <v>465</v>
-      </c>
-      <c r="I20" s="5">
+      <c r="B21" s="5">
+        <v>15568</v>
+      </c>
+      <c r="C21" s="5">
+        <v>4940</v>
+      </c>
+      <c r="D21" s="5">
+        <v>4856</v>
+      </c>
+      <c r="E21" s="5">
+        <v>3074</v>
+      </c>
+      <c r="F21" s="5">
+        <v>1549</v>
+      </c>
+      <c r="G21" s="5">
+        <v>633</v>
+      </c>
+      <c r="H21" s="5">
+        <v>487</v>
+      </c>
+      <c r="I21" s="5">
         <v>28</v>
       </c>
-      <c r="J20" s="5">
+      <c r="J21" s="5">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Categorise 128777 and add the two cards published beside it
128777 is love_iloveyou_kisses, published 2026-08-21 01:04:38 and first
sent at 09:37 the same morning. It was the only real card in twenty-one
days with no q1_value; its 4 sends move from uncategorised into Love &
romance, and iloveyou_kisses appears as a sub-category for the first time.

128778 gen_monblues and 128779 love_foreverlove came in the same export and
have no sends yet. Zero recategorisations against the 107,206 already
there; the catalogue is now 107,209.

Every card id in the tracker now maps. What remains uncategorised is the
pivot's 'desktop' row alone - 696 sends over twenty-one days, sitting only
in the two (Desktop) columns, which is the surface total rather than a card
and needs the card number captured upstream.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9KsXegBwxB1sWdCzRVLrr
</commit_message>
<xml_diff>
--- a/reports/daily_tracking.xlsx
+++ b/reports/daily_tracking.xlsx
@@ -886,10 +886,10 @@
         <v>228</v>
       </c>
       <c r="E22" s="2">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="F22" s="2">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="G22" s="2">
         <v>255</v>
@@ -914,10 +914,10 @@
         <v>5684</v>
       </c>
       <c r="E23" s="5">
-        <v>16395</v>
+        <v>16399</v>
       </c>
       <c r="F23" s="5">
-        <v>700</v>
+        <v>696</v>
       </c>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -2274,7 +2274,7 @@
         </is>
       </c>
       <c r="B22" s="2">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="C22" s="2">
         <v>506</v>
@@ -2292,7 +2292,7 @@
         <v>21</v>
       </c>
       <c r="H22" s="2">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I22" s="2">
         <v>11</v>
@@ -2335,7 +2335,7 @@
         </is>
       </c>
       <c r="B23" s="5">
-        <v>16395</v>
+        <v>16399</v>
       </c>
       <c r="C23" s="5">
         <v>10803</v>
@@ -2353,7 +2353,7 @@
         <v>590</v>
       </c>
       <c r="H23" s="5">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="I23" s="5">
         <v>341</v>
@@ -12258,7 +12258,7 @@
         <v>506</v>
       </c>
       <c r="G314" s="3">
-        <v>0.6884353741496598</v>
+        <v>0.6847090663058186</v>
       </c>
       <c r="H314" s="2">
         <v>123</v>
@@ -12290,7 +12290,7 @@
         <v>55</v>
       </c>
       <c r="G315" s="3">
-        <v>0.07482993197278912</v>
+        <v>0.07442489851150202</v>
       </c>
       <c r="H315" s="2">
         <v>26</v>
@@ -12322,7 +12322,7 @@
         <v>43</v>
       </c>
       <c r="G316" s="3">
-        <v>0.058503401360544216</v>
+        <v>0.058186738836265225</v>
       </c>
       <c r="H316" s="2">
         <v>22</v>
@@ -12354,7 +12354,7 @@
         <v>25</v>
       </c>
       <c r="G317" s="3">
-        <v>0.034013605442176874</v>
+        <v>0.03382949932341001</v>
       </c>
       <c r="H317" s="2">
         <v>18</v>
@@ -12386,7 +12386,7 @@
         <v>25</v>
       </c>
       <c r="G318" s="3">
-        <v>0.034013605442176874</v>
+        <v>0.03382949932341001</v>
       </c>
       <c r="H318" s="2">
         <v>9</v>
@@ -12418,7 +12418,7 @@
         <v>21</v>
       </c>
       <c r="G319" s="3">
-        <v>0.02857142857142857</v>
+        <v>0.028416779431664412</v>
       </c>
       <c r="H319" s="2">
         <v>9</v>
@@ -12441,19 +12441,19 @@
         </is>
       </c>
       <c r="D320" s="2">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E320" s="2">
         <v>3</v>
       </c>
       <c r="F320" s="2">
+        <v>20</v>
+      </c>
+      <c r="G320" s="3">
+        <v>0.02706359945872801</v>
+      </c>
+      <c r="H320" s="2">
         <v>16</v>
-      </c>
-      <c r="G320" s="3">
-        <v>0.021768707482993196</v>
-      </c>
-      <c r="H320" s="2">
-        <v>15</v>
       </c>
     </row>
     <row r="321">
@@ -12482,7 +12482,7 @@
         <v>15</v>
       </c>
       <c r="G321" s="3">
-        <v>0.02040816326530612</v>
+        <v>0.02029769959404601</v>
       </c>
       <c r="H321" s="2">
         <v>10</v>
@@ -12514,7 +12514,7 @@
         <v>11</v>
       </c>
       <c r="G322" s="3">
-        <v>0.014965986394557823</v>
+        <v>0.014884979702300407</v>
       </c>
       <c r="H322" s="2">
         <v>9</v>
@@ -12546,7 +12546,7 @@
         <v>5</v>
       </c>
       <c r="G323" s="3">
-        <v>0.006802721088435374</v>
+        <v>0.006765899864682003</v>
       </c>
       <c r="H323" s="2">
         <v>2</v>
@@ -12578,7 +12578,7 @@
         <v>5</v>
       </c>
       <c r="G324" s="3">
-        <v>0.006802721088435374</v>
+        <v>0.006765899864682003</v>
       </c>
       <c r="H324" s="2">
         <v>5</v>
@@ -12610,7 +12610,7 @@
         <v>4</v>
       </c>
       <c r="G325" s="3">
-        <v>0.005442176870748299</v>
+        <v>0.005412719891745603</v>
       </c>
       <c r="H325" s="2">
         <v>2</v>
@@ -12642,7 +12642,7 @@
         <v>3</v>
       </c>
       <c r="G326" s="3">
-        <v>0.004081632653061225</v>
+        <v>0.0040595399188092015</v>
       </c>
       <c r="H326" s="2">
         <v>2</v>
@@ -12674,7 +12674,7 @@
         <v>1</v>
       </c>
       <c r="G327" s="3">
-        <v>0.0013605442176870747</v>
+        <v>0.0013531799729364006</v>
       </c>
       <c r="H327" s="2">
         <v>1</v>
@@ -12689,13 +12689,13 @@
       <c r="B328" s="4"/>
       <c r="C328" s="4"/>
       <c r="D328" s="5">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="E328" s="5">
         <v>198</v>
       </c>
       <c r="F328" s="5">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="G328" s="5">
         <v>1.0</v>
@@ -60446,19 +60446,19 @@
       </c>
       <c r="C1715" s="0" t="inlineStr">
         <is>
-          <t>sweetheart</t>
+          <t>iloveyou_kisses</t>
         </is>
       </c>
       <c r="D1715" s="0" t="inlineStr">
         <is>
-          <t>love_sweetheart</t>
+          <t>love_iloveyou_kisses</t>
         </is>
       </c>
       <c r="E1715" s="2">
         <v>4</v>
       </c>
       <c r="F1715" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1716">
@@ -60469,24 +60469,24 @@
       </c>
       <c r="B1716" s="0" t="inlineStr">
         <is>
-          <t>Thank you</t>
+          <t>Love &amp; romance</t>
         </is>
       </c>
       <c r="C1716" s="0" t="inlineStr">
         <is>
-          <t>inspirational</t>
+          <t>sweetheart</t>
         </is>
       </c>
       <c r="D1716" s="0" t="inlineStr">
         <is>
-          <t>thank_inspirational</t>
+          <t>love_sweetheart</t>
         </is>
       </c>
       <c r="E1716" s="2">
         <v>4</v>
       </c>
       <c r="F1716" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="1717">
@@ -60497,24 +60497,24 @@
       </c>
       <c r="B1717" s="0" t="inlineStr">
         <is>
-          <t>Events cards</t>
+          <t>Thank you</t>
         </is>
       </c>
       <c r="C1717" s="0" t="inlineStr">
         <is>
-          <t>wed_flowers</t>
+          <t>inspirational</t>
         </is>
       </c>
       <c r="D1717" s="0" t="inlineStr">
         <is>
-          <t>wed_flowers</t>
+          <t>thank_inspirational</t>
         </is>
       </c>
       <c r="E1717" s="2">
         <v>4</v>
       </c>
       <c r="F1717" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1718">
@@ -60525,24 +60525,24 @@
       </c>
       <c r="B1718" s="0" t="inlineStr">
         <is>
-          <t>Birthday</t>
+          <t>Events cards</t>
         </is>
       </c>
       <c r="C1718" s="0" t="inlineStr">
         <is>
-          <t>milestone</t>
+          <t>wed_flowers</t>
         </is>
       </c>
       <c r="D1718" s="0" t="inlineStr">
         <is>
-          <t>birth_milestone</t>
+          <t>wed_flowers</t>
         </is>
       </c>
       <c r="E1718" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1718" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1719">
@@ -60558,12 +60558,12 @@
       </c>
       <c r="C1719" s="0" t="inlineStr">
         <is>
-          <t>momndad</t>
+          <t>milestone</t>
         </is>
       </c>
       <c r="D1719" s="0" t="inlineStr">
         <is>
-          <t>birth_momndad</t>
+          <t>birth_milestone</t>
         </is>
       </c>
       <c r="E1719" s="2">
@@ -60581,24 +60581,24 @@
       </c>
       <c r="B1720" s="0" t="inlineStr">
         <is>
-          <t>Flowers</t>
+          <t>Birthday</t>
         </is>
       </c>
       <c r="C1720" s="0" t="inlineStr">
         <is>
-          <t>love</t>
+          <t>momndad</t>
         </is>
       </c>
       <c r="D1720" s="0" t="inlineStr">
         <is>
-          <t>flwr_love</t>
+          <t>birth_momndad</t>
         </is>
       </c>
       <c r="E1720" s="2">
         <v>3</v>
       </c>
       <c r="F1720" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1721">
@@ -60609,17 +60609,17 @@
       </c>
       <c r="B1721" s="0" t="inlineStr">
         <is>
-          <t>Everyday greetings</t>
+          <t>Flowers</t>
         </is>
       </c>
       <c r="C1721" s="0" t="inlineStr">
         <is>
-          <t>morningquotes</t>
+          <t>love</t>
         </is>
       </c>
       <c r="D1721" s="0" t="inlineStr">
         <is>
-          <t>gen_morningquotes</t>
+          <t>flwr_love</t>
         </is>
       </c>
       <c r="E1721" s="2">
@@ -60637,24 +60637,24 @@
       </c>
       <c r="B1722" s="0" t="inlineStr">
         <is>
-          <t>Inspirational &amp; sympathy</t>
+          <t>Everyday greetings</t>
         </is>
       </c>
       <c r="C1722" s="0" t="inlineStr">
         <is>
-          <t>encour</t>
+          <t>morningquotes</t>
         </is>
       </c>
       <c r="D1722" s="0" t="inlineStr">
         <is>
-          <t>insp_encour</t>
+          <t>gen_morningquotes</t>
         </is>
       </c>
       <c r="E1722" s="2">
         <v>3</v>
       </c>
       <c r="F1722" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1723">
@@ -60665,24 +60665,24 @@
       </c>
       <c r="B1723" s="0" t="inlineStr">
         <is>
-          <t>Keeping in touch</t>
+          <t>Inspirational &amp; sympathy</t>
         </is>
       </c>
       <c r="C1723" s="0" t="inlineStr">
         <is>
-          <t>thinkingofyou</t>
+          <t>encour</t>
         </is>
       </c>
       <c r="D1723" s="0" t="inlineStr">
         <is>
-          <t>intouch_thinkingofyou</t>
+          <t>insp_encour</t>
         </is>
       </c>
       <c r="E1723" s="2">
         <v>3</v>
       </c>
       <c r="F1723" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1724">
@@ -60693,24 +60693,24 @@
       </c>
       <c r="B1724" s="0" t="inlineStr">
         <is>
-          <t>Pets</t>
+          <t>Keeping in touch</t>
         </is>
       </c>
       <c r="C1724" s="0" t="inlineStr">
         <is>
-          <t>getwell</t>
+          <t>thinkingofyou</t>
         </is>
       </c>
       <c r="D1724" s="0" t="inlineStr">
         <is>
-          <t>pet_getwell</t>
+          <t>intouch_thinkingofyou</t>
         </is>
       </c>
       <c r="E1724" s="2">
         <v>3</v>
       </c>
       <c r="F1724" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1725">
@@ -60721,24 +60721,24 @@
       </c>
       <c r="B1725" s="0" t="inlineStr">
         <is>
-          <t>Thank you</t>
+          <t>Pets</t>
         </is>
       </c>
       <c r="C1725" s="0" t="inlineStr">
         <is>
-          <t>everyday</t>
+          <t>getwell</t>
         </is>
       </c>
       <c r="D1725" s="0" t="inlineStr">
         <is>
-          <t>thank_everyday</t>
+          <t>pet_getwell</t>
         </is>
       </c>
       <c r="E1725" s="2">
         <v>3</v>
       </c>
       <c r="F1725" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1726">
@@ -60754,19 +60754,19 @@
       </c>
       <c r="C1726" s="0" t="inlineStr">
         <is>
-          <t>wedding</t>
+          <t>everyday</t>
         </is>
       </c>
       <c r="D1726" s="0" t="inlineStr">
         <is>
-          <t>thank_wedding</t>
+          <t>thank_everyday</t>
         </is>
       </c>
       <c r="E1726" s="2">
         <v>3</v>
       </c>
       <c r="F1726" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1727">
@@ -60777,21 +60777,21 @@
       </c>
       <c r="B1727" s="0" t="inlineStr">
         <is>
-          <t>Birthday</t>
+          <t>Thank you</t>
         </is>
       </c>
       <c r="C1727" s="0" t="inlineStr">
         <is>
-          <t>flowers</t>
+          <t>wedding</t>
         </is>
       </c>
       <c r="D1727" s="0" t="inlineStr">
         <is>
-          <t>birth_flowers</t>
+          <t>thank_wedding</t>
         </is>
       </c>
       <c r="E1727" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F1727" s="2">
         <v>1</v>
@@ -60810,12 +60810,12 @@
       </c>
       <c r="C1728" s="0" t="inlineStr">
         <is>
-          <t>missyou</t>
+          <t>flowers</t>
         </is>
       </c>
       <c r="D1728" s="0" t="inlineStr">
         <is>
-          <t>birth_missyou</t>
+          <t>birth_flowers</t>
         </is>
       </c>
       <c r="E1728" s="2">
@@ -60838,19 +60838,19 @@
       </c>
       <c r="C1729" s="0" t="inlineStr">
         <is>
-          <t>zodiac</t>
+          <t>missyou</t>
         </is>
       </c>
       <c r="D1729" s="0" t="inlineStr">
         <is>
-          <t>birth_zodiac</t>
+          <t>birth_missyou</t>
         </is>
       </c>
       <c r="E1729" s="2">
         <v>2</v>
       </c>
       <c r="F1729" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1730">
@@ -60861,24 +60861,24 @@
       </c>
       <c r="B1730" s="0" t="inlineStr">
         <is>
-          <t>Congratulations</t>
+          <t>Birthday</t>
         </is>
       </c>
       <c r="C1730" s="0" t="inlineStr">
         <is>
-          <t>newbaby</t>
+          <t>zodiac</t>
         </is>
       </c>
       <c r="D1730" s="0" t="inlineStr">
         <is>
-          <t>congrats_newbaby</t>
+          <t>birth_zodiac</t>
         </is>
       </c>
       <c r="E1730" s="2">
         <v>2</v>
       </c>
       <c r="F1730" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1731">
@@ -60894,19 +60894,19 @@
       </c>
       <c r="C1731" s="0" t="inlineStr">
         <is>
-          <t>newcarandlicense</t>
+          <t>newbaby</t>
         </is>
       </c>
       <c r="D1731" s="0" t="inlineStr">
         <is>
-          <t>congrats_newcarandlicense</t>
+          <t>congrats_newbaby</t>
         </is>
       </c>
       <c r="E1731" s="2">
         <v>2</v>
       </c>
       <c r="F1731" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1732">
@@ -60917,24 +60917,24 @@
       </c>
       <c r="B1732" s="0" t="inlineStr">
         <is>
-          <t>Events cards</t>
+          <t>Congratulations</t>
         </is>
       </c>
       <c r="C1732" s="0" t="inlineStr">
         <is>
-          <t>eaug_hugsweetheartday</t>
+          <t>newcarandlicense</t>
         </is>
       </c>
       <c r="D1732" s="0" t="inlineStr">
         <is>
-          <t>eaug_hugsweetheartday</t>
+          <t>congrats_newcarandlicense</t>
         </is>
       </c>
       <c r="E1732" s="2">
         <v>2</v>
       </c>
       <c r="F1732" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1733">
@@ -60950,12 +60950,12 @@
       </c>
       <c r="C1733" s="0" t="inlineStr">
         <is>
-          <t>esep_flowerofthemonth</t>
+          <t>eaug_hugsweetheartday</t>
         </is>
       </c>
       <c r="D1733" s="0" t="inlineStr">
         <is>
-          <t>esep_flowerofthemonth</t>
+          <t>eaug_hugsweetheartday</t>
         </is>
       </c>
       <c r="E1733" s="2">
@@ -60973,17 +60973,17 @@
       </c>
       <c r="B1734" s="0" t="inlineStr">
         <is>
-          <t>Everyday greetings</t>
+          <t>Events cards</t>
         </is>
       </c>
       <c r="C1734" s="0" t="inlineStr">
         <is>
-          <t>hi</t>
+          <t>esep_flowerofthemonth</t>
         </is>
       </c>
       <c r="D1734" s="0" t="inlineStr">
         <is>
-          <t>gen_hi</t>
+          <t>esep_flowerofthemonth</t>
         </is>
       </c>
       <c r="E1734" s="2">
@@ -61006,19 +61006,19 @@
       </c>
       <c r="C1735" s="0" t="inlineStr">
         <is>
-          <t>hvgtday</t>
+          <t>hi</t>
         </is>
       </c>
       <c r="D1735" s="0" t="inlineStr">
         <is>
-          <t>gen_hvgtday</t>
+          <t>gen_hi</t>
         </is>
       </c>
       <c r="E1735" s="2">
         <v>2</v>
       </c>
       <c r="F1735" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1736">
@@ -61034,12 +61034,12 @@
       </c>
       <c r="C1736" s="0" t="inlineStr">
         <is>
-          <t>morning</t>
+          <t>hvgtday</t>
         </is>
       </c>
       <c r="D1736" s="0" t="inlineStr">
         <is>
-          <t>gen_morning</t>
+          <t>gen_hvgtday</t>
         </is>
       </c>
       <c r="E1736" s="2">
@@ -61057,24 +61057,24 @@
       </c>
       <c r="B1737" s="0" t="inlineStr">
         <is>
-          <t>Keeping in touch</t>
+          <t>Everyday greetings</t>
         </is>
       </c>
       <c r="C1737" s="0" t="inlineStr">
         <is>
-          <t>justbecause</t>
+          <t>morning</t>
         </is>
       </c>
       <c r="D1737" s="0" t="inlineStr">
         <is>
-          <t>intouch_justbecause</t>
+          <t>gen_morning</t>
         </is>
       </c>
       <c r="E1737" s="2">
         <v>2</v>
       </c>
       <c r="F1737" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1738">
@@ -61085,17 +61085,17 @@
       </c>
       <c r="B1738" s="0" t="inlineStr">
         <is>
-          <t>Invitations &amp; parties</t>
+          <t>Keeping in touch</t>
         </is>
       </c>
       <c r="C1738" s="0" t="inlineStr">
         <is>
-          <t>otherinvitations</t>
+          <t>justbecause</t>
         </is>
       </c>
       <c r="D1738" s="0" t="inlineStr">
         <is>
-          <t>invp_otherinvitations</t>
+          <t>intouch_justbecause</t>
         </is>
       </c>
       <c r="E1738" s="2">
@@ -61113,24 +61113,24 @@
       </c>
       <c r="B1739" s="0" t="inlineStr">
         <is>
-          <t>Love &amp; romance</t>
+          <t>Invitations &amp; parties</t>
         </is>
       </c>
       <c r="C1739" s="0" t="inlineStr">
         <is>
-          <t>iloveyou_general</t>
+          <t>otherinvitations</t>
         </is>
       </c>
       <c r="D1739" s="0" t="inlineStr">
         <is>
-          <t>love_iloveyou_general</t>
+          <t>invp_otherinvitations</t>
         </is>
       </c>
       <c r="E1739" s="2">
         <v>2</v>
       </c>
       <c r="F1739" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1740">
@@ -61146,12 +61146,12 @@
       </c>
       <c r="C1740" s="0" t="inlineStr">
         <is>
-          <t>lovepoems</t>
+          <t>iloveyou_general</t>
         </is>
       </c>
       <c r="D1740" s="0" t="inlineStr">
         <is>
-          <t>love_lovepoems</t>
+          <t>love_iloveyou_general</t>
         </is>
       </c>
       <c r="E1740" s="2">
@@ -61169,17 +61169,17 @@
       </c>
       <c r="B1741" s="0" t="inlineStr">
         <is>
-          <t>Thank you</t>
+          <t>Love &amp; romance</t>
         </is>
       </c>
       <c r="C1741" s="0" t="inlineStr">
         <is>
-          <t>love</t>
+          <t>lovepoems</t>
         </is>
       </c>
       <c r="D1741" s="0" t="inlineStr">
         <is>
-          <t>thank_love</t>
+          <t>love_lovepoems</t>
         </is>
       </c>
       <c r="E1741" s="2">
@@ -61197,24 +61197,24 @@
       </c>
       <c r="B1742" s="0" t="inlineStr">
         <is>
-          <t>Anniversary</t>
+          <t>Thank you</t>
         </is>
       </c>
       <c r="C1742" s="0" t="inlineStr">
         <is>
-          <t>ouranniversary_forhim</t>
+          <t>love</t>
         </is>
       </c>
       <c r="D1742" s="0" t="inlineStr">
         <is>
-          <t>anniv_ouranniversary_forhim</t>
+          <t>thank_love</t>
         </is>
       </c>
       <c r="E1742" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1742" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1743">
@@ -61225,17 +61225,17 @@
       </c>
       <c r="B1743" s="0" t="inlineStr">
         <is>
-          <t>Birthday</t>
+          <t>Anniversary</t>
         </is>
       </c>
       <c r="C1743" s="0" t="inlineStr">
         <is>
-          <t>forher</t>
+          <t>ouranniversary_forhim</t>
         </is>
       </c>
       <c r="D1743" s="0" t="inlineStr">
         <is>
-          <t>birth_forher</t>
+          <t>anniv_ouranniversary_forhim</t>
         </is>
       </c>
       <c r="E1743" s="2">
@@ -61258,12 +61258,12 @@
       </c>
       <c r="C1744" s="0" t="inlineStr">
         <is>
-          <t>forhim</t>
+          <t>forher</t>
         </is>
       </c>
       <c r="D1744" s="0" t="inlineStr">
         <is>
-          <t>birth_forhim</t>
+          <t>birth_forher</t>
         </is>
       </c>
       <c r="E1744" s="2">
@@ -61286,12 +61286,12 @@
       </c>
       <c r="C1745" s="0" t="inlineStr">
         <is>
-          <t>grandparents</t>
+          <t>forhim</t>
         </is>
       </c>
       <c r="D1745" s="0" t="inlineStr">
         <is>
-          <t>birth_grandparents</t>
+          <t>birth_forhim</t>
         </is>
       </c>
       <c r="E1745" s="2">
@@ -61314,12 +61314,12 @@
       </c>
       <c r="C1746" s="0" t="inlineStr">
         <is>
-          <t>hubbywife</t>
+          <t>grandparents</t>
         </is>
       </c>
       <c r="D1746" s="0" t="inlineStr">
         <is>
-          <t>birth_hubbywife</t>
+          <t>birth_grandparents</t>
         </is>
       </c>
       <c r="E1746" s="2">
@@ -61342,12 +61342,12 @@
       </c>
       <c r="C1747" s="0" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>hubbywife</t>
         </is>
       </c>
       <c r="D1747" s="0" t="inlineStr">
         <is>
-          <t>birth_kids</t>
+          <t>birth_hubbywife</t>
         </is>
       </c>
       <c r="E1747" s="2">
@@ -61370,12 +61370,12 @@
       </c>
       <c r="C1748" s="0" t="inlineStr">
         <is>
-          <t>specials</t>
+          <t>kids</t>
         </is>
       </c>
       <c r="D1748" s="0" t="inlineStr">
         <is>
-          <t>birth_specials</t>
+          <t>birth_kids</t>
         </is>
       </c>
       <c r="E1748" s="2">
@@ -61393,17 +61393,17 @@
       </c>
       <c r="B1749" s="0" t="inlineStr">
         <is>
-          <t>Business &amp; work</t>
+          <t>Birthday</t>
         </is>
       </c>
       <c r="C1749" s="0" t="inlineStr">
         <is>
-          <t>humor</t>
+          <t>specials</t>
         </is>
       </c>
       <c r="D1749" s="0" t="inlineStr">
         <is>
-          <t>bus_humor</t>
+          <t>birth_specials</t>
         </is>
       </c>
       <c r="E1749" s="2">
@@ -61421,17 +61421,17 @@
       </c>
       <c r="B1750" s="0" t="inlineStr">
         <is>
-          <t>Congratulations</t>
+          <t>Business &amp; work</t>
         </is>
       </c>
       <c r="C1750" s="0" t="inlineStr">
         <is>
-          <t>onotheroccasions</t>
+          <t>humor</t>
         </is>
       </c>
       <c r="D1750" s="0" t="inlineStr">
         <is>
-          <t>congrats_onotheroccasions</t>
+          <t>bus_humor</t>
         </is>
       </c>
       <c r="E1750" s="2">
@@ -61449,17 +61449,17 @@
       </c>
       <c r="B1751" s="0" t="inlineStr">
         <is>
-          <t>Events cards</t>
+          <t>Congratulations</t>
         </is>
       </c>
       <c r="C1751" s="0" t="inlineStr">
         <is>
-          <t>eapr_goodfriday</t>
+          <t>onotheroccasions</t>
         </is>
       </c>
       <c r="D1751" s="0" t="inlineStr">
         <is>
-          <t>eapr_goodfriday</t>
+          <t>congrats_onotheroccasions</t>
         </is>
       </c>
       <c r="E1751" s="2">
@@ -61482,12 +61482,12 @@
       </c>
       <c r="C1752" s="0" t="inlineStr">
         <is>
-          <t>eaug_bananasplit_day</t>
+          <t>eapr_goodfriday</t>
         </is>
       </c>
       <c r="D1752" s="0" t="inlineStr">
         <is>
-          <t>eaug_bananasplit_day</t>
+          <t>eapr_goodfriday</t>
         </is>
       </c>
       <c r="E1752" s="2">
@@ -61510,12 +61510,12 @@
       </c>
       <c r="C1753" s="0" t="inlineStr">
         <is>
-          <t>eaug_beanangelday</t>
+          <t>eaug_bananasplit_day</t>
         </is>
       </c>
       <c r="D1753" s="0" t="inlineStr">
         <is>
-          <t>eaug_beanangelday</t>
+          <t>eaug_bananasplit_day</t>
         </is>
       </c>
       <c r="E1753" s="2">
@@ -61538,12 +61538,12 @@
       </c>
       <c r="C1754" s="0" t="inlineStr">
         <is>
-          <t>eaug_cardssister</t>
+          <t>eaug_beanangelday</t>
         </is>
       </c>
       <c r="D1754" s="0" t="inlineStr">
         <is>
-          <t>eaug_cardssister</t>
+          <t>eaug_beanangelday</t>
         </is>
       </c>
       <c r="E1754" s="2">
@@ -61566,12 +61566,12 @@
       </c>
       <c r="C1755" s="0" t="inlineStr">
         <is>
-          <t>eaug_friendshipday_happy</t>
+          <t>eaug_cardssister</t>
         </is>
       </c>
       <c r="D1755" s="0" t="inlineStr">
         <is>
-          <t>eaug_friendshipday_happy</t>
+          <t>eaug_cardssister</t>
         </is>
       </c>
       <c r="E1755" s="2">
@@ -61594,12 +61594,12 @@
       </c>
       <c r="C1756" s="0" t="inlineStr">
         <is>
-          <t>eaug_rakshabandhan_happy</t>
+          <t>eaug_friendshipday_happy</t>
         </is>
       </c>
       <c r="D1756" s="0" t="inlineStr">
         <is>
-          <t>eaug_rakshabandhan_happy</t>
+          <t>eaug_friendshipday_happy</t>
         </is>
       </c>
       <c r="E1756" s="2">
@@ -61622,12 +61622,12 @@
       </c>
       <c r="C1757" s="0" t="inlineStr">
         <is>
-          <t>eaug_rakshabandhan_interactive</t>
+          <t>eaug_rakshabandhan_happy</t>
         </is>
       </c>
       <c r="D1757" s="0" t="inlineStr">
         <is>
-          <t>eaug_rakshabandhan_interactive</t>
+          <t>eaug_rakshabandhan_happy</t>
         </is>
       </c>
       <c r="E1757" s="2">
@@ -61650,12 +61650,12 @@
       </c>
       <c r="C1758" s="0" t="inlineStr">
         <is>
-          <t>eaug_romawaremonth</t>
+          <t>eaug_rakshabandhan_interactive</t>
         </is>
       </c>
       <c r="D1758" s="0" t="inlineStr">
         <is>
-          <t>eaug_romawaremonth</t>
+          <t>eaug_rakshabandhan_interactive</t>
         </is>
       </c>
       <c r="E1758" s="2">
@@ -61678,12 +61678,12 @@
       </c>
       <c r="C1759" s="0" t="inlineStr">
         <is>
-          <t>eaug_womensequality_day</t>
+          <t>eaug_romawaremonth</t>
         </is>
       </c>
       <c r="D1759" s="0" t="inlineStr">
         <is>
-          <t>eaug_womensequality_day</t>
+          <t>eaug_romawaremonth</t>
         </is>
       </c>
       <c r="E1759" s="2">
@@ -61706,12 +61706,12 @@
       </c>
       <c r="C1760" s="0" t="inlineStr">
         <is>
-          <t>ejan_thankyoucards</t>
+          <t>eaug_womensequality_day</t>
         </is>
       </c>
       <c r="D1760" s="0" t="inlineStr">
         <is>
-          <t>ejan_thankyoucards</t>
+          <t>eaug_womensequality_day</t>
         </is>
       </c>
       <c r="E1760" s="2">
@@ -61734,12 +61734,12 @@
       </c>
       <c r="C1761" s="0" t="inlineStr">
         <is>
-          <t>eoct_nationaliloveyou_day</t>
+          <t>ejan_thankyoucards</t>
         </is>
       </c>
       <c r="D1761" s="0" t="inlineStr">
         <is>
-          <t>eoct_nationaliloveyou_day</t>
+          <t>ejan_thankyoucards</t>
         </is>
       </c>
       <c r="E1761" s="2">
@@ -61762,12 +61762,12 @@
       </c>
       <c r="C1762" s="0" t="inlineStr">
         <is>
-          <t>eoct_sweetday_hugnkiss</t>
+          <t>eoct_nationaliloveyou_day</t>
         </is>
       </c>
       <c r="D1762" s="0" t="inlineStr">
         <is>
-          <t>eoct_sweetday_hugnkiss</t>
+          <t>eoct_nationaliloveyou_day</t>
         </is>
       </c>
       <c r="E1762" s="2">
@@ -61790,12 +61790,12 @@
       </c>
       <c r="C1763" s="0" t="inlineStr">
         <is>
-          <t>esep_fall_poem</t>
+          <t>eoct_sweetday_hugnkiss</t>
         </is>
       </c>
       <c r="D1763" s="0" t="inlineStr">
         <is>
-          <t>esep_fall_poem</t>
+          <t>eoct_sweetday_hugnkiss</t>
         </is>
       </c>
       <c r="E1763" s="2">
@@ -61813,17 +61813,17 @@
       </c>
       <c r="B1764" s="0" t="inlineStr">
         <is>
-          <t>Flowers</t>
+          <t>Events cards</t>
         </is>
       </c>
       <c r="C1764" s="0" t="inlineStr">
         <is>
-          <t>flrwishes</t>
+          <t>esep_fall_poem</t>
         </is>
       </c>
       <c r="D1764" s="0" t="inlineStr">
         <is>
-          <t>flwr_flrwishes</t>
+          <t>esep_fall_poem</t>
         </is>
       </c>
       <c r="E1764" s="2">
@@ -61841,17 +61841,17 @@
       </c>
       <c r="B1765" s="0" t="inlineStr">
         <is>
-          <t>Everyday greetings</t>
+          <t>Flowers</t>
         </is>
       </c>
       <c r="C1765" s="0" t="inlineStr">
         <is>
-          <t>goodnight</t>
+          <t>flrwishes</t>
         </is>
       </c>
       <c r="D1765" s="0" t="inlineStr">
         <is>
-          <t>gen_goodnight</t>
+          <t>flwr_flrwishes</t>
         </is>
       </c>
       <c r="E1765" s="2">
@@ -61874,12 +61874,12 @@
       </c>
       <c r="C1766" s="0" t="inlineStr">
         <is>
-          <t>quotesmessages_images_getwell_messages</t>
+          <t>goodnight</t>
         </is>
       </c>
       <c r="D1766" s="0" t="inlineStr">
         <is>
-          <t>gen_quotesmessages_images_getwell_messages</t>
+          <t>gen_goodnight</t>
         </is>
       </c>
       <c r="E1766" s="2">
@@ -61902,12 +61902,12 @@
       </c>
       <c r="C1767" s="0" t="inlineStr">
         <is>
-          <t>sorry</t>
+          <t>quotesmessages_images_getwell_messages</t>
         </is>
       </c>
       <c r="D1767" s="0" t="inlineStr">
         <is>
-          <t>gen_sorry</t>
+          <t>gen_quotesmessages_images_getwell_messages</t>
         </is>
       </c>
       <c r="E1767" s="2">
@@ -61930,12 +61930,12 @@
       </c>
       <c r="C1768" s="0" t="inlineStr">
         <is>
-          <t>voyage</t>
+          <t>sorry</t>
         </is>
       </c>
       <c r="D1768" s="0" t="inlineStr">
         <is>
-          <t>gen_voyage</t>
+          <t>gen_sorry</t>
         </is>
       </c>
       <c r="E1768" s="2">
@@ -61958,12 +61958,12 @@
       </c>
       <c r="C1769" s="0" t="inlineStr">
         <is>
-          <t>weekend</t>
+          <t>voyage</t>
         </is>
       </c>
       <c r="D1769" s="0" t="inlineStr">
         <is>
-          <t>gen_weekend</t>
+          <t>gen_voyage</t>
         </is>
       </c>
       <c r="E1769" s="2">
@@ -61981,17 +61981,17 @@
       </c>
       <c r="B1770" s="0" t="inlineStr">
         <is>
-          <t>Inspirational &amp; sympathy</t>
+          <t>Everyday greetings</t>
         </is>
       </c>
       <c r="C1770" s="0" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>weekend</t>
         </is>
       </c>
       <c r="D1770" s="0" t="inlineStr">
         <is>
-          <t>insp_health</t>
+          <t>gen_weekend</t>
         </is>
       </c>
       <c r="E1770" s="2">
@@ -62014,12 +62014,12 @@
       </c>
       <c r="C1771" s="0" t="inlineStr">
         <is>
-          <t>recovery</t>
+          <t>health</t>
         </is>
       </c>
       <c r="D1771" s="0" t="inlineStr">
         <is>
-          <t>insp_recovery</t>
+          <t>insp_health</t>
         </is>
       </c>
       <c r="E1771" s="2">
@@ -62037,17 +62037,17 @@
       </c>
       <c r="B1772" s="0" t="inlineStr">
         <is>
-          <t>Invitations &amp; parties</t>
+          <t>Inspirational &amp; sympathy</t>
         </is>
       </c>
       <c r="C1772" s="0" t="inlineStr">
         <is>
-          <t>birth_gen</t>
+          <t>recovery</t>
         </is>
       </c>
       <c r="D1772" s="0" t="inlineStr">
         <is>
-          <t>invp_birth_gen</t>
+          <t>insp_recovery</t>
         </is>
       </c>
       <c r="E1772" s="2">
@@ -62065,17 +62065,17 @@
       </c>
       <c r="B1773" s="0" t="inlineStr">
         <is>
-          <t>Love &amp; romance</t>
+          <t>Invitations &amp; parties</t>
         </is>
       </c>
       <c r="C1773" s="0" t="inlineStr">
         <is>
-          <t>iloveyou_couples</t>
+          <t>birth_gen</t>
         </is>
       </c>
       <c r="D1773" s="0" t="inlineStr">
         <is>
-          <t>love_iloveyou_couples</t>
+          <t>invp_birth_gen</t>
         </is>
       </c>
       <c r="E1773" s="2">
@@ -62098,12 +62098,12 @@
       </c>
       <c r="C1774" s="0" t="inlineStr">
         <is>
-          <t>missing_forher</t>
+          <t>iloveyou_couples</t>
         </is>
       </c>
       <c r="D1774" s="0" t="inlineStr">
         <is>
-          <t>love_missing_forher</t>
+          <t>love_iloveyou_couples</t>
         </is>
       </c>
       <c r="E1774" s="2">
@@ -62126,12 +62126,12 @@
       </c>
       <c r="C1775" s="0" t="inlineStr">
         <is>
-          <t>newlove</t>
+          <t>missing_forher</t>
         </is>
       </c>
       <c r="D1775" s="0" t="inlineStr">
         <is>
-          <t>love_newlove</t>
+          <t>love_missing_forher</t>
         </is>
       </c>
       <c r="E1775" s="2">
@@ -62149,17 +62149,17 @@
       </c>
       <c r="B1776" s="0" t="inlineStr">
         <is>
-          <t>Pets</t>
+          <t>Love &amp; romance</t>
         </is>
       </c>
       <c r="C1776" s="0" t="inlineStr">
         <is>
-          <t>hihello</t>
+          <t>newlove</t>
         </is>
       </c>
       <c r="D1776" s="0" t="inlineStr">
         <is>
-          <t>pet_hihello</t>
+          <t>love_newlove</t>
         </is>
       </c>
       <c r="E1776" s="2">
@@ -62182,12 +62182,12 @@
       </c>
       <c r="C1777" s="0" t="inlineStr">
         <is>
-          <t>lossofpet</t>
+          <t>hihello</t>
         </is>
       </c>
       <c r="D1777" s="0" t="inlineStr">
         <is>
-          <t>pet_lossofpet</t>
+          <t>pet_hihello</t>
         </is>
       </c>
       <c r="E1777" s="2">
@@ -62205,17 +62205,17 @@
       </c>
       <c r="B1778" s="0" t="inlineStr">
         <is>
-          <t>Events cards</t>
+          <t>Pets</t>
         </is>
       </c>
       <c r="C1778" s="0" t="inlineStr">
         <is>
-          <t>wed_justmarried</t>
+          <t>lossofpet</t>
         </is>
       </c>
       <c r="D1778" s="0" t="inlineStr">
         <is>
-          <t>wed_justmarried</t>
+          <t>pet_lossofpet</t>
         </is>
       </c>
       <c r="E1778" s="2">
@@ -62238,12 +62238,12 @@
       </c>
       <c r="C1779" s="0" t="inlineStr">
         <is>
-          <t>wed_wed_congrats</t>
+          <t>wed_justmarried</t>
         </is>
       </c>
       <c r="D1779" s="0" t="inlineStr">
         <is>
-          <t>wed_wed_congrats</t>
+          <t>wed_justmarried</t>
         </is>
       </c>
       <c r="E1779" s="2">
@@ -62266,34 +62266,62 @@
       </c>
       <c r="C1780" s="0" t="inlineStr">
         <is>
+          <t>wed_wed_congrats</t>
+        </is>
+      </c>
+      <c r="D1780" s="0" t="inlineStr">
+        <is>
+          <t>wed_wed_congrats</t>
+        </is>
+      </c>
+      <c r="E1780" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1780" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1781">
+      <c r="A1781" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B1781" s="0" t="inlineStr">
+        <is>
+          <t>Events cards</t>
+        </is>
+      </c>
+      <c r="C1781" s="0" t="inlineStr">
+        <is>
           <t>wed_weddingetc</t>
         </is>
       </c>
-      <c r="D1780" s="0" t="inlineStr">
+      <c r="D1781" s="0" t="inlineStr">
         <is>
           <t>wed_weddingetc</t>
         </is>
       </c>
-      <c r="E1780" s="2">
-        <v>1</v>
-      </c>
-      <c r="F1780" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1781">
-      <c r="A1781" s="4" t="inlineStr">
+      <c r="E1781" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1781" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1782">
+      <c r="A1782" s="4" t="inlineStr">
         <is>
           <t>TOTAL 2026-08-21</t>
         </is>
       </c>
-      <c r="B1781" s="4"/>
-      <c r="C1781" s="4"/>
-      <c r="D1781" s="4"/>
-      <c r="E1781" s="5">
-        <v>735</v>
-      </c>
-      <c r="F1781" s="4"/>
+      <c r="B1782" s="4"/>
+      <c r="C1782" s="4"/>
+      <c r="D1782" s="4"/>
+      <c r="E1782" s="5">
+        <v>739</v>
+      </c>
+      <c r="F1782" s="4"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>